<commit_message>
Daily scrape: 2026-03-27 10:08 UTC
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -456,6 +456,18 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:08:17 NZT</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fri 27 Mar 2026 Last Update 16:40:00 AEDT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-03-31
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Futures Prices" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Futures Prices" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +40,12 @@
       <color rgb="00808080"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +55,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF3FB"/>
       </patternFill>
     </fill>
   </fills>
@@ -77,13 +94,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -450,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -488,6 +523,834 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Base Month – Mar 2026</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>152.6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Base Month – Apr 2026</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Base Month – May 2026</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>204.95</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Base Month – Jun 2026</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>211.6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Base Month – Jul 2026</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>226.8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Base Month – Aug 2026</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Base Month – Sep 2026</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>157.15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q1 2026</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>69.8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q2 2026</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>200.9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q3 2026</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>203.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q4 2026</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>106.85</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q1 2027</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q2 2027</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>202.75</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q3 2027</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q4 2027</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>87.75</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q1 2028</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q2 2028</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>193.6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q3 2028</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>189.85</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q4 2028</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>84.75</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q1 2029</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q2 2029</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q3 2029</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Otahuhu</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q4 2029</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>84.75</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Base Month – Mar 2026</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>141.4</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Base Month – Apr 2026</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>168.05</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Base Month – May 2026</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>186.55</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Base Month – Jun 2026</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>192.8</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Base Month – Jul 2026</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>213.95</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Base Month – Aug 2026</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>213.5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Base Month – Sep 2026</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q1 2026</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q2 2026</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>182.5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q3 2026</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q4 2026</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q1 2027</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>131.1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q2 2027</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="n">
+        <v>182.75</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q3 2027</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q4 2027</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="n">
+        <v>69.95</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q1 2028</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>108.65</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q2 2028</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>171.1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q3 2028</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q4 2028</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="n">
+        <v>67.55</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q1 2029</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="n">
+        <v>107.3</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q2 2029</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>170.75</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q3 2029</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="n">
+        <v>172.2</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Benmore</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Base Quarter – Q4 2029</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="n">
+        <v>68.05</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:D2"/>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-01
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -17,8 +17,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="166" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -128,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -151,7 +151,7 @@
     <xf numFmtId="4" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -160,7 +160,7 @@
     <xf numFmtId="4" fontId="2" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -168,6 +168,12 @@
     </xf>
     <xf numFmtId="4" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -534,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1629,7 +1635,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="n">
+      <c r="A48" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B48" s="9" t="inlineStr">
@@ -1652,7 +1658,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="11" t="n">
+      <c r="A49" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B49" s="12" t="inlineStr">
@@ -1675,7 +1681,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="n">
+      <c r="A50" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B50" s="9" t="inlineStr">
@@ -1698,7 +1704,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="11" t="n">
+      <c r="A51" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B51" s="12" t="inlineStr">
@@ -1721,7 +1727,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="n">
+      <c r="A52" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B52" s="9" t="inlineStr">
@@ -1744,7 +1750,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="11" t="n">
+      <c r="A53" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B53" s="12" t="inlineStr">
@@ -1767,7 +1773,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="8" t="n">
+      <c r="A54" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B54" s="9" t="inlineStr">
@@ -1790,7 +1796,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="11" t="n">
+      <c r="A55" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B55" s="12" t="inlineStr">
@@ -1813,7 +1819,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="n">
+      <c r="A56" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B56" s="9" t="inlineStr">
@@ -1836,7 +1842,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="11" t="n">
+      <c r="A57" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B57" s="12" t="inlineStr">
@@ -1859,7 +1865,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="8" t="n">
+      <c r="A58" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B58" s="9" t="inlineStr">
@@ -1882,7 +1888,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="n">
+      <c r="A59" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B59" s="12" t="inlineStr">
@@ -1905,7 +1911,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="n">
+      <c r="A60" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B60" s="9" t="inlineStr">
@@ -1928,7 +1934,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="11" t="n">
+      <c r="A61" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B61" s="12" t="inlineStr">
@@ -1951,7 +1957,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="8" t="n">
+      <c r="A62" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B62" s="9" t="inlineStr">
@@ -1974,7 +1980,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="11" t="n">
+      <c r="A63" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B63" s="12" t="inlineStr">
@@ -1997,7 +2003,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="n">
+      <c r="A64" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B64" s="9" t="inlineStr">
@@ -2020,7 +2026,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="11" t="n">
+      <c r="A65" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B65" s="12" t="inlineStr">
@@ -2043,7 +2049,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="8" t="n">
+      <c r="A66" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B66" s="9" t="inlineStr">
@@ -2066,7 +2072,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="11" t="n">
+      <c r="A67" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B67" s="12" t="inlineStr">
@@ -2089,7 +2095,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="8" t="n">
+      <c r="A68" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B68" s="9" t="inlineStr">
@@ -2112,7 +2118,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="11" t="n">
+      <c r="A69" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B69" s="12" t="inlineStr">
@@ -2135,7 +2141,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="8" t="n">
+      <c r="A70" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B70" s="9" t="inlineStr">
@@ -2158,7 +2164,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="11" t="n">
+      <c r="A71" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B71" s="12" t="inlineStr">
@@ -2181,7 +2187,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="8" t="n">
+      <c r="A72" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B72" s="9" t="inlineStr">
@@ -2204,7 +2210,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="11" t="n">
+      <c r="A73" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B73" s="12" t="inlineStr">
@@ -2227,7 +2233,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="8" t="n">
+      <c r="A74" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B74" s="9" t="inlineStr">
@@ -2250,7 +2256,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="11" t="n">
+      <c r="A75" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B75" s="12" t="inlineStr">
@@ -2273,7 +2279,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="8" t="n">
+      <c r="A76" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B76" s="9" t="inlineStr">
@@ -2296,7 +2302,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="11" t="n">
+      <c r="A77" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B77" s="12" t="inlineStr">
@@ -2319,7 +2325,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="8" t="n">
+      <c r="A78" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B78" s="9" t="inlineStr">
@@ -2342,7 +2348,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="11" t="n">
+      <c r="A79" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B79" s="12" t="inlineStr">
@@ -2365,7 +2371,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="n">
+      <c r="A80" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B80" s="9" t="inlineStr">
@@ -2388,7 +2394,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="11" t="n">
+      <c r="A81" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B81" s="12" t="inlineStr">
@@ -2411,7 +2417,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="8" t="n">
+      <c r="A82" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B82" s="9" t="inlineStr">
@@ -2434,7 +2440,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="11" t="n">
+      <c r="A83" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B83" s="12" t="inlineStr">
@@ -2457,7 +2463,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="8" t="n">
+      <c r="A84" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B84" s="9" t="inlineStr">
@@ -2480,7 +2486,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="11" t="n">
+      <c r="A85" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B85" s="12" t="inlineStr">
@@ -2503,7 +2509,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="8" t="n">
+      <c r="A86" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B86" s="9" t="inlineStr">
@@ -2526,7 +2532,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="11" t="n">
+      <c r="A87" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B87" s="12" t="inlineStr">
@@ -2549,7 +2555,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="8" t="n">
+      <c r="A88" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B88" s="9" t="inlineStr">
@@ -2572,7 +2578,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="11" t="n">
+      <c r="A89" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B89" s="12" t="inlineStr">
@@ -2595,7 +2601,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="8" t="n">
+      <c r="A90" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B90" s="9" t="inlineStr">
@@ -2618,7 +2624,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="11" t="n">
+      <c r="A91" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B91" s="12" t="inlineStr">
@@ -2641,7 +2647,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="8" t="n">
+      <c r="A92" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B92" s="9" t="inlineStr">
@@ -2664,7 +2670,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="11" t="n">
+      <c r="A93" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B93" s="12" t="inlineStr">
@@ -2687,7 +2693,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="8" t="n">
+      <c r="A94" s="14" t="n">
         <v>46113</v>
       </c>
       <c r="B94" s="9" t="inlineStr">
@@ -2710,7 +2716,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="11" t="n">
+      <c r="A95" s="15" t="n">
         <v>46113</v>
       </c>
       <c r="B95" s="12" t="inlineStr">
@@ -2729,6 +2735,1110 @@
         </is>
       </c>
       <c r="E95" s="13" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B96" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D96" s="9" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E96" s="10" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B97" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C97" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D97" s="12" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E97" s="13" t="n">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B98" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C98" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D98" s="9" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E98" s="10" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B99" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C99" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D99" s="12" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E99" s="13" t="n">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B100" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C100" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D100" s="9" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E100" s="10" t="n">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B101" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C101" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D101" s="12" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E101" s="13" t="n">
+        <v>151.15</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B102" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C102" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D102" s="9" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E102" s="10" t="n">
+        <v>102.25</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B103" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C103" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D103" s="12" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E103" s="13" t="n">
+        <v>102.25</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B104" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C104" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D104" s="9" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E104" s="10" t="n">
+        <v>102.25</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B105" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C105" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D105" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E105" s="13" t="n">
+        <v>185.4</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B106" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C106" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D106" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E106" s="10" t="n">
+        <v>194.2</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B107" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C107" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D107" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E107" s="13" t="n">
+        <v>102.25</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B108" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C108" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D108" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E108" s="10" t="n">
+        <v>151.95</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B109" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C109" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D109" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E109" s="13" t="n">
+        <v>197.6</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B110" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C110" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D110" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E110" s="10" t="n">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B111" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C111" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D111" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E111" s="13" t="n">
+        <v>84.5</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B112" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C112" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D112" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E112" s="10" t="n">
+        <v>126.45</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B113" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C113" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D113" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E113" s="13" t="n">
+        <v>192.55</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B114" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C114" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D114" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E114" s="10" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B115" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C115" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D115" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E115" s="13" t="n">
+        <v>84.84999999999999</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B116" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C116" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D116" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E116" s="10" t="n">
+        <v>124.5</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B117" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C117" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D117" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E117" s="13" t="n">
+        <v>185.25</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B118" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C118" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D118" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E118" s="10" t="n">
+        <v>187.75</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B119" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C119" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D119" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E119" s="13" t="n">
+        <v>83.25</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B120" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C120" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D120" s="9" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E120" s="10" t="n">
+        <v>156.15</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B121" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C121" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D121" s="12" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E121" s="13" t="n">
+        <v>182.5</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B122" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C122" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D122" s="9" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E122" s="10" t="n">
+        <v>186.1</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B123" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C123" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D123" s="12" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E123" s="13" t="n">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B124" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C124" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D124" s="9" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E124" s="10" t="n">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B125" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C125" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D125" s="12" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E125" s="13" t="n">
+        <v>141.15</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B126" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C126" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D126" s="9" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E126" s="10" t="n">
+        <v>86.25</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B127" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C127" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D127" s="12" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E127" s="13" t="n">
+        <v>86.25</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B128" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C128" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D128" s="9" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E128" s="10" t="n">
+        <v>86.25</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B129" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C129" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D129" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E129" s="13" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B130" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C130" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D130" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E130" s="10" t="n">
+        <v>182.85</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B131" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C131" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D131" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E131" s="13" t="n">
+        <v>86.25</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B132" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C132" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D132" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E132" s="10" t="n">
+        <v>129.15</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B133" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C133" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D133" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E133" s="13" t="n">
+        <v>178.6</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B134" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D134" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E134" s="10" t="n">
+        <v>178.6</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B135" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C135" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D135" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E135" s="13" t="n">
+        <v>67.95</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B136" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C136" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D136" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E136" s="10" t="n">
+        <v>106.35</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B137" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C137" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D137" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E137" s="13" t="n">
+        <v>171.55</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B138" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C138" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D138" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E138" s="10" t="n">
+        <v>170.35</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B139" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C139" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D139" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E139" s="13" t="n">
+        <v>66.5</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B140" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C140" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D140" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E140" s="10" t="n">
+        <v>108.1</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B141" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C141" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D141" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E141" s="13" t="n">
+        <v>166.75</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B142" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C142" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D142" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E142" s="10" t="n">
+        <v>165.25</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="15" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B143" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C143" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D143" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E143" s="13" t="n">
         <v>67</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-02
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -540,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E143"/>
+  <dimension ref="A1:E191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3842,6 +3842,1110 @@
         <v>67</v>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B144" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C144" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D144" s="9" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E144" s="10" t="n">
+        <v>156.6</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B145" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C145" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D145" s="12" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E145" s="13" t="n">
+        <v>179.45</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B146" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C146" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D146" s="9" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E146" s="10" t="n">
+        <v>186.7</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B147" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C147" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D147" s="12" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E147" s="13" t="n">
+        <v>203.65</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B148" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C148" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D148" s="9" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E148" s="10" t="n">
+        <v>203.75</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B149" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C149" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D149" s="12" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E149" s="13" t="n">
+        <v>147.5</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B150" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C150" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D150" s="9" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E150" s="10" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B151" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C151" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D151" s="12" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E151" s="13" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B152" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C152" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D152" s="9" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E152" s="10" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B153" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C153" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D153" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E153" s="13" t="n">
+        <v>174.3</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B154" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C154" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D154" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E154" s="10" t="n">
+        <v>185.4</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B155" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C155" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D155" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E155" s="13" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B156" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C156" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D156" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E156" s="10" t="n">
+        <v>151.95</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B157" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C157" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D157" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E157" s="13" t="n">
+        <v>196.7</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B158" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C158" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D158" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E158" s="10" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B159" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C159" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D159" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E159" s="13" t="n">
+        <v>82.75</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B160" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C160" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D160" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E160" s="10" t="n">
+        <v>126.45</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B161" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C161" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D161" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E161" s="13" t="n">
+        <v>188.2</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B162" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D162" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E162" s="10" t="n">
+        <v>188.75</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B163" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C163" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D163" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E163" s="13" t="n">
+        <v>81.59999999999999</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B164" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C164" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D164" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E164" s="10" t="n">
+        <v>127.15</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B165" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C165" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D165" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E165" s="13" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B166" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C166" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D166" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E166" s="10" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B167" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C167" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D167" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E167" s="13" t="n">
+        <v>82.25</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B168" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D168" s="9" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E168" s="10" t="n">
+        <v>146.9</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B169" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C169" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D169" s="12" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E169" s="13" t="n">
+        <v>166.95</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B170" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C170" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D170" s="9" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E170" s="10" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B171" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C171" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D171" s="12" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E171" s="13" t="n">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B172" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C172" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D172" s="9" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E172" s="10" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B173" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C173" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D173" s="12" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E173" s="13" t="n">
+        <v>137.5</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B174" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C174" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D174" s="9" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E174" s="10" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B175" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C175" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D175" s="12" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E175" s="13" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B176" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C176" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D176" s="9" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E176" s="10" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B177" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C177" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D177" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E177" s="13" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B178" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C178" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D178" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E178" s="10" t="n">
+        <v>172.2</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B179" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C179" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D179" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E179" s="13" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B180" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C180" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D180" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E180" s="10" t="n">
+        <v>127.9</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B181" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C181" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D181" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E181" s="13" t="n">
+        <v>177.5</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B182" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C182" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D182" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E182" s="10" t="n">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B183" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C183" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D183" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E183" s="13" t="n">
+        <v>65.3</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B184" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C184" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D184" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E184" s="10" t="n">
+        <v>106.35</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B185" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C185" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D185" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E185" s="13" t="n">
+        <v>166.9</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B186" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C186" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D186" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E186" s="10" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B187" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C187" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D187" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E187" s="13" t="n">
+        <v>65.05</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B188" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C188" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D188" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E188" s="10" t="n">
+        <v>106.35</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B189" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C189" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D189" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E189" s="13" t="n">
+        <v>164.25</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="14" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B190" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C190" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D190" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E190" s="10" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="15" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B191" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C191" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D191" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E191" s="13" t="n">
+        <v>65.09999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-03
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -540,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E191"/>
+  <dimension ref="A1:E239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4946,6 +4946,1110 @@
         <v>65.09999999999999</v>
       </c>
     </row>
+    <row r="192">
+      <c r="A192" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B192" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C192" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D192" s="9" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E192" s="10" t="n">
+        <v>156.6</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B193" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C193" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D193" s="12" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E193" s="13" t="n">
+        <v>179.45</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B194" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C194" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D194" s="9" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E194" s="10" t="n">
+        <v>186.7</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B195" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C195" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D195" s="12" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E195" s="13" t="n">
+        <v>203.65</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B196" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C196" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D196" s="9" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E196" s="10" t="n">
+        <v>203.75</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B197" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C197" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D197" s="12" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E197" s="13" t="n">
+        <v>147.5</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B198" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C198" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D198" s="9" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E198" s="10" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B199" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C199" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D199" s="12" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E199" s="13" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B200" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C200" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D200" s="9" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E200" s="10" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B201" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C201" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D201" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E201" s="13" t="n">
+        <v>174.3</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B202" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C202" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D202" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E202" s="10" t="n">
+        <v>185.4</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B203" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C203" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D203" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E203" s="13" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B204" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C204" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D204" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E204" s="10" t="n">
+        <v>151.95</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B205" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C205" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D205" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E205" s="13" t="n">
+        <v>196.7</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B206" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C206" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D206" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E206" s="10" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B207" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C207" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D207" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E207" s="13" t="n">
+        <v>82.75</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B208" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C208" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D208" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E208" s="10" t="n">
+        <v>126.45</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B209" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C209" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D209" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E209" s="13" t="n">
+        <v>188.2</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B210" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C210" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D210" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E210" s="10" t="n">
+        <v>188.75</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B211" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C211" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D211" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E211" s="13" t="n">
+        <v>81.59999999999999</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B212" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C212" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D212" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E212" s="10" t="n">
+        <v>127.15</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B213" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C213" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D213" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E213" s="13" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B214" s="9" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C214" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D214" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E214" s="10" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B215" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C215" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D215" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E215" s="13" t="n">
+        <v>82.25</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B216" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C216" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D216" s="9" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E216" s="10" t="n">
+        <v>146.9</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B217" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C217" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D217" s="12" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E217" s="13" t="n">
+        <v>166.95</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B218" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C218" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D218" s="9" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E218" s="10" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B219" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C219" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D219" s="12" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E219" s="13" t="n">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B220" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C220" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D220" s="9" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E220" s="10" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B221" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C221" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D221" s="12" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E221" s="13" t="n">
+        <v>137.5</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B222" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C222" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D222" s="9" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E222" s="10" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B223" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C223" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D223" s="12" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E223" s="13" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B224" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C224" s="9" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D224" s="9" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E224" s="10" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B225" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C225" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D225" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E225" s="13" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B226" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C226" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D226" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E226" s="10" t="n">
+        <v>172.2</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B227" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C227" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D227" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E227" s="13" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B228" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C228" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D228" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E228" s="10" t="n">
+        <v>127.9</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B229" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C229" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D229" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E229" s="13" t="n">
+        <v>177.5</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B230" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C230" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D230" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E230" s="10" t="n">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B231" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C231" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D231" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E231" s="13" t="n">
+        <v>65.3</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B232" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C232" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D232" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E232" s="10" t="n">
+        <v>106.35</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B233" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C233" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D233" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E233" s="13" t="n">
+        <v>166.9</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B234" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C234" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D234" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E234" s="10" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B235" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C235" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D235" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E235" s="13" t="n">
+        <v>65.05</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B236" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C236" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D236" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E236" s="10" t="n">
+        <v>106.35</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B237" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C237" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D237" s="12" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E237" s="13" t="n">
+        <v>164.25</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="14" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B238" s="9" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C238" s="9" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D238" s="9" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E238" s="10" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="15" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B239" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C239" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D239" s="12" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E239" s="13" t="n">
+        <v>65.09999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-05
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -17,8 +17,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="166" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -148,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -180,7 +180,7 @@
     <xf numFmtId="164" fontId="2" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -189,7 +189,7 @@
     <xf numFmtId="4" fontId="2" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -197,6 +197,12 @@
     </xf>
     <xf numFmtId="4" fontId="2" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -563,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E239"/>
+  <dimension ref="A1:E287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.98828125" customWidth="1" min="1" max="1"/>
@@ -4970,7 +4976,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="11" t="n">
+      <c r="A192" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B192" s="12" t="inlineStr">
@@ -4993,7 +4999,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="14" t="n">
+      <c r="A193" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B193" s="15" t="inlineStr">
@@ -5016,7 +5022,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="11" t="n">
+      <c r="A194" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B194" s="12" t="inlineStr">
@@ -5039,7 +5045,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="14" t="n">
+      <c r="A195" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B195" s="15" t="inlineStr">
@@ -5062,7 +5068,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="11" t="n">
+      <c r="A196" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B196" s="12" t="inlineStr">
@@ -5085,7 +5091,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="14" t="n">
+      <c r="A197" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B197" s="15" t="inlineStr">
@@ -5108,7 +5114,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="11" t="n">
+      <c r="A198" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B198" s="12" t="inlineStr">
@@ -5131,7 +5137,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="14" t="n">
+      <c r="A199" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B199" s="15" t="inlineStr">
@@ -5154,7 +5160,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="11" t="n">
+      <c r="A200" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B200" s="12" t="inlineStr">
@@ -5177,7 +5183,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="14" t="n">
+      <c r="A201" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B201" s="15" t="inlineStr">
@@ -5200,7 +5206,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="11" t="n">
+      <c r="A202" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B202" s="12" t="inlineStr">
@@ -5223,7 +5229,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="14" t="n">
+      <c r="A203" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B203" s="15" t="inlineStr">
@@ -5246,7 +5252,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="11" t="n">
+      <c r="A204" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B204" s="12" t="inlineStr">
@@ -5269,7 +5275,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="14" t="n">
+      <c r="A205" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B205" s="15" t="inlineStr">
@@ -5292,7 +5298,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="11" t="n">
+      <c r="A206" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B206" s="12" t="inlineStr">
@@ -5315,7 +5321,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="14" t="n">
+      <c r="A207" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B207" s="15" t="inlineStr">
@@ -5338,7 +5344,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="11" t="n">
+      <c r="A208" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B208" s="12" t="inlineStr">
@@ -5361,7 +5367,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="14" t="n">
+      <c r="A209" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B209" s="15" t="inlineStr">
@@ -5384,7 +5390,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="11" t="n">
+      <c r="A210" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B210" s="12" t="inlineStr">
@@ -5407,7 +5413,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="14" t="n">
+      <c r="A211" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B211" s="15" t="inlineStr">
@@ -5430,7 +5436,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="11" t="n">
+      <c r="A212" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B212" s="12" t="inlineStr">
@@ -5453,7 +5459,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="14" t="n">
+      <c r="A213" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B213" s="15" t="inlineStr">
@@ -5476,7 +5482,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="11" t="n">
+      <c r="A214" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B214" s="12" t="inlineStr">
@@ -5499,7 +5505,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="14" t="n">
+      <c r="A215" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B215" s="15" t="inlineStr">
@@ -5522,7 +5528,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="11" t="n">
+      <c r="A216" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B216" s="12" t="inlineStr">
@@ -5545,7 +5551,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="14" t="n">
+      <c r="A217" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B217" s="15" t="inlineStr">
@@ -5568,7 +5574,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="11" t="n">
+      <c r="A218" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B218" s="12" t="inlineStr">
@@ -5591,7 +5597,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="14" t="n">
+      <c r="A219" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B219" s="15" t="inlineStr">
@@ -5614,7 +5620,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="11" t="n">
+      <c r="A220" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B220" s="12" t="inlineStr">
@@ -5637,7 +5643,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="14" t="n">
+      <c r="A221" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B221" s="15" t="inlineStr">
@@ -5660,7 +5666,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="11" t="n">
+      <c r="A222" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B222" s="12" t="inlineStr">
@@ -5683,7 +5689,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="14" t="n">
+      <c r="A223" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B223" s="15" t="inlineStr">
@@ -5706,7 +5712,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="11" t="n">
+      <c r="A224" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B224" s="12" t="inlineStr">
@@ -5729,7 +5735,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="14" t="n">
+      <c r="A225" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B225" s="15" t="inlineStr">
@@ -5752,7 +5758,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="11" t="n">
+      <c r="A226" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B226" s="12" t="inlineStr">
@@ -5775,7 +5781,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="14" t="n">
+      <c r="A227" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B227" s="15" t="inlineStr">
@@ -5798,7 +5804,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="11" t="n">
+      <c r="A228" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B228" s="12" t="inlineStr">
@@ -5821,7 +5827,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="14" t="n">
+      <c r="A229" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B229" s="15" t="inlineStr">
@@ -5844,7 +5850,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="11" t="n">
+      <c r="A230" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B230" s="12" t="inlineStr">
@@ -5867,7 +5873,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="14" t="n">
+      <c r="A231" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B231" s="15" t="inlineStr">
@@ -5890,7 +5896,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="11" t="n">
+      <c r="A232" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B232" s="12" t="inlineStr">
@@ -5913,7 +5919,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="14" t="n">
+      <c r="A233" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B233" s="15" t="inlineStr">
@@ -5936,7 +5942,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="11" t="n">
+      <c r="A234" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B234" s="12" t="inlineStr">
@@ -5959,7 +5965,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="14" t="n">
+      <c r="A235" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B235" s="15" t="inlineStr">
@@ -5982,7 +5988,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="11" t="n">
+      <c r="A236" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B236" s="12" t="inlineStr">
@@ -6005,7 +6011,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="14" t="n">
+      <c r="A237" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B237" s="15" t="inlineStr">
@@ -6028,7 +6034,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="11" t="n">
+      <c r="A238" s="17" t="n">
         <v>46116</v>
       </c>
       <c r="B238" s="12" t="inlineStr">
@@ -6051,7 +6057,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="14" t="n">
+      <c r="A239" s="18" t="n">
         <v>46116</v>
       </c>
       <c r="B239" s="15" t="inlineStr">
@@ -6070,6 +6076,1110 @@
         </is>
       </c>
       <c r="E239" s="16" t="n">
+        <v>65.09999999999999</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B240" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C240" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D240" s="12" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E240" s="13" t="n">
+        <v>156.6</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B241" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C241" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D241" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E241" s="16" t="n">
+        <v>179.45</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B242" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C242" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D242" s="12" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E242" s="13" t="n">
+        <v>186.7</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B243" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C243" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D243" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E243" s="16" t="n">
+        <v>203.65</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B244" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C244" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D244" s="12" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E244" s="13" t="n">
+        <v>203.75</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B245" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C245" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D245" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E245" s="16" t="n">
+        <v>147.5</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B246" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C246" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D246" s="12" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E246" s="13" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B247" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C247" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D247" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E247" s="16" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B248" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C248" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D248" s="12" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E248" s="13" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B249" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C249" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D249" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E249" s="16" t="n">
+        <v>174.3</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B250" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C250" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D250" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E250" s="13" t="n">
+        <v>185.4</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B251" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C251" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D251" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E251" s="16" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B252" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C252" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D252" s="12" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E252" s="13" t="n">
+        <v>151.95</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B253" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C253" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D253" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E253" s="16" t="n">
+        <v>196.7</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B254" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C254" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D254" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E254" s="13" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B255" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C255" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D255" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E255" s="16" t="n">
+        <v>82.75</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B256" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C256" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D256" s="12" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E256" s="13" t="n">
+        <v>126.45</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B257" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C257" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D257" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E257" s="16" t="n">
+        <v>188.2</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B258" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C258" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D258" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E258" s="13" t="n">
+        <v>188.75</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B259" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C259" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D259" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E259" s="16" t="n">
+        <v>81.59999999999999</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B260" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C260" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D260" s="12" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E260" s="13" t="n">
+        <v>127.15</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B261" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C261" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D261" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E261" s="16" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B262" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C262" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D262" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E262" s="13" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B263" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C263" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D263" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E263" s="16" t="n">
+        <v>82.25</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B264" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C264" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D264" s="12" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E264" s="13" t="n">
+        <v>146.9</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B265" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C265" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D265" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E265" s="16" t="n">
+        <v>166.95</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B266" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C266" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D266" s="12" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E266" s="13" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B267" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C267" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D267" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E267" s="16" t="n">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B268" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C268" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D268" s="12" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E268" s="13" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B269" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C269" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D269" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E269" s="16" t="n">
+        <v>137.5</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B270" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C270" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D270" s="12" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E270" s="13" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B271" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C271" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D271" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E271" s="16" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B272" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C272" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D272" s="12" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E272" s="13" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B273" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C273" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D273" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E273" s="16" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B274" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C274" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D274" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E274" s="13" t="n">
+        <v>172.2</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B275" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C275" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D275" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E275" s="16" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B276" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C276" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D276" s="12" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E276" s="13" t="n">
+        <v>127.9</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B277" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C277" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D277" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E277" s="16" t="n">
+        <v>177.5</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B278" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C278" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D278" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E278" s="13" t="n">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B279" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C279" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D279" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E279" s="16" t="n">
+        <v>65.3</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B280" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C280" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D280" s="12" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E280" s="13" t="n">
+        <v>106.35</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B281" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C281" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D281" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E281" s="16" t="n">
+        <v>166.9</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B282" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C282" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D282" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E282" s="13" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B283" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C283" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D283" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E283" s="16" t="n">
+        <v>65.05</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B284" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C284" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D284" s="12" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E284" s="13" t="n">
+        <v>106.35</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B285" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C285" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D285" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E285" s="16" t="n">
+        <v>164.25</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="17" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B286" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C286" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D286" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E286" s="13" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="18" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B287" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C287" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D287" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E287" s="16" t="n">
         <v>65.09999999999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-06
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E287"/>
+  <dimension ref="A1:E335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.98828125" customWidth="1" min="1" max="1"/>
@@ -7183,6 +7183,1110 @@
         <v>65.09999999999999</v>
       </c>
     </row>
+    <row r="288">
+      <c r="A288" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B288" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C288" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D288" s="12" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E288" s="13" t="n">
+        <v>156.6</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B289" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C289" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D289" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E289" s="16" t="n">
+        <v>179.45</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B290" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C290" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D290" s="12" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E290" s="13" t="n">
+        <v>186.7</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B291" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C291" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D291" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E291" s="16" t="n">
+        <v>203.65</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B292" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C292" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D292" s="12" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E292" s="13" t="n">
+        <v>203.75</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B293" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C293" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D293" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E293" s="16" t="n">
+        <v>147.5</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B294" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C294" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D294" s="12" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E294" s="13" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B295" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C295" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D295" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E295" s="16" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B296" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C296" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D296" s="12" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E296" s="13" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B297" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C297" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D297" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E297" s="16" t="n">
+        <v>174.3</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B298" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C298" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D298" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E298" s="13" t="n">
+        <v>185.4</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B299" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C299" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D299" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E299" s="16" t="n">
+        <v>99.95</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B300" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C300" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D300" s="12" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E300" s="13" t="n">
+        <v>151.95</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B301" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C301" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D301" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E301" s="16" t="n">
+        <v>196.7</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B302" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C302" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D302" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E302" s="13" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B303" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C303" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D303" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E303" s="16" t="n">
+        <v>82.75</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B304" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C304" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D304" s="12" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E304" s="13" t="n">
+        <v>126.45</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B305" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C305" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D305" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E305" s="16" t="n">
+        <v>188.2</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B306" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C306" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D306" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E306" s="13" t="n">
+        <v>188.75</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B307" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C307" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D307" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E307" s="16" t="n">
+        <v>81.59999999999999</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B308" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C308" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D308" s="12" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E308" s="13" t="n">
+        <v>127.15</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B309" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C309" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D309" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E309" s="16" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B310" s="12" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C310" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D310" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E310" s="13" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B311" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C311" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D311" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E311" s="16" t="n">
+        <v>82.25</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B312" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C312" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D312" s="12" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E312" s="13" t="n">
+        <v>146.9</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B313" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C313" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D313" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E313" s="16" t="n">
+        <v>166.95</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B314" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C314" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D314" s="12" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E314" s="13" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B315" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C315" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D315" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E315" s="16" t="n">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B316" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C316" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D316" s="12" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E316" s="13" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B317" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C317" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D317" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E317" s="16" t="n">
+        <v>137.5</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B318" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C318" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D318" s="12" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E318" s="13" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B319" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C319" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D319" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E319" s="16" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B320" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C320" s="12" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D320" s="12" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E320" s="13" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B321" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C321" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D321" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E321" s="16" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B322" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C322" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D322" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E322" s="13" t="n">
+        <v>172.2</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B323" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C323" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D323" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E323" s="16" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B324" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C324" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D324" s="12" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E324" s="13" t="n">
+        <v>127.9</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B325" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C325" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D325" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E325" s="16" t="n">
+        <v>177.5</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B326" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C326" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D326" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E326" s="13" t="n">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B327" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C327" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D327" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E327" s="16" t="n">
+        <v>65.3</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B328" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C328" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D328" s="12" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E328" s="13" t="n">
+        <v>106.35</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B329" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C329" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D329" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E329" s="16" t="n">
+        <v>166.9</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B330" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C330" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D330" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E330" s="13" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B331" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C331" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D331" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E331" s="16" t="n">
+        <v>65.05</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B332" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C332" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D332" s="12" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E332" s="13" t="n">
+        <v>106.35</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B333" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C333" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D333" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E333" s="16" t="n">
+        <v>164.25</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="17" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B334" s="12" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C334" s="12" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D334" s="12" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E334" s="13" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="18" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B335" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C335" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D335" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E335" s="16" t="n">
+        <v>65.09999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-08
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -17,8 +17,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="166" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -153,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -194,7 +194,7 @@
     <xf numFmtId="4" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -203,7 +203,7 @@
     <xf numFmtId="4" fontId="2" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -211,6 +211,12 @@
     </xf>
     <xf numFmtId="4" fontId="2" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -577,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E337"/>
+  <dimension ref="A1:E385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7238,7 +7244,7 @@
       </c>
     </row>
     <row r="290">
-      <c r="A290" s="14" t="n">
+      <c r="A290" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B290" s="15" t="inlineStr">
@@ -7261,7 +7267,7 @@
       </c>
     </row>
     <row r="291">
-      <c r="A291" s="17" t="n">
+      <c r="A291" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B291" s="18" t="inlineStr">
@@ -7284,7 +7290,7 @@
       </c>
     </row>
     <row r="292">
-      <c r="A292" s="14" t="n">
+      <c r="A292" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B292" s="15" t="inlineStr">
@@ -7307,7 +7313,7 @@
       </c>
     </row>
     <row r="293">
-      <c r="A293" s="17" t="n">
+      <c r="A293" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B293" s="18" t="inlineStr">
@@ -7330,7 +7336,7 @@
       </c>
     </row>
     <row r="294">
-      <c r="A294" s="14" t="n">
+      <c r="A294" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B294" s="15" t="inlineStr">
@@ -7353,7 +7359,7 @@
       </c>
     </row>
     <row r="295">
-      <c r="A295" s="17" t="n">
+      <c r="A295" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B295" s="18" t="inlineStr">
@@ -7376,7 +7382,7 @@
       </c>
     </row>
     <row r="296">
-      <c r="A296" s="14" t="n">
+      <c r="A296" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B296" s="15" t="inlineStr">
@@ -7399,7 +7405,7 @@
       </c>
     </row>
     <row r="297">
-      <c r="A297" s="17" t="n">
+      <c r="A297" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B297" s="18" t="inlineStr">
@@ -7422,7 +7428,7 @@
       </c>
     </row>
     <row r="298">
-      <c r="A298" s="14" t="n">
+      <c r="A298" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B298" s="15" t="inlineStr">
@@ -7445,7 +7451,7 @@
       </c>
     </row>
     <row r="299">
-      <c r="A299" s="17" t="n">
+      <c r="A299" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B299" s="18" t="inlineStr">
@@ -7468,7 +7474,7 @@
       </c>
     </row>
     <row r="300">
-      <c r="A300" s="14" t="n">
+      <c r="A300" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B300" s="15" t="inlineStr">
@@ -7491,7 +7497,7 @@
       </c>
     </row>
     <row r="301">
-      <c r="A301" s="17" t="n">
+      <c r="A301" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B301" s="18" t="inlineStr">
@@ -7514,7 +7520,7 @@
       </c>
     </row>
     <row r="302">
-      <c r="A302" s="14" t="n">
+      <c r="A302" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B302" s="15" t="inlineStr">
@@ -7537,7 +7543,7 @@
       </c>
     </row>
     <row r="303">
-      <c r="A303" s="17" t="n">
+      <c r="A303" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B303" s="18" t="inlineStr">
@@ -7560,7 +7566,7 @@
       </c>
     </row>
     <row r="304">
-      <c r="A304" s="14" t="n">
+      <c r="A304" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B304" s="15" t="inlineStr">
@@ -7583,7 +7589,7 @@
       </c>
     </row>
     <row r="305">
-      <c r="A305" s="17" t="n">
+      <c r="A305" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B305" s="18" t="inlineStr">
@@ -7606,7 +7612,7 @@
       </c>
     </row>
     <row r="306">
-      <c r="A306" s="14" t="n">
+      <c r="A306" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B306" s="15" t="inlineStr">
@@ -7629,7 +7635,7 @@
       </c>
     </row>
     <row r="307">
-      <c r="A307" s="17" t="n">
+      <c r="A307" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B307" s="18" t="inlineStr">
@@ -7652,7 +7658,7 @@
       </c>
     </row>
     <row r="308">
-      <c r="A308" s="14" t="n">
+      <c r="A308" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B308" s="15" t="inlineStr">
@@ -7675,7 +7681,7 @@
       </c>
     </row>
     <row r="309">
-      <c r="A309" s="17" t="n">
+      <c r="A309" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B309" s="18" t="inlineStr">
@@ -7698,7 +7704,7 @@
       </c>
     </row>
     <row r="310">
-      <c r="A310" s="14" t="n">
+      <c r="A310" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B310" s="15" t="inlineStr">
@@ -7721,7 +7727,7 @@
       </c>
     </row>
     <row r="311">
-      <c r="A311" s="17" t="n">
+      <c r="A311" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B311" s="18" t="inlineStr">
@@ -7744,7 +7750,7 @@
       </c>
     </row>
     <row r="312">
-      <c r="A312" s="14" t="n">
+      <c r="A312" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B312" s="15" t="inlineStr">
@@ -7767,7 +7773,7 @@
       </c>
     </row>
     <row r="313">
-      <c r="A313" s="17" t="n">
+      <c r="A313" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B313" s="18" t="inlineStr">
@@ -7790,7 +7796,7 @@
       </c>
     </row>
     <row r="314">
-      <c r="A314" s="14" t="n">
+      <c r="A314" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B314" s="15" t="inlineStr">
@@ -7813,7 +7819,7 @@
       </c>
     </row>
     <row r="315">
-      <c r="A315" s="17" t="n">
+      <c r="A315" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B315" s="18" t="inlineStr">
@@ -7836,7 +7842,7 @@
       </c>
     </row>
     <row r="316">
-      <c r="A316" s="14" t="n">
+      <c r="A316" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B316" s="15" t="inlineStr">
@@ -7859,7 +7865,7 @@
       </c>
     </row>
     <row r="317">
-      <c r="A317" s="17" t="n">
+      <c r="A317" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B317" s="18" t="inlineStr">
@@ -7882,7 +7888,7 @@
       </c>
     </row>
     <row r="318">
-      <c r="A318" s="14" t="n">
+      <c r="A318" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B318" s="15" t="inlineStr">
@@ -7905,7 +7911,7 @@
       </c>
     </row>
     <row r="319">
-      <c r="A319" s="17" t="n">
+      <c r="A319" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B319" s="18" t="inlineStr">
@@ -7928,7 +7934,7 @@
       </c>
     </row>
     <row r="320">
-      <c r="A320" s="14" t="n">
+      <c r="A320" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B320" s="15" t="inlineStr">
@@ -7951,7 +7957,7 @@
       </c>
     </row>
     <row r="321">
-      <c r="A321" s="17" t="n">
+      <c r="A321" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B321" s="18" t="inlineStr">
@@ -7974,7 +7980,7 @@
       </c>
     </row>
     <row r="322">
-      <c r="A322" s="14" t="n">
+      <c r="A322" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B322" s="15" t="inlineStr">
@@ -7997,7 +8003,7 @@
       </c>
     </row>
     <row r="323">
-      <c r="A323" s="17" t="n">
+      <c r="A323" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B323" s="18" t="inlineStr">
@@ -8020,7 +8026,7 @@
       </c>
     </row>
     <row r="324">
-      <c r="A324" s="14" t="n">
+      <c r="A324" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B324" s="15" t="inlineStr">
@@ -8043,7 +8049,7 @@
       </c>
     </row>
     <row r="325">
-      <c r="A325" s="17" t="n">
+      <c r="A325" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B325" s="18" t="inlineStr">
@@ -8066,7 +8072,7 @@
       </c>
     </row>
     <row r="326">
-      <c r="A326" s="14" t="n">
+      <c r="A326" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B326" s="15" t="inlineStr">
@@ -8089,7 +8095,7 @@
       </c>
     </row>
     <row r="327">
-      <c r="A327" s="17" t="n">
+      <c r="A327" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B327" s="18" t="inlineStr">
@@ -8112,7 +8118,7 @@
       </c>
     </row>
     <row r="328">
-      <c r="A328" s="14" t="n">
+      <c r="A328" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B328" s="15" t="inlineStr">
@@ -8135,7 +8141,7 @@
       </c>
     </row>
     <row r="329">
-      <c r="A329" s="17" t="n">
+      <c r="A329" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B329" s="18" t="inlineStr">
@@ -8158,7 +8164,7 @@
       </c>
     </row>
     <row r="330">
-      <c r="A330" s="14" t="n">
+      <c r="A330" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B330" s="15" t="inlineStr">
@@ -8181,7 +8187,7 @@
       </c>
     </row>
     <row r="331">
-      <c r="A331" s="17" t="n">
+      <c r="A331" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B331" s="18" t="inlineStr">
@@ -8204,7 +8210,7 @@
       </c>
     </row>
     <row r="332">
-      <c r="A332" s="14" t="n">
+      <c r="A332" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B332" s="15" t="inlineStr">
@@ -8227,7 +8233,7 @@
       </c>
     </row>
     <row r="333">
-      <c r="A333" s="17" t="n">
+      <c r="A333" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B333" s="18" t="inlineStr">
@@ -8250,7 +8256,7 @@
       </c>
     </row>
     <row r="334">
-      <c r="A334" s="14" t="n">
+      <c r="A334" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B334" s="15" t="inlineStr">
@@ -8273,7 +8279,7 @@
       </c>
     </row>
     <row r="335">
-      <c r="A335" s="17" t="n">
+      <c r="A335" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B335" s="18" t="inlineStr">
@@ -8296,7 +8302,7 @@
       </c>
     </row>
     <row r="336">
-      <c r="A336" s="14" t="n">
+      <c r="A336" s="20" t="n">
         <v>46119</v>
       </c>
       <c r="B336" s="15" t="inlineStr">
@@ -8319,7 +8325,7 @@
       </c>
     </row>
     <row r="337">
-      <c r="A337" s="17" t="n">
+      <c r="A337" s="21" t="n">
         <v>46119</v>
       </c>
       <c r="B337" s="18" t="inlineStr">
@@ -8339,6 +8345,1110 @@
       </c>
       <c r="E337" s="19" t="n">
         <v>65.09999999999999</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B338" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C338" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D338" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E338" s="16" t="n">
+        <v>134.55</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B339" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C339" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D339" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E339" s="19" t="n">
+        <v>171.1</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B340" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C340" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D340" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E340" s="16" t="n">
+        <v>179.05</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B341" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C341" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D341" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E341" s="19" t="n">
+        <v>197.95</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B342" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C342" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D342" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E342" s="16" t="n">
+        <v>194.75</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B343" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C343" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D343" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E343" s="19" t="n">
+        <v>142.85</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B344" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C344" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D344" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E344" s="16" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B345" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C345" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D345" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E345" s="19" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B346" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C346" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D346" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E346" s="16" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B347" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C347" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D347" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E347" s="19" t="n">
+        <v>161.65</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B348" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C348" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D348" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E348" s="16" t="n">
+        <v>178.9</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B349" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C349" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D349" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E349" s="19" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B350" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C350" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D350" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E350" s="16" t="n">
+        <v>142.5</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B351" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C351" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D351" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E351" s="19" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B352" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C352" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D352" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E352" s="16" t="n">
+        <v>193.5</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B353" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C353" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D353" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E353" s="19" t="n">
+        <v>84.34999999999999</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B354" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C354" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D354" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E354" s="16" t="n">
+        <v>127.3</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B355" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C355" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D355" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E355" s="19" t="n">
+        <v>185.5</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B356" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C356" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D356" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E356" s="16" t="n">
+        <v>187.25</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B357" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C357" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D357" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E357" s="19" t="n">
+        <v>85.65000000000001</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B358" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C358" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D358" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E358" s="16" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B359" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C359" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D359" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E359" s="19" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B360" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C360" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D360" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E360" s="16" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B361" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C361" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D361" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E361" s="19" t="n">
+        <v>82.25</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B362" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C362" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D362" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E362" s="16" t="n">
+        <v>133.3</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B363" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C363" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D363" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E363" s="19" t="n">
+        <v>159.15</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B364" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C364" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D364" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E364" s="16" t="n">
+        <v>168.35</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B365" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C365" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D365" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E365" s="19" t="n">
+        <v>183.25</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B366" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C366" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D366" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E366" s="16" t="n">
+        <v>180.75</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B367" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C367" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D367" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E367" s="19" t="n">
+        <v>134.6</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B368" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C368" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D368" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E368" s="16" t="n">
+        <v>80.90000000000001</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B369" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C369" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D369" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E369" s="19" t="n">
+        <v>80.90000000000001</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B370" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C370" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D370" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E370" s="16" t="n">
+        <v>80.90000000000001</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B371" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C371" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D371" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E371" s="19" t="n">
+        <v>153.65</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B372" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C372" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D372" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E372" s="16" t="n">
+        <v>166.55</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B373" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C373" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D373" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E373" s="19" t="n">
+        <v>80.90000000000001</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B374" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C374" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D374" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E374" s="16" t="n">
+        <v>118.5</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B375" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C375" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D375" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E375" s="19" t="n">
+        <v>175.35</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B376" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C376" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D376" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E376" s="16" t="n">
+        <v>174.95</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B377" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C377" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D377" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E377" s="19" t="n">
+        <v>66.95</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B378" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C378" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D378" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E378" s="16" t="n">
+        <v>108.65</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B379" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C379" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D379" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E379" s="19" t="n">
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B380" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C380" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D380" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E380" s="16" t="n">
+        <v>165.75</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B381" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C381" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D381" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E381" s="19" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B382" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C382" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D382" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E382" s="16" t="n">
+        <v>108.95</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B383" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C383" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D383" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E383" s="19" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="20" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B384" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C384" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D384" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E384" s="16" t="n">
+        <v>163.15</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="21" t="n">
+        <v>46120</v>
+      </c>
+      <c r="B385" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C385" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D385" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E385" s="19" t="n">
+        <v>68.59999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-09
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E385"/>
+  <dimension ref="A1:E433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9451,6 +9451,1110 @@
         <v>68.59999999999999</v>
       </c>
     </row>
+    <row r="386">
+      <c r="A386" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B386" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C386" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D386" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E386" s="16" t="n">
+        <v>125.45</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B387" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C387" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D387" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E387" s="19" t="n">
+        <v>160.5</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B388" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C388" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D388" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E388" s="16" t="n">
+        <v>169.05</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B389" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C389" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D389" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E389" s="19" t="n">
+        <v>187.4</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B390" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C390" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D390" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E390" s="16" t="n">
+        <v>186.5</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B391" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C391" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D391" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E391" s="19" t="n">
+        <v>136.75</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B392" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C392" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D392" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E392" s="16" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B393" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C393" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D393" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E393" s="19" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B394" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C394" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D394" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E394" s="16" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B395" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C395" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D395" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E395" s="19" t="n">
+        <v>151.75</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B396" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C396" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D396" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E396" s="16" t="n">
+        <v>170.6</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B397" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C397" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D397" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E397" s="19" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B398" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C398" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D398" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E398" s="16" t="n">
+        <v>140.35</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B399" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C399" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D399" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E399" s="19" t="n">
+        <v>188.75</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B400" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C400" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D400" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E400" s="16" t="n">
+        <v>188.45</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B401" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C401" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D401" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E401" s="19" t="n">
+        <v>84.5</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B402" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C402" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D402" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E402" s="16" t="n">
+        <v>127.3</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B403" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C403" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D403" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E403" s="19" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B404" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C404" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D404" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E404" s="16" t="n">
+        <v>186.95</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B405" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C405" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D405" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E405" s="19" t="n">
+        <v>83.84999999999999</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B406" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C406" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D406" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E406" s="16" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B407" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C407" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D407" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E407" s="19" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B408" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C408" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D408" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E408" s="16" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B409" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C409" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D409" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E409" s="19" t="n">
+        <v>83.25</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B410" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C410" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D410" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E410" s="16" t="n">
+        <v>119.1</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B411" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C411" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D411" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E411" s="19" t="n">
+        <v>145.05</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B412" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C412" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D412" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E412" s="16" t="n">
+        <v>154.35</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B413" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C413" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D413" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E413" s="19" t="n">
+        <v>176.3</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B414" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C414" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D414" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E414" s="16" t="n">
+        <v>175.15</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B415" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C415" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D415" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E415" s="19" t="n">
+        <v>127.45</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B416" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C416" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D416" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E416" s="16" t="n">
+        <v>82.45</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B417" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C417" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D417" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E417" s="19" t="n">
+        <v>82.45</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B418" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C418" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D418" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E418" s="16" t="n">
+        <v>82.45</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B419" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C419" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D419" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E419" s="19" t="n">
+        <v>139.55</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B420" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C420" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D420" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E420" s="16" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B421" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C421" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D421" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E421" s="19" t="n">
+        <v>82.45</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B422" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C422" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D422" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E422" s="16" t="n">
+        <v>117.25</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B423" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C423" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D423" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E423" s="19" t="n">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B424" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C424" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D424" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E424" s="16" t="n">
+        <v>171.2</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B425" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C425" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D425" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E425" s="19" t="n">
+        <v>70.5</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B426" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C426" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D426" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E426" s="16" t="n">
+        <v>108.65</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B427" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C427" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D427" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E427" s="19" t="n">
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B428" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C428" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D428" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E428" s="16" t="n">
+        <v>165.75</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B429" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C429" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D429" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E429" s="19" t="n">
+        <v>69.3</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B430" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C430" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D430" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E430" s="16" t="n">
+        <v>108.95</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B431" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C431" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D431" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E431" s="19" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="20" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B432" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C432" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D432" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E432" s="16" t="n">
+        <v>163.15</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="21" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B433" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C433" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D433" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E433" s="19" t="n">
+        <v>69.15000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-10
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E433"/>
+  <dimension ref="A1:E481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10555,6 +10555,1110 @@
         <v>69.15000000000001</v>
       </c>
     </row>
+    <row r="434">
+      <c r="A434" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B434" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C434" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D434" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E434" s="16" t="n">
+        <v>106.85</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B435" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C435" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D435" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E435" s="19" t="n">
+        <v>142.4</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B436" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C436" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D436" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E436" s="16" t="n">
+        <v>175.3</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B437" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C437" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D437" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E437" s="19" t="n">
+        <v>188.6</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B438" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C438" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D438" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E438" s="16" t="n">
+        <v>186.5</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B439" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C439" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D439" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E439" s="19" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B440" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C440" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D440" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E440" s="16" t="n">
+        <v>97.05</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B441" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C441" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D441" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E441" s="19" t="n">
+        <v>97.05</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B442" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C442" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D442" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E442" s="16" t="n">
+        <v>97.05</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B443" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C443" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D443" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E443" s="19" t="n">
+        <v>141.5</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B444" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C444" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D444" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E444" s="16" t="n">
+        <v>168.8</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B445" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C445" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D445" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E445" s="19" t="n">
+        <v>97.05</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B446" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C446" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D446" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E446" s="16" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B447" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C447" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D447" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E447" s="19" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B448" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C448" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D448" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E448" s="16" t="n">
+        <v>187.65</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B449" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C449" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D449" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E449" s="19" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B450" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C450" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D450" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E450" s="16" t="n">
+        <v>129.75</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B451" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C451" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D451" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E451" s="19" t="n">
+        <v>183.5</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B452" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C452" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D452" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E452" s="16" t="n">
+        <v>186.95</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B453" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C453" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D453" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E453" s="19" t="n">
+        <v>85.40000000000001</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B454" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C454" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D454" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E454" s="16" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B455" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C455" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D455" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E455" s="19" t="n">
+        <v>182.05</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B456" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C456" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D456" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E456" s="16" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B457" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C457" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D457" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E457" s="19" t="n">
+        <v>85.5</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B458" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C458" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D458" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E458" s="16" t="n">
+        <v>99.84999999999999</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B459" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C459" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D459" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E459" s="19" t="n">
+        <v>139.25</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B460" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C460" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D460" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E460" s="16" t="n">
+        <v>156.9</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B461" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C461" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D461" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E461" s="19" t="n">
+        <v>181.7</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B462" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C462" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D462" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E462" s="16" t="n">
+        <v>181.2</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B463" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C463" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D463" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E463" s="19" t="n">
+        <v>121.75</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B464" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C464" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D464" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E464" s="16" t="n">
+        <v>82.2</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B465" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C465" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D465" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E465" s="19" t="n">
+        <v>82.2</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B466" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C466" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D466" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E466" s="16" t="n">
+        <v>82.2</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B467" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C467" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D467" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E467" s="19" t="n">
+        <v>132.05</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B468" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C468" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D468" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E468" s="16" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B469" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C469" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D469" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E469" s="19" t="n">
+        <v>82.2</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B470" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C470" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D470" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E470" s="16" t="n">
+        <v>121.5</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B471" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C471" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D471" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E471" s="19" t="n">
+        <v>171.5</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B472" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C472" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D472" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E472" s="16" t="n">
+        <v>169.95</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B473" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C473" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D473" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E473" s="19" t="n">
+        <v>71.55</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B474" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C474" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D474" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E474" s="16" t="n">
+        <v>111.75</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B475" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C475" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D475" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E475" s="19" t="n">
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B476" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C476" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D476" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E476" s="16" t="n">
+        <v>165.75</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B477" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C477" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D477" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E477" s="19" t="n">
+        <v>72.34999999999999</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B478" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C478" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D478" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E478" s="16" t="n">
+        <v>110.7</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B479" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C479" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D479" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E479" s="19" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="20" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B480" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C480" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D480" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E480" s="16" t="n">
+        <v>166.85</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="21" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B481" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C481" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D481" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E481" s="19" t="n">
+        <v>71.40000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-11
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E481"/>
+  <dimension ref="A1:E529"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11659,6 +11659,1110 @@
         <v>71.40000000000001</v>
       </c>
     </row>
+    <row r="482">
+      <c r="A482" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B482" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C482" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D482" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E482" s="16" t="n">
+        <v>106.85</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B483" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C483" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D483" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E483" s="19" t="n">
+        <v>142.4</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B484" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C484" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D484" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E484" s="16" t="n">
+        <v>175.3</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B485" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C485" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D485" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E485" s="19" t="n">
+        <v>188.6</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B486" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C486" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D486" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E486" s="16" t="n">
+        <v>186.5</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B487" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C487" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D487" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E487" s="19" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B488" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C488" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D488" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E488" s="16" t="n">
+        <v>97.05</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B489" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C489" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D489" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E489" s="19" t="n">
+        <v>97.05</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B490" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C490" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D490" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E490" s="16" t="n">
+        <v>97.05</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B491" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C491" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D491" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E491" s="19" t="n">
+        <v>141.5</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B492" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C492" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D492" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E492" s="16" t="n">
+        <v>168.8</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B493" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C493" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D493" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E493" s="19" t="n">
+        <v>97.05</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B494" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C494" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D494" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E494" s="16" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B495" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C495" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D495" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E495" s="19" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B496" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C496" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D496" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E496" s="16" t="n">
+        <v>187.65</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B497" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C497" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D497" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E497" s="19" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B498" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C498" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D498" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E498" s="16" t="n">
+        <v>129.75</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B499" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C499" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D499" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E499" s="19" t="n">
+        <v>183.5</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B500" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C500" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D500" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E500" s="16" t="n">
+        <v>186.95</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B501" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C501" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D501" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E501" s="19" t="n">
+        <v>85.40000000000001</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B502" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C502" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D502" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E502" s="16" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B503" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C503" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D503" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E503" s="19" t="n">
+        <v>182.05</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B504" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C504" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D504" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E504" s="16" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B505" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C505" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D505" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E505" s="19" t="n">
+        <v>85.5</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B506" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C506" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D506" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E506" s="16" t="n">
+        <v>99.84999999999999</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B507" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C507" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D507" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E507" s="19" t="n">
+        <v>139.25</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B508" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C508" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D508" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E508" s="16" t="n">
+        <v>156.9</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B509" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C509" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D509" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E509" s="19" t="n">
+        <v>181.7</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B510" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C510" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D510" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E510" s="16" t="n">
+        <v>181.2</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B511" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C511" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D511" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E511" s="19" t="n">
+        <v>121.75</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B512" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C512" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D512" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E512" s="16" t="n">
+        <v>82.2</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B513" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C513" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D513" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E513" s="19" t="n">
+        <v>82.2</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B514" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C514" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D514" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E514" s="16" t="n">
+        <v>82.2</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B515" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C515" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D515" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E515" s="19" t="n">
+        <v>132.05</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B516" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C516" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D516" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E516" s="16" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B517" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C517" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D517" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E517" s="19" t="n">
+        <v>82.2</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B518" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C518" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D518" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E518" s="16" t="n">
+        <v>121.5</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B519" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C519" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D519" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E519" s="19" t="n">
+        <v>171.5</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B520" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C520" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D520" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E520" s="16" t="n">
+        <v>169.95</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B521" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C521" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D521" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E521" s="19" t="n">
+        <v>71.55</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B522" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C522" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D522" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E522" s="16" t="n">
+        <v>111.75</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B523" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C523" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D523" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E523" s="19" t="n">
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B524" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C524" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D524" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E524" s="16" t="n">
+        <v>165.75</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B525" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C525" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D525" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E525" s="19" t="n">
+        <v>72.34999999999999</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B526" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C526" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D526" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E526" s="16" t="n">
+        <v>110.7</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B527" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C527" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D527" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E527" s="19" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="20" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B528" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C528" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D528" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E528" s="16" t="n">
+        <v>166.85</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="21" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B529" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C529" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D529" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E529" s="19" t="n">
+        <v>71.40000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-12
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E529"/>
+  <dimension ref="A1:E577"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12763,6 +12763,1110 @@
         <v>71.40000000000001</v>
       </c>
     </row>
+    <row r="530">
+      <c r="A530" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B530" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C530" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D530" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E530" s="16" t="n">
+        <v>106.85</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B531" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C531" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D531" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E531" s="19" t="n">
+        <v>142.4</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B532" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C532" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D532" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E532" s="16" t="n">
+        <v>175.3</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B533" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C533" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D533" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E533" s="19" t="n">
+        <v>188.6</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B534" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C534" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D534" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E534" s="16" t="n">
+        <v>186.5</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B535" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C535" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D535" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E535" s="19" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B536" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C536" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D536" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E536" s="16" t="n">
+        <v>97.05</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B537" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C537" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D537" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E537" s="19" t="n">
+        <v>97.05</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B538" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C538" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D538" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E538" s="16" t="n">
+        <v>97.05</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B539" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C539" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D539" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E539" s="19" t="n">
+        <v>141.5</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B540" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C540" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D540" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E540" s="16" t="n">
+        <v>168.8</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B541" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C541" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D541" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E541" s="19" t="n">
+        <v>97.05</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B542" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C542" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D542" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E542" s="16" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B543" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C543" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D543" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E543" s="19" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B544" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C544" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D544" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E544" s="16" t="n">
+        <v>187.65</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B545" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C545" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D545" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E545" s="19" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B546" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C546" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D546" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E546" s="16" t="n">
+        <v>129.75</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B547" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C547" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D547" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E547" s="19" t="n">
+        <v>183.5</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B548" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C548" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D548" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E548" s="16" t="n">
+        <v>186.95</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B549" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C549" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D549" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E549" s="19" t="n">
+        <v>85.40000000000001</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B550" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C550" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D550" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E550" s="16" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B551" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C551" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D551" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E551" s="19" t="n">
+        <v>182.05</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B552" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C552" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D552" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E552" s="16" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B553" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C553" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D553" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E553" s="19" t="n">
+        <v>85.5</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B554" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C554" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D554" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E554" s="16" t="n">
+        <v>99.84999999999999</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B555" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C555" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D555" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E555" s="19" t="n">
+        <v>139.25</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B556" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C556" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D556" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E556" s="16" t="n">
+        <v>156.9</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B557" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C557" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D557" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E557" s="19" t="n">
+        <v>181.7</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B558" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C558" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D558" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E558" s="16" t="n">
+        <v>181.2</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B559" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C559" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D559" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E559" s="19" t="n">
+        <v>121.75</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B560" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C560" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D560" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E560" s="16" t="n">
+        <v>82.2</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B561" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C561" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D561" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E561" s="19" t="n">
+        <v>82.2</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B562" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C562" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D562" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E562" s="16" t="n">
+        <v>82.2</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B563" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C563" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D563" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E563" s="19" t="n">
+        <v>132.05</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B564" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C564" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D564" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E564" s="16" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B565" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C565" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D565" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E565" s="19" t="n">
+        <v>82.2</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B566" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C566" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D566" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E566" s="16" t="n">
+        <v>121.5</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B567" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C567" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D567" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E567" s="19" t="n">
+        <v>171.5</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B568" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C568" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D568" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E568" s="16" t="n">
+        <v>169.95</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B569" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C569" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D569" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E569" s="19" t="n">
+        <v>71.55</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B570" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C570" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D570" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E570" s="16" t="n">
+        <v>111.75</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B571" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C571" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D571" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E571" s="19" t="n">
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B572" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C572" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D572" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E572" s="16" t="n">
+        <v>165.75</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B573" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C573" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D573" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E573" s="19" t="n">
+        <v>72.34999999999999</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B574" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C574" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D574" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E574" s="16" t="n">
+        <v>110.7</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B575" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C575" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D575" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E575" s="19" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="20" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B576" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C576" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D576" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E576" s="16" t="n">
+        <v>166.85</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="21" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B577" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C577" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D577" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E577" s="19" t="n">
+        <v>71.40000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-13
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E577"/>
+  <dimension ref="A1:E625"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13867,6 +13867,1110 @@
         <v>71.40000000000001</v>
       </c>
     </row>
+    <row r="578">
+      <c r="A578" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B578" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C578" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D578" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E578" s="16" t="n">
+        <v>103.35</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B579" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C579" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D579" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E579" s="19" t="n">
+        <v>142.4</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B580" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C580" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D580" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E580" s="16" t="n">
+        <v>177.25</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B581" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C581" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D581" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E581" s="19" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B582" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C582" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D582" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E582" s="16" t="n">
+        <v>188.4</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B583" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C583" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D583" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E583" s="19" t="n">
+        <v>132.8</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B584" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C584" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D584" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E584" s="16" t="n">
+        <v>95.15000000000001</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B585" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C585" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D585" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E585" s="19" t="n">
+        <v>95.15000000000001</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B586" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C586" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D586" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E586" s="16" t="n">
+        <v>95.15000000000001</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B587" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C587" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D587" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E587" s="19" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B588" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C588" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D588" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E588" s="16" t="n">
+        <v>171.15</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B589" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C589" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D589" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E589" s="19" t="n">
+        <v>95.15000000000001</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B590" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C590" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D590" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E590" s="16" t="n">
+        <v>143.15</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B591" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C591" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D591" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E591" s="19" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B592" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C592" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D592" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E592" s="16" t="n">
+        <v>187.75</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B593" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C593" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D593" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E593" s="19" t="n">
+        <v>89.5</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B594" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C594" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D594" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E594" s="16" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B595" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C595" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D595" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E595" s="19" t="n">
+        <v>183.55</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B596" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C596" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D596" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E596" s="16" t="n">
+        <v>186.95</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B597" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C597" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D597" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E597" s="19" t="n">
+        <v>89.5</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B598" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C598" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D598" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E598" s="16" t="n">
+        <v>132.45</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B599" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C599" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D599" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E599" s="19" t="n">
+        <v>182.05</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B600" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C600" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D600" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E600" s="16" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B601" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C601" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D601" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E601" s="19" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B602" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C602" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D602" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E602" s="16" t="n">
+        <v>97.90000000000001</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B603" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C603" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D603" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E603" s="19" t="n">
+        <v>134.85</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B604" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C604" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D604" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E604" s="16" t="n">
+        <v>161.05</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B605" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C605" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D605" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E605" s="19" t="n">
+        <v>182.55</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B606" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C606" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D606" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E606" s="16" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B607" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C607" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D607" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E607" s="19" t="n">
+        <v>125.15</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B608" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C608" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D608" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E608" s="16" t="n">
+        <v>80.55</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B609" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C609" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D609" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E609" s="19" t="n">
+        <v>80.55</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B610" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C610" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D610" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E610" s="16" t="n">
+        <v>80.55</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B611" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C611" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D611" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E611" s="19" t="n">
+        <v>131.3</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B612" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C612" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D612" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E612" s="16" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B613" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C613" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D613" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E613" s="19" t="n">
+        <v>80.55</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B614" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C614" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D614" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E614" s="16" t="n">
+        <v>122.05</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B615" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C615" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D615" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E615" s="19" t="n">
+        <v>171.2</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B616" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C616" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D616" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E616" s="16" t="n">
+        <v>170.45</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B617" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C617" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D617" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E617" s="19" t="n">
+        <v>72.59999999999999</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B618" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C618" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D618" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E618" s="16" t="n">
+        <v>112.3</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B619" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C619" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D619" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E619" s="19" t="n">
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B620" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C620" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D620" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E620" s="16" t="n">
+        <v>165.75</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B621" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C621" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D621" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E621" s="19" t="n">
+        <v>73.7</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B622" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C622" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D622" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E622" s="16" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B623" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C623" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D623" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E623" s="19" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="20" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B624" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C624" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D624" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E624" s="16" t="n">
+        <v>166.85</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="21" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B625" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C625" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D625" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E625" s="19" t="n">
+        <v>73.09999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-14
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E625"/>
+  <dimension ref="A1:E673"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14971,6 +14971,1110 @@
         <v>73.09999999999999</v>
       </c>
     </row>
+    <row r="626">
+      <c r="A626" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B626" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C626" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D626" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E626" s="16" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B627" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C627" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D627" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E627" s="19" t="n">
+        <v>137.05</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B628" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C628" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D628" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E628" s="16" t="n">
+        <v>171.9</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B629" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C629" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D629" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E629" s="19" t="n">
+        <v>190.9</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B630" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C630" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D630" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E630" s="16" t="n">
+        <v>189.6</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B631" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C631" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D631" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E631" s="19" t="n">
+        <v>131.05</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B632" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C632" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D632" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E632" s="16" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B633" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C633" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D633" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E633" s="19" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B634" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C634" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D634" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E634" s="16" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B635" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C635" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D635" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E635" s="19" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B636" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C636" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D636" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E636" s="16" t="n">
+        <v>170.95</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B637" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C637" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D637" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E637" s="19" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B638" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C638" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D638" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E638" s="16" t="n">
+        <v>139.85</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B639" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C639" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D639" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E639" s="19" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B640" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C640" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D640" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E640" s="16" t="n">
+        <v>187.75</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B641" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C641" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D641" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E641" s="19" t="n">
+        <v>88.5</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B642" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C642" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D642" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E642" s="16" t="n">
+        <v>129.15</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B643" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C643" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D643" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E643" s="19" t="n">
+        <v>183.6</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B644" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C644" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D644" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E644" s="16" t="n">
+        <v>186.95</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B645" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C645" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D645" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E645" s="19" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B646" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C646" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D646" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E646" s="16" t="n">
+        <v>129.15</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B647" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C647" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D647" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E647" s="19" t="n">
+        <v>182.05</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B648" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C648" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D648" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E648" s="16" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B649" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C649" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D649" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E649" s="19" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B650" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C650" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D650" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E650" s="16" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B651" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C651" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D651" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E651" s="19" t="n">
+        <v>131.45</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B652" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C652" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D652" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E652" s="16" t="n">
+        <v>164.55</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B653" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C653" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D653" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E653" s="19" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B654" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C654" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D654" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E654" s="16" t="n">
+        <v>179.55</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B655" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C655" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D655" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E655" s="19" t="n">
+        <v>121.95</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B656" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C656" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D656" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E656" s="16" t="n">
+        <v>77.7</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B657" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C657" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D657" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E657" s="19" t="n">
+        <v>77.7</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B658" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C658" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D658" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E658" s="16" t="n">
+        <v>77.7</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B659" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C659" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D659" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E659" s="19" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B660" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C660" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D660" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E660" s="16" t="n">
+        <v>160.25</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B661" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C661" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D661" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E661" s="19" t="n">
+        <v>77.7</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B662" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C662" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D662" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E662" s="16" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B663" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C663" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D663" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E663" s="19" t="n">
+        <v>170.95</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B664" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C664" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D664" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E664" s="16" t="n">
+        <v>170.45</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B665" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C665" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D665" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E665" s="19" t="n">
+        <v>72.5</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B666" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C666" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D666" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E666" s="16" t="n">
+        <v>112.3</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B667" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C667" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D667" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E667" s="19" t="n">
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B668" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C668" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D668" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E668" s="16" t="n">
+        <v>165.75</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B669" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C669" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D669" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E669" s="19" t="n">
+        <v>73.7</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B670" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C670" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D670" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E670" s="16" t="n">
+        <v>112.75</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B671" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C671" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D671" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E671" s="19" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="20" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B672" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C672" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D672" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E672" s="16" t="n">
+        <v>166.85</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="21" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B673" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C673" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D673" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E673" s="19" t="n">
+        <v>73.09999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-15
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E673"/>
+  <dimension ref="A1:E721"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16075,6 +16075,1110 @@
         <v>73.09999999999999</v>
       </c>
     </row>
+    <row r="674">
+      <c r="A674" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B674" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C674" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D674" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E674" s="16" t="n">
+        <v>88.8</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B675" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C675" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D675" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E675" s="19" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B676" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C676" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D676" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E676" s="16" t="n">
+        <v>158.95</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B677" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C677" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D677" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E677" s="19" t="n">
+        <v>189.35</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B678" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C678" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D678" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E678" s="16" t="n">
+        <v>187.05</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B679" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C679" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D679" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E679" s="19" t="n">
+        <v>127.1</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B680" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C680" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D680" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E680" s="16" t="n">
+        <v>89.84999999999999</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B681" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C681" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D681" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E681" s="19" t="n">
+        <v>89.84999999999999</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B682" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C682" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D682" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E682" s="16" t="n">
+        <v>89.84999999999999</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B683" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C683" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D683" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E683" s="19" t="n">
+        <v>125.6</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B684" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C684" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D684" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E684" s="16" t="n">
+        <v>168.3</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B685" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C685" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D685" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E685" s="19" t="n">
+        <v>89.84999999999999</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B686" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C686" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D686" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E686" s="16" t="n">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B687" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C687" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D687" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E687" s="19" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B688" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C688" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D688" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E688" s="16" t="n">
+        <v>187.75</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B689" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C689" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D689" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E689" s="19" t="n">
+        <v>88.5</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B690" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C690" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D690" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E690" s="16" t="n">
+        <v>129.15</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B691" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C691" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D691" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E691" s="19" t="n">
+        <v>183.6</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B692" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C692" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D692" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E692" s="16" t="n">
+        <v>186.95</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B693" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C693" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D693" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E693" s="19" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B694" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C694" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D694" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E694" s="16" t="n">
+        <v>129.15</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B695" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C695" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D695" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E695" s="19" t="n">
+        <v>182.25</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B696" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C696" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D696" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E696" s="16" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B697" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C697" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D697" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E697" s="19" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B698" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C698" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D698" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E698" s="16" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B699" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C699" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D699" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E699" s="19" t="n">
+        <v>125.2</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B700" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C700" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D700" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E700" s="16" t="n">
+        <v>145.75</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B701" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C701" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D701" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E701" s="19" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B702" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C702" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D702" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E702" s="16" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B703" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C703" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D703" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E703" s="19" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B704" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C704" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D704" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E704" s="16" t="n">
+        <v>72.55</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B705" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C705" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D705" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E705" s="19" t="n">
+        <v>72.55</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B706" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C706" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D706" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E706" s="16" t="n">
+        <v>72.55</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B707" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C707" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D707" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E707" s="19" t="n">
+        <v>119.35</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B708" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C708" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D708" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E708" s="16" t="n">
+        <v>158.45</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B709" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C709" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D709" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E709" s="19" t="n">
+        <v>72.55</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B710" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C710" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D710" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E710" s="16" t="n">
+        <v>117.5</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B711" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C711" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D711" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E711" s="19" t="n">
+        <v>172.05</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B712" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C712" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D712" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E712" s="16" t="n">
+        <v>170.45</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B713" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C713" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D713" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E713" s="19" t="n">
+        <v>70.34999999999999</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B714" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C714" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D714" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E714" s="16" t="n">
+        <v>112.3</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B715" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C715" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D715" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E715" s="19" t="n">
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B716" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C716" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D716" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E716" s="16" t="n">
+        <v>165.75</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B717" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C717" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D717" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E717" s="19" t="n">
+        <v>73.7</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B718" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C718" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D718" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E718" s="16" t="n">
+        <v>112.75</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B719" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C719" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D719" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E719" s="19" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="20" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B720" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C720" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D720" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E720" s="16" t="n">
+        <v>166.85</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="21" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B721" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C721" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D721" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E721" s="19" t="n">
+        <v>73.09999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-16
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E721"/>
+  <dimension ref="A1:E769"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17179,6 +17179,1110 @@
         <v>73.09999999999999</v>
       </c>
     </row>
+    <row r="722">
+      <c r="A722" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B722" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C722" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D722" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E722" s="16" t="n">
+        <v>83.65000000000001</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B723" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C723" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D723" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E723" s="19" t="n">
+        <v>115.15</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B724" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C724" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D724" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E724" s="16" t="n">
+        <v>150.8</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B725" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C725" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D725" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E725" s="19" t="n">
+        <v>186.4</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B726" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C726" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D726" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E726" s="16" t="n">
+        <v>184.8</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B727" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C727" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D727" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E727" s="19" t="n">
+        <v>128.75</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B728" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C728" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D728" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E728" s="16" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B729" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C729" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D729" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E729" s="19" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B730" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C730" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D730" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E730" s="16" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B731" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C731" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D731" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E731" s="19" t="n">
+        <v>116.5</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B732" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C732" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D732" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E732" s="16" t="n">
+        <v>167.1</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B733" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C733" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D733" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E733" s="19" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B734" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C734" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D734" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E734" s="16" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B735" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C735" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D735" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E735" s="19" t="n">
+        <v>189.1</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B736" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C736" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D736" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E736" s="16" t="n">
+        <v>190.1</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B737" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C737" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D737" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E737" s="19" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B738" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C738" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D738" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E738" s="16" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B739" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C739" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D739" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E739" s="19" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B740" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C740" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D740" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E740" s="16" t="n">
+        <v>186.95</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B741" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C741" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D741" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E741" s="19" t="n">
+        <v>90.65000000000001</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B742" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C742" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D742" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E742" s="16" t="n">
+        <v>130.85</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B743" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C743" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D743" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E743" s="19" t="n">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B744" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C744" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D744" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E744" s="16" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B745" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C745" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D745" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E745" s="19" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B746" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C746" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D746" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E746" s="16" t="n">
+        <v>82.7</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B747" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C747" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D747" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E747" s="19" t="n">
+        <v>119.4</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B748" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C748" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D748" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E748" s="16" t="n">
+        <v>141.7</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B749" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C749" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D749" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E749" s="19" t="n">
+        <v>177.1</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B750" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C750" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D750" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E750" s="16" t="n">
+        <v>177.9</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B751" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C751" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D751" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E751" s="19" t="n">
+        <v>120.55</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B752" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C752" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D752" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E752" s="16" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B753" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C753" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D753" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E753" s="19" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B754" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C754" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D754" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E754" s="16" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B755" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C755" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D755" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E755" s="19" t="n">
+        <v>114.65</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B756" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C756" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D756" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E756" s="16" t="n">
+        <v>158.95</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B757" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C757" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D757" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E757" s="19" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B758" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C758" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D758" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E758" s="16" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B759" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C759" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D759" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E759" s="19" t="n">
+        <v>172.05</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B760" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C760" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D760" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E760" s="16" t="n">
+        <v>170.45</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B761" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C761" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D761" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E761" s="19" t="n">
+        <v>71.05</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B762" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C762" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D762" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E762" s="16" t="n">
+        <v>114.9</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B763" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C763" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D763" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E763" s="19" t="n">
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B764" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C764" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D764" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E764" s="16" t="n">
+        <v>165.75</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B765" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C765" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D765" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E765" s="19" t="n">
+        <v>74.65000000000001</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B766" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C766" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D766" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E766" s="16" t="n">
+        <v>113.6</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B767" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C767" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D767" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E767" s="19" t="n">
+        <v>167.35</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="20" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B768" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C768" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D768" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E768" s="16" t="n">
+        <v>167.35</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="21" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B769" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C769" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D769" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E769" s="19" t="n">
+        <v>72.55</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-17
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E769"/>
+  <dimension ref="A1:E817"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18283,6 +18283,1110 @@
         <v>72.55</v>
       </c>
     </row>
+    <row r="770">
+      <c r="A770" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B770" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C770" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D770" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E770" s="16" t="n">
+        <v>93.15000000000001</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B771" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C771" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D771" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E771" s="19" t="n">
+        <v>120.85</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B772" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C772" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D772" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E772" s="16" t="n">
+        <v>159.95</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B773" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C773" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D773" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E773" s="19" t="n">
+        <v>195.65</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B774" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C774" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D774" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E774" s="16" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B775" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C775" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D775" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E775" s="19" t="n">
+        <v>133.45</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B776" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C776" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D776" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E776" s="16" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B777" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C777" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D777" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E777" s="19" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B778" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C778" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D778" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E778" s="16" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B779" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C779" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D779" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E779" s="19" t="n">
+        <v>124.6</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B780" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C780" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D780" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E780" s="16" t="n">
+        <v>175.5</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B781" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C781" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D781" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E781" s="19" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B782" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C782" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D782" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E782" s="16" t="n">
+        <v>140.6</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B783" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C783" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D783" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E783" s="19" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B784" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C784" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D784" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E784" s="16" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B785" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C785" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D785" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E785" s="19" t="n">
+        <v>88.2</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B786" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C786" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D786" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E786" s="16" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B787" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C787" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D787" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E787" s="19" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B788" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C788" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D788" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E788" s="16" t="n">
+        <v>191.05</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B789" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C789" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D789" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E789" s="19" t="n">
+        <v>89.75</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B790" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C790" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D790" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E790" s="16" t="n">
+        <v>130.85</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B791" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C791" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D791" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E791" s="19" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B792" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C792" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D792" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E792" s="16" t="n">
+        <v>189.6</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B793" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C793" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D793" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E793" s="19" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B794" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C794" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D794" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E794" s="16" t="n">
+        <v>92.90000000000001</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B795" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C795" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D795" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E795" s="19" t="n">
+        <v>120.45</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B796" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C796" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D796" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E796" s="16" t="n">
+        <v>150.8</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B797" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C797" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D797" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E797" s="19" t="n">
+        <v>183.05</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B798" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C798" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D798" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E798" s="16" t="n">
+        <v>189.3</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B799" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C799" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D799" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E799" s="19" t="n">
+        <v>125.8</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B800" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C800" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D800" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E800" s="16" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B801" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C801" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D801" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E801" s="19" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B802" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C802" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D802" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E802" s="16" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B803" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C803" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D803" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E803" s="19" t="n">
+        <v>121.35</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B804" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C804" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D804" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E804" s="16" t="n">
+        <v>166.5</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B805" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C805" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D805" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E805" s="19" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B806" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C806" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D806" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E806" s="16" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B807" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C807" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D807" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E807" s="19" t="n">
+        <v>174.5</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B808" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C808" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D808" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E808" s="16" t="n">
+        <v>174.5</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B809" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C809" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D809" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E809" s="19" t="n">
+        <v>71.05</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B810" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C810" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D810" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E810" s="16" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B811" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C811" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D811" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E811" s="19" t="n">
+        <v>171.5</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B812" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C812" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D812" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E812" s="16" t="n">
+        <v>170.5</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B813" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C813" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D813" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E813" s="19" t="n">
+        <v>74.65000000000001</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B814" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C814" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D814" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E814" s="16" t="n">
+        <v>113.6</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B815" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C815" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D815" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E815" s="19" t="n">
+        <v>170.25</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="20" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B816" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C816" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D816" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E816" s="16" t="n">
+        <v>170.25</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="21" t="n">
+        <v>46129</v>
+      </c>
+      <c r="B817" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C817" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D817" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E817" s="19" t="n">
+        <v>72.55</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-18
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E817"/>
+  <dimension ref="A1:E865"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19387,6 +19387,1110 @@
         <v>72.55</v>
       </c>
     </row>
+    <row r="818">
+      <c r="A818" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B818" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C818" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D818" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E818" s="16" t="n">
+        <v>93.15000000000001</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B819" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C819" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D819" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E819" s="19" t="n">
+        <v>120.85</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B820" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C820" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D820" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E820" s="16" t="n">
+        <v>159.95</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B821" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C821" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D821" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E821" s="19" t="n">
+        <v>195.65</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B822" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C822" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D822" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E822" s="16" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B823" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C823" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D823" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E823" s="19" t="n">
+        <v>133.45</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B824" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C824" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D824" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E824" s="16" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B825" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C825" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D825" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E825" s="19" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B826" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C826" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D826" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E826" s="16" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B827" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C827" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D827" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E827" s="19" t="n">
+        <v>124.6</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B828" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C828" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D828" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E828" s="16" t="n">
+        <v>175.5</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B829" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C829" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D829" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E829" s="19" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B830" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C830" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D830" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E830" s="16" t="n">
+        <v>140.6</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B831" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C831" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D831" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E831" s="19" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B832" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C832" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D832" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E832" s="16" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B833" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C833" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D833" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E833" s="19" t="n">
+        <v>88.2</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B834" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C834" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D834" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E834" s="16" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B835" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C835" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D835" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E835" s="19" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B836" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C836" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D836" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E836" s="16" t="n">
+        <v>191.05</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B837" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C837" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D837" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E837" s="19" t="n">
+        <v>89.75</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B838" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C838" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D838" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E838" s="16" t="n">
+        <v>130.85</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B839" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C839" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D839" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E839" s="19" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B840" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C840" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D840" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E840" s="16" t="n">
+        <v>189.6</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B841" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C841" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D841" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E841" s="19" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B842" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C842" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D842" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E842" s="16" t="n">
+        <v>92.90000000000001</v>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B843" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C843" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D843" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E843" s="19" t="n">
+        <v>120.45</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B844" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C844" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D844" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E844" s="16" t="n">
+        <v>150.8</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B845" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C845" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D845" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E845" s="19" t="n">
+        <v>183.05</v>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B846" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C846" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D846" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E846" s="16" t="n">
+        <v>189.3</v>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B847" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C847" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D847" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E847" s="19" t="n">
+        <v>125.8</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B848" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C848" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D848" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E848" s="16" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B849" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C849" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D849" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E849" s="19" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B850" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C850" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D850" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E850" s="16" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B851" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C851" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D851" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E851" s="19" t="n">
+        <v>121.35</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B852" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C852" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D852" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E852" s="16" t="n">
+        <v>166.5</v>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B853" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C853" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D853" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E853" s="19" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B854" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C854" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D854" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E854" s="16" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B855" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C855" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D855" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E855" s="19" t="n">
+        <v>174.5</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B856" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C856" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D856" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E856" s="16" t="n">
+        <v>174.5</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B857" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C857" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D857" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E857" s="19" t="n">
+        <v>71.05</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B858" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C858" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D858" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E858" s="16" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B859" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C859" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D859" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E859" s="19" t="n">
+        <v>171.5</v>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B860" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C860" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D860" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E860" s="16" t="n">
+        <v>170.5</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B861" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C861" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D861" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E861" s="19" t="n">
+        <v>74.65000000000001</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B862" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C862" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D862" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E862" s="16" t="n">
+        <v>113.6</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B863" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C863" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D863" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E863" s="19" t="n">
+        <v>170.25</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="20" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B864" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C864" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D864" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E864" s="16" t="n">
+        <v>170.25</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="21" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B865" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C865" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D865" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E865" s="19" t="n">
+        <v>72.55</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-19
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E865"/>
+  <dimension ref="A1:E913"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20491,6 +20491,1110 @@
         <v>72.55</v>
       </c>
     </row>
+    <row r="866">
+      <c r="A866" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B866" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C866" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D866" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E866" s="16" t="n">
+        <v>93.15000000000001</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B867" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C867" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D867" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E867" s="19" t="n">
+        <v>120.85</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B868" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C868" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D868" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E868" s="16" t="n">
+        <v>159.95</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B869" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C869" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D869" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E869" s="19" t="n">
+        <v>195.65</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B870" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C870" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D870" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E870" s="16" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B871" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C871" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D871" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E871" s="19" t="n">
+        <v>133.45</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B872" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C872" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D872" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E872" s="16" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B873" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C873" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D873" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E873" s="19" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B874" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C874" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D874" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E874" s="16" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B875" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C875" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D875" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E875" s="19" t="n">
+        <v>124.6</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B876" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C876" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D876" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E876" s="16" t="n">
+        <v>175.5</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B877" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C877" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D877" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E877" s="19" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B878" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C878" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D878" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E878" s="16" t="n">
+        <v>140.6</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B879" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C879" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D879" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E879" s="19" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B880" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C880" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D880" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E880" s="16" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B881" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C881" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D881" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E881" s="19" t="n">
+        <v>88.2</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B882" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C882" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D882" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E882" s="16" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B883" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C883" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D883" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E883" s="19" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B884" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C884" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D884" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E884" s="16" t="n">
+        <v>191.05</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B885" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C885" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D885" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E885" s="19" t="n">
+        <v>89.75</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B886" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C886" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D886" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E886" s="16" t="n">
+        <v>130.85</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B887" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C887" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D887" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E887" s="19" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B888" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C888" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D888" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E888" s="16" t="n">
+        <v>189.6</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B889" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C889" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D889" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E889" s="19" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B890" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C890" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D890" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E890" s="16" t="n">
+        <v>92.90000000000001</v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B891" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C891" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D891" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E891" s="19" t="n">
+        <v>120.45</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B892" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C892" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D892" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E892" s="16" t="n">
+        <v>150.8</v>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B893" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C893" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D893" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E893" s="19" t="n">
+        <v>183.05</v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B894" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C894" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D894" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E894" s="16" t="n">
+        <v>189.3</v>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B895" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C895" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D895" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E895" s="19" t="n">
+        <v>125.8</v>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B896" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C896" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D896" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E896" s="16" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B897" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C897" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D897" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E897" s="19" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B898" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C898" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D898" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E898" s="16" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B899" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C899" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D899" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E899" s="19" t="n">
+        <v>121.35</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B900" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C900" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D900" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E900" s="16" t="n">
+        <v>166.5</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B901" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C901" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D901" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E901" s="19" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B902" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C902" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D902" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E902" s="16" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B903" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C903" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D903" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E903" s="19" t="n">
+        <v>174.5</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B904" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C904" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D904" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E904" s="16" t="n">
+        <v>174.5</v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B905" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C905" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D905" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E905" s="19" t="n">
+        <v>71.05</v>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B906" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C906" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D906" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E906" s="16" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B907" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C907" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D907" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E907" s="19" t="n">
+        <v>171.5</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B908" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C908" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D908" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E908" s="16" t="n">
+        <v>170.5</v>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B909" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C909" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D909" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E909" s="19" t="n">
+        <v>74.65000000000001</v>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B910" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C910" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D910" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E910" s="16" t="n">
+        <v>113.6</v>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B911" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C911" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D911" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E911" s="19" t="n">
+        <v>170.25</v>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" s="20" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B912" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C912" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D912" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E912" s="16" t="n">
+        <v>170.25</v>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" s="21" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B913" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C913" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D913" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E913" s="19" t="n">
+        <v>72.55</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-20
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E913"/>
+  <dimension ref="A1:E961"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21595,6 +21595,1110 @@
         <v>72.55</v>
       </c>
     </row>
+    <row r="914">
+      <c r="A914" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B914" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C914" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D914" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E914" s="16" t="n">
+        <v>90.5</v>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B915" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C915" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D915" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E915" s="19" t="n">
+        <v>109.2</v>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B916" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C916" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D916" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E916" s="16" t="n">
+        <v>140.05</v>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B917" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C917" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D917" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E917" s="19" t="n">
+        <v>175.05</v>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B918" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C918" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D918" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E918" s="16" t="n">
+        <v>178.1</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B919" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C919" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D919" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E919" s="19" t="n">
+        <v>126.5</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B920" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C920" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D920" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E920" s="16" t="n">
+        <v>78.45</v>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B921" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C921" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D921" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E921" s="19" t="n">
+        <v>78.45</v>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B922" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C922" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D922" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E922" s="16" t="n">
+        <v>78.45</v>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B923" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C923" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D923" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E923" s="19" t="n">
+        <v>113.2</v>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B924" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C924" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D924" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E924" s="16" t="n">
+        <v>160.25</v>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B925" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C925" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D925" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E925" s="19" t="n">
+        <v>78.45</v>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B926" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C926" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D926" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E926" s="16" t="n">
+        <v>136.5</v>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B927" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C927" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D927" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E927" s="19" t="n">
+        <v>192.8</v>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B928" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C928" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D928" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E928" s="16" t="n">
+        <v>190.4</v>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B929" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C929" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D929" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E929" s="19" t="n">
+        <v>83.5</v>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B930" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C930" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D930" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E930" s="16" t="n">
+        <v>127.1</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B931" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C931" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D931" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E931" s="19" t="n">
+        <v>185.8</v>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B932" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C932" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D932" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E932" s="16" t="n">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B933" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C933" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D933" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E933" s="19" t="n">
+        <v>84.15000000000001</v>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B934" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C934" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D934" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E934" s="16" t="n">
+        <v>125.2</v>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B935" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C935" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D935" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E935" s="19" t="n">
+        <v>183.5</v>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B936" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C936" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D936" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E936" s="16" t="n">
+        <v>184.55</v>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B937" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C937" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D937" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E937" s="19" t="n">
+        <v>83.25</v>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B938" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C938" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D938" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E938" s="16" t="n">
+        <v>89.5</v>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B939" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C939" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D939" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E939" s="19" t="n">
+        <v>106.6</v>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B940" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C940" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D940" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E940" s="16" t="n">
+        <v>131.5</v>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B941" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C941" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D941" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E941" s="19" t="n">
+        <v>161.95</v>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B942" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C942" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D942" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E942" s="16" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B943" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C943" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D943" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E943" s="19" t="n">
+        <v>116.6</v>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B944" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C944" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D944" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E944" s="16" t="n">
+        <v>67.95</v>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B945" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C945" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D945" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E945" s="19" t="n">
+        <v>67.95</v>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B946" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C946" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D946" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E946" s="16" t="n">
+        <v>67.95</v>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B947" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C947" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D947" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E947" s="19" t="n">
+        <v>109.15</v>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B948" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C948" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D948" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E948" s="16" t="n">
+        <v>148.2</v>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B949" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C949" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D949" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E949" s="19" t="n">
+        <v>67.95</v>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B950" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C950" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D950" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E950" s="16" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B951" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C951" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D951" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E951" s="19" t="n">
+        <v>172.3</v>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B952" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C952" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D952" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E952" s="16" t="n">
+        <v>171.55</v>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B953" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C953" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D953" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E953" s="19" t="n">
+        <v>67.3</v>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B954" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C954" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D954" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E954" s="16" t="n">
+        <v>112.15</v>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B955" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C955" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D955" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E955" s="19" t="n">
+        <v>166.5</v>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B956" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C956" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D956" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E956" s="16" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B957" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C957" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D957" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E957" s="19" t="n">
+        <v>69.8</v>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B958" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C958" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D958" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E958" s="16" t="n">
+        <v>109.2</v>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B959" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C959" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D959" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E959" s="19" t="n">
+        <v>163.8</v>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" s="20" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B960" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C960" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D960" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E960" s="16" t="n">
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" s="21" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B961" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C961" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D961" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E961" s="19" t="n">
+        <v>69</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-21
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E961"/>
+  <dimension ref="A1:E1009"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22699,6 +22699,1110 @@
         <v>69</v>
       </c>
     </row>
+    <row r="962">
+      <c r="A962" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B962" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C962" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D962" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E962" s="16" t="n">
+        <v>91.34999999999999</v>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B963" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C963" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D963" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E963" s="19" t="n">
+        <v>104.85</v>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B964" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C964" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D964" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E964" s="16" t="n">
+        <v>131.1</v>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B965" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C965" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D965" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E965" s="19" t="n">
+        <v>168.2</v>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B966" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C966" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D966" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E966" s="16" t="n">
+        <v>175.2</v>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B967" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C967" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D967" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E967" s="19" t="n">
+        <v>128.15</v>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B968" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C968" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D968" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E968" s="16" t="n">
+        <v>82.34999999999999</v>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B969" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C969" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D969" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E969" s="19" t="n">
+        <v>82.34999999999999</v>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B970" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C970" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D970" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E970" s="16" t="n">
+        <v>82.34999999999999</v>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B971" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C971" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D971" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E971" s="19" t="n">
+        <v>109.05</v>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B972" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C972" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D972" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E972" s="16" t="n">
+        <v>157.5</v>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B973" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C973" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D973" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E973" s="19" t="n">
+        <v>82.34999999999999</v>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B974" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C974" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D974" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E974" s="16" t="n">
+        <v>139.45</v>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B975" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C975" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D975" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E975" s="19" t="n">
+        <v>192.8</v>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B976" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C976" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D976" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E976" s="16" t="n">
+        <v>190.4</v>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B977" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C977" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D977" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E977" s="19" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B978" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C978" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D978" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E978" s="16" t="n">
+        <v>127.1</v>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B979" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C979" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D979" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E979" s="19" t="n">
+        <v>185.1</v>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B980" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C980" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D980" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E980" s="16" t="n">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B981" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C981" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D981" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E981" s="19" t="n">
+        <v>84.15000000000001</v>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B982" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C982" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D982" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E982" s="16" t="n">
+        <v>126.45</v>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B983" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C983" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D983" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E983" s="19" t="n">
+        <v>181.15</v>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B984" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C984" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D984" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E984" s="16" t="n">
+        <v>182.4</v>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B985" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C985" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D985" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E985" s="19" t="n">
+        <v>83.25</v>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B986" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C986" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D986" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E986" s="16" t="n">
+        <v>89.95</v>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B987" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C987" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D987" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E987" s="19" t="n">
+        <v>101.4</v>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B988" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C988" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D988" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E988" s="16" t="n">
+        <v>123.5</v>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B989" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C989" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D989" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E989" s="19" t="n">
+        <v>155.55</v>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B990" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C990" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D990" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E990" s="16" t="n">
+        <v>167.15</v>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B991" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C991" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D991" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E991" s="19" t="n">
+        <v>120.4</v>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B992" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C992" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D992" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E992" s="16" t="n">
+        <v>70.25</v>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B993" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C993" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D993" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E993" s="19" t="n">
+        <v>70.25</v>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B994" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C994" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D994" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E994" s="16" t="n">
+        <v>70.25</v>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B995" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C995" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D995" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E995" s="19" t="n">
+        <v>104.9</v>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B996" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C996" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D996" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E996" s="16" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B997" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C997" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D997" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E997" s="19" t="n">
+        <v>70.25</v>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B998" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C998" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D998" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E998" s="16" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B999" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C999" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D999" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E999" s="19" t="n">
+        <v>172.3</v>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B1000" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1000" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1000" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1000" s="16" t="n">
+        <v>171.55</v>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B1001" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1001" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1001" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1001" s="19" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B1002" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1002" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1002" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1002" s="16" t="n">
+        <v>110.15</v>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B1003" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1003" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1003" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1003" s="19" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B1004" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1004" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1004" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1004" s="16" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B1005" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1005" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1005" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1005" s="19" t="n">
+        <v>69.8</v>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B1006" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1006" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1006" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1006" s="16" t="n">
+        <v>109.2</v>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B1007" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1007" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1007" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1007" s="19" t="n">
+        <v>162.5</v>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" s="20" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B1008" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1008" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1008" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1008" s="16" t="n">
+        <v>163.5</v>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="21" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B1009" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1009" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1009" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1009" s="19" t="n">
+        <v>68.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-22
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1009"/>
+  <dimension ref="A1:E1057"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23803,6 +23803,1110 @@
         <v>68.75</v>
       </c>
     </row>
+    <row r="1010">
+      <c r="A1010" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1010" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1010" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1010" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1010" s="16" t="n">
+        <v>95.59999999999999</v>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1011" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1011" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1011" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1011" s="19" t="n">
+        <v>117.15</v>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1012" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1012" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1012" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1012" s="16" t="n">
+        <v>141.15</v>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1013" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1013" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1013" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1013" s="19" t="n">
+        <v>181.35</v>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1014" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1014" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1014" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1014" s="16" t="n">
+        <v>189.7</v>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1015" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1015" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1015" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1015" s="19" t="n">
+        <v>137.9</v>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1016" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1016" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1016" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1016" s="16" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1017" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1017" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1017" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1017" s="19" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1018" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1018" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1018" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1018" s="16" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1019" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1019" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1019" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1019" s="19" t="n">
+        <v>117.95</v>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1020" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1020" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1020" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1020" s="16" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1021" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1021" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1021" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1021" s="19" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1022" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1022" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1022" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1022" s="16" t="n">
+        <v>147.25</v>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1023" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1023" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1023" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1023" s="19" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1024" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1024" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1024" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1024" s="16" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1025" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1025" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1025" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1025" s="19" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1026" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1026" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1026" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1026" s="16" t="n">
+        <v>130.8</v>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1027" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1027" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1027" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1027" s="19" t="n">
+        <v>185.1</v>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1028" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1028" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1028" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1028" s="16" t="n">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1029" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1029" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1029" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1029" s="19" t="n">
+        <v>84.15000000000001</v>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1030" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1030" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1030" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1030" s="16" t="n">
+        <v>129.75</v>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1031" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1031" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1031" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1031" s="19" t="n">
+        <v>183.45</v>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1032" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1032" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1032" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1032" s="16" t="n">
+        <v>182.4</v>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1033" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1033" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1033" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1033" s="19" t="n">
+        <v>83.25</v>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1034" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1034" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1034" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1034" s="16" t="n">
+        <v>95.3</v>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1035" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1035" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1035" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1035" s="19" t="n">
+        <v>114.3</v>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1036" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1036" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1036" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1036" s="16" t="n">
+        <v>135.25</v>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1037" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1037" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1037" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1037" s="19" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1038" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1038" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1038" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1038" s="16" t="n">
+        <v>182.85</v>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1039" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1039" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1039" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1039" s="19" t="n">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1040" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1040" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1040" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1040" s="16" t="n">
+        <v>75.5</v>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1041" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1041" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1041" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1041" s="19" t="n">
+        <v>75.5</v>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1042" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1042" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1042" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1042" s="16" t="n">
+        <v>75.5</v>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1043" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1043" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1043" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1043" s="19" t="n">
+        <v>114.95</v>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1044" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1044" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1044" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1044" s="16" t="n">
+        <v>162.95</v>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1045" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1045" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1045" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1045" s="19" t="n">
+        <v>75.5</v>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1046" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1046" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1046" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1046" s="16" t="n">
+        <v>126.5</v>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1047" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1047" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1047" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1047" s="19" t="n">
+        <v>175.8</v>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1048" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1048" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1048" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1048" s="16" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1049" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1049" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1049" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1049" s="19" t="n">
+        <v>69.5</v>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1050" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1050" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1050" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1050" s="16" t="n">
+        <v>113.3</v>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1051" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1051" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1051" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1051" s="19" t="n">
+        <v>168.9</v>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1052" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1052" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1052" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1052" s="16" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1053" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1053" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1053" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1053" s="19" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1054" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1054" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1054" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1054" s="16" t="n">
+        <v>112.25</v>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1055" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1055" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1055" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1055" s="19" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" s="20" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1056" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1056" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1056" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1056" s="16" t="n">
+        <v>163.5</v>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="21" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B1057" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1057" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1057" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1057" s="19" t="n">
+        <v>68.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-23
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1057"/>
+  <dimension ref="A1:E1105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24907,6 +24907,1110 @@
         <v>68.75</v>
       </c>
     </row>
+    <row r="1058">
+      <c r="A1058" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1058" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1058" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1058" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1058" s="16" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1059" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1059" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1059" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1059" s="19" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1060" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1060" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1060" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1060" s="16" t="n">
+        <v>139.95</v>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1061" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1061" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1061" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1061" s="19" t="n">
+        <v>176.95</v>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1062" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1062" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1062" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1062" s="16" t="n">
+        <v>183.9</v>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1063" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1063" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1063" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1063" s="19" t="n">
+        <v>142.95</v>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1064" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1064" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1064" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1064" s="16" t="n">
+        <v>87.3</v>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1065" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1065" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1065" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1065" s="19" t="n">
+        <v>87.3</v>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1066" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1066" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1066" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1066" s="16" t="n">
+        <v>87.3</v>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1067" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1067" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1067" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1067" s="19" t="n">
+        <v>119.95</v>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1068" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1068" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1068" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1068" s="16" t="n">
+        <v>168.2</v>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1069" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1069" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1069" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1069" s="19" t="n">
+        <v>87.3</v>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1070" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1070" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1070" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1070" s="16" t="n">
+        <v>140.6</v>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1071" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1071" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1071" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1071" s="19" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1072" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1072" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1072" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1072" s="16" t="n">
+        <v>190.5</v>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1073" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1073" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1073" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1073" s="19" t="n">
+        <v>80.7</v>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1074" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1074" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1074" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1074" s="16" t="n">
+        <v>126.3</v>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1075" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1075" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1075" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1075" s="19" t="n">
+        <v>184.25</v>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1076" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1076" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1076" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1076" s="16" t="n">
+        <v>186.7</v>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1077" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1077" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1077" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1077" s="19" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1078" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1078" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1078" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1078" s="16" t="n">
+        <v>125.5</v>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1079" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1079" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1079" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1079" s="19" t="n">
+        <v>183.45</v>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1080" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1080" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1080" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1080" s="16" t="n">
+        <v>182.4</v>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1081" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1081" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1081" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1081" s="19" t="n">
+        <v>81.59999999999999</v>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1082" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1082" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1082" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1082" s="16" t="n">
+        <v>99.45</v>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1083" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1083" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1083" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1083" s="19" t="n">
+        <v>110.95</v>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1084" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1084" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1084" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1084" s="16" t="n">
+        <v>130.25</v>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1085" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1085" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1085" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1085" s="19" t="n">
+        <v>168.35</v>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1086" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1086" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1086" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1086" s="16" t="n">
+        <v>178.25</v>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1087" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1087" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1087" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1087" s="19" t="n">
+        <v>132.5</v>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1088" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1088" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1088" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1088" s="16" t="n">
+        <v>75.25</v>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1089" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1089" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1089" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1089" s="19" t="n">
+        <v>75.25</v>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1090" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1090" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1090" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1090" s="16" t="n">
+        <v>75.25</v>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1091" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1091" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1091" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1091" s="19" t="n">
+        <v>113.5</v>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1092" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1092" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1092" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1092" s="16" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1093" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1093" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1093" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1093" s="19" t="n">
+        <v>75.25</v>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1094" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1094" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1094" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1094" s="16" t="n">
+        <v>120.75</v>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1095" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1095" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1095" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1095" s="19" t="n">
+        <v>172.05</v>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1096" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1096" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1096" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1096" s="16" t="n">
+        <v>173.55</v>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1097" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1097" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1097" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1097" s="19" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1098" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1098" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1098" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1098" s="16" t="n">
+        <v>110.75</v>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1099" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1099" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1099" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1099" s="19" t="n">
+        <v>165.95</v>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1100" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1100" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1100" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1100" s="16" t="n">
+        <v>167.2</v>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1101" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1101" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1101" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1101" s="19" t="n">
+        <v>67.09999999999999</v>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1102" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1102" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1102" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1102" s="16" t="n">
+        <v>108.75</v>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1103" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1103" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1103" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1103" s="19" t="n">
+        <v>164.3</v>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="20" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1104" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1104" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1104" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1104" s="16" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="21" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1105" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1105" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1105" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1105" s="19" t="n">
+        <v>67</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-24
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1105"/>
+  <dimension ref="A1:E1153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26011,6 +26011,1110 @@
         <v>67</v>
       </c>
     </row>
+    <row r="1106">
+      <c r="A1106" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1106" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1106" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1106" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1106" s="16" t="n">
+        <v>100.6</v>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1107" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1107" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1107" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1107" s="19" t="n">
+        <v>111.15</v>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1108" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1108" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1108" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1108" s="16" t="n">
+        <v>130.3</v>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1109" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1109" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1109" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1109" s="19" t="n">
+        <v>169.1</v>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1110" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1110" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1110" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1110" s="16" t="n">
+        <v>175.1</v>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1111" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1111" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1111" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1111" s="19" t="n">
+        <v>131.9</v>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1112" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1112" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1112" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1112" s="16" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1113" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1113" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1113" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1113" s="19" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1114" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1114" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1114" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1114" s="16" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1115" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1115" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1115" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1115" s="19" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1116" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1116" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1116" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1116" s="16" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1117" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1117" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1117" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1117" s="19" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1118" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1118" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1118" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1118" s="16" t="n">
+        <v>135.95</v>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1119" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1119" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1119" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1119" s="19" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1120" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1120" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1120" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1120" s="16" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1121" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1121" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1121" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1121" s="19" t="n">
+        <v>77.09999999999999</v>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1122" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1122" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1122" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1122" s="16" t="n">
+        <v>121.75</v>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1123" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1123" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1123" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1123" s="19" t="n">
+        <v>178.7</v>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1124" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1124" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1124" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1124" s="16" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1125" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1125" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1125" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1125" s="19" t="n">
+        <v>77.95</v>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1126" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1126" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1126" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1126" s="16" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1127" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1127" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1127" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1127" s="19" t="n">
+        <v>175.8</v>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1128" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1128" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1128" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1128" s="16" t="n">
+        <v>176.75</v>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1129" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1129" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1129" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1129" s="19" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1130" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1130" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1130" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1130" s="16" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1131" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1131" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1131" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1131" s="19" t="n">
+        <v>104.6</v>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1132" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1132" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1132" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1132" s="16" t="n">
+        <v>120.15</v>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1133" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1133" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1133" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1133" s="19" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1134" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1134" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1134" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1134" s="16" t="n">
+        <v>168.45</v>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1135" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1135" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1135" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1135" s="19" t="n">
+        <v>123.65</v>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1136" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1136" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1136" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1136" s="16" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1137" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1137" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1137" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1137" s="19" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1138" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1138" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1138" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1138" s="16" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1139" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1139" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1139" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1139" s="19" t="n">
+        <v>107.55</v>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1140" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1140" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1140" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1140" s="16" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1141" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1141" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1141" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1141" s="19" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1142" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1142" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1142" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1142" s="16" t="n">
+        <v>118.8</v>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1143" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1143" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1143" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1143" s="19" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1144" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1144" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1144" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1144" s="16" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1145" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1145" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1145" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1145" s="19" t="n">
+        <v>65.75</v>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1146" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1146" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1146" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1146" s="16" t="n">
+        <v>106.05</v>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1147" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1147" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1147" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1147" s="19" t="n">
+        <v>158.5</v>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1148" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1148" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1148" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1148" s="16" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1149" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1149" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1149" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1149" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1150" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1150" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1150" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1150" s="16" t="n">
+        <v>105.75</v>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1151" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1151" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1151" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1151" s="19" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" s="20" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1152" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1152" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1152" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1152" s="16" t="n">
+        <v>158.75</v>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" s="21" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B1153" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1153" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1153" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1153" s="19" t="n">
+        <v>63</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-25
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1153"/>
+  <dimension ref="A1:E1201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27115,6 +27115,1110 @@
         <v>63</v>
       </c>
     </row>
+    <row r="1154">
+      <c r="A1154" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1154" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1154" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1154" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1154" s="16" t="n">
+        <v>100.6</v>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1155" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1155" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1155" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1155" s="19" t="n">
+        <v>111.15</v>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1156" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1156" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1156" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1156" s="16" t="n">
+        <v>130.3</v>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1157" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1157" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1157" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1157" s="19" t="n">
+        <v>169.1</v>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1158" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1158" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1158" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1158" s="16" t="n">
+        <v>175.1</v>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1159" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1159" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1159" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1159" s="19" t="n">
+        <v>131.9</v>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1160" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1160" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1160" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1160" s="16" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1161" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1161" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1161" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1161" s="19" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1162" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1162" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1162" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1162" s="16" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1163" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1163" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1163" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1163" s="19" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1164" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1164" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1164" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1164" s="16" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1165" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1165" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1165" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1165" s="19" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1166" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1166" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1166" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1166" s="16" t="n">
+        <v>135.95</v>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1167" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1167" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1167" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1167" s="19" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1168" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1168" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1168" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1168" s="16" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1169" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1169" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1169" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1169" s="19" t="n">
+        <v>77.09999999999999</v>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1170" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1170" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1170" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1170" s="16" t="n">
+        <v>121.75</v>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1171" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1171" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1171" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1171" s="19" t="n">
+        <v>178.7</v>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1172" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1172" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1172" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1172" s="16" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1173" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1173" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1173" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1173" s="19" t="n">
+        <v>77.95</v>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1174" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1174" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1174" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1174" s="16" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1175" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1175" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1175" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1175" s="19" t="n">
+        <v>175.8</v>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1176" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1176" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1176" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1176" s="16" t="n">
+        <v>176.75</v>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1177" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1177" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1177" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1177" s="19" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1178" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1178" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1178" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1178" s="16" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1179" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1179" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1179" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1179" s="19" t="n">
+        <v>104.6</v>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1180" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1180" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1180" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1180" s="16" t="n">
+        <v>120.15</v>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1181" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1181" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1181" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1181" s="19" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1182" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1182" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1182" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1182" s="16" t="n">
+        <v>168.45</v>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1183" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1183" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1183" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1183" s="19" t="n">
+        <v>123.65</v>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1184" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1184" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1184" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1184" s="16" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1185" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1185" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1185" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1185" s="19" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1186" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1186" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1186" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1186" s="16" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1187" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1187" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1187" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1187" s="19" t="n">
+        <v>107.55</v>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1188" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1188" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1188" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1188" s="16" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1189" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1189" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1189" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1189" s="19" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1190" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1190" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1190" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1190" s="16" t="n">
+        <v>118.8</v>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1191" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1191" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1191" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1191" s="19" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1192" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1192" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1192" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1192" s="16" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1193" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1193" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1193" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1193" s="19" t="n">
+        <v>65.75</v>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1194" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1194" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1194" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1194" s="16" t="n">
+        <v>106.05</v>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1195" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1195" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1195" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1195" s="19" t="n">
+        <v>158.5</v>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1196" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1196" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1196" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1196" s="16" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1197" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1197" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1197" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1197" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1198" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1198" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1198" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1198" s="16" t="n">
+        <v>105.75</v>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1199" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1199" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1199" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1199" s="19" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" s="20" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1200" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1200" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1200" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1200" s="16" t="n">
+        <v>158.75</v>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" s="21" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1201" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1201" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1201" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1201" s="19" t="n">
+        <v>63</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-26
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1201"/>
+  <dimension ref="A1:E1249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28219,6 +28219,1110 @@
         <v>63</v>
       </c>
     </row>
+    <row r="1202">
+      <c r="A1202" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1202" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1202" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1202" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1202" s="16" t="n">
+        <v>100.6</v>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1203" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1203" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1203" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1203" s="19" t="n">
+        <v>111.15</v>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1204" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1204" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1204" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1204" s="16" t="n">
+        <v>130.3</v>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1205" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1205" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1205" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1205" s="19" t="n">
+        <v>169.1</v>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1206" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1206" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1206" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1206" s="16" t="n">
+        <v>175.1</v>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1207" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1207" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1207" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1207" s="19" t="n">
+        <v>131.9</v>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1208" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1208" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1208" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1208" s="16" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1209" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1209" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1209" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1209" s="19" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1210" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1210" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1210" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1210" s="16" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1211" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1211" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1211" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1211" s="19" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1212" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1212" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1212" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1212" s="16" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1213" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1213" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1213" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1213" s="19" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1214" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1214" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1214" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1214" s="16" t="n">
+        <v>135.95</v>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1215" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1215" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1215" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1215" s="19" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1216" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1216" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1216" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1216" s="16" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1217" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1217" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1217" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1217" s="19" t="n">
+        <v>77.09999999999999</v>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1218" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1218" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1218" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1218" s="16" t="n">
+        <v>121.75</v>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1219" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1219" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1219" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1219" s="19" t="n">
+        <v>178.7</v>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1220" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1220" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1220" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1220" s="16" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1221" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1221" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1221" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1221" s="19" t="n">
+        <v>77.95</v>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1222" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1222" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1222" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1222" s="16" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1223" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1223" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1223" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1223" s="19" t="n">
+        <v>175.8</v>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1224" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1224" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1224" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1224" s="16" t="n">
+        <v>176.75</v>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1225" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1225" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1225" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1225" s="19" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1226" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1226" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1226" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1226" s="16" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1227" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1227" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1227" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1227" s="19" t="n">
+        <v>104.6</v>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1228" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1228" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1228" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1228" s="16" t="n">
+        <v>120.15</v>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1229" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1229" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1229" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1229" s="19" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1230" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1230" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1230" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1230" s="16" t="n">
+        <v>168.45</v>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1231" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1231" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1231" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1231" s="19" t="n">
+        <v>123.65</v>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1232" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1232" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1232" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1232" s="16" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1233" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1233" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1233" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1233" s="19" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1234" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1234" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1234" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1234" s="16" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1235" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1235" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1235" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1235" s="19" t="n">
+        <v>107.55</v>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1236" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1236" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1236" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1236" s="16" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1237" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1237" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1237" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1237" s="19" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1238" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1238" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1238" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1238" s="16" t="n">
+        <v>118.8</v>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1239" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1239" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1239" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1239" s="19" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1240" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1240" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1240" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1240" s="16" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1241" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1241" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1241" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1241" s="19" t="n">
+        <v>65.75</v>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1242" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1242" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1242" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1242" s="16" t="n">
+        <v>106.05</v>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1243" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1243" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1243" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1243" s="19" t="n">
+        <v>158.5</v>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1244" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1244" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1244" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1244" s="16" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1245" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1245" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1245" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1245" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1246" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1246" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1246" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1246" s="16" t="n">
+        <v>105.75</v>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1247" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1247" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1247" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1247" s="19" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" s="20" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1248" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1248" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1248" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1248" s="16" t="n">
+        <v>158.75</v>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" s="21" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B1249" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1249" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1249" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1249" s="19" t="n">
+        <v>63</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-27
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1249"/>
+  <dimension ref="A1:E1297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29323,6 +29323,1110 @@
         <v>63</v>
       </c>
     </row>
+    <row r="1250">
+      <c r="A1250" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1250" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1250" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1250" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1250" s="16" t="n">
+        <v>100.6</v>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1251" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1251" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1251" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1251" s="19" t="n">
+        <v>111.15</v>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1252" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1252" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1252" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1252" s="16" t="n">
+        <v>130.3</v>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1253" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1253" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1253" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1253" s="19" t="n">
+        <v>169.1</v>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1254" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1254" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1254" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1254" s="16" t="n">
+        <v>175.1</v>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1255" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1255" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1255" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1255" s="19" t="n">
+        <v>131.9</v>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1256" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1256" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1256" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1256" s="16" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1257" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1257" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1257" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1257" s="19" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1258" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1258" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1258" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1258" s="16" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1259" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1259" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1259" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1259" s="19" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1260" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1260" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1260" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1260" s="16" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1261" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1261" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1261" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1261" s="19" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1262" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1262" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1262" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1262" s="16" t="n">
+        <v>135.95</v>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1263" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1263" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1263" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1263" s="19" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1264" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1264" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1264" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1264" s="16" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1265" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1265" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1265" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1265" s="19" t="n">
+        <v>77.09999999999999</v>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1266" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1266" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1266" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1266" s="16" t="n">
+        <v>121.75</v>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1267" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1267" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1267" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1267" s="19" t="n">
+        <v>178.7</v>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1268" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1268" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1268" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1268" s="16" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1269" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1269" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1269" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1269" s="19" t="n">
+        <v>77.95</v>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1270" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1270" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1270" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1270" s="16" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1271" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1271" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1271" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1271" s="19" t="n">
+        <v>175.8</v>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1272" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1272" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1272" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1272" s="16" t="n">
+        <v>176.75</v>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1273" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1273" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1273" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1273" s="19" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1274" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1274" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1274" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1274" s="16" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1275" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1275" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1275" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1275" s="19" t="n">
+        <v>104.6</v>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1276" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1276" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1276" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1276" s="16" t="n">
+        <v>120.15</v>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1277" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1277" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1277" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1277" s="19" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1278" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1278" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1278" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1278" s="16" t="n">
+        <v>168.45</v>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1279" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1279" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1279" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1279" s="19" t="n">
+        <v>123.65</v>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1280" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1280" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1280" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1280" s="16" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1281" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1281" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1281" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1281" s="19" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1282" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1282" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1282" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1282" s="16" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1283" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1283" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1283" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1283" s="19" t="n">
+        <v>107.55</v>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1284" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1284" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1284" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1284" s="16" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1285" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1285" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1285" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1285" s="19" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1286" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1286" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1286" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1286" s="16" t="n">
+        <v>118.8</v>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1287" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1287" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1287" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1287" s="19" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1288" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1288" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1288" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1288" s="16" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1289" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1289" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1289" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1289" s="19" t="n">
+        <v>65.75</v>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1290" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1290" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1290" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1290" s="16" t="n">
+        <v>106.05</v>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1291" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1291" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1291" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1291" s="19" t="n">
+        <v>158.5</v>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1292" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1292" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1292" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1292" s="16" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1293" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1293" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1293" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1293" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1294" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1294" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1294" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1294" s="16" t="n">
+        <v>105.75</v>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1295" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1295" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1295" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1295" s="19" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" s="20" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1296" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1296" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1296" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1296" s="16" t="n">
+        <v>158.75</v>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" s="21" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B1297" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1297" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1297" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1297" s="19" t="n">
+        <v>63</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-28
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1297"/>
+  <dimension ref="A1:E1345"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30427,6 +30427,1110 @@
         <v>63</v>
       </c>
     </row>
+    <row r="1298">
+      <c r="A1298" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1298" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1298" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1298" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1298" s="16" t="n">
+        <v>102.05</v>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1299" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1299" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1299" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1299" s="19" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1300" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1300" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1300" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1300" s="16" t="n">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1301" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1301" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1301" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1301" s="19" t="n">
+        <v>165.7</v>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1302" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1302" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1302" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1302" s="16" t="n">
+        <v>168.5</v>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1303" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1303" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1303" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1303" s="19" t="n">
+        <v>130.75</v>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1304" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1304" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1304" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1304" s="16" t="n">
+        <v>85.2</v>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1305" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1305" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1305" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1305" s="19" t="n">
+        <v>85.2</v>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1306" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1306" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1306" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1306" s="16" t="n">
+        <v>85.2</v>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1307" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1307" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1307" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1307" s="19" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1308" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1308" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1308" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1308" s="16" t="n">
+        <v>155.25</v>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1309" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1309" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1309" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1309" s="19" t="n">
+        <v>85.2</v>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1310" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1310" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1310" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1310" s="16" t="n">
+        <v>136.25</v>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1311" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1311" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1311" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1311" s="19" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1312" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1312" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1312" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1312" s="16" t="n">
+        <v>186.8</v>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1313" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1313" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1313" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1313" s="19" t="n">
+        <v>78.7</v>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1314" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1314" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1314" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1314" s="16" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1315" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1315" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1315" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1315" s="19" t="n">
+        <v>178.7</v>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1316" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1316" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1316" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1316" s="16" t="n">
+        <v>178.2</v>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1317" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1317" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1317" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1317" s="19" t="n">
+        <v>75.5</v>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1318" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1318" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1318" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1318" s="16" t="n">
+        <v>119.15</v>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1319" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1319" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1319" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1319" s="19" t="n">
+        <v>174.5</v>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1320" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1320" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1320" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1320" s="16" t="n">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1321" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1321" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1321" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1321" s="19" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1322" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1322" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1322" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1322" s="16" t="n">
+        <v>98.09999999999999</v>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1323" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1323" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1323" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1323" s="19" t="n">
+        <v>107.5</v>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1324" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1324" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1324" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1324" s="16" t="n">
+        <v>124.95</v>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1325" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1325" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1325" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1325" s="19" t="n">
+        <v>155.5</v>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1326" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1326" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1326" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1326" s="16" t="n">
+        <v>161.3</v>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1327" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1327" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1327" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1327" s="19" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1328" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1328" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1328" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1328" s="16" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1329" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1329" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1329" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1329" s="19" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1330" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1330" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1330" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1330" s="16" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1331" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1331" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1331" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1331" s="19" t="n">
+        <v>110.15</v>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1332" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1332" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1332" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1332" s="16" t="n">
+        <v>148.5</v>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1333" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1333" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1333" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1333" s="19" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1334" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1334" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1334" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1334" s="16" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1335" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1335" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1335" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1335" s="19" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1336" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1336" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1336" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1336" s="16" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1337" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1337" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1337" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1337" s="19" t="n">
+        <v>66.5</v>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1338" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1338" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1338" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1338" s="16" t="n">
+        <v>105.4</v>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1339" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1339" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1339" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1339" s="19" t="n">
+        <v>159.75</v>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1340" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1340" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1340" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1340" s="16" t="n">
+        <v>160.5</v>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1341" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1341" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1341" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1341" s="19" t="n">
+        <v>65.09999999999999</v>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1342" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1342" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1342" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1342" s="16" t="n">
+        <v>101.4</v>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1343" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1343" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1343" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1343" s="19" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" s="20" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1344" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1344" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1344" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1344" s="16" t="n">
+        <v>155.15</v>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" s="21" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B1345" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1345" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1345" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1345" s="19" t="n">
+        <v>62.9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-29
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1345"/>
+  <dimension ref="A1:E1393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31531,6 +31531,1110 @@
         <v>62.9</v>
       </c>
     </row>
+    <row r="1346">
+      <c r="A1346" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1346" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1346" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1346" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1346" s="16" t="n">
+        <v>101.55</v>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1347" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1347" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1347" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1347" s="19" t="n">
+        <v>112.05</v>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1348" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1348" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1348" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1348" s="16" t="n">
+        <v>130.05</v>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1349" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1349" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1349" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1349" s="19" t="n">
+        <v>158.05</v>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1350" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1350" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1350" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1350" s="16" t="n">
+        <v>161.95</v>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1351" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1351" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1351" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1351" s="19" t="n">
+        <v>129.15</v>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1352" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1352" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1352" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1352" s="16" t="n">
+        <v>87.55</v>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1353" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1353" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1353" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1353" s="19" t="n">
+        <v>87.55</v>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1354" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1354" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1354" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1354" s="16" t="n">
+        <v>87.55</v>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1355" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1355" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1355" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1355" s="19" t="n">
+        <v>114.5</v>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1356" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1356" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1356" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1356" s="16" t="n">
+        <v>149.95</v>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1357" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1357" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1357" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1357" s="19" t="n">
+        <v>87.55</v>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1358" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1358" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1358" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1358" s="16" t="n">
+        <v>132.6</v>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1359" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1359" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1359" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1359" s="19" t="n">
+        <v>181.5</v>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1360" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1360" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1360" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1360" s="16" t="n">
+        <v>180.95</v>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1361" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1361" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1361" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1361" s="19" t="n">
+        <v>75.95</v>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1362" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1362" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1362" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1362" s="16" t="n">
+        <v>116.6</v>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1363" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1363" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1363" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1363" s="19" t="n">
+        <v>168.65</v>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1364" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1364" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1364" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1364" s="16" t="n">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1365" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1365" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1365" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1365" s="19" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1366" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1366" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1366" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1366" s="16" t="n">
+        <v>115.75</v>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1367" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1367" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1367" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1367" s="19" t="n">
+        <v>167.25</v>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1368" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1368" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1368" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1368" s="16" t="n">
+        <v>167.85</v>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1369" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1369" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1369" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1369" s="19" t="n">
+        <v>74.15000000000001</v>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1370" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1370" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1370" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1370" s="16" t="n">
+        <v>97.8</v>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1371" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1371" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1371" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1371" s="19" t="n">
+        <v>106.4</v>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1372" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1372" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1372" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1372" s="16" t="n">
+        <v>119.9</v>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1373" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1373" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1373" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1373" s="19" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1374" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1374" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1374" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1374" s="16" t="n">
+        <v>153.6</v>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1375" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1375" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1375" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1375" s="19" t="n">
+        <v>121.5</v>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1376" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1376" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1376" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1376" s="16" t="n">
+        <v>77.45</v>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1377" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1377" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1377" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1377" s="19" t="n">
+        <v>77.45</v>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1378" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1378" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1378" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1378" s="16" t="n">
+        <v>77.45</v>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1379" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1379" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1379" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1379" s="19" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1380" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1380" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1380" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1380" s="16" t="n">
+        <v>141.25</v>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1381" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1381" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1381" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1381" s="19" t="n">
+        <v>77.45</v>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1382" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1382" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1382" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1382" s="16" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1383" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1383" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1383" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1383" s="19" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1384" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1384" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1384" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1384" s="16" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1385" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1385" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1385" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1385" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1386" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1386" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1386" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1386" s="16" t="n">
+        <v>100.05</v>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1387" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1387" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1387" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1387" s="19" t="n">
+        <v>154.5</v>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1388" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1388" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1388" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1388" s="16" t="n">
+        <v>154.5</v>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1389" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1389" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1389" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1389" s="19" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1390" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1390" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1390" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1390" s="16" t="n">
+        <v>98.34999999999999</v>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1391" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1391" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1391" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1391" s="19" t="n">
+        <v>147.6</v>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" s="20" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1392" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1392" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1392" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1392" s="16" t="n">
+        <v>145.9</v>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" s="21" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B1393" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1393" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1393" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1393" s="19" t="n">
+        <v>62.7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-04-30
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1393"/>
+  <dimension ref="A1:E1441"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32635,6 +32635,1110 @@
         <v>62.7</v>
       </c>
     </row>
+    <row r="1394">
+      <c r="A1394" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1394" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1394" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1394" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1394" s="16" t="n">
+        <v>101.65</v>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1395" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1395" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1395" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1395" s="19" t="n">
+        <v>106.5</v>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1396" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1396" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1396" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1396" s="16" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1397" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1397" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1397" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1397" s="19" t="n">
+        <v>151.45</v>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1398" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1398" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1398" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1398" s="16" t="n">
+        <v>153.2</v>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1399" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1399" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1399" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1399" s="19" t="n">
+        <v>126.8</v>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1400" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1400" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1400" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1400" s="16" t="n">
+        <v>89.65000000000001</v>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1401" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1401" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1401" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1401" s="19" t="n">
+        <v>89.65000000000001</v>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1402" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1402" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1402" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1402" s="16" t="n">
+        <v>89.65000000000001</v>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1403" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1403" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1403" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1403" s="19" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1404" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1404" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1404" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1404" s="16" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1405" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1405" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1405" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1405" s="19" t="n">
+        <v>89.65000000000001</v>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1406" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1406" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1406" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1406" s="16" t="n">
+        <v>135.9</v>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1407" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1407" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1407" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1407" s="19" t="n">
+        <v>184.85</v>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1408" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1408" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1408" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1408" s="16" t="n">
+        <v>184.35</v>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1409" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1409" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1409" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1409" s="19" t="n">
+        <v>75.05</v>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1410" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1410" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1410" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1410" s="16" t="n">
+        <v>119.6</v>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1411" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1411" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1411" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1411" s="19" t="n">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1412" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1412" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1412" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1412" s="16" t="n">
+        <v>172.1</v>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1413" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1413" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1413" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1413" s="19" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1414" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1414" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1414" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1414" s="16" t="n">
+        <v>115.35</v>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1415" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1415" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1415" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1415" s="19" t="n">
+        <v>170.5</v>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1416" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1416" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1416" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1416" s="16" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1417" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1417" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1417" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1417" s="19" t="n">
+        <v>75.45</v>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1418" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1418" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1418" s="15" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="E1418" s="16" t="n">
+        <v>98.40000000000001</v>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1419" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1419" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1419" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1419" s="19" t="n">
+        <v>99.40000000000001</v>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1420" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1420" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1420" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1420" s="16" t="n">
+        <v>111.35</v>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1421" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1421" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1421" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1421" s="19" t="n">
+        <v>140.25</v>
+      </c>
+    </row>
+    <row r="1422">
+      <c r="A1422" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1422" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1422" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1422" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1422" s="16" t="n">
+        <v>143.55</v>
+      </c>
+    </row>
+    <row r="1423">
+      <c r="A1423" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1423" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1423" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1423" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1423" s="19" t="n">
+        <v>117.6</v>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1424" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1424" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1424" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1424" s="16" t="n">
+        <v>80.5</v>
+      </c>
+    </row>
+    <row r="1425">
+      <c r="A1425" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1425" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1425" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1425" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1425" s="19" t="n">
+        <v>80.5</v>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1426" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1426" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1426" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1426" s="16" t="n">
+        <v>80.5</v>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1427" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1427" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1427" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1427" s="19" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1428" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1428" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1428" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1428" s="16" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1429" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1429" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1429" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1429" s="19" t="n">
+        <v>80.5</v>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1430" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1430" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1430" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1430" s="16" t="n">
+        <v>118.5</v>
+      </c>
+    </row>
+    <row r="1431">
+      <c r="A1431" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1431" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1431" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1431" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1431" s="19" t="n">
+        <v>167.25</v>
+      </c>
+    </row>
+    <row r="1432">
+      <c r="A1432" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1432" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1432" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1432" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1432" s="16" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="1433">
+      <c r="A1433" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1433" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1433" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1433" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1433" s="19" t="n">
+        <v>66.3</v>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1434" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1434" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1434" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1434" s="16" t="n">
+        <v>103.55</v>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1435" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1435" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1435" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1435" s="19" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="1436">
+      <c r="A1436" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1436" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1436" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1436" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1436" s="16" t="n">
+        <v>157.05</v>
+      </c>
+    </row>
+    <row r="1437">
+      <c r="A1437" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1437" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1437" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1437" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1437" s="19" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="1438">
+      <c r="A1438" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1438" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1438" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1438" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1438" s="16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1439" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1439" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1439" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1439" s="19" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="1440">
+      <c r="A1440" s="20" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1440" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1440" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1440" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1440" s="16" t="n">
+        <v>150.35</v>
+      </c>
+    </row>
+    <row r="1441">
+      <c r="A1441" s="21" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1441" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1441" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1441" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1441" s="19" t="n">
+        <v>64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-01
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1441"/>
+  <dimension ref="A1:E1487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33739,6 +33739,1064 @@
         <v>64</v>
       </c>
     </row>
+    <row r="1442">
+      <c r="A1442" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1442" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1442" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1442" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1442" s="16" t="n">
+        <v>113.75</v>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1443" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1443" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1443" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1443" s="19" t="n">
+        <v>122.3</v>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1444" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1444" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1444" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1444" s="16" t="n">
+        <v>155.35</v>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1445" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1445" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1445" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1445" s="19" t="n">
+        <v>156.4</v>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1446" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1446" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1446" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1446" s="16" t="n">
+        <v>116.55</v>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1447" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1447" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1447" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1447" s="19" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1448" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1448" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1448" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1448" s="16" t="n">
+        <v>81.34999999999999</v>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1449" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1449" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1449" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1449" s="19" t="n">
+        <v>81.34999999999999</v>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1450" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1450" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1450" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1450" s="16" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1451" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1451" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1451" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1451" s="19" t="n">
+        <v>143.05</v>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1452" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1452" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1452" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1452" s="16" t="n">
+        <v>85.95</v>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1453" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1453" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1453" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1453" s="19" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1454" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1454" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1454" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1454" s="16" t="n">
+        <v>182.65</v>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1455" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1455" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1455" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1455" s="19" t="n">
+        <v>180.1</v>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1456" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1456" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1456" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1456" s="16" t="n">
+        <v>76.09999999999999</v>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1457" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1457" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1457" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1457" s="19" t="n">
+        <v>119.6</v>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1458" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1458" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1458" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1458" s="16" t="n">
+        <v>171.4</v>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1459" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1459" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1459" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1459" s="19" t="n">
+        <v>171.45</v>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1460" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1460" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1460" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1460" s="16" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1461" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1461" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1461" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1461" s="19" t="n">
+        <v>115.35</v>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1462" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1462" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1462" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1462" s="16" t="n">
+        <v>165.6</v>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1463" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1463" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1463" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1463" s="19" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1464" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1464" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1464" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1464" s="16" t="n">
+        <v>75.45</v>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1465" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1465" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1465" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1465" s="19" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1466" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1466" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1466" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1466" s="16" t="n">
+        <v>113.25</v>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1467" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1467" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1467" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1467" s="19" t="n">
+        <v>144.25</v>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1468" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1468" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1468" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1468" s="16" t="n">
+        <v>142.8</v>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1469" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1469" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1469" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1469" s="19" t="n">
+        <v>108.3</v>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1470" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1470" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1470" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1470" s="16" t="n">
+        <v>90.15000000000001</v>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1471" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1471" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1471" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1471" s="19" t="n">
+        <v>67.84999999999999</v>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1472" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1472" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1472" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1472" s="16" t="n">
+        <v>67.84999999999999</v>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1473" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1473" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1473" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1473" s="19" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1474" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1474" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1474" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1474" s="16" t="n">
+        <v>132.05</v>
+      </c>
+    </row>
+    <row r="1475">
+      <c r="A1475" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1475" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1475" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1475" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1475" s="19" t="n">
+        <v>75.34999999999999</v>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1476" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1476" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1476" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1476" s="16" t="n">
+        <v>117.85</v>
+      </c>
+    </row>
+    <row r="1477">
+      <c r="A1477" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1477" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1477" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1477" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1477" s="19" t="n">
+        <v>163.5</v>
+      </c>
+    </row>
+    <row r="1478">
+      <c r="A1478" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1478" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1478" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1478" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1478" s="16" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="1479">
+      <c r="A1479" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1479" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1479" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1479" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1479" s="19" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="1480">
+      <c r="A1480" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1480" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1480" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1480" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1480" s="16" t="n">
+        <v>103.55</v>
+      </c>
+    </row>
+    <row r="1481">
+      <c r="A1481" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1481" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1481" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1481" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1481" s="19" t="n">
+        <v>152.5</v>
+      </c>
+    </row>
+    <row r="1482">
+      <c r="A1482" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1482" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1482" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1482" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1482" s="16" t="n">
+        <v>153.7</v>
+      </c>
+    </row>
+    <row r="1483">
+      <c r="A1483" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1483" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1483" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1483" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1483" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1484">
+      <c r="A1484" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1484" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1484" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1484" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1484" s="16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="1485">
+      <c r="A1485" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1485" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1485" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1485" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1485" s="19" t="n">
+        <v>146.9</v>
+      </c>
+    </row>
+    <row r="1486">
+      <c r="A1486" s="20" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1486" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1486" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1486" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1486" s="16" t="n">
+        <v>147.8</v>
+      </c>
+    </row>
+    <row r="1487">
+      <c r="A1487" s="21" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1487" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1487" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1487" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1487" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-02
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1487"/>
+  <dimension ref="A1:E1533"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34797,6 +34797,1064 @@
         <v>65</v>
       </c>
     </row>
+    <row r="1488">
+      <c r="A1488" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1488" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1488" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1488" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1488" s="16" t="n">
+        <v>113.75</v>
+      </c>
+    </row>
+    <row r="1489">
+      <c r="A1489" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1489" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1489" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1489" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1489" s="19" t="n">
+        <v>122.3</v>
+      </c>
+    </row>
+    <row r="1490">
+      <c r="A1490" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1490" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1490" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1490" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1490" s="16" t="n">
+        <v>155.35</v>
+      </c>
+    </row>
+    <row r="1491">
+      <c r="A1491" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1491" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1491" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1491" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1491" s="19" t="n">
+        <v>156.4</v>
+      </c>
+    </row>
+    <row r="1492">
+      <c r="A1492" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1492" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1492" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1492" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1492" s="16" t="n">
+        <v>116.55</v>
+      </c>
+    </row>
+    <row r="1493">
+      <c r="A1493" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1493" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1493" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1493" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1493" s="19" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="1494">
+      <c r="A1494" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1494" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1494" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1494" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1494" s="16" t="n">
+        <v>81.34999999999999</v>
+      </c>
+    </row>
+    <row r="1495">
+      <c r="A1495" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1495" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1495" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1495" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1495" s="19" t="n">
+        <v>81.34999999999999</v>
+      </c>
+    </row>
+    <row r="1496">
+      <c r="A1496" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1496" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1496" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1496" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1496" s="16" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="1497">
+      <c r="A1497" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1497" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1497" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1497" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1497" s="19" t="n">
+        <v>143.05</v>
+      </c>
+    </row>
+    <row r="1498">
+      <c r="A1498" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1498" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1498" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1498" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1498" s="16" t="n">
+        <v>85.95</v>
+      </c>
+    </row>
+    <row r="1499">
+      <c r="A1499" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1499" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1499" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1499" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1499" s="19" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="1500">
+      <c r="A1500" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1500" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1500" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1500" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1500" s="16" t="n">
+        <v>182.65</v>
+      </c>
+    </row>
+    <row r="1501">
+      <c r="A1501" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1501" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1501" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1501" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1501" s="19" t="n">
+        <v>180.1</v>
+      </c>
+    </row>
+    <row r="1502">
+      <c r="A1502" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1502" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1502" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1502" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1502" s="16" t="n">
+        <v>76.09999999999999</v>
+      </c>
+    </row>
+    <row r="1503">
+      <c r="A1503" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1503" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1503" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1503" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1503" s="19" t="n">
+        <v>119.6</v>
+      </c>
+    </row>
+    <row r="1504">
+      <c r="A1504" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1504" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1504" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1504" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1504" s="16" t="n">
+        <v>171.4</v>
+      </c>
+    </row>
+    <row r="1505">
+      <c r="A1505" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1505" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1505" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1505" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1505" s="19" t="n">
+        <v>171.45</v>
+      </c>
+    </row>
+    <row r="1506">
+      <c r="A1506" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1506" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1506" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1506" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1506" s="16" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="1507">
+      <c r="A1507" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1507" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1507" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1507" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1507" s="19" t="n">
+        <v>115.35</v>
+      </c>
+    </row>
+    <row r="1508">
+      <c r="A1508" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1508" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1508" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1508" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1508" s="16" t="n">
+        <v>165.6</v>
+      </c>
+    </row>
+    <row r="1509">
+      <c r="A1509" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1509" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1509" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1509" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1509" s="19" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="1510">
+      <c r="A1510" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1510" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1510" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1510" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1510" s="16" t="n">
+        <v>75.45</v>
+      </c>
+    </row>
+    <row r="1511">
+      <c r="A1511" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1511" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1511" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1511" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1511" s="19" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="1512">
+      <c r="A1512" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1512" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1512" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1512" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1512" s="16" t="n">
+        <v>113.25</v>
+      </c>
+    </row>
+    <row r="1513">
+      <c r="A1513" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1513" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1513" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1513" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1513" s="19" t="n">
+        <v>144.25</v>
+      </c>
+    </row>
+    <row r="1514">
+      <c r="A1514" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1514" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1514" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1514" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1514" s="16" t="n">
+        <v>142.8</v>
+      </c>
+    </row>
+    <row r="1515">
+      <c r="A1515" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1515" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1515" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1515" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1515" s="19" t="n">
+        <v>108.3</v>
+      </c>
+    </row>
+    <row r="1516">
+      <c r="A1516" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1516" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1516" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1516" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1516" s="16" t="n">
+        <v>90.15000000000001</v>
+      </c>
+    </row>
+    <row r="1517">
+      <c r="A1517" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1517" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1517" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1517" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1517" s="19" t="n">
+        <v>67.84999999999999</v>
+      </c>
+    </row>
+    <row r="1518">
+      <c r="A1518" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1518" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1518" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1518" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1518" s="16" t="n">
+        <v>67.84999999999999</v>
+      </c>
+    </row>
+    <row r="1519">
+      <c r="A1519" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1519" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1519" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1519" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1519" s="19" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="1520">
+      <c r="A1520" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1520" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1520" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1520" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1520" s="16" t="n">
+        <v>132.05</v>
+      </c>
+    </row>
+    <row r="1521">
+      <c r="A1521" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1521" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1521" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1521" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1521" s="19" t="n">
+        <v>75.34999999999999</v>
+      </c>
+    </row>
+    <row r="1522">
+      <c r="A1522" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1522" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1522" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1522" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1522" s="16" t="n">
+        <v>117.85</v>
+      </c>
+    </row>
+    <row r="1523">
+      <c r="A1523" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1523" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1523" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1523" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1523" s="19" t="n">
+        <v>163.5</v>
+      </c>
+    </row>
+    <row r="1524">
+      <c r="A1524" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1524" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1524" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1524" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1524" s="16" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="1525">
+      <c r="A1525" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1525" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1525" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1525" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1525" s="19" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="1526">
+      <c r="A1526" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1526" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1526" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1526" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1526" s="16" t="n">
+        <v>103.55</v>
+      </c>
+    </row>
+    <row r="1527">
+      <c r="A1527" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1527" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1527" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1527" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1527" s="19" t="n">
+        <v>152.5</v>
+      </c>
+    </row>
+    <row r="1528">
+      <c r="A1528" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1528" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1528" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1528" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1528" s="16" t="n">
+        <v>153.7</v>
+      </c>
+    </row>
+    <row r="1529">
+      <c r="A1529" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1529" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1529" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1529" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1529" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1530">
+      <c r="A1530" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1530" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1530" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1530" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1530" s="16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="1531">
+      <c r="A1531" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1531" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1531" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1531" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1531" s="19" t="n">
+        <v>146.9</v>
+      </c>
+    </row>
+    <row r="1532">
+      <c r="A1532" s="20" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1532" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1532" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1532" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1532" s="16" t="n">
+        <v>147.8</v>
+      </c>
+    </row>
+    <row r="1533">
+      <c r="A1533" s="21" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1533" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1533" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1533" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1533" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-03
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1533"/>
+  <dimension ref="A1:E1579"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -35855,6 +35855,1064 @@
         <v>65</v>
       </c>
     </row>
+    <row r="1534">
+      <c r="A1534" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1534" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1534" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1534" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1534" s="16" t="n">
+        <v>113.75</v>
+      </c>
+    </row>
+    <row r="1535">
+      <c r="A1535" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1535" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1535" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1535" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1535" s="19" t="n">
+        <v>122.3</v>
+      </c>
+    </row>
+    <row r="1536">
+      <c r="A1536" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1536" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1536" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1536" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1536" s="16" t="n">
+        <v>155.35</v>
+      </c>
+    </row>
+    <row r="1537">
+      <c r="A1537" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1537" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1537" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1537" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1537" s="19" t="n">
+        <v>156.4</v>
+      </c>
+    </row>
+    <row r="1538">
+      <c r="A1538" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1538" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1538" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1538" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1538" s="16" t="n">
+        <v>116.55</v>
+      </c>
+    </row>
+    <row r="1539">
+      <c r="A1539" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1539" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1539" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1539" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1539" s="19" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="1540">
+      <c r="A1540" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1540" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1540" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1540" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1540" s="16" t="n">
+        <v>81.34999999999999</v>
+      </c>
+    </row>
+    <row r="1541">
+      <c r="A1541" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1541" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1541" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1541" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1541" s="19" t="n">
+        <v>81.34999999999999</v>
+      </c>
+    </row>
+    <row r="1542">
+      <c r="A1542" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1542" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1542" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1542" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1542" s="16" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="1543">
+      <c r="A1543" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1543" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1543" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1543" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1543" s="19" t="n">
+        <v>143.05</v>
+      </c>
+    </row>
+    <row r="1544">
+      <c r="A1544" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1544" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1544" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1544" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1544" s="16" t="n">
+        <v>85.95</v>
+      </c>
+    </row>
+    <row r="1545">
+      <c r="A1545" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1545" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1545" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1545" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1545" s="19" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="1546">
+      <c r="A1546" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1546" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1546" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1546" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1546" s="16" t="n">
+        <v>182.65</v>
+      </c>
+    </row>
+    <row r="1547">
+      <c r="A1547" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1547" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1547" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1547" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1547" s="19" t="n">
+        <v>180.1</v>
+      </c>
+    </row>
+    <row r="1548">
+      <c r="A1548" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1548" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1548" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1548" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1548" s="16" t="n">
+        <v>76.09999999999999</v>
+      </c>
+    </row>
+    <row r="1549">
+      <c r="A1549" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1549" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1549" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1549" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1549" s="19" t="n">
+        <v>119.6</v>
+      </c>
+    </row>
+    <row r="1550">
+      <c r="A1550" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1550" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1550" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1550" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1550" s="16" t="n">
+        <v>171.4</v>
+      </c>
+    </row>
+    <row r="1551">
+      <c r="A1551" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1551" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1551" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1551" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1551" s="19" t="n">
+        <v>171.45</v>
+      </c>
+    </row>
+    <row r="1552">
+      <c r="A1552" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1552" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1552" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1552" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1552" s="16" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="1553">
+      <c r="A1553" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1553" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1553" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1553" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1553" s="19" t="n">
+        <v>115.35</v>
+      </c>
+    </row>
+    <row r="1554">
+      <c r="A1554" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1554" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1554" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1554" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1554" s="16" t="n">
+        <v>165.6</v>
+      </c>
+    </row>
+    <row r="1555">
+      <c r="A1555" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1555" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1555" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1555" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1555" s="19" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="1556">
+      <c r="A1556" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1556" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1556" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1556" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1556" s="16" t="n">
+        <v>75.45</v>
+      </c>
+    </row>
+    <row r="1557">
+      <c r="A1557" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1557" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1557" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1557" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1557" s="19" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="1558">
+      <c r="A1558" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1558" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1558" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1558" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1558" s="16" t="n">
+        <v>113.25</v>
+      </c>
+    </row>
+    <row r="1559">
+      <c r="A1559" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1559" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1559" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1559" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1559" s="19" t="n">
+        <v>144.25</v>
+      </c>
+    </row>
+    <row r="1560">
+      <c r="A1560" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1560" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1560" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1560" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1560" s="16" t="n">
+        <v>142.8</v>
+      </c>
+    </row>
+    <row r="1561">
+      <c r="A1561" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1561" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1561" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1561" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1561" s="19" t="n">
+        <v>108.3</v>
+      </c>
+    </row>
+    <row r="1562">
+      <c r="A1562" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1562" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1562" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1562" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1562" s="16" t="n">
+        <v>90.15000000000001</v>
+      </c>
+    </row>
+    <row r="1563">
+      <c r="A1563" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1563" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1563" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1563" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1563" s="19" t="n">
+        <v>67.84999999999999</v>
+      </c>
+    </row>
+    <row r="1564">
+      <c r="A1564" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1564" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1564" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1564" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1564" s="16" t="n">
+        <v>67.84999999999999</v>
+      </c>
+    </row>
+    <row r="1565">
+      <c r="A1565" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1565" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1565" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1565" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1565" s="19" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="1566">
+      <c r="A1566" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1566" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1566" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1566" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1566" s="16" t="n">
+        <v>132.05</v>
+      </c>
+    </row>
+    <row r="1567">
+      <c r="A1567" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1567" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1567" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1567" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1567" s="19" t="n">
+        <v>75.34999999999999</v>
+      </c>
+    </row>
+    <row r="1568">
+      <c r="A1568" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1568" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1568" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1568" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1568" s="16" t="n">
+        <v>117.85</v>
+      </c>
+    </row>
+    <row r="1569">
+      <c r="A1569" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1569" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1569" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1569" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1569" s="19" t="n">
+        <v>163.5</v>
+      </c>
+    </row>
+    <row r="1570">
+      <c r="A1570" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1570" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1570" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1570" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1570" s="16" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="1571">
+      <c r="A1571" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1571" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1571" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1571" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1571" s="19" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="1572">
+      <c r="A1572" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1572" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1572" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1572" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1572" s="16" t="n">
+        <v>103.55</v>
+      </c>
+    </row>
+    <row r="1573">
+      <c r="A1573" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1573" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1573" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1573" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1573" s="19" t="n">
+        <v>152.5</v>
+      </c>
+    </row>
+    <row r="1574">
+      <c r="A1574" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1574" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1574" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1574" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1574" s="16" t="n">
+        <v>153.7</v>
+      </c>
+    </row>
+    <row r="1575">
+      <c r="A1575" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1575" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1575" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1575" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1575" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1576">
+      <c r="A1576" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1576" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1576" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1576" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1576" s="16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="1577">
+      <c r="A1577" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1577" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1577" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1577" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1577" s="19" t="n">
+        <v>146.9</v>
+      </c>
+    </row>
+    <row r="1578">
+      <c r="A1578" s="20" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1578" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1578" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1578" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1578" s="16" t="n">
+        <v>147.8</v>
+      </c>
+    </row>
+    <row r="1579">
+      <c r="A1579" s="21" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1579" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1579" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1579" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1579" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-04
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1579"/>
+  <dimension ref="A1:E1625"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36913,6 +36913,1064 @@
         <v>65</v>
       </c>
     </row>
+    <row r="1580">
+      <c r="A1580" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1580" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1580" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1580" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1580" s="16" t="n">
+        <v>100.4</v>
+      </c>
+    </row>
+    <row r="1581">
+      <c r="A1581" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1581" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1581" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1581" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1581" s="19" t="n">
+        <v>110.9</v>
+      </c>
+    </row>
+    <row r="1582">
+      <c r="A1582" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1582" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1582" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1582" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1582" s="16" t="n">
+        <v>141.55</v>
+      </c>
+    </row>
+    <row r="1583">
+      <c r="A1583" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1583" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1583" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1583" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1583" s="19" t="n">
+        <v>141.55</v>
+      </c>
+    </row>
+    <row r="1584">
+      <c r="A1584" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1584" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1584" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1584" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1584" s="16" t="n">
+        <v>107.65</v>
+      </c>
+    </row>
+    <row r="1585">
+      <c r="A1585" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1585" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1585" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1585" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1585" s="19" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="1586">
+      <c r="A1586" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1586" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1586" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1586" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1586" s="16" t="n">
+        <v>81.45</v>
+      </c>
+    </row>
+    <row r="1587">
+      <c r="A1587" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1587" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1587" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1587" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1587" s="19" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="1588">
+      <c r="A1588" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1588" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1588" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1588" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1588" s="16" t="n">
+        <v>104.95</v>
+      </c>
+    </row>
+    <row r="1589">
+      <c r="A1589" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1589" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1589" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1589" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1589" s="19" t="n">
+        <v>130.5</v>
+      </c>
+    </row>
+    <row r="1590">
+      <c r="A1590" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1590" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1590" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1590" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1590" s="16" t="n">
+        <v>82.5</v>
+      </c>
+    </row>
+    <row r="1591">
+      <c r="A1591" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1591" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1591" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1591" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1591" s="19" t="n">
+        <v>128.5</v>
+      </c>
+    </row>
+    <row r="1592">
+      <c r="A1592" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1592" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1592" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1592" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1592" s="16" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="1593">
+      <c r="A1593" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1593" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1593" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1593" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1593" s="19" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="1594">
+      <c r="A1594" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1594" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1594" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1594" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1594" s="16" t="n">
+        <v>76.09999999999999</v>
+      </c>
+    </row>
+    <row r="1595">
+      <c r="A1595" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1595" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1595" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1595" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1595" s="19" t="n">
+        <v>117.9</v>
+      </c>
+    </row>
+    <row r="1596">
+      <c r="A1596" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1596" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1596" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1596" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1596" s="16" t="n">
+        <v>166.95</v>
+      </c>
+    </row>
+    <row r="1597">
+      <c r="A1597" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1597" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1597" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1597" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1597" s="19" t="n">
+        <v>163.9</v>
+      </c>
+    </row>
+    <row r="1598">
+      <c r="A1598" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1598" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1598" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1598" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1598" s="16" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="1599">
+      <c r="A1599" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1599" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1599" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1599" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1599" s="19" t="n">
+        <v>115.35</v>
+      </c>
+    </row>
+    <row r="1600">
+      <c r="A1600" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1600" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1600" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1600" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1600" s="16" t="n">
+        <v>161.45</v>
+      </c>
+    </row>
+    <row r="1601">
+      <c r="A1601" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1601" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1601" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1601" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1601" s="19" t="n">
+        <v>159.05</v>
+      </c>
+    </row>
+    <row r="1602">
+      <c r="A1602" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1602" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1602" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1602" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1602" s="16" t="n">
+        <v>75.45</v>
+      </c>
+    </row>
+    <row r="1603">
+      <c r="A1603" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1603" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1603" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1603" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1603" s="19" t="n">
+        <v>88.8</v>
+      </c>
+    </row>
+    <row r="1604">
+      <c r="A1604" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1604" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1604" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1604" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1604" s="16" t="n">
+        <v>100.55</v>
+      </c>
+    </row>
+    <row r="1605">
+      <c r="A1605" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1605" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1605" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1605" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1605" s="19" t="n">
+        <v>132.4</v>
+      </c>
+    </row>
+    <row r="1606">
+      <c r="A1606" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1606" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1606" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1606" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1606" s="16" t="n">
+        <v>131.65</v>
+      </c>
+    </row>
+    <row r="1607">
+      <c r="A1607" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1607" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1607" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1607" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1607" s="19" t="n">
+        <v>98.2</v>
+      </c>
+    </row>
+    <row r="1608">
+      <c r="A1608" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1608" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1608" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1608" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1608" s="16" t="n">
+        <v>82.8</v>
+      </c>
+    </row>
+    <row r="1609">
+      <c r="A1609" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1609" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1609" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1609" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1609" s="19" t="n">
+        <v>67.05</v>
+      </c>
+    </row>
+    <row r="1610">
+      <c r="A1610" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1610" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1610" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1610" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1610" s="16" t="n">
+        <v>62.3</v>
+      </c>
+    </row>
+    <row r="1611">
+      <c r="A1611" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1611" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1611" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1611" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1611" s="19" t="n">
+        <v>96.3</v>
+      </c>
+    </row>
+    <row r="1612">
+      <c r="A1612" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1612" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1612" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1612" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1612" s="16" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1613">
+      <c r="A1613" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1613" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1613" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1613" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1613" s="19" t="n">
+        <v>70.75</v>
+      </c>
+    </row>
+    <row r="1614">
+      <c r="A1614" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1614" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1614" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1614" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1614" s="16" t="n">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="1615">
+      <c r="A1615" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1615" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1615" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1615" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1615" s="19" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="1616">
+      <c r="A1616" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1616" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1616" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1616" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1616" s="16" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="1617">
+      <c r="A1617" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1617" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1617" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1617" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1617" s="19" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="1618">
+      <c r="A1618" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1618" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1618" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1618" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1618" s="16" t="n">
+        <v>103.55</v>
+      </c>
+    </row>
+    <row r="1619">
+      <c r="A1619" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1619" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1619" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1619" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1619" s="19" t="n">
+        <v>149.35</v>
+      </c>
+    </row>
+    <row r="1620">
+      <c r="A1620" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1620" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1620" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1620" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1620" s="16" t="n">
+        <v>149.5</v>
+      </c>
+    </row>
+    <row r="1621">
+      <c r="A1621" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1621" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1621" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1621" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1621" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1622">
+      <c r="A1622" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1622" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1622" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1622" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1622" s="16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="1623">
+      <c r="A1623" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1623" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1623" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1623" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1623" s="19" t="n">
+        <v>143.9</v>
+      </c>
+    </row>
+    <row r="1624">
+      <c r="A1624" s="20" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1624" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1624" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1624" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1624" s="16" t="n">
+        <v>144.5</v>
+      </c>
+    </row>
+    <row r="1625">
+      <c r="A1625" s="21" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1625" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1625" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1625" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1625" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-05
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1625"/>
+  <dimension ref="A1:E1671"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37971,6 +37971,1064 @@
         <v>65</v>
       </c>
     </row>
+    <row r="1626">
+      <c r="A1626" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1626" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1626" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1626" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1626" s="16" t="n">
+        <v>87.8</v>
+      </c>
+    </row>
+    <row r="1627">
+      <c r="A1627" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1627" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1627" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1627" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1627" s="19" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="1628">
+      <c r="A1628" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1628" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1628" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1628" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1628" s="16" t="n">
+        <v>141.3</v>
+      </c>
+    </row>
+    <row r="1629">
+      <c r="A1629" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1629" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1629" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1629" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1629" s="19" t="n">
+        <v>143.75</v>
+      </c>
+    </row>
+    <row r="1630">
+      <c r="A1630" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1630" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1630" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1630" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1630" s="16" t="n">
+        <v>104.2</v>
+      </c>
+    </row>
+    <row r="1631">
+      <c r="A1631" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1631" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1631" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1631" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1631" s="19" t="n">
+        <v>81.40000000000001</v>
+      </c>
+    </row>
+    <row r="1632">
+      <c r="A1632" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1632" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1632" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1632" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1632" s="16" t="n">
+        <v>77.90000000000001</v>
+      </c>
+    </row>
+    <row r="1633">
+      <c r="A1633" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1633" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1633" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1633" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1633" s="19" t="n">
+        <v>71.75</v>
+      </c>
+    </row>
+    <row r="1634">
+      <c r="A1634" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1634" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1634" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1634" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1634" s="16" t="n">
+        <v>97.5</v>
+      </c>
+    </row>
+    <row r="1635">
+      <c r="A1635" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1635" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1635" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1635" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1635" s="19" t="n">
+        <v>130.05</v>
+      </c>
+    </row>
+    <row r="1636">
+      <c r="A1636" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1636" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1636" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1636" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1636" s="16" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="1637">
+      <c r="A1637" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1637" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1637" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1637" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1637" s="19" t="n">
+        <v>127.55</v>
+      </c>
+    </row>
+    <row r="1638">
+      <c r="A1638" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1638" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1638" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1638" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1638" s="16" t="n">
+        <v>177.8</v>
+      </c>
+    </row>
+    <row r="1639">
+      <c r="A1639" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1639" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1639" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1639" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1639" s="19" t="n">
+        <v>178.15</v>
+      </c>
+    </row>
+    <row r="1640">
+      <c r="A1640" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1640" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1640" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1640" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1640" s="16" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="1641">
+      <c r="A1641" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1641" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1641" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1641" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1641" s="19" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1642">
+      <c r="A1642" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1642" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1642" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1642" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1642" s="16" t="n">
+        <v>168.9</v>
+      </c>
+    </row>
+    <row r="1643">
+      <c r="A1643" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1643" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1643" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1643" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1643" s="19" t="n">
+        <v>168.95</v>
+      </c>
+    </row>
+    <row r="1644">
+      <c r="A1644" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1644" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1644" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1644" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1644" s="16" t="n">
+        <v>77.25</v>
+      </c>
+    </row>
+    <row r="1645">
+      <c r="A1645" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1645" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1645" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1645" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1645" s="19" t="n">
+        <v>119.25</v>
+      </c>
+    </row>
+    <row r="1646">
+      <c r="A1646" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1646" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1646" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1646" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1646" s="16" t="n">
+        <v>167.5</v>
+      </c>
+    </row>
+    <row r="1647">
+      <c r="A1647" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1647" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1647" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1647" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1647" s="19" t="n">
+        <v>164.45</v>
+      </c>
+    </row>
+    <row r="1648">
+      <c r="A1648" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1648" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1648" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1648" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1648" s="16" t="n">
+        <v>75.45</v>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1649" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1649" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1649" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1649" s="19" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1650" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1650" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1650" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1650" s="16" t="n">
+        <v>96.40000000000001</v>
+      </c>
+    </row>
+    <row r="1651">
+      <c r="A1651" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1651" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1651" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1651" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1651" s="19" t="n">
+        <v>131.9</v>
+      </c>
+    </row>
+    <row r="1652">
+      <c r="A1652" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1652" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1652" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1652" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1652" s="16" t="n">
+        <v>136.15</v>
+      </c>
+    </row>
+    <row r="1653">
+      <c r="A1653" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1653" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1653" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1653" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1653" s="19" t="n">
+        <v>97.09999999999999</v>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1654" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1654" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1654" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1654" s="16" t="n">
+        <v>78.95</v>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1655" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1655" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1655" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1655" s="19" t="n">
+        <v>67.90000000000001</v>
+      </c>
+    </row>
+    <row r="1656">
+      <c r="A1656" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1656" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1656" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1656" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1656" s="16" t="n">
+        <v>63.1</v>
+      </c>
+    </row>
+    <row r="1657">
+      <c r="A1657" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1657" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1657" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1657" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1657" s="19" t="n">
+        <v>91.84999999999999</v>
+      </c>
+    </row>
+    <row r="1658">
+      <c r="A1658" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1658" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1658" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1658" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1658" s="16" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="1659">
+      <c r="A1659" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1659" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1659" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1659" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1659" s="19" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="1660">
+      <c r="A1660" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1660" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1660" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1660" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1660" s="16" t="n">
+        <v>108.85</v>
+      </c>
+    </row>
+    <row r="1661">
+      <c r="A1661" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1661" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1661" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1661" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1661" s="19" t="n">
+        <v>160.15</v>
+      </c>
+    </row>
+    <row r="1662">
+      <c r="A1662" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1662" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1662" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1662" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1662" s="16" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1663" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1663" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1663" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1663" s="19" t="n">
+        <v>68.59999999999999</v>
+      </c>
+    </row>
+    <row r="1664">
+      <c r="A1664" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1664" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1664" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1664" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1664" s="16" t="n">
+        <v>106.25</v>
+      </c>
+    </row>
+    <row r="1665">
+      <c r="A1665" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1665" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1665" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1665" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1665" s="19" t="n">
+        <v>152.7</v>
+      </c>
+    </row>
+    <row r="1666">
+      <c r="A1666" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1666" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1666" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1666" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1666" s="16" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="1667">
+      <c r="A1667" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1667" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1667" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1667" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1667" s="19" t="n">
+        <v>66.5</v>
+      </c>
+    </row>
+    <row r="1668">
+      <c r="A1668" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1668" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1668" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1668" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1668" s="16" t="n">
+        <v>104.05</v>
+      </c>
+    </row>
+    <row r="1669">
+      <c r="A1669" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1669" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1669" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1669" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1669" s="19" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="1670">
+      <c r="A1670" s="20" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1670" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1670" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1670" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1670" s="16" t="n">
+        <v>149.55</v>
+      </c>
+    </row>
+    <row r="1671">
+      <c r="A1671" s="21" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1671" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1671" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1671" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1671" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-06
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1671"/>
+  <dimension ref="A1:E1717"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -39029,6 +39029,1064 @@
         <v>65</v>
       </c>
     </row>
+    <row r="1672">
+      <c r="A1672" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1672" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1672" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1672" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1672" s="16" t="n">
+        <v>77.2</v>
+      </c>
+    </row>
+    <row r="1673">
+      <c r="A1673" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1673" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1673" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1673" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1673" s="19" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="1674">
+      <c r="A1674" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1674" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1674" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1674" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1674" s="16" t="n">
+        <v>136.05</v>
+      </c>
+    </row>
+    <row r="1675">
+      <c r="A1675" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1675" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1675" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1675" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1675" s="19" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="1676">
+      <c r="A1676" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1676" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1676" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1676" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1676" s="16" t="n">
+        <v>101.15</v>
+      </c>
+    </row>
+    <row r="1677">
+      <c r="A1677" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1677" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1677" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1677" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1677" s="19" t="n">
+        <v>81.7</v>
+      </c>
+    </row>
+    <row r="1678">
+      <c r="A1678" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1678" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1678" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1678" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1678" s="16" t="n">
+        <v>76.15000000000001</v>
+      </c>
+    </row>
+    <row r="1679">
+      <c r="A1679" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1679" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1679" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1679" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1679" s="19" t="n">
+        <v>70.15000000000001</v>
+      </c>
+    </row>
+    <row r="1680">
+      <c r="A1680" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1680" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1680" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1680" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1680" s="16" t="n">
+        <v>93.3</v>
+      </c>
+    </row>
+    <row r="1681">
+      <c r="A1681" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1681" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1681" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1681" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1681" s="19" t="n">
+        <v>126.35</v>
+      </c>
+    </row>
+    <row r="1682">
+      <c r="A1682" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1682" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1682" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1682" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1682" s="16" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="1683">
+      <c r="A1683" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1683" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1683" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1683" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1683" s="19" t="n">
+        <v>127.2</v>
+      </c>
+    </row>
+    <row r="1684">
+      <c r="A1684" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1684" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1684" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1684" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1684" s="16" t="n">
+        <v>181.2</v>
+      </c>
+    </row>
+    <row r="1685">
+      <c r="A1685" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1685" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1685" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1685" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1685" s="19" t="n">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="1686">
+      <c r="A1686" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1686" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1686" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1686" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1686" s="16" t="n">
+        <v>79.15000000000001</v>
+      </c>
+    </row>
+    <row r="1687">
+      <c r="A1687" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1687" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1687" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1687" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1687" s="19" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1688">
+      <c r="A1688" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1688" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1688" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1688" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1688" s="16" t="n">
+        <v>169.65</v>
+      </c>
+    </row>
+    <row r="1689">
+      <c r="A1689" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1689" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1689" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1689" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1689" s="19" t="n">
+        <v>169.7</v>
+      </c>
+    </row>
+    <row r="1690">
+      <c r="A1690" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1690" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1690" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1690" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1690" s="16" t="n">
+        <v>77.59999999999999</v>
+      </c>
+    </row>
+    <row r="1691">
+      <c r="A1691" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1691" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1691" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1691" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1691" s="19" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="1692">
+      <c r="A1692" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1692" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1692" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1692" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1692" s="16" t="n">
+        <v>169.55</v>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1693" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1693" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1693" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1693" s="19" t="n">
+        <v>170.3</v>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1694" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1694" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1694" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1694" s="16" t="n">
+        <v>76.25</v>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1695" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1695" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1695" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1695" s="19" t="n">
+        <v>69.34999999999999</v>
+      </c>
+    </row>
+    <row r="1696">
+      <c r="A1696" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1696" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1696" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1696" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1696" s="16" t="n">
+        <v>90.84999999999999</v>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1697" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1697" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1697" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1697" s="19" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1698" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1698" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1698" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1698" s="16" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1699" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1699" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1699" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1699" s="19" t="n">
+        <v>94.5</v>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1700" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1700" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1700" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1700" s="16" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1701" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1701" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1701" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1701" s="19" t="n">
+        <v>65.8</v>
+      </c>
+    </row>
+    <row r="1702">
+      <c r="A1702" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1702" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1702" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1702" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1702" s="16" t="n">
+        <v>61.15</v>
+      </c>
+    </row>
+    <row r="1703">
+      <c r="A1703" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1703" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1703" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1703" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1703" s="19" t="n">
+        <v>86.2</v>
+      </c>
+    </row>
+    <row r="1704">
+      <c r="A1704" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1704" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1704" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1704" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1704" s="16" t="n">
+        <v>118.1</v>
+      </c>
+    </row>
+    <row r="1705">
+      <c r="A1705" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1705" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1705" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1705" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1705" s="19" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="1706">
+      <c r="A1706" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1706" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1706" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1706" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1706" s="16" t="n">
+        <v>106.75</v>
+      </c>
+    </row>
+    <row r="1707">
+      <c r="A1707" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1707" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1707" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1707" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1707" s="19" t="n">
+        <v>162.1</v>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1708" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1708" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1708" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1708" s="16" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="1709">
+      <c r="A1709" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1709" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1709" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1709" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1709" s="19" t="n">
+        <v>68.90000000000001</v>
+      </c>
+    </row>
+    <row r="1710">
+      <c r="A1710" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1710" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1710" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1710" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1710" s="16" t="n">
+        <v>106.9</v>
+      </c>
+    </row>
+    <row r="1711">
+      <c r="A1711" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1711" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1711" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1711" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1711" s="19" t="n">
+        <v>154.2</v>
+      </c>
+    </row>
+    <row r="1712">
+      <c r="A1712" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1712" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1712" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1712" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1712" s="16" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="1713">
+      <c r="A1713" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1713" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1713" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1713" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1713" s="19" t="n">
+        <v>66.75</v>
+      </c>
+    </row>
+    <row r="1714">
+      <c r="A1714" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1714" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1714" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1714" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1714" s="16" t="n">
+        <v>102.1</v>
+      </c>
+    </row>
+    <row r="1715">
+      <c r="A1715" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1715" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1715" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1715" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1715" s="19" t="n">
+        <v>151.9</v>
+      </c>
+    </row>
+    <row r="1716">
+      <c r="A1716" s="20" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1716" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1716" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1716" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1716" s="16" t="n">
+        <v>152.5</v>
+      </c>
+    </row>
+    <row r="1717">
+      <c r="A1717" s="21" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B1717" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1717" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1717" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1717" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-07
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1717"/>
+  <dimension ref="A1:E1763"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -40087,6 +40087,1064 @@
         <v>65</v>
       </c>
     </row>
+    <row r="1718">
+      <c r="A1718" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1718" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1718" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1718" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1718" s="16" t="n">
+        <v>75.40000000000001</v>
+      </c>
+    </row>
+    <row r="1719">
+      <c r="A1719" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1719" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1719" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1719" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1719" s="19" t="n">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1720" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1720" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1720" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1720" s="16" t="n">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1721" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1721" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1721" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1721" s="19" t="n">
+        <v>145.9</v>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1722" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1722" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1722" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1722" s="16" t="n">
+        <v>107.1</v>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1723" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1723" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1723" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1723" s="19" t="n">
+        <v>81.59999999999999</v>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1724" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1724" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1724" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1724" s="16" t="n">
+        <v>75.8</v>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1725" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1725" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1725" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1725" s="19" t="n">
+        <v>69.84999999999999</v>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1726" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1726" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1726" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1726" s="16" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="1727">
+      <c r="A1727" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1727" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1727" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1727" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1727" s="19" t="n">
+        <v>132.95</v>
+      </c>
+    </row>
+    <row r="1728">
+      <c r="A1728" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1728" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1728" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1728" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1728" s="16" t="n">
+        <v>75.75</v>
+      </c>
+    </row>
+    <row r="1729">
+      <c r="A1729" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1729" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1729" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1729" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1729" s="19" t="n">
+        <v>124.8</v>
+      </c>
+    </row>
+    <row r="1730">
+      <c r="A1730" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1730" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1730" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1730" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1730" s="16" t="n">
+        <v>181.2</v>
+      </c>
+    </row>
+    <row r="1731">
+      <c r="A1731" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1731" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1731" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1731" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1731" s="19" t="n">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="1732">
+      <c r="A1732" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1732" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1732" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1732" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1732" s="16" t="n">
+        <v>77.7</v>
+      </c>
+    </row>
+    <row r="1733">
+      <c r="A1733" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1733" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1733" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1733" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1733" s="19" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="1734">
+      <c r="A1734" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1734" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1734" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1734" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1734" s="16" t="n">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="1735">
+      <c r="A1735" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1735" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1735" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1735" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1735" s="19" t="n">
+        <v>169.7</v>
+      </c>
+    </row>
+    <row r="1736">
+      <c r="A1736" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1736" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1736" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1736" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1736" s="16" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="1737">
+      <c r="A1737" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1737" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1737" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1737" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1737" s="19" t="n">
+        <v>116.75</v>
+      </c>
+    </row>
+    <row r="1738">
+      <c r="A1738" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1738" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1738" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1738" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1738" s="16" t="n">
+        <v>167.4</v>
+      </c>
+    </row>
+    <row r="1739">
+      <c r="A1739" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1739" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1739" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1739" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1739" s="19" t="n">
+        <v>167.4</v>
+      </c>
+    </row>
+    <row r="1740">
+      <c r="A1740" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1740" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1740" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1740" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1740" s="16" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="1741">
+      <c r="A1741" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1741" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1741" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1741" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1741" s="19" t="n">
+        <v>68.75</v>
+      </c>
+    </row>
+    <row r="1742">
+      <c r="A1742" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1742" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1742" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1742" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1742" s="16" t="n">
+        <v>102.25</v>
+      </c>
+    </row>
+    <row r="1743">
+      <c r="A1743" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1743" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1743" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1743" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1743" s="19" t="n">
+        <v>134.65</v>
+      </c>
+    </row>
+    <row r="1744">
+      <c r="A1744" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1744" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1744" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1744" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1744" s="16" t="n">
+        <v>139.15</v>
+      </c>
+    </row>
+    <row r="1745">
+      <c r="A1745" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1745" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1745" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1745" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1745" s="19" t="n">
+        <v>100.4</v>
+      </c>
+    </row>
+    <row r="1746">
+      <c r="A1746" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1746" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1746" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1746" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1746" s="16" t="n">
+        <v>74.7</v>
+      </c>
+    </row>
+    <row r="1747">
+      <c r="A1747" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1747" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1747" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1747" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1747" s="19" t="n">
+        <v>64.65000000000001</v>
+      </c>
+    </row>
+    <row r="1748">
+      <c r="A1748" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1748" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1748" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1748" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1748" s="16" t="n">
+        <v>60.1</v>
+      </c>
+    </row>
+    <row r="1749">
+      <c r="A1749" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1749" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1749" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1749" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1749" s="19" t="n">
+        <v>89.75</v>
+      </c>
+    </row>
+    <row r="1750">
+      <c r="A1750" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1750" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1750" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1750" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1750" s="16" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="1751">
+      <c r="A1751" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1751" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1751" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1751" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1751" s="19" t="n">
+        <v>66.5</v>
+      </c>
+    </row>
+    <row r="1752">
+      <c r="A1752" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1752" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1752" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1752" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1752" s="16" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="1753">
+      <c r="A1753" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1753" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1753" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1753" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1753" s="19" t="n">
+        <v>162.1</v>
+      </c>
+    </row>
+    <row r="1754">
+      <c r="A1754" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1754" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1754" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1754" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1754" s="16" t="n">
+        <v>161.55</v>
+      </c>
+    </row>
+    <row r="1755">
+      <c r="A1755" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1755" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1755" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1755" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1755" s="19" t="n">
+        <v>68.09999999999999</v>
+      </c>
+    </row>
+    <row r="1756">
+      <c r="A1756" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1756" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1756" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1756" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1756" s="16" t="n">
+        <v>104.3</v>
+      </c>
+    </row>
+    <row r="1757">
+      <c r="A1757" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1757" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1757" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1757" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1757" s="19" t="n">
+        <v>154.25</v>
+      </c>
+    </row>
+    <row r="1758">
+      <c r="A1758" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1758" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1758" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1758" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1758" s="16" t="n">
+        <v>154.5</v>
+      </c>
+    </row>
+    <row r="1759">
+      <c r="A1759" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1759" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1759" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1759" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1759" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1760">
+      <c r="A1760" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1760" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1760" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1760" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1760" s="16" t="n">
+        <v>97.95</v>
+      </c>
+    </row>
+    <row r="1761">
+      <c r="A1761" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1761" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1761" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1761" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1761" s="19" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="1762">
+      <c r="A1762" s="20" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1762" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1762" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1762" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1762" s="16" t="n">
+        <v>149.9</v>
+      </c>
+    </row>
+    <row r="1763">
+      <c r="A1763" s="21" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1763" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1763" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1763" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1763" s="19" t="n">
+        <v>63.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-08
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1763"/>
+  <dimension ref="A1:E1809"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -41145,6 +41145,1064 @@
         <v>63.2</v>
       </c>
     </row>
+    <row r="1764">
+      <c r="A1764" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1764" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1764" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1764" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1764" s="16" t="n">
+        <v>77.95</v>
+      </c>
+    </row>
+    <row r="1765">
+      <c r="A1765" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1765" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1765" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1765" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1765" s="19" t="n">
+        <v>111.4</v>
+      </c>
+    </row>
+    <row r="1766">
+      <c r="A1766" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1766" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1766" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1766" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1766" s="16" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="1767">
+      <c r="A1767" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1767" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1767" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1767" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1767" s="19" t="n">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="1768">
+      <c r="A1768" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1768" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1768" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1768" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1768" s="16" t="n">
+        <v>109.65</v>
+      </c>
+    </row>
+    <row r="1769">
+      <c r="A1769" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1769" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1769" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1769" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1769" s="19" t="n">
+        <v>86.7</v>
+      </c>
+    </row>
+    <row r="1770">
+      <c r="A1770" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1770" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1770" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1770" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1770" s="16" t="n">
+        <v>79.05</v>
+      </c>
+    </row>
+    <row r="1771">
+      <c r="A1771" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1771" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1771" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1771" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1771" s="19" t="n">
+        <v>72.84999999999999</v>
+      </c>
+    </row>
+    <row r="1772">
+      <c r="A1772" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1772" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1772" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1772" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1772" s="16" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="1773">
+      <c r="A1773" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1773" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1773" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1773" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1773" s="19" t="n">
+        <v>134.5</v>
+      </c>
+    </row>
+    <row r="1774">
+      <c r="A1774" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1774" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1774" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1774" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1774" s="16" t="n">
+        <v>79.55</v>
+      </c>
+    </row>
+    <row r="1775">
+      <c r="A1775" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1775" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1775" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1775" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1775" s="19" t="n">
+        <v>127.25</v>
+      </c>
+    </row>
+    <row r="1776">
+      <c r="A1776" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1776" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1776" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1776" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1776" s="16" t="n">
+        <v>181.2</v>
+      </c>
+    </row>
+    <row r="1777">
+      <c r="A1777" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1777" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1777" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1777" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1777" s="19" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="1778">
+      <c r="A1778" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1778" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1778" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1778" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1778" s="16" t="n">
+        <v>79.5</v>
+      </c>
+    </row>
+    <row r="1779">
+      <c r="A1779" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1779" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1779" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1779" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1779" s="19" t="n">
+        <v>121.1</v>
+      </c>
+    </row>
+    <row r="1780">
+      <c r="A1780" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1780" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1780" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1780" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1780" s="16" t="n">
+        <v>169.75</v>
+      </c>
+    </row>
+    <row r="1781">
+      <c r="A1781" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1781" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1781" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1781" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1781" s="19" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="1782">
+      <c r="A1782" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1782" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1782" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1782" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1782" s="16" t="n">
+        <v>77.55</v>
+      </c>
+    </row>
+    <row r="1783">
+      <c r="A1783" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1783" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1783" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1783" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1783" s="19" t="n">
+        <v>117.95</v>
+      </c>
+    </row>
+    <row r="1784">
+      <c r="A1784" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1784" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1784" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1784" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1784" s="16" t="n">
+        <v>167.4</v>
+      </c>
+    </row>
+    <row r="1785">
+      <c r="A1785" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1785" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1785" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1785" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1785" s="19" t="n">
+        <v>167.4</v>
+      </c>
+    </row>
+    <row r="1786">
+      <c r="A1786" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1786" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1786" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1786" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1786" s="16" t="n">
+        <v>76.7</v>
+      </c>
+    </row>
+    <row r="1787">
+      <c r="A1787" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1787" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1787" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1787" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1787" s="19" t="n">
+        <v>72.55</v>
+      </c>
+    </row>
+    <row r="1788">
+      <c r="A1788" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1788" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1788" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1788" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1788" s="16" t="n">
+        <v>102.9</v>
+      </c>
+    </row>
+    <row r="1789">
+      <c r="A1789" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1789" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1789" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1789" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1789" s="19" t="n">
+        <v>138.35</v>
+      </c>
+    </row>
+    <row r="1790">
+      <c r="A1790" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1790" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1790" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1790" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1790" s="16" t="n">
+        <v>141.05</v>
+      </c>
+    </row>
+    <row r="1791">
+      <c r="A1791" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1791" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1791" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1791" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1791" s="19" t="n">
+        <v>102.85</v>
+      </c>
+    </row>
+    <row r="1792">
+      <c r="A1792" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1792" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1792" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1792" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1792" s="16" t="n">
+        <v>77.25</v>
+      </c>
+    </row>
+    <row r="1793">
+      <c r="A1793" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1793" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1793" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1793" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1793" s="19" t="n">
+        <v>66.45</v>
+      </c>
+    </row>
+    <row r="1794">
+      <c r="A1794" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1794" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1794" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1794" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1794" s="16" t="n">
+        <v>61.75</v>
+      </c>
+    </row>
+    <row r="1795">
+      <c r="A1795" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1795" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1795" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1795" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1795" s="19" t="n">
+        <v>91.25</v>
+      </c>
+    </row>
+    <row r="1796">
+      <c r="A1796" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1796" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1796" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1796" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1796" s="16" t="n">
+        <v>127.7</v>
+      </c>
+    </row>
+    <row r="1797">
+      <c r="A1797" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1797" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1797" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1797" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1797" s="19" t="n">
+        <v>68.5</v>
+      </c>
+    </row>
+    <row r="1798">
+      <c r="A1798" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1798" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1798" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1798" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1798" s="16" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="1799">
+      <c r="A1799" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1799" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1799" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1799" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1799" s="19" t="n">
+        <v>162.1</v>
+      </c>
+    </row>
+    <row r="1800">
+      <c r="A1800" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1800" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1800" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1800" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1800" s="16" t="n">
+        <v>163.5</v>
+      </c>
+    </row>
+    <row r="1801">
+      <c r="A1801" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1801" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1801" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1801" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1801" s="19" t="n">
+        <v>69.3</v>
+      </c>
+    </row>
+    <row r="1802">
+      <c r="A1802" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1802" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1802" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1802" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1802" s="16" t="n">
+        <v>104.5</v>
+      </c>
+    </row>
+    <row r="1803">
+      <c r="A1803" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1803" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1803" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1803" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1803" s="19" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="1804">
+      <c r="A1804" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1804" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1804" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1804" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1804" s="16" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="1805">
+      <c r="A1805" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1805" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1805" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1805" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1805" s="19" t="n">
+        <v>66.25</v>
+      </c>
+    </row>
+    <row r="1806">
+      <c r="A1806" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1806" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1806" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1806" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1806" s="16" t="n">
+        <v>99.5</v>
+      </c>
+    </row>
+    <row r="1807">
+      <c r="A1807" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1807" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1807" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1807" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1807" s="19" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="1808">
+      <c r="A1808" s="20" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1808" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1808" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1808" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1808" s="16" t="n">
+        <v>149.9</v>
+      </c>
+    </row>
+    <row r="1809">
+      <c r="A1809" s="21" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B1809" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1809" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1809" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1809" s="19" t="n">
+        <v>64.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-09
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1809"/>
+  <dimension ref="A1:E1855"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -42203,6 +42203,1064 @@
         <v>64.75</v>
       </c>
     </row>
+    <row r="1810">
+      <c r="A1810" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1810" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1810" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1810" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1810" s="16" t="n">
+        <v>77.95</v>
+      </c>
+    </row>
+    <row r="1811">
+      <c r="A1811" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1811" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1811" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1811" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1811" s="19" t="n">
+        <v>111.4</v>
+      </c>
+    </row>
+    <row r="1812">
+      <c r="A1812" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1812" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1812" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1812" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1812" s="16" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="1813">
+      <c r="A1813" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1813" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1813" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1813" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1813" s="19" t="n">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="1814">
+      <c r="A1814" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1814" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1814" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1814" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1814" s="16" t="n">
+        <v>109.65</v>
+      </c>
+    </row>
+    <row r="1815">
+      <c r="A1815" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1815" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1815" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1815" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1815" s="19" t="n">
+        <v>86.7</v>
+      </c>
+    </row>
+    <row r="1816">
+      <c r="A1816" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1816" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1816" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1816" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1816" s="16" t="n">
+        <v>79.05</v>
+      </c>
+    </row>
+    <row r="1817">
+      <c r="A1817" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1817" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1817" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1817" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1817" s="19" t="n">
+        <v>72.84999999999999</v>
+      </c>
+    </row>
+    <row r="1818">
+      <c r="A1818" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1818" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1818" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1818" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1818" s="16" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="1819">
+      <c r="A1819" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1819" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1819" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1819" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1819" s="19" t="n">
+        <v>134.5</v>
+      </c>
+    </row>
+    <row r="1820">
+      <c r="A1820" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1820" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1820" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1820" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1820" s="16" t="n">
+        <v>79.55</v>
+      </c>
+    </row>
+    <row r="1821">
+      <c r="A1821" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1821" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1821" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1821" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1821" s="19" t="n">
+        <v>127.25</v>
+      </c>
+    </row>
+    <row r="1822">
+      <c r="A1822" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1822" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1822" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1822" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1822" s="16" t="n">
+        <v>181.2</v>
+      </c>
+    </row>
+    <row r="1823">
+      <c r="A1823" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1823" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1823" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1823" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1823" s="19" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="1824">
+      <c r="A1824" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1824" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1824" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1824" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1824" s="16" t="n">
+        <v>79.5</v>
+      </c>
+    </row>
+    <row r="1825">
+      <c r="A1825" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1825" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1825" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1825" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1825" s="19" t="n">
+        <v>121.1</v>
+      </c>
+    </row>
+    <row r="1826">
+      <c r="A1826" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1826" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1826" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1826" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1826" s="16" t="n">
+        <v>169.75</v>
+      </c>
+    </row>
+    <row r="1827">
+      <c r="A1827" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1827" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1827" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1827" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1827" s="19" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="1828">
+      <c r="A1828" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1828" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1828" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1828" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1828" s="16" t="n">
+        <v>77.55</v>
+      </c>
+    </row>
+    <row r="1829">
+      <c r="A1829" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1829" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1829" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1829" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1829" s="19" t="n">
+        <v>117.95</v>
+      </c>
+    </row>
+    <row r="1830">
+      <c r="A1830" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1830" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1830" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1830" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1830" s="16" t="n">
+        <v>167.4</v>
+      </c>
+    </row>
+    <row r="1831">
+      <c r="A1831" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1831" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1831" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1831" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1831" s="19" t="n">
+        <v>167.4</v>
+      </c>
+    </row>
+    <row r="1832">
+      <c r="A1832" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1832" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1832" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1832" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1832" s="16" t="n">
+        <v>76.7</v>
+      </c>
+    </row>
+    <row r="1833">
+      <c r="A1833" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1833" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1833" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1833" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1833" s="19" t="n">
+        <v>72.55</v>
+      </c>
+    </row>
+    <row r="1834">
+      <c r="A1834" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1834" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1834" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1834" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1834" s="16" t="n">
+        <v>102.9</v>
+      </c>
+    </row>
+    <row r="1835">
+      <c r="A1835" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1835" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1835" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1835" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1835" s="19" t="n">
+        <v>138.35</v>
+      </c>
+    </row>
+    <row r="1836">
+      <c r="A1836" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1836" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1836" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1836" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1836" s="16" t="n">
+        <v>141.05</v>
+      </c>
+    </row>
+    <row r="1837">
+      <c r="A1837" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1837" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1837" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1837" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1837" s="19" t="n">
+        <v>102.85</v>
+      </c>
+    </row>
+    <row r="1838">
+      <c r="A1838" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1838" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1838" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1838" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1838" s="16" t="n">
+        <v>77.25</v>
+      </c>
+    </row>
+    <row r="1839">
+      <c r="A1839" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1839" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1839" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1839" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1839" s="19" t="n">
+        <v>66.45</v>
+      </c>
+    </row>
+    <row r="1840">
+      <c r="A1840" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1840" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1840" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1840" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1840" s="16" t="n">
+        <v>61.75</v>
+      </c>
+    </row>
+    <row r="1841">
+      <c r="A1841" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1841" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1841" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1841" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1841" s="19" t="n">
+        <v>91.25</v>
+      </c>
+    </row>
+    <row r="1842">
+      <c r="A1842" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1842" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1842" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1842" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1842" s="16" t="n">
+        <v>127.7</v>
+      </c>
+    </row>
+    <row r="1843">
+      <c r="A1843" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1843" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1843" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1843" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1843" s="19" t="n">
+        <v>68.5</v>
+      </c>
+    </row>
+    <row r="1844">
+      <c r="A1844" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1844" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1844" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1844" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1844" s="16" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="1845">
+      <c r="A1845" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1845" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1845" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1845" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1845" s="19" t="n">
+        <v>162.1</v>
+      </c>
+    </row>
+    <row r="1846">
+      <c r="A1846" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1846" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1846" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1846" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1846" s="16" t="n">
+        <v>163.5</v>
+      </c>
+    </row>
+    <row r="1847">
+      <c r="A1847" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1847" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1847" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1847" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1847" s="19" t="n">
+        <v>69.3</v>
+      </c>
+    </row>
+    <row r="1848">
+      <c r="A1848" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1848" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1848" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1848" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1848" s="16" t="n">
+        <v>104.5</v>
+      </c>
+    </row>
+    <row r="1849">
+      <c r="A1849" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1849" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1849" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1849" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1849" s="19" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="1850">
+      <c r="A1850" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1850" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1850" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1850" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1850" s="16" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="1851">
+      <c r="A1851" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1851" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1851" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1851" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1851" s="19" t="n">
+        <v>66.25</v>
+      </c>
+    </row>
+    <row r="1852">
+      <c r="A1852" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1852" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1852" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1852" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1852" s="16" t="n">
+        <v>99.5</v>
+      </c>
+    </row>
+    <row r="1853">
+      <c r="A1853" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1853" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1853" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1853" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1853" s="19" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="1854">
+      <c r="A1854" s="20" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1854" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1854" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1854" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1854" s="16" t="n">
+        <v>149.9</v>
+      </c>
+    </row>
+    <row r="1855">
+      <c r="A1855" s="21" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1855" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1855" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1855" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1855" s="19" t="n">
+        <v>64.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-10
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1855"/>
+  <dimension ref="A1:E1901"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -43261,6 +43261,1064 @@
         <v>64.75</v>
       </c>
     </row>
+    <row r="1856">
+      <c r="A1856" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1856" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1856" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1856" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1856" s="16" t="n">
+        <v>77.95</v>
+      </c>
+    </row>
+    <row r="1857">
+      <c r="A1857" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1857" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1857" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1857" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1857" s="19" t="n">
+        <v>111.4</v>
+      </c>
+    </row>
+    <row r="1858">
+      <c r="A1858" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1858" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1858" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1858" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1858" s="16" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="1859">
+      <c r="A1859" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1859" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1859" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1859" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1859" s="19" t="n">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="1860">
+      <c r="A1860" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1860" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1860" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1860" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1860" s="16" t="n">
+        <v>109.65</v>
+      </c>
+    </row>
+    <row r="1861">
+      <c r="A1861" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1861" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1861" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1861" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1861" s="19" t="n">
+        <v>86.7</v>
+      </c>
+    </row>
+    <row r="1862">
+      <c r="A1862" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1862" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1862" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1862" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1862" s="16" t="n">
+        <v>79.05</v>
+      </c>
+    </row>
+    <row r="1863">
+      <c r="A1863" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1863" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1863" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1863" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1863" s="19" t="n">
+        <v>72.84999999999999</v>
+      </c>
+    </row>
+    <row r="1864">
+      <c r="A1864" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1864" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1864" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1864" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1864" s="16" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="1865">
+      <c r="A1865" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1865" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1865" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1865" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1865" s="19" t="n">
+        <v>134.5</v>
+      </c>
+    </row>
+    <row r="1866">
+      <c r="A1866" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1866" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1866" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1866" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1866" s="16" t="n">
+        <v>79.55</v>
+      </c>
+    </row>
+    <row r="1867">
+      <c r="A1867" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1867" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1867" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1867" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1867" s="19" t="n">
+        <v>127.25</v>
+      </c>
+    </row>
+    <row r="1868">
+      <c r="A1868" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1868" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1868" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1868" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1868" s="16" t="n">
+        <v>181.2</v>
+      </c>
+    </row>
+    <row r="1869">
+      <c r="A1869" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1869" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1869" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1869" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1869" s="19" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="1870">
+      <c r="A1870" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1870" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1870" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1870" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1870" s="16" t="n">
+        <v>79.5</v>
+      </c>
+    </row>
+    <row r="1871">
+      <c r="A1871" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1871" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1871" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1871" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1871" s="19" t="n">
+        <v>121.1</v>
+      </c>
+    </row>
+    <row r="1872">
+      <c r="A1872" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1872" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1872" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1872" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1872" s="16" t="n">
+        <v>169.75</v>
+      </c>
+    </row>
+    <row r="1873">
+      <c r="A1873" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1873" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1873" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1873" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1873" s="19" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="1874">
+      <c r="A1874" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1874" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1874" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1874" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1874" s="16" t="n">
+        <v>77.55</v>
+      </c>
+    </row>
+    <row r="1875">
+      <c r="A1875" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1875" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1875" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1875" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1875" s="19" t="n">
+        <v>117.95</v>
+      </c>
+    </row>
+    <row r="1876">
+      <c r="A1876" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1876" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1876" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1876" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1876" s="16" t="n">
+        <v>167.4</v>
+      </c>
+    </row>
+    <row r="1877">
+      <c r="A1877" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1877" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1877" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1877" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1877" s="19" t="n">
+        <v>167.4</v>
+      </c>
+    </row>
+    <row r="1878">
+      <c r="A1878" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1878" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1878" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1878" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1878" s="16" t="n">
+        <v>76.7</v>
+      </c>
+    </row>
+    <row r="1879">
+      <c r="A1879" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1879" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1879" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1879" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1879" s="19" t="n">
+        <v>72.55</v>
+      </c>
+    </row>
+    <row r="1880">
+      <c r="A1880" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1880" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1880" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1880" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1880" s="16" t="n">
+        <v>102.9</v>
+      </c>
+    </row>
+    <row r="1881">
+      <c r="A1881" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1881" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1881" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1881" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1881" s="19" t="n">
+        <v>138.35</v>
+      </c>
+    </row>
+    <row r="1882">
+      <c r="A1882" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1882" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1882" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1882" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1882" s="16" t="n">
+        <v>141.05</v>
+      </c>
+    </row>
+    <row r="1883">
+      <c r="A1883" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1883" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1883" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1883" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1883" s="19" t="n">
+        <v>102.85</v>
+      </c>
+    </row>
+    <row r="1884">
+      <c r="A1884" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1884" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1884" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1884" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1884" s="16" t="n">
+        <v>77.25</v>
+      </c>
+    </row>
+    <row r="1885">
+      <c r="A1885" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1885" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1885" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1885" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1885" s="19" t="n">
+        <v>66.45</v>
+      </c>
+    </row>
+    <row r="1886">
+      <c r="A1886" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1886" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1886" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1886" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1886" s="16" t="n">
+        <v>61.75</v>
+      </c>
+    </row>
+    <row r="1887">
+      <c r="A1887" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1887" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1887" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1887" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1887" s="19" t="n">
+        <v>91.25</v>
+      </c>
+    </row>
+    <row r="1888">
+      <c r="A1888" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1888" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1888" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1888" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1888" s="16" t="n">
+        <v>127.7</v>
+      </c>
+    </row>
+    <row r="1889">
+      <c r="A1889" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1889" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1889" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1889" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1889" s="19" t="n">
+        <v>68.5</v>
+      </c>
+    </row>
+    <row r="1890">
+      <c r="A1890" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1890" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1890" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1890" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1890" s="16" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="1891">
+      <c r="A1891" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1891" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1891" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1891" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1891" s="19" t="n">
+        <v>162.1</v>
+      </c>
+    </row>
+    <row r="1892">
+      <c r="A1892" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1892" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1892" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1892" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1892" s="16" t="n">
+        <v>163.5</v>
+      </c>
+    </row>
+    <row r="1893">
+      <c r="A1893" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1893" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1893" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1893" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1893" s="19" t="n">
+        <v>69.3</v>
+      </c>
+    </row>
+    <row r="1894">
+      <c r="A1894" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1894" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1894" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1894" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1894" s="16" t="n">
+        <v>104.5</v>
+      </c>
+    </row>
+    <row r="1895">
+      <c r="A1895" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1895" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1895" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1895" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1895" s="19" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="1896">
+      <c r="A1896" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1896" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1896" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1896" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1896" s="16" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="1897">
+      <c r="A1897" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1897" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1897" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1897" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1897" s="19" t="n">
+        <v>66.25</v>
+      </c>
+    </row>
+    <row r="1898">
+      <c r="A1898" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1898" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1898" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1898" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1898" s="16" t="n">
+        <v>99.5</v>
+      </c>
+    </row>
+    <row r="1899">
+      <c r="A1899" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1899" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1899" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1899" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1899" s="19" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="1900">
+      <c r="A1900" s="20" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1900" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1900" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1900" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1900" s="16" t="n">
+        <v>149.9</v>
+      </c>
+    </row>
+    <row r="1901">
+      <c r="A1901" s="21" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B1901" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1901" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1901" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1901" s="19" t="n">
+        <v>64.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-11
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1901"/>
+  <dimension ref="A1:E1947"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -44319,6 +44319,1064 @@
         <v>64.75</v>
       </c>
     </row>
+    <row r="1902">
+      <c r="A1902" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1902" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1902" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1902" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1902" s="16" t="n">
+        <v>78.40000000000001</v>
+      </c>
+    </row>
+    <row r="1903">
+      <c r="A1903" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1903" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1903" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1903" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1903" s="19" t="n">
+        <v>115.65</v>
+      </c>
+    </row>
+    <row r="1904">
+      <c r="A1904" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1904" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1904" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1904" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1904" s="16" t="n">
+        <v>152.25</v>
+      </c>
+    </row>
+    <row r="1905">
+      <c r="A1905" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1905" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1905" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1905" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1905" s="19" t="n">
+        <v>153.35</v>
+      </c>
+    </row>
+    <row r="1906">
+      <c r="A1906" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1906" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1906" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1906" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1906" s="16" t="n">
+        <v>114.65</v>
+      </c>
+    </row>
+    <row r="1907">
+      <c r="A1907" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1907" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1907" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1907" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1907" s="19" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="1908">
+      <c r="A1908" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1908" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1908" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1908" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1908" s="16" t="n">
+        <v>81.5</v>
+      </c>
+    </row>
+    <row r="1909">
+      <c r="A1909" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1909" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1909" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1909" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1909" s="19" t="n">
+        <v>75.15000000000001</v>
+      </c>
+    </row>
+    <row r="1910">
+      <c r="A1910" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1910" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1910" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1910" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1910" s="16" t="n">
+        <v>98.55</v>
+      </c>
+    </row>
+    <row r="1911">
+      <c r="A1911" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1911" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1911" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1911" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1911" s="19" t="n">
+        <v>140.4</v>
+      </c>
+    </row>
+    <row r="1912">
+      <c r="A1912" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1912" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1912" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1912" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1912" s="16" t="n">
+        <v>82.90000000000001</v>
+      </c>
+    </row>
+    <row r="1913">
+      <c r="A1913" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1913" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1913" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1913" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1913" s="19" t="n">
+        <v>130.5</v>
+      </c>
+    </row>
+    <row r="1914">
+      <c r="A1914" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1914" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1914" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1914" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1914" s="16" t="n">
+        <v>183.9</v>
+      </c>
+    </row>
+    <row r="1915">
+      <c r="A1915" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1915" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1915" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1915" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1915" s="19" t="n">
+        <v>183.25</v>
+      </c>
+    </row>
+    <row r="1916">
+      <c r="A1916" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1916" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1916" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1916" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1916" s="16" t="n">
+        <v>80.84999999999999</v>
+      </c>
+    </row>
+    <row r="1917">
+      <c r="A1917" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1917" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1917" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1917" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1917" s="19" t="n">
+        <v>123.15</v>
+      </c>
+    </row>
+    <row r="1918">
+      <c r="A1918" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1918" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1918" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1918" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1918" s="16" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="1919">
+      <c r="A1919" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1919" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1919" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1919" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1919" s="19" t="n">
+        <v>174.15</v>
+      </c>
+    </row>
+    <row r="1920">
+      <c r="A1920" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1920" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1920" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1920" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1920" s="16" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="1921">
+      <c r="A1921" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1921" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1921" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1921" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1921" s="19" t="n">
+        <v>117.95</v>
+      </c>
+    </row>
+    <row r="1922">
+      <c r="A1922" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1922" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1922" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1922" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1922" s="16" t="n">
+        <v>170.5</v>
+      </c>
+    </row>
+    <row r="1923">
+      <c r="A1923" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1923" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1923" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1923" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1923" s="19" t="n">
+        <v>169.85</v>
+      </c>
+    </row>
+    <row r="1924">
+      <c r="A1924" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1924" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1924" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1924" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1924" s="16" t="n">
+        <v>76.7</v>
+      </c>
+    </row>
+    <row r="1925">
+      <c r="A1925" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1925" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1925" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1925" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1925" s="19" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="1926">
+      <c r="A1926" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1926" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1926" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1926" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1926" s="16" t="n">
+        <v>107.5</v>
+      </c>
+    </row>
+    <row r="1927">
+      <c r="A1927" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1927" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1927" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1927" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1927" s="19" t="n">
+        <v>142.3</v>
+      </c>
+    </row>
+    <row r="1928">
+      <c r="A1928" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1928" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1928" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1928" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1928" s="16" t="n">
+        <v>142.45</v>
+      </c>
+    </row>
+    <row r="1929">
+      <c r="A1929" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1929" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1929" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1929" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1929" s="19" t="n">
+        <v>106.3</v>
+      </c>
+    </row>
+    <row r="1930">
+      <c r="A1930" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1930" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1930" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1930" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1930" s="16" t="n">
+        <v>83.15000000000001</v>
+      </c>
+    </row>
+    <row r="1931">
+      <c r="A1931" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1931" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1931" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1931" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1931" s="19" t="n">
+        <v>68.40000000000001</v>
+      </c>
+    </row>
+    <row r="1932">
+      <c r="A1932" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1932" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1932" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1932" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1932" s="16" t="n">
+        <v>63.6</v>
+      </c>
+    </row>
+    <row r="1933">
+      <c r="A1933" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1933" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1933" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1933" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1933" s="19" t="n">
+        <v>93.59999999999999</v>
+      </c>
+    </row>
+    <row r="1934">
+      <c r="A1934" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1934" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1934" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1934" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1934" s="16" t="n">
+        <v>130.6</v>
+      </c>
+    </row>
+    <row r="1935">
+      <c r="A1935" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1935" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1935" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1935" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1935" s="19" t="n">
+        <v>71.75</v>
+      </c>
+    </row>
+    <row r="1936">
+      <c r="A1936" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1936" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1936" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1936" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1936" s="16" t="n">
+        <v>111.15</v>
+      </c>
+    </row>
+    <row r="1937">
+      <c r="A1937" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1937" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1937" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1937" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1937" s="19" t="n">
+        <v>166.5</v>
+      </c>
+    </row>
+    <row r="1938">
+      <c r="A1938" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1938" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1938" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1938" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1938" s="16" t="n">
+        <v>166.6</v>
+      </c>
+    </row>
+    <row r="1939">
+      <c r="A1939" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1939" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1939" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1939" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1939" s="19" t="n">
+        <v>69.5</v>
+      </c>
+    </row>
+    <row r="1940">
+      <c r="A1940" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1940" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1940" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1940" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1940" s="16" t="n">
+        <v>105.3</v>
+      </c>
+    </row>
+    <row r="1941">
+      <c r="A1941" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1941" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1941" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1941" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1941" s="19" t="n">
+        <v>155.55</v>
+      </c>
+    </row>
+    <row r="1942">
+      <c r="A1942" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1942" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1942" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1942" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1942" s="16" t="n">
+        <v>155.55</v>
+      </c>
+    </row>
+    <row r="1943">
+      <c r="A1943" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1943" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1943" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1943" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1943" s="19" t="n">
+        <v>67.75</v>
+      </c>
+    </row>
+    <row r="1944">
+      <c r="A1944" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1944" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1944" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1944" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1944" s="16" t="n">
+        <v>100.9</v>
+      </c>
+    </row>
+    <row r="1945">
+      <c r="A1945" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1945" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1945" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1945" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1945" s="19" t="n">
+        <v>151.95</v>
+      </c>
+    </row>
+    <row r="1946">
+      <c r="A1946" s="20" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1946" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1946" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1946" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1946" s="16" t="n">
+        <v>151.65</v>
+      </c>
+    </row>
+    <row r="1947">
+      <c r="A1947" s="21" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B1947" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1947" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1947" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1947" s="19" t="n">
+        <v>65.95</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-12
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1947"/>
+  <dimension ref="A1:E1993"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -45377,6 +45377,1064 @@
         <v>65.95</v>
       </c>
     </row>
+    <row r="1948">
+      <c r="A1948" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1948" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1948" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1948" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1948" s="16" t="n">
+        <v>77.05</v>
+      </c>
+    </row>
+    <row r="1949">
+      <c r="A1949" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1949" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1949" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1949" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1949" s="19" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="1950">
+      <c r="A1950" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1950" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1950" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1950" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1950" s="16" t="n">
+        <v>153.5</v>
+      </c>
+    </row>
+    <row r="1951">
+      <c r="A1951" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1951" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1951" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1951" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1951" s="19" t="n">
+        <v>156.5</v>
+      </c>
+    </row>
+    <row r="1952">
+      <c r="A1952" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1952" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1952" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1952" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1952" s="16" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="1953">
+      <c r="A1953" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1953" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1953" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1953" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1953" s="19" t="n">
+        <v>96.15000000000001</v>
+      </c>
+    </row>
+    <row r="1954">
+      <c r="A1954" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1954" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1954" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1954" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1954" s="16" t="n">
+        <v>81.34999999999999</v>
+      </c>
+    </row>
+    <row r="1955">
+      <c r="A1955" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1955" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1955" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1955" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1955" s="19" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="1956">
+      <c r="A1956" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1956" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1956" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1956" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1956" s="16" t="n">
+        <v>97.55</v>
+      </c>
+    </row>
+    <row r="1957">
+      <c r="A1957" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1957" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1957" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1957" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1957" s="19" t="n">
+        <v>142.3</v>
+      </c>
+    </row>
+    <row r="1958">
+      <c r="A1958" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1958" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1958" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1958" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1958" s="16" t="n">
+        <v>84.2</v>
+      </c>
+    </row>
+    <row r="1959">
+      <c r="A1959" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1959" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1959" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1959" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1959" s="19" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="1960">
+      <c r="A1960" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1960" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1960" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1960" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1960" s="16" t="n">
+        <v>184.35</v>
+      </c>
+    </row>
+    <row r="1961">
+      <c r="A1961" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1961" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1961" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1961" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1961" s="19" t="n">
+        <v>183.25</v>
+      </c>
+    </row>
+    <row r="1962">
+      <c r="A1962" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1962" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1962" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1962" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1962" s="16" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="1963">
+      <c r="A1963" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1963" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1963" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1963" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1963" s="19" t="n">
+        <v>122.75</v>
+      </c>
+    </row>
+    <row r="1964">
+      <c r="A1964" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1964" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1964" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1964" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1964" s="16" t="n">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="1965">
+      <c r="A1965" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1965" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1965" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1965" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1965" s="19" t="n">
+        <v>174.15</v>
+      </c>
+    </row>
+    <row r="1966">
+      <c r="A1966" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1966" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1966" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1966" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1966" s="16" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="1967">
+      <c r="A1967" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1967" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1967" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1967" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1967" s="19" t="n">
+        <v>117.95</v>
+      </c>
+    </row>
+    <row r="1968">
+      <c r="A1968" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1968" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1968" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1968" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1968" s="16" t="n">
+        <v>170.5</v>
+      </c>
+    </row>
+    <row r="1969">
+      <c r="A1969" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1969" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1969" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1969" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1969" s="19" t="n">
+        <v>169.85</v>
+      </c>
+    </row>
+    <row r="1970">
+      <c r="A1970" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1970" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1970" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1970" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1970" s="16" t="n">
+        <v>76.7</v>
+      </c>
+    </row>
+    <row r="1971">
+      <c r="A1971" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1971" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1971" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1971" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1971" s="19" t="n">
+        <v>70.05</v>
+      </c>
+    </row>
+    <row r="1972">
+      <c r="A1972" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1972" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1972" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1972" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1972" s="16" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="1973">
+      <c r="A1973" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1973" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1973" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1973" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1973" s="19" t="n">
+        <v>143.55</v>
+      </c>
+    </row>
+    <row r="1974">
+      <c r="A1974" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1974" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1974" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1974" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1974" s="16" t="n">
+        <v>143.8</v>
+      </c>
+    </row>
+    <row r="1975">
+      <c r="A1975" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1975" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1975" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1975" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1975" s="19" t="n">
+        <v>107.8</v>
+      </c>
+    </row>
+    <row r="1976">
+      <c r="A1976" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1976" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1976" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1976" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1976" s="16" t="n">
+        <v>87.5</v>
+      </c>
+    </row>
+    <row r="1977">
+      <c r="A1977" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1977" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1977" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1977" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E1977" s="19" t="n">
+        <v>68.25</v>
+      </c>
+    </row>
+    <row r="1978">
+      <c r="A1978" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1978" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1978" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1978" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E1978" s="16" t="n">
+        <v>63.45</v>
+      </c>
+    </row>
+    <row r="1979">
+      <c r="A1979" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1979" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1979" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1979" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E1979" s="19" t="n">
+        <v>91.09999999999999</v>
+      </c>
+    </row>
+    <row r="1980">
+      <c r="A1980" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1980" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1980" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1980" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E1980" s="16" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="1981">
+      <c r="A1981" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1981" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1981" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1981" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E1981" s="19" t="n">
+        <v>73.15000000000001</v>
+      </c>
+    </row>
+    <row r="1982">
+      <c r="A1982" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1982" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1982" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1982" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E1982" s="16" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="1983">
+      <c r="A1983" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1983" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1983" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1983" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E1983" s="19" t="n">
+        <v>166.5</v>
+      </c>
+    </row>
+    <row r="1984">
+      <c r="A1984" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1984" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1984" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1984" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E1984" s="16" t="n">
+        <v>166.6</v>
+      </c>
+    </row>
+    <row r="1985">
+      <c r="A1985" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1985" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1985" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1985" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E1985" s="19" t="n">
+        <v>69.8</v>
+      </c>
+    </row>
+    <row r="1986">
+      <c r="A1986" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1986" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1986" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1986" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E1986" s="16" t="n">
+        <v>105.5</v>
+      </c>
+    </row>
+    <row r="1987">
+      <c r="A1987" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1987" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1987" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1987" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E1987" s="19" t="n">
+        <v>156.25</v>
+      </c>
+    </row>
+    <row r="1988">
+      <c r="A1988" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1988" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1988" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1988" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E1988" s="16" t="n">
+        <v>155.55</v>
+      </c>
+    </row>
+    <row r="1989">
+      <c r="A1989" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1989" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1989" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1989" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E1989" s="19" t="n">
+        <v>67.75</v>
+      </c>
+    </row>
+    <row r="1990">
+      <c r="A1990" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1990" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1990" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1990" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E1990" s="16" t="n">
+        <v>100.9</v>
+      </c>
+    </row>
+    <row r="1991">
+      <c r="A1991" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1991" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1991" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1991" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E1991" s="19" t="n">
+        <v>151.95</v>
+      </c>
+    </row>
+    <row r="1992">
+      <c r="A1992" s="20" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1992" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1992" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1992" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E1992" s="16" t="n">
+        <v>151.65</v>
+      </c>
+    </row>
+    <row r="1993">
+      <c r="A1993" s="21" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B1993" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C1993" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D1993" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E1993" s="19" t="n">
+        <v>65.95</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-13
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1993"/>
+  <dimension ref="A1:E2039"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -46435,6 +46435,1064 @@
         <v>65.95</v>
       </c>
     </row>
+    <row r="1994">
+      <c r="A1994" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B1994" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1994" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1994" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E1994" s="16" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="1995">
+      <c r="A1995" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B1995" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1995" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1995" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E1995" s="19" t="n">
+        <v>102.95</v>
+      </c>
+    </row>
+    <row r="1996">
+      <c r="A1996" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B1996" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1996" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1996" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E1996" s="16" t="n">
+        <v>145.95</v>
+      </c>
+    </row>
+    <row r="1997">
+      <c r="A1997" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B1997" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1997" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1997" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E1997" s="19" t="n">
+        <v>147.9</v>
+      </c>
+    </row>
+    <row r="1998">
+      <c r="A1998" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B1998" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1998" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1998" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E1998" s="16" t="n">
+        <v>110.5</v>
+      </c>
+    </row>
+    <row r="1999">
+      <c r="A1999" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B1999" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C1999" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D1999" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E1999" s="19" t="n">
+        <v>94.15000000000001</v>
+      </c>
+    </row>
+    <row r="2000">
+      <c r="A2000" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2000" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2000" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2000" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2000" s="16" t="n">
+        <v>84.05</v>
+      </c>
+    </row>
+    <row r="2001">
+      <c r="A2001" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2001" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2001" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2001" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2001" s="19" t="n">
+        <v>77.45</v>
+      </c>
+    </row>
+    <row r="2002">
+      <c r="A2002" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2002" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2002" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2002" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2002" s="16" t="n">
+        <v>92.2</v>
+      </c>
+    </row>
+    <row r="2003">
+      <c r="A2003" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2003" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2003" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2003" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2003" s="19" t="n">
+        <v>135.05</v>
+      </c>
+    </row>
+    <row r="2004">
+      <c r="A2004" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2004" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2004" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2004" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2004" s="16" t="n">
+        <v>85.25</v>
+      </c>
+    </row>
+    <row r="2005">
+      <c r="A2005" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2005" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2005" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2005" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2005" s="19" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2006">
+      <c r="A2006" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2006" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2006" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2006" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2006" s="16" t="n">
+        <v>181.9</v>
+      </c>
+    </row>
+    <row r="2007">
+      <c r="A2007" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2007" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2007" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2007" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2007" s="19" t="n">
+        <v>180.6</v>
+      </c>
+    </row>
+    <row r="2008">
+      <c r="A2008" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2008" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2008" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2008" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2008" s="16" t="n">
+        <v>78.2</v>
+      </c>
+    </row>
+    <row r="2009">
+      <c r="A2009" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2009" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2009" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2009" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2009" s="19" t="n">
+        <v>120.4</v>
+      </c>
+    </row>
+    <row r="2010">
+      <c r="A2010" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2010" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2010" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2010" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2010" s="16" t="n">
+        <v>171.9</v>
+      </c>
+    </row>
+    <row r="2011">
+      <c r="A2011" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2011" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2011" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2011" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2011" s="19" t="n">
+        <v>172.1</v>
+      </c>
+    </row>
+    <row r="2012">
+      <c r="A2012" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2012" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2012" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2012" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2012" s="16" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2013">
+      <c r="A2013" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2013" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2013" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2013" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2013" s="19" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2014">
+      <c r="A2014" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2014" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2014" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2014" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2014" s="16" t="n">
+        <v>168.5</v>
+      </c>
+    </row>
+    <row r="2015">
+      <c r="A2015" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2015" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2015" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2015" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2015" s="19" t="n">
+        <v>167.7</v>
+      </c>
+    </row>
+    <row r="2016">
+      <c r="A2016" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2016" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2016" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2016" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2016" s="16" t="n">
+        <v>76.09999999999999</v>
+      </c>
+    </row>
+    <row r="2017">
+      <c r="A2017" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2017" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2017" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2017" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2017" s="19" t="n">
+        <v>67.15000000000001</v>
+      </c>
+    </row>
+    <row r="2018">
+      <c r="A2018" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2018" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2018" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2018" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2018" s="16" t="n">
+        <v>93.8</v>
+      </c>
+    </row>
+    <row r="2019">
+      <c r="A2019" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2019" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2019" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2019" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2019" s="19" t="n">
+        <v>135.5</v>
+      </c>
+    </row>
+    <row r="2020">
+      <c r="A2020" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2020" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2020" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2020" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2020" s="16" t="n">
+        <v>136.75</v>
+      </c>
+    </row>
+    <row r="2021">
+      <c r="A2021" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2021" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2021" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2021" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2021" s="19" t="n">
+        <v>103.35</v>
+      </c>
+    </row>
+    <row r="2022">
+      <c r="A2022" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2022" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2022" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2022" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2022" s="16" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2023">
+      <c r="A2023" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2023" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2023" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2023" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2023" s="19" t="n">
+        <v>74.34999999999999</v>
+      </c>
+    </row>
+    <row r="2024">
+      <c r="A2024" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2024" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2024" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2024" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2024" s="16" t="n">
+        <v>69.09999999999999</v>
+      </c>
+    </row>
+    <row r="2025">
+      <c r="A2025" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2025" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2025" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2025" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2025" s="19" t="n">
+        <v>86.40000000000001</v>
+      </c>
+    </row>
+    <row r="2026">
+      <c r="A2026" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2026" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2026" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2026" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2026" s="16" t="n">
+        <v>125.45</v>
+      </c>
+    </row>
+    <row r="2027">
+      <c r="A2027" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2027" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2027" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2027" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2027" s="19" t="n">
+        <v>76.5</v>
+      </c>
+    </row>
+    <row r="2028">
+      <c r="A2028" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2028" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2028" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2028" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2028" s="16" t="n">
+        <v>109.35</v>
+      </c>
+    </row>
+    <row r="2029">
+      <c r="A2029" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2029" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2029" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2029" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2029" s="19" t="n">
+        <v>163.9</v>
+      </c>
+    </row>
+    <row r="2030">
+      <c r="A2030" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2030" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2030" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2030" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2030" s="16" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="2031">
+      <c r="A2031" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2031" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2031" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2031" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2031" s="19" t="n">
+        <v>66.8</v>
+      </c>
+    </row>
+    <row r="2032">
+      <c r="A2032" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2032" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2032" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2032" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2032" s="16" t="n">
+        <v>101.9</v>
+      </c>
+    </row>
+    <row r="2033">
+      <c r="A2033" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2033" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2033" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2033" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2033" s="19" t="n">
+        <v>153.2</v>
+      </c>
+    </row>
+    <row r="2034">
+      <c r="A2034" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2034" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2034" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2034" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2034" s="16" t="n">
+        <v>153.5</v>
+      </c>
+    </row>
+    <row r="2035">
+      <c r="A2035" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2035" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2035" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2035" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2035" s="19" t="n">
+        <v>65.09999999999999</v>
+      </c>
+    </row>
+    <row r="2036">
+      <c r="A2036" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2036" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2036" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2036" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2036" s="16" t="n">
+        <v>97.45</v>
+      </c>
+    </row>
+    <row r="2037">
+      <c r="A2037" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2037" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2037" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2037" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2037" s="19" t="n">
+        <v>148.55</v>
+      </c>
+    </row>
+    <row r="2038">
+      <c r="A2038" s="20" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2038" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2038" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2038" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2038" s="16" t="n">
+        <v>148.5</v>
+      </c>
+    </row>
+    <row r="2039">
+      <c r="A2039" s="21" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B2039" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2039" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2039" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2039" s="19" t="n">
+        <v>64.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-14
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2039"/>
+  <dimension ref="A1:E2085"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -47493,6 +47493,1064 @@
         <v>64.5</v>
       </c>
     </row>
+    <row r="2040">
+      <c r="A2040" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2040" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2040" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2040" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2040" s="16" t="n">
+        <v>76.65000000000001</v>
+      </c>
+    </row>
+    <row r="2041">
+      <c r="A2041" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2041" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2041" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2041" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2041" s="19" t="n">
+        <v>102.55</v>
+      </c>
+    </row>
+    <row r="2042">
+      <c r="A2042" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2042" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2042" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2042" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2042" s="16" t="n">
+        <v>147.25</v>
+      </c>
+    </row>
+    <row r="2043">
+      <c r="A2043" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2043" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2043" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2043" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2043" s="19" t="n">
+        <v>148.65</v>
+      </c>
+    </row>
+    <row r="2044">
+      <c r="A2044" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2044" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2044" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2044" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2044" s="16" t="n">
+        <v>109.75</v>
+      </c>
+    </row>
+    <row r="2045">
+      <c r="A2045" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2045" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2045" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2045" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2045" s="19" t="n">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2046">
+      <c r="A2046" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2046" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2046" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2046" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2046" s="16" t="n">
+        <v>87.7</v>
+      </c>
+    </row>
+    <row r="2047">
+      <c r="A2047" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2047" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2047" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2047" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2047" s="19" t="n">
+        <v>80.8</v>
+      </c>
+    </row>
+    <row r="2048">
+      <c r="A2048" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2048" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2048" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2048" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2048" s="16" t="n">
+        <v>93.65000000000001</v>
+      </c>
+    </row>
+    <row r="2049">
+      <c r="A2049" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2049" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2049" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2049" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2049" s="19" t="n">
+        <v>135.5</v>
+      </c>
+    </row>
+    <row r="2050">
+      <c r="A2050" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2050" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2050" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2050" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2050" s="16" t="n">
+        <v>87.15000000000001</v>
+      </c>
+    </row>
+    <row r="2051">
+      <c r="A2051" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2051" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2051" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2051" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2051" s="19" t="n">
+        <v>131.9</v>
+      </c>
+    </row>
+    <row r="2052">
+      <c r="A2052" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2052" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2052" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2052" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2052" s="16" t="n">
+        <v>178.2</v>
+      </c>
+    </row>
+    <row r="2053">
+      <c r="A2053" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2053" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2053" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2053" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2053" s="19" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="2054">
+      <c r="A2054" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2054" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2054" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2054" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2054" s="16" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2055">
+      <c r="A2055" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2055" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2055" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2055" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2055" s="19" t="n">
+        <v>119.25</v>
+      </c>
+    </row>
+    <row r="2056">
+      <c r="A2056" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2056" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2056" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2056" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2056" s="16" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2057">
+      <c r="A2057" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2057" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2057" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2057" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2057" s="19" t="n">
+        <v>168.5</v>
+      </c>
+    </row>
+    <row r="2058">
+      <c r="A2058" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2058" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2058" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2058" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2058" s="16" t="n">
+        <v>76.65000000000001</v>
+      </c>
+    </row>
+    <row r="2059">
+      <c r="A2059" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2059" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2059" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2059" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2059" s="19" t="n">
+        <v>114.25</v>
+      </c>
+    </row>
+    <row r="2060">
+      <c r="A2060" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2060" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2060" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2060" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2060" s="16" t="n">
+        <v>168.5</v>
+      </c>
+    </row>
+    <row r="2061">
+      <c r="A2061" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2061" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2061" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2061" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2061" s="19" t="n">
+        <v>167.7</v>
+      </c>
+    </row>
+    <row r="2062">
+      <c r="A2062" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2062" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2062" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2062" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2062" s="16" t="n">
+        <v>75.5</v>
+      </c>
+    </row>
+    <row r="2063">
+      <c r="A2063" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2063" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2063" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2063" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2063" s="19" t="n">
+        <v>74.65000000000001</v>
+      </c>
+    </row>
+    <row r="2064">
+      <c r="A2064" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2064" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2064" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2064" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2064" s="16" t="n">
+        <v>92.8</v>
+      </c>
+    </row>
+    <row r="2065">
+      <c r="A2065" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2065" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2065" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2065" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2065" s="19" t="n">
+        <v>136.55</v>
+      </c>
+    </row>
+    <row r="2066">
+      <c r="A2066" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2066" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2066" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2066" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2066" s="16" t="n">
+        <v>137.8</v>
+      </c>
+    </row>
+    <row r="2067">
+      <c r="A2067" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2067" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2067" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2067" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2067" s="19" t="n">
+        <v>102.9</v>
+      </c>
+    </row>
+    <row r="2068">
+      <c r="A2068" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2068" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2068" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2068" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2068" s="16" t="n">
+        <v>82.5</v>
+      </c>
+    </row>
+    <row r="2069">
+      <c r="A2069" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2069" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2069" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2069" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2069" s="19" t="n">
+        <v>76.34999999999999</v>
+      </c>
+    </row>
+    <row r="2070">
+      <c r="A2070" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2070" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2070" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2070" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2070" s="16" t="n">
+        <v>70.95</v>
+      </c>
+    </row>
+    <row r="2071">
+      <c r="A2071" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2071" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2071" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2071" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2071" s="19" t="n">
+        <v>88.65000000000001</v>
+      </c>
+    </row>
+    <row r="2072">
+      <c r="A2072" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2072" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2072" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2072" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2072" s="16" t="n">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2073">
+      <c r="A2073" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2073" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2073" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2073" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2073" s="19" t="n">
+        <v>76.59999999999999</v>
+      </c>
+    </row>
+    <row r="2074">
+      <c r="A2074" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2074" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2074" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2074" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2074" s="16" t="n">
+        <v>111.3</v>
+      </c>
+    </row>
+    <row r="2075">
+      <c r="A2075" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2075" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2075" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2075" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2075" s="19" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2076">
+      <c r="A2076" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2076" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2076" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2076" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2076" s="16" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2077">
+      <c r="A2077" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2077" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2077" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2077" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2077" s="19" t="n">
+        <v>66.59999999999999</v>
+      </c>
+    </row>
+    <row r="2078">
+      <c r="A2078" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2078" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2078" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2078" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2078" s="16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2079">
+      <c r="A2079" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2079" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2079" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2079" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2079" s="19" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2080">
+      <c r="A2080" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2080" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2080" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2080" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2080" s="16" t="n">
+        <v>153.25</v>
+      </c>
+    </row>
+    <row r="2081">
+      <c r="A2081" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2081" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2081" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2081" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2081" s="19" t="n">
+        <v>64.5</v>
+      </c>
+    </row>
+    <row r="2082">
+      <c r="A2082" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2082" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2082" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2082" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2082" s="16" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2083">
+      <c r="A2083" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2083" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2083" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2083" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2083" s="19" t="n">
+        <v>150.5</v>
+      </c>
+    </row>
+    <row r="2084">
+      <c r="A2084" s="20" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2084" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2084" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2084" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2084" s="16" t="n">
+        <v>148.5</v>
+      </c>
+    </row>
+    <row r="2085">
+      <c r="A2085" s="21" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B2085" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2085" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2085" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2085" s="19" t="n">
+        <v>63.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-15
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2085"/>
+  <dimension ref="A1:E2131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -48551,6 +48551,1064 @@
         <v>63.5</v>
       </c>
     </row>
+    <row r="2086">
+      <c r="A2086" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2086" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2086" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2086" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2086" s="16" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2087">
+      <c r="A2087" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2087" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2087" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2087" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2087" s="19" t="n">
+        <v>103.1</v>
+      </c>
+    </row>
+    <row r="2088">
+      <c r="A2088" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2088" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2088" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2088" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2088" s="16" t="n">
+        <v>151.95</v>
+      </c>
+    </row>
+    <row r="2089">
+      <c r="A2089" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2089" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2089" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2089" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2089" s="19" t="n">
+        <v>155.65</v>
+      </c>
+    </row>
+    <row r="2090">
+      <c r="A2090" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2090" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2090" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2090" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2090" s="16" t="n">
+        <v>114.5</v>
+      </c>
+    </row>
+    <row r="2091">
+      <c r="A2091" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2091" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2091" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2091" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2091" s="19" t="n">
+        <v>87.05</v>
+      </c>
+    </row>
+    <row r="2092">
+      <c r="A2092" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2092" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2092" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2092" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2092" s="16" t="n">
+        <v>84.3</v>
+      </c>
+    </row>
+    <row r="2093">
+      <c r="A2093" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2093" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2093" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2093" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2093" s="19" t="n">
+        <v>77.7</v>
+      </c>
+    </row>
+    <row r="2094">
+      <c r="A2094" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2094" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2094" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2094" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2094" s="16" t="n">
+        <v>93.59999999999999</v>
+      </c>
+    </row>
+    <row r="2095">
+      <c r="A2095" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2095" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2095" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2095" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2095" s="19" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2096">
+      <c r="A2096" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2096" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2096" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2096" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2096" s="16" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2097">
+      <c r="A2097" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2097" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2097" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2097" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2097" s="19" t="n">
+        <v>131.9</v>
+      </c>
+    </row>
+    <row r="2098">
+      <c r="A2098" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2098" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2098" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2098" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2098" s="16" t="n">
+        <v>178.2</v>
+      </c>
+    </row>
+    <row r="2099">
+      <c r="A2099" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2099" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2099" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2099" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2099" s="19" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="2100">
+      <c r="A2100" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2100" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2100" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2100" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2100" s="16" t="n">
+        <v>76.59999999999999</v>
+      </c>
+    </row>
+    <row r="2101">
+      <c r="A2101" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2101" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2101" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2101" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2101" s="19" t="n">
+        <v>118.5</v>
+      </c>
+    </row>
+    <row r="2102">
+      <c r="A2102" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2102" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2102" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2102" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2102" s="16" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2103">
+      <c r="A2103" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2103" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2103" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2103" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2103" s="19" t="n">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2104">
+      <c r="A2104" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2104" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2104" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2104" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2104" s="16" t="n">
+        <v>75.3</v>
+      </c>
+    </row>
+    <row r="2105">
+      <c r="A2105" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2105" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2105" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2105" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2105" s="19" t="n">
+        <v>114.25</v>
+      </c>
+    </row>
+    <row r="2106">
+      <c r="A2106" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2106" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2106" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2106" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2106" s="16" t="n">
+        <v>168.5</v>
+      </c>
+    </row>
+    <row r="2107">
+      <c r="A2107" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2107" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2107" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2107" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2107" s="19" t="n">
+        <v>167.7</v>
+      </c>
+    </row>
+    <row r="2108">
+      <c r="A2108" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2108" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2108" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2108" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2108" s="16" t="n">
+        <v>73.75</v>
+      </c>
+    </row>
+    <row r="2109">
+      <c r="A2109" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2109" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2109" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2109" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2109" s="19" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="2110">
+      <c r="A2110" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2110" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2110" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2110" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2110" s="16" t="n">
+        <v>91.5</v>
+      </c>
+    </row>
+    <row r="2111">
+      <c r="A2111" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2111" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2111" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2111" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2111" s="19" t="n">
+        <v>143.15</v>
+      </c>
+    </row>
+    <row r="2112">
+      <c r="A2112" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2112" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2112" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2112" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2112" s="16" t="n">
+        <v>144.75</v>
+      </c>
+    </row>
+    <row r="2113">
+      <c r="A2113" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2113" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2113" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2113" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2113" s="19" t="n">
+        <v>106.05</v>
+      </c>
+    </row>
+    <row r="2114">
+      <c r="A2114" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2114" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2114" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2114" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2114" s="16" t="n">
+        <v>76.5</v>
+      </c>
+    </row>
+    <row r="2115">
+      <c r="A2115" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2115" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2115" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2115" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2115" s="19" t="n">
+        <v>70.75</v>
+      </c>
+    </row>
+    <row r="2116">
+      <c r="A2116" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2116" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2116" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2116" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2116" s="16" t="n">
+        <v>65.75</v>
+      </c>
+    </row>
+    <row r="2117">
+      <c r="A2117" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2117" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2117" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2117" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2117" s="19" t="n">
+        <v>87.25</v>
+      </c>
+    </row>
+    <row r="2118">
+      <c r="A2118" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2118" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2118" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2118" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2118" s="16" t="n">
+        <v>131.6</v>
+      </c>
+    </row>
+    <row r="2119">
+      <c r="A2119" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2119" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2119" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2119" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2119" s="19" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2120">
+      <c r="A2120" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2120" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2120" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2120" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2120" s="16" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2121">
+      <c r="A2121" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2121" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2121" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2121" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2121" s="19" t="n">
+        <v>159.25</v>
+      </c>
+    </row>
+    <row r="2122">
+      <c r="A2122" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2122" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2122" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2122" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2122" s="16" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="2123">
+      <c r="A2123" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2123" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2123" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2123" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2123" s="19" t="n">
+        <v>66.5</v>
+      </c>
+    </row>
+    <row r="2124">
+      <c r="A2124" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2124" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2124" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2124" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2124" s="16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2125">
+      <c r="A2125" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2125" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2125" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2125" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2125" s="19" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2126">
+      <c r="A2126" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2126" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2126" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2126" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2126" s="16" t="n">
+        <v>152.25</v>
+      </c>
+    </row>
+    <row r="2127">
+      <c r="A2127" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2127" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2127" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2127" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2127" s="19" t="n">
+        <v>63.5</v>
+      </c>
+    </row>
+    <row r="2128">
+      <c r="A2128" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2128" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2128" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2128" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2128" s="16" t="n">
+        <v>96.59999999999999</v>
+      </c>
+    </row>
+    <row r="2129">
+      <c r="A2129" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2129" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2129" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2129" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2129" s="19" t="n">
+        <v>150.5</v>
+      </c>
+    </row>
+    <row r="2130">
+      <c r="A2130" s="20" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2130" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2130" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2130" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2130" s="16" t="n">
+        <v>148.5</v>
+      </c>
+    </row>
+    <row r="2131">
+      <c r="A2131" s="21" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B2131" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2131" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2131" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2131" s="19" t="n">
+        <v>62.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-16
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2131"/>
+  <dimension ref="A1:E2177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -49609,6 +49609,1064 @@
         <v>62.6</v>
       </c>
     </row>
+    <row r="2132">
+      <c r="A2132" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2132" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2132" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2132" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2132" s="16" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2133">
+      <c r="A2133" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2133" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2133" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2133" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2133" s="19" t="n">
+        <v>103.1</v>
+      </c>
+    </row>
+    <row r="2134">
+      <c r="A2134" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2134" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2134" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2134" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2134" s="16" t="n">
+        <v>151.95</v>
+      </c>
+    </row>
+    <row r="2135">
+      <c r="A2135" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2135" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2135" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2135" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2135" s="19" t="n">
+        <v>155.65</v>
+      </c>
+    </row>
+    <row r="2136">
+      <c r="A2136" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2136" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2136" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2136" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2136" s="16" t="n">
+        <v>114.5</v>
+      </c>
+    </row>
+    <row r="2137">
+      <c r="A2137" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2137" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2137" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2137" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2137" s="19" t="n">
+        <v>87.05</v>
+      </c>
+    </row>
+    <row r="2138">
+      <c r="A2138" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2138" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2138" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2138" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2138" s="16" t="n">
+        <v>84.3</v>
+      </c>
+    </row>
+    <row r="2139">
+      <c r="A2139" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2139" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2139" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2139" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2139" s="19" t="n">
+        <v>77.7</v>
+      </c>
+    </row>
+    <row r="2140">
+      <c r="A2140" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2140" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2140" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2140" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2140" s="16" t="n">
+        <v>93.59999999999999</v>
+      </c>
+    </row>
+    <row r="2141">
+      <c r="A2141" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2141" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2141" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2141" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2141" s="19" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2142">
+      <c r="A2142" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2142" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2142" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2142" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2142" s="16" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2143">
+      <c r="A2143" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2143" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2143" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2143" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2143" s="19" t="n">
+        <v>131.9</v>
+      </c>
+    </row>
+    <row r="2144">
+      <c r="A2144" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2144" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2144" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2144" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2144" s="16" t="n">
+        <v>178.2</v>
+      </c>
+    </row>
+    <row r="2145">
+      <c r="A2145" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2145" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2145" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2145" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2145" s="19" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="2146">
+      <c r="A2146" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2146" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2146" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2146" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2146" s="16" t="n">
+        <v>76.59999999999999</v>
+      </c>
+    </row>
+    <row r="2147">
+      <c r="A2147" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2147" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2147" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2147" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2147" s="19" t="n">
+        <v>118.5</v>
+      </c>
+    </row>
+    <row r="2148">
+      <c r="A2148" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2148" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2148" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2148" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2148" s="16" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2149">
+      <c r="A2149" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2149" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2149" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2149" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2149" s="19" t="n">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2150">
+      <c r="A2150" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2150" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2150" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2150" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2150" s="16" t="n">
+        <v>75.3</v>
+      </c>
+    </row>
+    <row r="2151">
+      <c r="A2151" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2151" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2151" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2151" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2151" s="19" t="n">
+        <v>114.25</v>
+      </c>
+    </row>
+    <row r="2152">
+      <c r="A2152" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2152" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2152" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2152" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2152" s="16" t="n">
+        <v>168.5</v>
+      </c>
+    </row>
+    <row r="2153">
+      <c r="A2153" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2153" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2153" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2153" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2153" s="19" t="n">
+        <v>167.7</v>
+      </c>
+    </row>
+    <row r="2154">
+      <c r="A2154" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2154" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2154" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2154" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2154" s="16" t="n">
+        <v>73.75</v>
+      </c>
+    </row>
+    <row r="2155">
+      <c r="A2155" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2155" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2155" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2155" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2155" s="19" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="2156">
+      <c r="A2156" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2156" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2156" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2156" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2156" s="16" t="n">
+        <v>91.5</v>
+      </c>
+    </row>
+    <row r="2157">
+      <c r="A2157" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2157" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2157" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2157" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2157" s="19" t="n">
+        <v>143.15</v>
+      </c>
+    </row>
+    <row r="2158">
+      <c r="A2158" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2158" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2158" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2158" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2158" s="16" t="n">
+        <v>144.75</v>
+      </c>
+    </row>
+    <row r="2159">
+      <c r="A2159" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2159" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2159" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2159" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2159" s="19" t="n">
+        <v>106.05</v>
+      </c>
+    </row>
+    <row r="2160">
+      <c r="A2160" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2160" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2160" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2160" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2160" s="16" t="n">
+        <v>76.5</v>
+      </c>
+    </row>
+    <row r="2161">
+      <c r="A2161" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2161" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2161" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2161" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2161" s="19" t="n">
+        <v>70.75</v>
+      </c>
+    </row>
+    <row r="2162">
+      <c r="A2162" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2162" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2162" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2162" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2162" s="16" t="n">
+        <v>65.75</v>
+      </c>
+    </row>
+    <row r="2163">
+      <c r="A2163" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2163" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2163" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2163" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2163" s="19" t="n">
+        <v>87.25</v>
+      </c>
+    </row>
+    <row r="2164">
+      <c r="A2164" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2164" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2164" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2164" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2164" s="16" t="n">
+        <v>131.6</v>
+      </c>
+    </row>
+    <row r="2165">
+      <c r="A2165" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2165" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2165" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2165" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2165" s="19" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2166">
+      <c r="A2166" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2166" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2166" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2166" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2166" s="16" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2167">
+      <c r="A2167" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2167" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2167" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2167" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2167" s="19" t="n">
+        <v>159.25</v>
+      </c>
+    </row>
+    <row r="2168">
+      <c r="A2168" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2168" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2168" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2168" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2168" s="16" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="2169">
+      <c r="A2169" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2169" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2169" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2169" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2169" s="19" t="n">
+        <v>66.5</v>
+      </c>
+    </row>
+    <row r="2170">
+      <c r="A2170" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2170" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2170" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2170" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2170" s="16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2171">
+      <c r="A2171" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2171" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2171" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2171" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2171" s="19" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2172">
+      <c r="A2172" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2172" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2172" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2172" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2172" s="16" t="n">
+        <v>152.25</v>
+      </c>
+    </row>
+    <row r="2173">
+      <c r="A2173" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2173" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2173" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2173" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2173" s="19" t="n">
+        <v>63.5</v>
+      </c>
+    </row>
+    <row r="2174">
+      <c r="A2174" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2174" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2174" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2174" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2174" s="16" t="n">
+        <v>96.59999999999999</v>
+      </c>
+    </row>
+    <row r="2175">
+      <c r="A2175" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2175" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2175" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2175" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2175" s="19" t="n">
+        <v>150.5</v>
+      </c>
+    </row>
+    <row r="2176">
+      <c r="A2176" s="20" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2176" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2176" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2176" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2176" s="16" t="n">
+        <v>148.5</v>
+      </c>
+    </row>
+    <row r="2177">
+      <c r="A2177" s="21" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B2177" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2177" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2177" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2177" s="19" t="n">
+        <v>62.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-17
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2177"/>
+  <dimension ref="A1:E2223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -50667,6 +50667,1064 @@
         <v>62.6</v>
       </c>
     </row>
+    <row r="2178">
+      <c r="A2178" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2178" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2178" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2178" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2178" s="16" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2179">
+      <c r="A2179" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2179" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2179" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2179" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2179" s="19" t="n">
+        <v>103.1</v>
+      </c>
+    </row>
+    <row r="2180">
+      <c r="A2180" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2180" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2180" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2180" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2180" s="16" t="n">
+        <v>151.95</v>
+      </c>
+    </row>
+    <row r="2181">
+      <c r="A2181" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2181" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2181" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2181" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2181" s="19" t="n">
+        <v>155.65</v>
+      </c>
+    </row>
+    <row r="2182">
+      <c r="A2182" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2182" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2182" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2182" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2182" s="16" t="n">
+        <v>114.5</v>
+      </c>
+    </row>
+    <row r="2183">
+      <c r="A2183" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2183" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2183" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2183" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2183" s="19" t="n">
+        <v>87.05</v>
+      </c>
+    </row>
+    <row r="2184">
+      <c r="A2184" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2184" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2184" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2184" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2184" s="16" t="n">
+        <v>84.3</v>
+      </c>
+    </row>
+    <row r="2185">
+      <c r="A2185" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2185" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2185" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2185" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2185" s="19" t="n">
+        <v>77.7</v>
+      </c>
+    </row>
+    <row r="2186">
+      <c r="A2186" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2186" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2186" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2186" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2186" s="16" t="n">
+        <v>93.59999999999999</v>
+      </c>
+    </row>
+    <row r="2187">
+      <c r="A2187" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2187" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2187" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2187" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2187" s="19" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2188">
+      <c r="A2188" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2188" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2188" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2188" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2188" s="16" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2189">
+      <c r="A2189" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2189" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2189" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2189" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2189" s="19" t="n">
+        <v>131.9</v>
+      </c>
+    </row>
+    <row r="2190">
+      <c r="A2190" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2190" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2190" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2190" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2190" s="16" t="n">
+        <v>178.2</v>
+      </c>
+    </row>
+    <row r="2191">
+      <c r="A2191" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2191" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2191" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2191" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2191" s="19" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="2192">
+      <c r="A2192" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2192" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2192" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2192" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2192" s="16" t="n">
+        <v>76.59999999999999</v>
+      </c>
+    </row>
+    <row r="2193">
+      <c r="A2193" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2193" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2193" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2193" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2193" s="19" t="n">
+        <v>118.5</v>
+      </c>
+    </row>
+    <row r="2194">
+      <c r="A2194" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2194" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2194" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2194" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2194" s="16" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2195">
+      <c r="A2195" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2195" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2195" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2195" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2195" s="19" t="n">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2196">
+      <c r="A2196" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2196" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2196" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2196" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2196" s="16" t="n">
+        <v>75.3</v>
+      </c>
+    </row>
+    <row r="2197">
+      <c r="A2197" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2197" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2197" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2197" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2197" s="19" t="n">
+        <v>114.25</v>
+      </c>
+    </row>
+    <row r="2198">
+      <c r="A2198" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2198" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2198" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2198" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2198" s="16" t="n">
+        <v>168.5</v>
+      </c>
+    </row>
+    <row r="2199">
+      <c r="A2199" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2199" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2199" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2199" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2199" s="19" t="n">
+        <v>167.7</v>
+      </c>
+    </row>
+    <row r="2200">
+      <c r="A2200" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2200" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2200" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2200" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2200" s="16" t="n">
+        <v>73.75</v>
+      </c>
+    </row>
+    <row r="2201">
+      <c r="A2201" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2201" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2201" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2201" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2201" s="19" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="2202">
+      <c r="A2202" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2202" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2202" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2202" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2202" s="16" t="n">
+        <v>91.5</v>
+      </c>
+    </row>
+    <row r="2203">
+      <c r="A2203" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2203" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2203" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2203" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2203" s="19" t="n">
+        <v>143.15</v>
+      </c>
+    </row>
+    <row r="2204">
+      <c r="A2204" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2204" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2204" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2204" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2204" s="16" t="n">
+        <v>144.75</v>
+      </c>
+    </row>
+    <row r="2205">
+      <c r="A2205" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2205" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2205" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2205" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2205" s="19" t="n">
+        <v>106.05</v>
+      </c>
+    </row>
+    <row r="2206">
+      <c r="A2206" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2206" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2206" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2206" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2206" s="16" t="n">
+        <v>76.5</v>
+      </c>
+    </row>
+    <row r="2207">
+      <c r="A2207" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2207" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2207" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2207" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2207" s="19" t="n">
+        <v>70.75</v>
+      </c>
+    </row>
+    <row r="2208">
+      <c r="A2208" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2208" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2208" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2208" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2208" s="16" t="n">
+        <v>65.75</v>
+      </c>
+    </row>
+    <row r="2209">
+      <c r="A2209" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2209" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2209" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2209" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2209" s="19" t="n">
+        <v>87.25</v>
+      </c>
+    </row>
+    <row r="2210">
+      <c r="A2210" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2210" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2210" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2210" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2210" s="16" t="n">
+        <v>131.6</v>
+      </c>
+    </row>
+    <row r="2211">
+      <c r="A2211" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2211" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2211" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2211" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2211" s="19" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2212">
+      <c r="A2212" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2212" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2212" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2212" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2212" s="16" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2213">
+      <c r="A2213" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2213" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2213" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2213" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2213" s="19" t="n">
+        <v>159.25</v>
+      </c>
+    </row>
+    <row r="2214">
+      <c r="A2214" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2214" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2214" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2214" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2214" s="16" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="2215">
+      <c r="A2215" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2215" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2215" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2215" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2215" s="19" t="n">
+        <v>66.5</v>
+      </c>
+    </row>
+    <row r="2216">
+      <c r="A2216" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2216" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2216" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2216" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2216" s="16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2217">
+      <c r="A2217" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2217" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2217" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2217" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2217" s="19" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2218">
+      <c r="A2218" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2218" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2218" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2218" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2218" s="16" t="n">
+        <v>152.25</v>
+      </c>
+    </row>
+    <row r="2219">
+      <c r="A2219" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2219" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2219" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2219" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2219" s="19" t="n">
+        <v>63.5</v>
+      </c>
+    </row>
+    <row r="2220">
+      <c r="A2220" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2220" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2220" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2220" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2220" s="16" t="n">
+        <v>96.59999999999999</v>
+      </c>
+    </row>
+    <row r="2221">
+      <c r="A2221" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2221" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2221" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2221" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2221" s="19" t="n">
+        <v>150.5</v>
+      </c>
+    </row>
+    <row r="2222">
+      <c r="A2222" s="20" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2222" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2222" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2222" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2222" s="16" t="n">
+        <v>148.5</v>
+      </c>
+    </row>
+    <row r="2223">
+      <c r="A2223" s="21" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B2223" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2223" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2223" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2223" s="19" t="n">
+        <v>62.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-18
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2223"/>
+  <dimension ref="A1:E2269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -51725,6 +51725,1064 @@
         <v>62.6</v>
       </c>
     </row>
+    <row r="2224">
+      <c r="A2224" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2224" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2224" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2224" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2224" s="16" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2225">
+      <c r="A2225" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2225" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2225" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2225" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2225" s="19" t="n">
+        <v>105.5</v>
+      </c>
+    </row>
+    <row r="2226">
+      <c r="A2226" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2226" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2226" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2226" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2226" s="16" t="n">
+        <v>153.15</v>
+      </c>
+    </row>
+    <row r="2227">
+      <c r="A2227" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2227" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2227" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2227" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2227" s="19" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="2228">
+      <c r="A2228" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2228" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2228" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2228" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2228" s="16" t="n">
+        <v>114.25</v>
+      </c>
+    </row>
+    <row r="2229">
+      <c r="A2229" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2229" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2229" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2229" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2229" s="19" t="n">
+        <v>88.25</v>
+      </c>
+    </row>
+    <row r="2230">
+      <c r="A2230" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2230" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2230" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2230" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2230" s="16" t="n">
+        <v>87.75</v>
+      </c>
+    </row>
+    <row r="2231">
+      <c r="A2231" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2231" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2231" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2231" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2231" s="19" t="n">
+        <v>80.90000000000001</v>
+      </c>
+    </row>
+    <row r="2232">
+      <c r="A2232" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2232" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2232" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2232" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2232" s="16" t="n">
+        <v>94.40000000000001</v>
+      </c>
+    </row>
+    <row r="2233">
+      <c r="A2233" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2233" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2233" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2233" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2233" s="19" t="n">
+        <v>141.1</v>
+      </c>
+    </row>
+    <row r="2234">
+      <c r="A2234" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2234" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2234" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2234" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2234" s="16" t="n">
+        <v>85.59999999999999</v>
+      </c>
+    </row>
+    <row r="2235">
+      <c r="A2235" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2235" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2235" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2235" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2235" s="19" t="n">
+        <v>134.9</v>
+      </c>
+    </row>
+    <row r="2236">
+      <c r="A2236" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2236" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2236" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2236" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2236" s="16" t="n">
+        <v>178.2</v>
+      </c>
+    </row>
+    <row r="2237">
+      <c r="A2237" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2237" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2237" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2237" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2237" s="19" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="2238">
+      <c r="A2238" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2238" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2238" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2238" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2238" s="16" t="n">
+        <v>74.84999999999999</v>
+      </c>
+    </row>
+    <row r="2239">
+      <c r="A2239" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2239" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2239" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2239" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2239" s="19" t="n">
+        <v>120.45</v>
+      </c>
+    </row>
+    <row r="2240">
+      <c r="A2240" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2240" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2240" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2240" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2240" s="16" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2241">
+      <c r="A2241" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2241" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2241" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2241" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2241" s="19" t="n">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2242">
+      <c r="A2242" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2242" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2242" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2242" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2242" s="16" t="n">
+        <v>72.25</v>
+      </c>
+    </row>
+    <row r="2243">
+      <c r="A2243" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2243" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2243" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2243" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2243" s="19" t="n">
+        <v>114.25</v>
+      </c>
+    </row>
+    <row r="2244">
+      <c r="A2244" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2244" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2244" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2244" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2244" s="16" t="n">
+        <v>168.5</v>
+      </c>
+    </row>
+    <row r="2245">
+      <c r="A2245" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2245" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2245" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2245" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2245" s="19" t="n">
+        <v>167.7</v>
+      </c>
+    </row>
+    <row r="2246">
+      <c r="A2246" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2246" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2246" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2246" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2246" s="16" t="n">
+        <v>71.59999999999999</v>
+      </c>
+    </row>
+    <row r="2247">
+      <c r="A2247" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2247" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2247" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2247" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2247" s="19" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="2248">
+      <c r="A2248" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2248" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2248" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2248" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2248" s="16" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2249">
+      <c r="A2249" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2249" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2249" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2249" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2249" s="19" t="n">
+        <v>143.5</v>
+      </c>
+    </row>
+    <row r="2250">
+      <c r="A2250" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2250" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2250" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2250" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2250" s="16" t="n">
+        <v>141.2</v>
+      </c>
+    </row>
+    <row r="2251">
+      <c r="A2251" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2251" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2251" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2251" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2251" s="19" t="n">
+        <v>104.45</v>
+      </c>
+    </row>
+    <row r="2252">
+      <c r="A2252" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2252" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2252" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2252" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2252" s="16" t="n">
+        <v>79.25</v>
+      </c>
+    </row>
+    <row r="2253">
+      <c r="A2253" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2253" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2253" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2253" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2253" s="19" t="n">
+        <v>74.59999999999999</v>
+      </c>
+    </row>
+    <row r="2254">
+      <c r="A2254" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2254" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2254" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2254" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2254" s="16" t="n">
+        <v>69.3</v>
+      </c>
+    </row>
+    <row r="2255">
+      <c r="A2255" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2255" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2255" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2255" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2255" s="19" t="n">
+        <v>89.05</v>
+      </c>
+    </row>
+    <row r="2256">
+      <c r="A2256" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2256" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2256" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2256" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2256" s="16" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2257">
+      <c r="A2257" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2257" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2257" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2257" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2257" s="19" t="n">
+        <v>74.40000000000001</v>
+      </c>
+    </row>
+    <row r="2258">
+      <c r="A2258" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2258" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2258" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2258" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2258" s="16" t="n">
+        <v>116.2</v>
+      </c>
+    </row>
+    <row r="2259">
+      <c r="A2259" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2259" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2259" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2259" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2259" s="19" t="n">
+        <v>159.25</v>
+      </c>
+    </row>
+    <row r="2260">
+      <c r="A2260" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2260" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2260" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2260" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2260" s="16" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="2261">
+      <c r="A2261" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2261" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2261" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2261" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2261" s="19" t="n">
+        <v>66.09999999999999</v>
+      </c>
+    </row>
+    <row r="2262">
+      <c r="A2262" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2262" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2262" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2262" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2262" s="16" t="n">
+        <v>101.25</v>
+      </c>
+    </row>
+    <row r="2263">
+      <c r="A2263" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2263" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2263" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2263" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2263" s="19" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2264">
+      <c r="A2264" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2264" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2264" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2264" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2264" s="16" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2265">
+      <c r="A2265" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2265" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2265" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2265" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2265" s="19" t="n">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="2266">
+      <c r="A2266" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2266" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2266" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2266" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2266" s="16" t="n">
+        <v>96.5</v>
+      </c>
+    </row>
+    <row r="2267">
+      <c r="A2267" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2267" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2267" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2267" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2267" s="19" t="n">
+        <v>150.5</v>
+      </c>
+    </row>
+    <row r="2268">
+      <c r="A2268" s="20" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2268" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2268" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2268" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2268" s="16" t="n">
+        <v>148.5</v>
+      </c>
+    </row>
+    <row r="2269">
+      <c r="A2269" s="21" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2269" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2269" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2269" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2269" s="19" t="n">
+        <v>61.3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-19
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2269"/>
+  <dimension ref="A1:E2315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -52783,6 +52783,1064 @@
         <v>61.3</v>
       </c>
     </row>
+    <row r="2270">
+      <c r="A2270" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2270" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2270" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2270" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2270" s="16" t="n">
+        <v>78.45</v>
+      </c>
+    </row>
+    <row r="2271">
+      <c r="A2271" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2271" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2271" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2271" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2271" s="19" t="n">
+        <v>115.6</v>
+      </c>
+    </row>
+    <row r="2272">
+      <c r="A2272" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2272" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2272" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2272" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2272" s="16" t="n">
+        <v>155.1</v>
+      </c>
+    </row>
+    <row r="2273">
+      <c r="A2273" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2273" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2273" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2273" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2273" s="19" t="n">
+        <v>158.2</v>
+      </c>
+    </row>
+    <row r="2274">
+      <c r="A2274" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2274" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2274" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2274" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2274" s="16" t="n">
+        <v>118.9</v>
+      </c>
+    </row>
+    <row r="2275">
+      <c r="A2275" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2275" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2275" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2275" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2275" s="19" t="n">
+        <v>89.90000000000001</v>
+      </c>
+    </row>
+    <row r="2276">
+      <c r="A2276" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2276" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2276" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2276" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2276" s="16" t="n">
+        <v>88.25</v>
+      </c>
+    </row>
+    <row r="2277">
+      <c r="A2277" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2277" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2277" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2277" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2277" s="19" t="n">
+        <v>81.34999999999999</v>
+      </c>
+    </row>
+    <row r="2278">
+      <c r="A2278" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2278" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2278" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2278" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2278" s="16" t="n">
+        <v>98.55</v>
+      </c>
+    </row>
+    <row r="2279">
+      <c r="A2279" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2279" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2279" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2279" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2279" s="19" t="n">
+        <v>144.35</v>
+      </c>
+    </row>
+    <row r="2280">
+      <c r="A2280" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2280" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2280" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2280" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2280" s="16" t="n">
+        <v>86.5</v>
+      </c>
+    </row>
+    <row r="2281">
+      <c r="A2281" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2281" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2281" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2281" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2281" s="19" t="n">
+        <v>135.25</v>
+      </c>
+    </row>
+    <row r="2282">
+      <c r="A2282" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2282" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2282" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2282" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2282" s="16" t="n">
+        <v>181.5</v>
+      </c>
+    </row>
+    <row r="2283">
+      <c r="A2283" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2283" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2283" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2283" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2283" s="19" t="n">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2284">
+      <c r="A2284" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2284" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2284" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2284" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2284" s="16" t="n">
+        <v>74.84999999999999</v>
+      </c>
+    </row>
+    <row r="2285">
+      <c r="A2285" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2285" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2285" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2285" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2285" s="19" t="n">
+        <v>120.45</v>
+      </c>
+    </row>
+    <row r="2286">
+      <c r="A2286" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2286" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2286" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2286" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2286" s="16" t="n">
+        <v>172.5</v>
+      </c>
+    </row>
+    <row r="2287">
+      <c r="A2287" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2287" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2287" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2287" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2287" s="19" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="2288">
+      <c r="A2288" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2288" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2288" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2288" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2288" s="16" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2289">
+      <c r="A2289" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2289" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2289" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2289" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2289" s="19" t="n">
+        <v>114.25</v>
+      </c>
+    </row>
+    <row r="2290">
+      <c r="A2290" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2290" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2290" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2290" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2290" s="16" t="n">
+        <v>168.6</v>
+      </c>
+    </row>
+    <row r="2291">
+      <c r="A2291" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2291" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2291" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2291" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2291" s="19" t="n">
+        <v>169.15</v>
+      </c>
+    </row>
+    <row r="2292">
+      <c r="A2292" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2292" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2292" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2292" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2292" s="16" t="n">
+        <v>71.59999999999999</v>
+      </c>
+    </row>
+    <row r="2293">
+      <c r="A2293" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2293" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2293" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2293" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2293" s="19" t="n">
+        <v>74.75</v>
+      </c>
+    </row>
+    <row r="2294">
+      <c r="A2294" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2294" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2294" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2294" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2294" s="16" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2295">
+      <c r="A2295" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2295" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2295" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2295" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2295" s="19" t="n">
+        <v>146.8</v>
+      </c>
+    </row>
+    <row r="2296">
+      <c r="A2296" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2296" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2296" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2296" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2296" s="16" t="n">
+        <v>147.15</v>
+      </c>
+    </row>
+    <row r="2297">
+      <c r="A2297" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2297" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2297" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2297" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2297" s="19" t="n">
+        <v>109.75</v>
+      </c>
+    </row>
+    <row r="2298">
+      <c r="A2298" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2298" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2298" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2298" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2298" s="16" t="n">
+        <v>83.25</v>
+      </c>
+    </row>
+    <row r="2299">
+      <c r="A2299" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2299" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2299" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2299" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2299" s="19" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2300">
+      <c r="A2300" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2300" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2300" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2300" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2300" s="16" t="n">
+        <v>72.45</v>
+      </c>
+    </row>
+    <row r="2301">
+      <c r="A2301" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2301" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2301" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2301" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2301" s="19" t="n">
+        <v>93.34999999999999</v>
+      </c>
+    </row>
+    <row r="2302">
+      <c r="A2302" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2302" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2302" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2302" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2302" s="16" t="n">
+        <v>134.85</v>
+      </c>
+    </row>
+    <row r="2303">
+      <c r="A2303" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2303" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2303" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2303" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2303" s="19" t="n">
+        <v>77.90000000000001</v>
+      </c>
+    </row>
+    <row r="2304">
+      <c r="A2304" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2304" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2304" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2304" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2304" s="16" t="n">
+        <v>118.1</v>
+      </c>
+    </row>
+    <row r="2305">
+      <c r="A2305" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2305" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2305" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2305" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2305" s="19" t="n">
+        <v>165.1</v>
+      </c>
+    </row>
+    <row r="2306">
+      <c r="A2306" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2306" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2306" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2306" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2306" s="16" t="n">
+        <v>165.4</v>
+      </c>
+    </row>
+    <row r="2307">
+      <c r="A2307" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2307" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2307" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2307" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2307" s="19" t="n">
+        <v>66.09999999999999</v>
+      </c>
+    </row>
+    <row r="2308">
+      <c r="A2308" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2308" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2308" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2308" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2308" s="16" t="n">
+        <v>101.25</v>
+      </c>
+    </row>
+    <row r="2309">
+      <c r="A2309" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2309" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2309" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2309" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2309" s="19" t="n">
+        <v>154.5</v>
+      </c>
+    </row>
+    <row r="2310">
+      <c r="A2310" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2310" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2310" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2310" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2310" s="16" t="n">
+        <v>154.55</v>
+      </c>
+    </row>
+    <row r="2311">
+      <c r="A2311" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2311" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2311" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2311" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2311" s="19" t="n">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="2312">
+      <c r="A2312" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2312" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2312" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2312" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2312" s="16" t="n">
+        <v>96.5</v>
+      </c>
+    </row>
+    <row r="2313">
+      <c r="A2313" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2313" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2313" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2313" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2313" s="19" t="n">
+        <v>153.2</v>
+      </c>
+    </row>
+    <row r="2314">
+      <c r="A2314" s="20" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2314" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2314" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2314" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2314" s="16" t="n">
+        <v>152.6</v>
+      </c>
+    </row>
+    <row r="2315">
+      <c r="A2315" s="21" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2315" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2315" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2315" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2315" s="19" t="n">
+        <v>61.3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-20
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2315"/>
+  <dimension ref="A1:E2361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -53841,6 +53841,1064 @@
         <v>61.3</v>
       </c>
     </row>
+    <row r="2316">
+      <c r="A2316" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2316" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2316" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2316" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2316" s="16" t="n">
+        <v>78.25</v>
+      </c>
+    </row>
+    <row r="2317">
+      <c r="A2317" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2317" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2317" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2317" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2317" s="19" t="n">
+        <v>109.8</v>
+      </c>
+    </row>
+    <row r="2318">
+      <c r="A2318" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2318" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2318" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2318" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2318" s="16" t="n">
+        <v>150.4</v>
+      </c>
+    </row>
+    <row r="2319">
+      <c r="A2319" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2319" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2319" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2319" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2319" s="19" t="n">
+        <v>154.2</v>
+      </c>
+    </row>
+    <row r="2320">
+      <c r="A2320" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2320" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2320" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2320" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2320" s="16" t="n">
+        <v>112.35</v>
+      </c>
+    </row>
+    <row r="2321">
+      <c r="A2321" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2321" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2321" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2321" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2321" s="19" t="n">
+        <v>88.45</v>
+      </c>
+    </row>
+    <row r="2322">
+      <c r="A2322" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2322" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2322" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2322" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2322" s="16" t="n">
+        <v>87.40000000000001</v>
+      </c>
+    </row>
+    <row r="2323">
+      <c r="A2323" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2323" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2323" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2323" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2323" s="19" t="n">
+        <v>80.55</v>
+      </c>
+    </row>
+    <row r="2324">
+      <c r="A2324" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2324" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2324" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2324" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2324" s="16" t="n">
+        <v>96.59999999999999</v>
+      </c>
+    </row>
+    <row r="2325">
+      <c r="A2325" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2325" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2325" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2325" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2325" s="19" t="n">
+        <v>139.3</v>
+      </c>
+    </row>
+    <row r="2326">
+      <c r="A2326" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2326" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2326" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2326" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2326" s="16" t="n">
+        <v>85.45</v>
+      </c>
+    </row>
+    <row r="2327">
+      <c r="A2327" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2327" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2327" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2327" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2327" s="19" t="n">
+        <v>139.35</v>
+      </c>
+    </row>
+    <row r="2328">
+      <c r="A2328" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2328" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2328" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2328" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2328" s="16" t="n">
+        <v>181.5</v>
+      </c>
+    </row>
+    <row r="2329">
+      <c r="A2329" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2329" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2329" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2329" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2329" s="19" t="n">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2330">
+      <c r="A2330" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2330" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2330" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2330" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2330" s="16" t="n">
+        <v>74.84999999999999</v>
+      </c>
+    </row>
+    <row r="2331">
+      <c r="A2331" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2331" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2331" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2331" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2331" s="19" t="n">
+        <v>120.45</v>
+      </c>
+    </row>
+    <row r="2332">
+      <c r="A2332" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2332" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2332" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2332" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2332" s="16" t="n">
+        <v>173.5</v>
+      </c>
+    </row>
+    <row r="2333">
+      <c r="A2333" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2333" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2333" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2333" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2333" s="19" t="n">
+        <v>174.5</v>
+      </c>
+    </row>
+    <row r="2334">
+      <c r="A2334" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2334" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2334" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2334" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2334" s="16" t="n">
+        <v>74.8</v>
+      </c>
+    </row>
+    <row r="2335">
+      <c r="A2335" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2335" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2335" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2335" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2335" s="19" t="n">
+        <v>114.25</v>
+      </c>
+    </row>
+    <row r="2336">
+      <c r="A2336" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2336" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2336" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2336" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2336" s="16" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2337">
+      <c r="A2337" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2337" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2337" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2337" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2337" s="19" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2338">
+      <c r="A2338" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2338" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2338" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2338" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2338" s="16" t="n">
+        <v>73.75</v>
+      </c>
+    </row>
+    <row r="2339">
+      <c r="A2339" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2339" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2339" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2339" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2339" s="19" t="n">
+        <v>72.09999999999999</v>
+      </c>
+    </row>
+    <row r="2340">
+      <c r="A2340" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2340" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2340" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2340" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2340" s="16" t="n">
+        <v>100.05</v>
+      </c>
+    </row>
+    <row r="2341">
+      <c r="A2341" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2341" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2341" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2341" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2341" s="19" t="n">
+        <v>137.7</v>
+      </c>
+    </row>
+    <row r="2342">
+      <c r="A2342" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2342" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2342" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2342" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2342" s="16" t="n">
+        <v>140.85</v>
+      </c>
+    </row>
+    <row r="2343">
+      <c r="A2343" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2343" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2343" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2343" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2343" s="19" t="n">
+        <v>105.55</v>
+      </c>
+    </row>
+    <row r="2344">
+      <c r="A2344" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2344" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2344" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2344" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2344" s="16" t="n">
+        <v>81.55</v>
+      </c>
+    </row>
+    <row r="2345">
+      <c r="A2345" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2345" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2345" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2345" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2345" s="19" t="n">
+        <v>75.95</v>
+      </c>
+    </row>
+    <row r="2346">
+      <c r="A2346" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2346" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2346" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2346" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2346" s="16" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="2347">
+      <c r="A2347" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2347" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2347" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2347" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2347" s="19" t="n">
+        <v>90.15000000000001</v>
+      </c>
+    </row>
+    <row r="2348">
+      <c r="A2348" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2348" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2348" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2348" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2348" s="16" t="n">
+        <v>128.3</v>
+      </c>
+    </row>
+    <row r="2349">
+      <c r="A2349" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2349" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2349" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2349" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2349" s="19" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2350">
+      <c r="A2350" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2350" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2350" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2350" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2350" s="16" t="n">
+        <v>119.9</v>
+      </c>
+    </row>
+    <row r="2351">
+      <c r="A2351" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2351" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2351" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2351" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2351" s="19" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="2352">
+      <c r="A2352" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2352" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2352" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2352" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2352" s="16" t="n">
+        <v>165.55</v>
+      </c>
+    </row>
+    <row r="2353">
+      <c r="A2353" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2353" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2353" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2353" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2353" s="19" t="n">
+        <v>67.3</v>
+      </c>
+    </row>
+    <row r="2354">
+      <c r="A2354" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2354" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2354" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2354" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2354" s="16" t="n">
+        <v>102.6</v>
+      </c>
+    </row>
+    <row r="2355">
+      <c r="A2355" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2355" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2355" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2355" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2355" s="19" t="n">
+        <v>158.3</v>
+      </c>
+    </row>
+    <row r="2356">
+      <c r="A2356" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2356" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2356" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2356" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2356" s="16" t="n">
+        <v>160.85</v>
+      </c>
+    </row>
+    <row r="2357">
+      <c r="A2357" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2357" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2357" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2357" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2357" s="19" t="n">
+        <v>64.45</v>
+      </c>
+    </row>
+    <row r="2358">
+      <c r="A2358" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2358" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2358" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2358" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2358" s="16" t="n">
+        <v>96.8</v>
+      </c>
+    </row>
+    <row r="2359">
+      <c r="A2359" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2359" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2359" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2359" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2359" s="19" t="n">
+        <v>153.5</v>
+      </c>
+    </row>
+    <row r="2360">
+      <c r="A2360" s="20" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2360" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2360" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2360" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2360" s="16" t="n">
+        <v>153.5</v>
+      </c>
+    </row>
+    <row r="2361">
+      <c r="A2361" s="21" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2361" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2361" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2361" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2361" s="19" t="n">
+        <v>64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-21
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2361"/>
+  <dimension ref="A1:E2407"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -54899,6 +54899,1064 @@
         <v>64</v>
       </c>
     </row>
+    <row r="2362">
+      <c r="A2362" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2362" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2362" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2362" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2362" s="16" t="n">
+        <v>75.55</v>
+      </c>
+    </row>
+    <row r="2363">
+      <c r="A2363" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2363" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2363" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2363" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2363" s="19" t="n">
+        <v>104.2</v>
+      </c>
+    </row>
+    <row r="2364">
+      <c r="A2364" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2364" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2364" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2364" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2364" s="16" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2365">
+      <c r="A2365" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2365" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2365" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2365" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2365" s="19" t="n">
+        <v>144.5</v>
+      </c>
+    </row>
+    <row r="2366">
+      <c r="A2366" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2366" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2366" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2366" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2366" s="16" t="n">
+        <v>110.25</v>
+      </c>
+    </row>
+    <row r="2367">
+      <c r="A2367" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2367" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2367" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2367" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2367" s="19" t="n">
+        <v>84.5</v>
+      </c>
+    </row>
+    <row r="2368">
+      <c r="A2368" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2368" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2368" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2368" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2368" s="16" t="n">
+        <v>81.40000000000001</v>
+      </c>
+    </row>
+    <row r="2369">
+      <c r="A2369" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2369" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2369" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2369" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2369" s="19" t="n">
+        <v>75.05</v>
+      </c>
+    </row>
+    <row r="2370">
+      <c r="A2370" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2370" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2370" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2370" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2370" s="16" t="n">
+        <v>93.8</v>
+      </c>
+    </row>
+    <row r="2371">
+      <c r="A2371" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2371" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2371" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2371" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2371" s="19" t="n">
+        <v>132.5</v>
+      </c>
+    </row>
+    <row r="2372">
+      <c r="A2372" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2372" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2372" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2372" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2372" s="16" t="n">
+        <v>80.3</v>
+      </c>
+    </row>
+    <row r="2373">
+      <c r="A2373" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2373" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2373" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2373" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2373" s="19" t="n">
+        <v>135.7</v>
+      </c>
+    </row>
+    <row r="2374">
+      <c r="A2374" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2374" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2374" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2374" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2374" s="16" t="n">
+        <v>175.35</v>
+      </c>
+    </row>
+    <row r="2375">
+      <c r="A2375" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2375" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2375" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2375" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2375" s="19" t="n">
+        <v>175.95</v>
+      </c>
+    </row>
+    <row r="2376">
+      <c r="A2376" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2376" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2376" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2376" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2376" s="16" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="2377">
+      <c r="A2377" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2377" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2377" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2377" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2377" s="19" t="n">
+        <v>116.15</v>
+      </c>
+    </row>
+    <row r="2378">
+      <c r="A2378" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2378" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2378" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2378" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2378" s="16" t="n">
+        <v>168.45</v>
+      </c>
+    </row>
+    <row r="2379">
+      <c r="A2379" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2379" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2379" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2379" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2379" s="19" t="n">
+        <v>167.25</v>
+      </c>
+    </row>
+    <row r="2380">
+      <c r="A2380" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2380" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2380" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2380" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2380" s="16" t="n">
+        <v>73.2</v>
+      </c>
+    </row>
+    <row r="2381">
+      <c r="A2381" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2381" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2381" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2381" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2381" s="19" t="n">
+        <v>113.4</v>
+      </c>
+    </row>
+    <row r="2382">
+      <c r="A2382" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2382" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2382" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2382" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2382" s="16" t="n">
+        <v>163.3</v>
+      </c>
+    </row>
+    <row r="2383">
+      <c r="A2383" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2383" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2383" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2383" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2383" s="19" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="2384">
+      <c r="A2384" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2384" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2384" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2384" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2384" s="16" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2385">
+      <c r="A2385" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2385" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2385" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2385" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2385" s="19" t="n">
+        <v>69.15000000000001</v>
+      </c>
+    </row>
+    <row r="2386">
+      <c r="A2386" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2386" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2386" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2386" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2386" s="16" t="n">
+        <v>94.2</v>
+      </c>
+    </row>
+    <row r="2387">
+      <c r="A2387" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2387" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2387" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2387" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2387" s="19" t="n">
+        <v>130.2</v>
+      </c>
+    </row>
+    <row r="2388">
+      <c r="A2388" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2388" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2388" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2388" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2388" s="16" t="n">
+        <v>134.2</v>
+      </c>
+    </row>
+    <row r="2389">
+      <c r="A2389" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2389" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2389" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2389" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2389" s="19" t="n">
+        <v>102.65</v>
+      </c>
+    </row>
+    <row r="2390">
+      <c r="A2390" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2390" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2390" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2390" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2390" s="16" t="n">
+        <v>74.45</v>
+      </c>
+    </row>
+    <row r="2391">
+      <c r="A2391" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2391" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2391" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2391" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2391" s="19" t="n">
+        <v>71.15000000000001</v>
+      </c>
+    </row>
+    <row r="2392">
+      <c r="A2392" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2392" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2392" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2392" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2392" s="16" t="n">
+        <v>66.09999999999999</v>
+      </c>
+    </row>
+    <row r="2393">
+      <c r="A2393" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2393" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2393" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2393" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2393" s="19" t="n">
+        <v>87.25</v>
+      </c>
+    </row>
+    <row r="2394">
+      <c r="A2394" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2394" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2394" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2394" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2394" s="16" t="n">
+        <v>122.6</v>
+      </c>
+    </row>
+    <row r="2395">
+      <c r="A2395" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2395" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2395" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2395" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2395" s="19" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="2396">
+      <c r="A2396" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2396" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2396" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2396" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2396" s="16" t="n">
+        <v>115.6</v>
+      </c>
+    </row>
+    <row r="2397">
+      <c r="A2397" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2397" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2397" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2397" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2397" s="19" t="n">
+        <v>162.8</v>
+      </c>
+    </row>
+    <row r="2398">
+      <c r="A2398" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2398" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2398" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2398" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2398" s="16" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2399">
+      <c r="A2399" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2399" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2399" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2399" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2399" s="19" t="n">
+        <v>64.95</v>
+      </c>
+    </row>
+    <row r="2400">
+      <c r="A2400" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2400" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2400" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2400" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2400" s="16" t="n">
+        <v>100.5</v>
+      </c>
+    </row>
+    <row r="2401">
+      <c r="A2401" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2401" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2401" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2401" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2401" s="19" t="n">
+        <v>150.1</v>
+      </c>
+    </row>
+    <row r="2402">
+      <c r="A2402" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2402" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2402" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2402" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2402" s="16" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="2403">
+      <c r="A2403" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2403" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2403" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2403" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2403" s="19" t="n">
+        <v>63.95</v>
+      </c>
+    </row>
+    <row r="2404">
+      <c r="A2404" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2404" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2404" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2404" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2404" s="16" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2405">
+      <c r="A2405" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2405" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2405" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2405" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2405" s="19" t="n">
+        <v>146.45</v>
+      </c>
+    </row>
+    <row r="2406">
+      <c r="A2406" s="20" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2406" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2406" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2406" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2406" s="16" t="n">
+        <v>147.15</v>
+      </c>
+    </row>
+    <row r="2407">
+      <c r="A2407" s="21" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B2407" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2407" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2407" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2407" s="19" t="n">
+        <v>62.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-22
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2407"/>
+  <dimension ref="A1:E2453"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -55957,6 +55957,1064 @@
         <v>62.5</v>
       </c>
     </row>
+    <row r="2408">
+      <c r="A2408" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2408" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2408" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2408" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2408" s="16" t="n">
+        <v>76.25</v>
+      </c>
+    </row>
+    <row r="2409">
+      <c r="A2409" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2409" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2409" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2409" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2409" s="19" t="n">
+        <v>103.3</v>
+      </c>
+    </row>
+    <row r="2410">
+      <c r="A2410" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2410" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2410" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2410" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2410" s="16" t="n">
+        <v>139.95</v>
+      </c>
+    </row>
+    <row r="2411">
+      <c r="A2411" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2411" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2411" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2411" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2411" s="19" t="n">
+        <v>141.95</v>
+      </c>
+    </row>
+    <row r="2412">
+      <c r="A2412" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2412" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2412" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2412" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2412" s="16" t="n">
+        <v>110.2</v>
+      </c>
+    </row>
+    <row r="2413">
+      <c r="A2413" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2413" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2413" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2413" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2413" s="19" t="n">
+        <v>85.45</v>
+      </c>
+    </row>
+    <row r="2414">
+      <c r="A2414" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2414" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2414" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2414" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2414" s="16" t="n">
+        <v>82.34999999999999</v>
+      </c>
+    </row>
+    <row r="2415">
+      <c r="A2415" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2415" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2415" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2415" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2415" s="19" t="n">
+        <v>75.90000000000001</v>
+      </c>
+    </row>
+    <row r="2416">
+      <c r="A2416" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2416" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2416" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2416" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2416" s="16" t="n">
+        <v>93.75</v>
+      </c>
+    </row>
+    <row r="2417">
+      <c r="A2417" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2417" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2417" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2417" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2417" s="19" t="n">
+        <v>130.95</v>
+      </c>
+    </row>
+    <row r="2418">
+      <c r="A2418" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2418" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2418" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2418" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2418" s="16" t="n">
+        <v>81.2</v>
+      </c>
+    </row>
+    <row r="2419">
+      <c r="A2419" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2419" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2419" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2419" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2419" s="19" t="n">
+        <v>135.7</v>
+      </c>
+    </row>
+    <row r="2420">
+      <c r="A2420" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2420" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2420" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2420" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2420" s="16" t="n">
+        <v>179.2</v>
+      </c>
+    </row>
+    <row r="2421">
+      <c r="A2421" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2421" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2421" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2421" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2421" s="19" t="n">
+        <v>178.05</v>
+      </c>
+    </row>
+    <row r="2422">
+      <c r="A2422" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2422" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2422" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2422" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2422" s="16" t="n">
+        <v>73.34999999999999</v>
+      </c>
+    </row>
+    <row r="2423">
+      <c r="A2423" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2423" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2423" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2423" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2423" s="19" t="n">
+        <v>117.45</v>
+      </c>
+    </row>
+    <row r="2424">
+      <c r="A2424" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2424" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2424" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2424" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2424" s="16" t="n">
+        <v>169.7</v>
+      </c>
+    </row>
+    <row r="2425">
+      <c r="A2425" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2425" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2425" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2425" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2425" s="19" t="n">
+        <v>169.5</v>
+      </c>
+    </row>
+    <row r="2426">
+      <c r="A2426" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2426" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2426" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2426" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2426" s="16" t="n">
+        <v>72.90000000000001</v>
+      </c>
+    </row>
+    <row r="2427">
+      <c r="A2427" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2427" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2427" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2427" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2427" s="19" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2428">
+      <c r="A2428" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2428" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2428" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2428" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2428" s="16" t="n">
+        <v>164.15</v>
+      </c>
+    </row>
+    <row r="2429">
+      <c r="A2429" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2429" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2429" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2429" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2429" s="19" t="n">
+        <v>165.25</v>
+      </c>
+    </row>
+    <row r="2430">
+      <c r="A2430" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2430" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2430" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2430" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2430" s="16" t="n">
+        <v>71.95</v>
+      </c>
+    </row>
+    <row r="2431">
+      <c r="A2431" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2431" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2431" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2431" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2431" s="19" t="n">
+        <v>70.09999999999999</v>
+      </c>
+    </row>
+    <row r="2432">
+      <c r="A2432" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2432" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2432" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2432" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2432" s="16" t="n">
+        <v>92.55</v>
+      </c>
+    </row>
+    <row r="2433">
+      <c r="A2433" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2433" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2433" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2433" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2433" s="19" t="n">
+        <v>127.55</v>
+      </c>
+    </row>
+    <row r="2434">
+      <c r="A2434" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2434" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2434" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2434" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2434" s="16" t="n">
+        <v>132.35</v>
+      </c>
+    </row>
+    <row r="2435">
+      <c r="A2435" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2435" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2435" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2435" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2435" s="19" t="n">
+        <v>99.25</v>
+      </c>
+    </row>
+    <row r="2436">
+      <c r="A2436" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2436" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2436" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2436" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2436" s="16" t="n">
+        <v>75.5</v>
+      </c>
+    </row>
+    <row r="2437">
+      <c r="A2437" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2437" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2437" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2437" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2437" s="19" t="n">
+        <v>72.15000000000001</v>
+      </c>
+    </row>
+    <row r="2438">
+      <c r="A2438" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2438" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2438" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2438" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2438" s="16" t="n">
+        <v>67.05</v>
+      </c>
+    </row>
+    <row r="2439">
+      <c r="A2439" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2439" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2439" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2439" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2439" s="19" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2440">
+      <c r="A2440" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2440" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2440" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2440" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2440" s="16" t="n">
+        <v>119.95</v>
+      </c>
+    </row>
+    <row r="2441">
+      <c r="A2441" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2441" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2441" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2441" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2441" s="19" t="n">
+        <v>71.55</v>
+      </c>
+    </row>
+    <row r="2442">
+      <c r="A2442" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2442" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2442" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2442" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2442" s="16" t="n">
+        <v>115.7</v>
+      </c>
+    </row>
+    <row r="2443">
+      <c r="A2443" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2443" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2443" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2443" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2443" s="19" t="n">
+        <v>163.7</v>
+      </c>
+    </row>
+    <row r="2444">
+      <c r="A2444" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2444" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2444" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2444" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2444" s="16" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2445">
+      <c r="A2445" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2445" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2445" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2445" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2445" s="19" t="n">
+        <v>64.65000000000001</v>
+      </c>
+    </row>
+    <row r="2446">
+      <c r="A2446" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2446" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2446" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2446" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2446" s="16" t="n">
+        <v>100.5</v>
+      </c>
+    </row>
+    <row r="2447">
+      <c r="A2447" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2447" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2447" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2447" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2447" s="19" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2448">
+      <c r="A2448" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2448" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2448" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2448" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2448" s="16" t="n">
+        <v>155.5</v>
+      </c>
+    </row>
+    <row r="2449">
+      <c r="A2449" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2449" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2449" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2449" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2449" s="19" t="n">
+        <v>62.7</v>
+      </c>
+    </row>
+    <row r="2450">
+      <c r="A2450" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2450" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2450" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2450" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2450" s="16" t="n">
+        <v>95.15000000000001</v>
+      </c>
+    </row>
+    <row r="2451">
+      <c r="A2451" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2451" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2451" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2451" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2451" s="19" t="n">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="2452">
+      <c r="A2452" s="20" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2452" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2452" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2452" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2452" s="16" t="n">
+        <v>147.1</v>
+      </c>
+    </row>
+    <row r="2453">
+      <c r="A2453" s="21" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B2453" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2453" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2453" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2453" s="19" t="n">
+        <v>60.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-23
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2453"/>
+  <dimension ref="A1:E2499"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -57015,6 +57015,1064 @@
         <v>60.75</v>
       </c>
     </row>
+    <row r="2454">
+      <c r="A2454" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2454" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2454" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2454" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2454" s="16" t="n">
+        <v>76.25</v>
+      </c>
+    </row>
+    <row r="2455">
+      <c r="A2455" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2455" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2455" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2455" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2455" s="19" t="n">
+        <v>103.3</v>
+      </c>
+    </row>
+    <row r="2456">
+      <c r="A2456" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2456" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2456" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2456" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2456" s="16" t="n">
+        <v>139.95</v>
+      </c>
+    </row>
+    <row r="2457">
+      <c r="A2457" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2457" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2457" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2457" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2457" s="19" t="n">
+        <v>141.95</v>
+      </c>
+    </row>
+    <row r="2458">
+      <c r="A2458" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2458" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2458" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2458" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2458" s="16" t="n">
+        <v>110.2</v>
+      </c>
+    </row>
+    <row r="2459">
+      <c r="A2459" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2459" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2459" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2459" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2459" s="19" t="n">
+        <v>85.45</v>
+      </c>
+    </row>
+    <row r="2460">
+      <c r="A2460" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2460" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2460" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2460" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2460" s="16" t="n">
+        <v>82.34999999999999</v>
+      </c>
+    </row>
+    <row r="2461">
+      <c r="A2461" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2461" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2461" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2461" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2461" s="19" t="n">
+        <v>75.90000000000001</v>
+      </c>
+    </row>
+    <row r="2462">
+      <c r="A2462" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2462" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2462" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2462" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2462" s="16" t="n">
+        <v>93.75</v>
+      </c>
+    </row>
+    <row r="2463">
+      <c r="A2463" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2463" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2463" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2463" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2463" s="19" t="n">
+        <v>130.95</v>
+      </c>
+    </row>
+    <row r="2464">
+      <c r="A2464" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2464" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2464" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2464" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2464" s="16" t="n">
+        <v>81.2</v>
+      </c>
+    </row>
+    <row r="2465">
+      <c r="A2465" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2465" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2465" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2465" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2465" s="19" t="n">
+        <v>135.7</v>
+      </c>
+    </row>
+    <row r="2466">
+      <c r="A2466" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2466" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2466" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2466" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2466" s="16" t="n">
+        <v>179.2</v>
+      </c>
+    </row>
+    <row r="2467">
+      <c r="A2467" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2467" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2467" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2467" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2467" s="19" t="n">
+        <v>178.05</v>
+      </c>
+    </row>
+    <row r="2468">
+      <c r="A2468" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2468" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2468" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2468" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2468" s="16" t="n">
+        <v>73.34999999999999</v>
+      </c>
+    </row>
+    <row r="2469">
+      <c r="A2469" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2469" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2469" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2469" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2469" s="19" t="n">
+        <v>117.45</v>
+      </c>
+    </row>
+    <row r="2470">
+      <c r="A2470" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2470" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2470" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2470" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2470" s="16" t="n">
+        <v>169.7</v>
+      </c>
+    </row>
+    <row r="2471">
+      <c r="A2471" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2471" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2471" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2471" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2471" s="19" t="n">
+        <v>169.5</v>
+      </c>
+    </row>
+    <row r="2472">
+      <c r="A2472" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2472" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2472" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2472" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2472" s="16" t="n">
+        <v>72.90000000000001</v>
+      </c>
+    </row>
+    <row r="2473">
+      <c r="A2473" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2473" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2473" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2473" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2473" s="19" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2474">
+      <c r="A2474" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2474" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2474" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2474" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2474" s="16" t="n">
+        <v>164.15</v>
+      </c>
+    </row>
+    <row r="2475">
+      <c r="A2475" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2475" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2475" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2475" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2475" s="19" t="n">
+        <v>165.25</v>
+      </c>
+    </row>
+    <row r="2476">
+      <c r="A2476" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2476" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2476" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2476" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2476" s="16" t="n">
+        <v>71.95</v>
+      </c>
+    </row>
+    <row r="2477">
+      <c r="A2477" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2477" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2477" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2477" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2477" s="19" t="n">
+        <v>70.09999999999999</v>
+      </c>
+    </row>
+    <row r="2478">
+      <c r="A2478" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2478" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2478" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2478" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2478" s="16" t="n">
+        <v>92.55</v>
+      </c>
+    </row>
+    <row r="2479">
+      <c r="A2479" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2479" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2479" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2479" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2479" s="19" t="n">
+        <v>127.55</v>
+      </c>
+    </row>
+    <row r="2480">
+      <c r="A2480" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2480" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2480" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2480" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2480" s="16" t="n">
+        <v>132.35</v>
+      </c>
+    </row>
+    <row r="2481">
+      <c r="A2481" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2481" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2481" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2481" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2481" s="19" t="n">
+        <v>99.25</v>
+      </c>
+    </row>
+    <row r="2482">
+      <c r="A2482" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2482" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2482" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2482" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2482" s="16" t="n">
+        <v>75.5</v>
+      </c>
+    </row>
+    <row r="2483">
+      <c r="A2483" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2483" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2483" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2483" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2483" s="19" t="n">
+        <v>72.15000000000001</v>
+      </c>
+    </row>
+    <row r="2484">
+      <c r="A2484" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2484" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2484" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2484" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2484" s="16" t="n">
+        <v>67.05</v>
+      </c>
+    </row>
+    <row r="2485">
+      <c r="A2485" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2485" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2485" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2485" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2485" s="19" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2486">
+      <c r="A2486" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2486" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2486" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2486" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2486" s="16" t="n">
+        <v>119.95</v>
+      </c>
+    </row>
+    <row r="2487">
+      <c r="A2487" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2487" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2487" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2487" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2487" s="19" t="n">
+        <v>71.55</v>
+      </c>
+    </row>
+    <row r="2488">
+      <c r="A2488" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2488" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2488" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2488" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2488" s="16" t="n">
+        <v>115.7</v>
+      </c>
+    </row>
+    <row r="2489">
+      <c r="A2489" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2489" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2489" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2489" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2489" s="19" t="n">
+        <v>163.7</v>
+      </c>
+    </row>
+    <row r="2490">
+      <c r="A2490" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2490" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2490" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2490" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2490" s="16" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2491">
+      <c r="A2491" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2491" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2491" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2491" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2491" s="19" t="n">
+        <v>64.65000000000001</v>
+      </c>
+    </row>
+    <row r="2492">
+      <c r="A2492" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2492" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2492" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2492" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2492" s="16" t="n">
+        <v>100.5</v>
+      </c>
+    </row>
+    <row r="2493">
+      <c r="A2493" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2493" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2493" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2493" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2493" s="19" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2494">
+      <c r="A2494" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2494" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2494" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2494" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2494" s="16" t="n">
+        <v>155.5</v>
+      </c>
+    </row>
+    <row r="2495">
+      <c r="A2495" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2495" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2495" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2495" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2495" s="19" t="n">
+        <v>62.7</v>
+      </c>
+    </row>
+    <row r="2496">
+      <c r="A2496" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2496" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2496" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2496" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2496" s="16" t="n">
+        <v>95.15000000000001</v>
+      </c>
+    </row>
+    <row r="2497">
+      <c r="A2497" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2497" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2497" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2497" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2497" s="19" t="n">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="2498">
+      <c r="A2498" s="20" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2498" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2498" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2498" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2498" s="16" t="n">
+        <v>147.1</v>
+      </c>
+    </row>
+    <row r="2499">
+      <c r="A2499" s="21" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B2499" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2499" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2499" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2499" s="19" t="n">
+        <v>60.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-24
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2499"/>
+  <dimension ref="A1:E2545"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -58073,6 +58073,1064 @@
         <v>60.75</v>
       </c>
     </row>
+    <row r="2500">
+      <c r="A2500" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2500" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2500" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2500" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2500" s="16" t="n">
+        <v>76.25</v>
+      </c>
+    </row>
+    <row r="2501">
+      <c r="A2501" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2501" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2501" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2501" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2501" s="19" t="n">
+        <v>103.3</v>
+      </c>
+    </row>
+    <row r="2502">
+      <c r="A2502" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2502" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2502" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2502" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2502" s="16" t="n">
+        <v>139.95</v>
+      </c>
+    </row>
+    <row r="2503">
+      <c r="A2503" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2503" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2503" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2503" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2503" s="19" t="n">
+        <v>141.95</v>
+      </c>
+    </row>
+    <row r="2504">
+      <c r="A2504" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2504" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2504" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2504" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2504" s="16" t="n">
+        <v>110.2</v>
+      </c>
+    </row>
+    <row r="2505">
+      <c r="A2505" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2505" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2505" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2505" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2505" s="19" t="n">
+        <v>85.45</v>
+      </c>
+    </row>
+    <row r="2506">
+      <c r="A2506" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2506" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2506" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2506" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2506" s="16" t="n">
+        <v>82.34999999999999</v>
+      </c>
+    </row>
+    <row r="2507">
+      <c r="A2507" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2507" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2507" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2507" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2507" s="19" t="n">
+        <v>75.90000000000001</v>
+      </c>
+    </row>
+    <row r="2508">
+      <c r="A2508" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2508" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2508" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2508" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2508" s="16" t="n">
+        <v>93.75</v>
+      </c>
+    </row>
+    <row r="2509">
+      <c r="A2509" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2509" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2509" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2509" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2509" s="19" t="n">
+        <v>130.95</v>
+      </c>
+    </row>
+    <row r="2510">
+      <c r="A2510" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2510" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2510" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2510" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2510" s="16" t="n">
+        <v>81.2</v>
+      </c>
+    </row>
+    <row r="2511">
+      <c r="A2511" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2511" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2511" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2511" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2511" s="19" t="n">
+        <v>135.7</v>
+      </c>
+    </row>
+    <row r="2512">
+      <c r="A2512" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2512" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2512" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2512" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2512" s="16" t="n">
+        <v>179.2</v>
+      </c>
+    </row>
+    <row r="2513">
+      <c r="A2513" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2513" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2513" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2513" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2513" s="19" t="n">
+        <v>178.05</v>
+      </c>
+    </row>
+    <row r="2514">
+      <c r="A2514" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2514" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2514" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2514" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2514" s="16" t="n">
+        <v>73.34999999999999</v>
+      </c>
+    </row>
+    <row r="2515">
+      <c r="A2515" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2515" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2515" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2515" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2515" s="19" t="n">
+        <v>117.45</v>
+      </c>
+    </row>
+    <row r="2516">
+      <c r="A2516" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2516" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2516" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2516" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2516" s="16" t="n">
+        <v>169.7</v>
+      </c>
+    </row>
+    <row r="2517">
+      <c r="A2517" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2517" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2517" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2517" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2517" s="19" t="n">
+        <v>169.5</v>
+      </c>
+    </row>
+    <row r="2518">
+      <c r="A2518" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2518" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2518" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2518" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2518" s="16" t="n">
+        <v>72.90000000000001</v>
+      </c>
+    </row>
+    <row r="2519">
+      <c r="A2519" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2519" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2519" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2519" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2519" s="19" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2520">
+      <c r="A2520" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2520" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2520" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2520" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2520" s="16" t="n">
+        <v>164.15</v>
+      </c>
+    </row>
+    <row r="2521">
+      <c r="A2521" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2521" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2521" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2521" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2521" s="19" t="n">
+        <v>165.25</v>
+      </c>
+    </row>
+    <row r="2522">
+      <c r="A2522" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2522" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2522" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2522" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2522" s="16" t="n">
+        <v>71.95</v>
+      </c>
+    </row>
+    <row r="2523">
+      <c r="A2523" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2523" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2523" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2523" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2523" s="19" t="n">
+        <v>70.09999999999999</v>
+      </c>
+    </row>
+    <row r="2524">
+      <c r="A2524" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2524" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2524" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2524" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2524" s="16" t="n">
+        <v>92.55</v>
+      </c>
+    </row>
+    <row r="2525">
+      <c r="A2525" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2525" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2525" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2525" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2525" s="19" t="n">
+        <v>127.55</v>
+      </c>
+    </row>
+    <row r="2526">
+      <c r="A2526" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2526" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2526" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2526" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2526" s="16" t="n">
+        <v>132.35</v>
+      </c>
+    </row>
+    <row r="2527">
+      <c r="A2527" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2527" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2527" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2527" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2527" s="19" t="n">
+        <v>99.25</v>
+      </c>
+    </row>
+    <row r="2528">
+      <c r="A2528" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2528" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2528" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2528" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2528" s="16" t="n">
+        <v>75.5</v>
+      </c>
+    </row>
+    <row r="2529">
+      <c r="A2529" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2529" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2529" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2529" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2529" s="19" t="n">
+        <v>72.15000000000001</v>
+      </c>
+    </row>
+    <row r="2530">
+      <c r="A2530" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2530" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2530" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2530" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2530" s="16" t="n">
+        <v>67.05</v>
+      </c>
+    </row>
+    <row r="2531">
+      <c r="A2531" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2531" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2531" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2531" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2531" s="19" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2532">
+      <c r="A2532" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2532" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2532" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2532" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2532" s="16" t="n">
+        <v>119.95</v>
+      </c>
+    </row>
+    <row r="2533">
+      <c r="A2533" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2533" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2533" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2533" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2533" s="19" t="n">
+        <v>71.55</v>
+      </c>
+    </row>
+    <row r="2534">
+      <c r="A2534" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2534" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2534" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2534" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2534" s="16" t="n">
+        <v>115.7</v>
+      </c>
+    </row>
+    <row r="2535">
+      <c r="A2535" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2535" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2535" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2535" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2535" s="19" t="n">
+        <v>163.7</v>
+      </c>
+    </row>
+    <row r="2536">
+      <c r="A2536" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2536" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2536" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2536" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2536" s="16" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2537">
+      <c r="A2537" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2537" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2537" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2537" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2537" s="19" t="n">
+        <v>64.65000000000001</v>
+      </c>
+    </row>
+    <row r="2538">
+      <c r="A2538" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2538" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2538" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2538" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2538" s="16" t="n">
+        <v>100.5</v>
+      </c>
+    </row>
+    <row r="2539">
+      <c r="A2539" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2539" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2539" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2539" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2539" s="19" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2540">
+      <c r="A2540" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2540" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2540" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2540" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2540" s="16" t="n">
+        <v>155.5</v>
+      </c>
+    </row>
+    <row r="2541">
+      <c r="A2541" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2541" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2541" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2541" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2541" s="19" t="n">
+        <v>62.7</v>
+      </c>
+    </row>
+    <row r="2542">
+      <c r="A2542" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2542" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2542" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2542" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2542" s="16" t="n">
+        <v>95.15000000000001</v>
+      </c>
+    </row>
+    <row r="2543">
+      <c r="A2543" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2543" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2543" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2543" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2543" s="19" t="n">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="2544">
+      <c r="A2544" s="20" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2544" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2544" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2544" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2544" s="16" t="n">
+        <v>147.1</v>
+      </c>
+    </row>
+    <row r="2545">
+      <c r="A2545" s="21" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2545" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2545" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2545" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2545" s="19" t="n">
+        <v>60.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-25
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2545"/>
+  <dimension ref="A1:E2591"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -59131,6 +59131,1064 @@
         <v>60.75</v>
       </c>
     </row>
+    <row r="2546">
+      <c r="A2546" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2546" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2546" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2546" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2546" s="16" t="n">
+        <v>78.5</v>
+      </c>
+    </row>
+    <row r="2547">
+      <c r="A2547" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2547" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2547" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2547" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2547" s="19" t="n">
+        <v>95.05</v>
+      </c>
+    </row>
+    <row r="2548">
+      <c r="A2548" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2548" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2548" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2548" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2548" s="16" t="n">
+        <v>130.65</v>
+      </c>
+    </row>
+    <row r="2549">
+      <c r="A2549" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2549" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2549" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2549" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2549" s="19" t="n">
+        <v>132.5</v>
+      </c>
+    </row>
+    <row r="2550">
+      <c r="A2550" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2550" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2550" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2550" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2550" s="16" t="n">
+        <v>102.2</v>
+      </c>
+    </row>
+    <row r="2551">
+      <c r="A2551" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2551" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2551" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2551" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2551" s="19" t="n">
+        <v>81.09999999999999</v>
+      </c>
+    </row>
+    <row r="2552">
+      <c r="A2552" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2552" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2552" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2552" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2552" s="16" t="n">
+        <v>79.5</v>
+      </c>
+    </row>
+    <row r="2553">
+      <c r="A2553" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2553" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2553" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2553" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2553" s="19" t="n">
+        <v>73.3</v>
+      </c>
+    </row>
+    <row r="2554">
+      <c r="A2554" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2554" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2554" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2554" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2554" s="16" t="n">
+        <v>91.8</v>
+      </c>
+    </row>
+    <row r="2555">
+      <c r="A2555" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2555" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2555" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2555" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2555" s="19" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="2556">
+      <c r="A2556" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2556" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2556" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2556" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2556" s="16" t="n">
+        <v>77.95</v>
+      </c>
+    </row>
+    <row r="2557">
+      <c r="A2557" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2557" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2557" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2557" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2557" s="19" t="n">
+        <v>133.6</v>
+      </c>
+    </row>
+    <row r="2558">
+      <c r="A2558" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2558" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2558" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2558" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2558" s="16" t="n">
+        <v>179.2</v>
+      </c>
+    </row>
+    <row r="2559">
+      <c r="A2559" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2559" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2559" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2559" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2559" s="19" t="n">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="2560">
+      <c r="A2560" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2560" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2560" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2560" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2560" s="16" t="n">
+        <v>73.59999999999999</v>
+      </c>
+    </row>
+    <row r="2561">
+      <c r="A2561" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2561" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2561" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2561" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2561" s="19" t="n">
+        <v>117.45</v>
+      </c>
+    </row>
+    <row r="2562">
+      <c r="A2562" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2562" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2562" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2562" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2562" s="16" t="n">
+        <v>167.45</v>
+      </c>
+    </row>
+    <row r="2563">
+      <c r="A2563" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2563" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2563" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2563" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2563" s="19" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2564">
+      <c r="A2564" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2564" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2564" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2564" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2564" s="16" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="2565">
+      <c r="A2565" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2565" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2565" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2565" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2565" s="19" t="n">
+        <v>111.1</v>
+      </c>
+    </row>
+    <row r="2566">
+      <c r="A2566" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2566" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2566" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2566" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2566" s="16" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="2567">
+      <c r="A2567" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2567" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2567" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2567" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2567" s="19" t="n">
+        <v>165.8</v>
+      </c>
+    </row>
+    <row r="2568">
+      <c r="A2568" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2568" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2568" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2568" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2568" s="16" t="n">
+        <v>71.95</v>
+      </c>
+    </row>
+    <row r="2569">
+      <c r="A2569" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2569" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2569" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2569" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2569" s="19" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2570">
+      <c r="A2570" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2570" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2570" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2570" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2570" s="16" t="n">
+        <v>86.5</v>
+      </c>
+    </row>
+    <row r="2571">
+      <c r="A2571" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2571" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2571" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2571" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2571" s="19" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2572">
+      <c r="A2572" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2572" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2572" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2572" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2572" s="16" t="n">
+        <v>119.75</v>
+      </c>
+    </row>
+    <row r="2573">
+      <c r="A2573" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2573" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2573" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2573" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2573" s="19" t="n">
+        <v>91.7</v>
+      </c>
+    </row>
+    <row r="2574">
+      <c r="A2574" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2574" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2574" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2574" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2574" s="16" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="2575">
+      <c r="A2575" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2575" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2575" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2575" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2575" s="19" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2576">
+      <c r="A2576" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2576" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2576" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2576" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2576" s="16" t="n">
+        <v>63.2</v>
+      </c>
+    </row>
+    <row r="2577">
+      <c r="A2577" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2577" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2577" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2577" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2577" s="19" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2578">
+      <c r="A2578" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2578" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2578" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2578" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2578" s="16" t="n">
+        <v>109.35</v>
+      </c>
+    </row>
+    <row r="2579">
+      <c r="A2579" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2579" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2579" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2579" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2579" s="19" t="n">
+        <v>67.5</v>
+      </c>
+    </row>
+    <row r="2580">
+      <c r="A2580" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2580" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2580" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2580" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2580" s="16" t="n">
+        <v>112.6</v>
+      </c>
+    </row>
+    <row r="2581">
+      <c r="A2581" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2581" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2581" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2581" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2581" s="19" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="2582">
+      <c r="A2582" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2582" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2582" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2582" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2582" s="16" t="n">
+        <v>161.2</v>
+      </c>
+    </row>
+    <row r="2583">
+      <c r="A2583" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2583" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2583" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2583" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2583" s="19" t="n">
+        <v>63.5</v>
+      </c>
+    </row>
+    <row r="2584">
+      <c r="A2584" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2584" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2584" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2584" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2584" s="16" t="n">
+        <v>97.8</v>
+      </c>
+    </row>
+    <row r="2585">
+      <c r="A2585" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2585" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2585" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2585" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2585" s="19" t="n">
+        <v>151.95</v>
+      </c>
+    </row>
+    <row r="2586">
+      <c r="A2586" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2586" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2586" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2586" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2586" s="16" t="n">
+        <v>155.4</v>
+      </c>
+    </row>
+    <row r="2587">
+      <c r="A2587" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2587" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2587" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2587" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2587" s="19" t="n">
+        <v>62.7</v>
+      </c>
+    </row>
+    <row r="2588">
+      <c r="A2588" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2588" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2588" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2588" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2588" s="16" t="n">
+        <v>92.75</v>
+      </c>
+    </row>
+    <row r="2589">
+      <c r="A2589" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2589" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2589" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2589" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2589" s="19" t="n">
+        <v>150.2</v>
+      </c>
+    </row>
+    <row r="2590">
+      <c r="A2590" s="20" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2590" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2590" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2590" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2590" s="16" t="n">
+        <v>150.05</v>
+      </c>
+    </row>
+    <row r="2591">
+      <c r="A2591" s="21" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B2591" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2591" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2591" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2591" s="19" t="n">
+        <v>60.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-27
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2591"/>
+  <dimension ref="A1:E2637"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -60189,6 +60189,1064 @@
         <v>60.75</v>
       </c>
     </row>
+    <row r="2592">
+      <c r="A2592" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2592" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2592" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2592" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2592" s="16" t="n">
+        <v>80.25</v>
+      </c>
+    </row>
+    <row r="2593">
+      <c r="A2593" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2593" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2593" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2593" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2593" s="19" t="n">
+        <v>88.7</v>
+      </c>
+    </row>
+    <row r="2594">
+      <c r="A2594" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2594" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2594" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2594" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2594" s="16" t="n">
+        <v>125.25</v>
+      </c>
+    </row>
+    <row r="2595">
+      <c r="A2595" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2595" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2595" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2595" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2595" s="19" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2596">
+      <c r="A2596" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2596" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2596" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2596" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2596" s="16" t="n">
+        <v>100.35</v>
+      </c>
+    </row>
+    <row r="2597">
+      <c r="A2597" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2597" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2597" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2597" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2597" s="19" t="n">
+        <v>83.05</v>
+      </c>
+    </row>
+    <row r="2598">
+      <c r="A2598" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2598" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2598" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2598" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2598" s="16" t="n">
+        <v>78.55</v>
+      </c>
+    </row>
+    <row r="2599">
+      <c r="A2599" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2599" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2599" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2599" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2599" s="19" t="n">
+        <v>72.40000000000001</v>
+      </c>
+    </row>
+    <row r="2600">
+      <c r="A2600" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2600" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2600" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2600" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2600" s="16" t="n">
+        <v>90.3</v>
+      </c>
+    </row>
+    <row r="2601">
+      <c r="A2601" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2601" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2601" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2601" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2601" s="19" t="n">
+        <v>119.4</v>
+      </c>
+    </row>
+    <row r="2602">
+      <c r="A2602" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2602" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2602" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2602" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2602" s="16" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2603">
+      <c r="A2603" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2603" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2603" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2603" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2603" s="19" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2604">
+      <c r="A2604" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2604" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2604" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2604" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2604" s="16" t="n">
+        <v>175.2</v>
+      </c>
+    </row>
+    <row r="2605">
+      <c r="A2605" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2605" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2605" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2605" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2605" s="19" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="2606">
+      <c r="A2606" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2606" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2606" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2606" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2606" s="16" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2607">
+      <c r="A2607" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2607" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2607" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2607" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2607" s="19" t="n">
+        <v>113.35</v>
+      </c>
+    </row>
+    <row r="2608">
+      <c r="A2608" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2608" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2608" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2608" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2608" s="16" t="n">
+        <v>169.5</v>
+      </c>
+    </row>
+    <row r="2609">
+      <c r="A2609" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2609" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2609" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2609" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2609" s="19" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2610">
+      <c r="A2610" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2610" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2610" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2610" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2610" s="16" t="n">
+        <v>68.5</v>
+      </c>
+    </row>
+    <row r="2611">
+      <c r="A2611" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2611" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2611" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2611" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2611" s="19" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2612">
+      <c r="A2612" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2612" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2612" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2612" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2612" s="16" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="2613">
+      <c r="A2613" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2613" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2613" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2613" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2613" s="19" t="n">
+        <v>163.75</v>
+      </c>
+    </row>
+    <row r="2614">
+      <c r="A2614" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2614" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2614" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2614" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2614" s="16" t="n">
+        <v>68.5</v>
+      </c>
+    </row>
+    <row r="2615">
+      <c r="A2615" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2615" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2615" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2615" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2615" s="19" t="n">
+        <v>74.25</v>
+      </c>
+    </row>
+    <row r="2616">
+      <c r="A2616" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2616" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2616" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2616" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2616" s="16" t="n">
+        <v>79.90000000000001</v>
+      </c>
+    </row>
+    <row r="2617">
+      <c r="A2617" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2617" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2617" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2617" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2617" s="19" t="n">
+        <v>113.85</v>
+      </c>
+    </row>
+    <row r="2618">
+      <c r="A2618" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2618" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2618" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2618" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2618" s="16" t="n">
+        <v>123.15</v>
+      </c>
+    </row>
+    <row r="2619">
+      <c r="A2619" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2619" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2619" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2619" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2619" s="19" t="n">
+        <v>92.7</v>
+      </c>
+    </row>
+    <row r="2620">
+      <c r="A2620" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2620" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2620" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2620" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2620" s="16" t="n">
+        <v>75.55</v>
+      </c>
+    </row>
+    <row r="2621">
+      <c r="A2621" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2621" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2621" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2621" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2621" s="19" t="n">
+        <v>63.15</v>
+      </c>
+    </row>
+    <row r="2622">
+      <c r="A2622" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2622" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2622" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2622" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2622" s="16" t="n">
+        <v>58.75</v>
+      </c>
+    </row>
+    <row r="2623">
+      <c r="A2623" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2623" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2623" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2623" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2623" s="19" t="n">
+        <v>84.25</v>
+      </c>
+    </row>
+    <row r="2624">
+      <c r="A2624" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2624" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2624" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2624" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2624" s="16" t="n">
+        <v>110.1</v>
+      </c>
+    </row>
+    <row r="2625">
+      <c r="A2625" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2625" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2625" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2625" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2625" s="19" t="n">
+        <v>65.84999999999999</v>
+      </c>
+    </row>
+    <row r="2626">
+      <c r="A2626" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2626" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2626" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2626" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2626" s="16" t="n">
+        <v>110.5</v>
+      </c>
+    </row>
+    <row r="2627">
+      <c r="A2627" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2627" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2627" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2627" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2627" s="19" t="n">
+        <v>159.55</v>
+      </c>
+    </row>
+    <row r="2628">
+      <c r="A2628" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2628" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2628" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2628" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2628" s="16" t="n">
+        <v>158.75</v>
+      </c>
+    </row>
+    <row r="2629">
+      <c r="A2629" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2629" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2629" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2629" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2629" s="19" t="n">
+        <v>60.9</v>
+      </c>
+    </row>
+    <row r="2630">
+      <c r="A2630" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2630" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2630" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2630" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2630" s="16" t="n">
+        <v>95.75</v>
+      </c>
+    </row>
+    <row r="2631">
+      <c r="A2631" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2631" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2631" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2631" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2631" s="19" t="n">
+        <v>152.6</v>
+      </c>
+    </row>
+    <row r="2632">
+      <c r="A2632" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2632" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2632" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2632" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2632" s="16" t="n">
+        <v>154.5</v>
+      </c>
+    </row>
+    <row r="2633">
+      <c r="A2633" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2633" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2633" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2633" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2633" s="19" t="n">
+        <v>59.35</v>
+      </c>
+    </row>
+    <row r="2634">
+      <c r="A2634" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2634" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2634" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2634" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2634" s="16" t="n">
+        <v>89.3</v>
+      </c>
+    </row>
+    <row r="2635">
+      <c r="A2635" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2635" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2635" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2635" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2635" s="19" t="n">
+        <v>147.3</v>
+      </c>
+    </row>
+    <row r="2636">
+      <c r="A2636" s="20" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2636" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2636" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2636" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2636" s="16" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2637">
+      <c r="A2637" s="21" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2637" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2637" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2637" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2637" s="19" t="n">
+        <v>59.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-28
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2637"/>
+  <dimension ref="A1:E2683"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -61247,6 +61247,1064 @@
         <v>59.75</v>
       </c>
     </row>
+    <row r="2638">
+      <c r="A2638" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2638" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2638" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2638" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2638" s="16" t="n">
+        <v>80.55</v>
+      </c>
+    </row>
+    <row r="2639">
+      <c r="A2639" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2639" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2639" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2639" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2639" s="19" t="n">
+        <v>85.34999999999999</v>
+      </c>
+    </row>
+    <row r="2640">
+      <c r="A2640" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2640" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2640" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2640" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2640" s="16" t="n">
+        <v>129.25</v>
+      </c>
+    </row>
+    <row r="2641">
+      <c r="A2641" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2641" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2641" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2641" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2641" s="19" t="n">
+        <v>136.3</v>
+      </c>
+    </row>
+    <row r="2642">
+      <c r="A2642" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2642" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2642" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2642" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2642" s="16" t="n">
+        <v>103.8</v>
+      </c>
+    </row>
+    <row r="2643">
+      <c r="A2643" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2643" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2643" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2643" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2643" s="19" t="n">
+        <v>87.40000000000001</v>
+      </c>
+    </row>
+    <row r="2644">
+      <c r="A2644" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2644" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2644" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2644" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2644" s="16" t="n">
+        <v>79.40000000000001</v>
+      </c>
+    </row>
+    <row r="2645">
+      <c r="A2645" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2645" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2645" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2645" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2645" s="19" t="n">
+        <v>73.15000000000001</v>
+      </c>
+    </row>
+    <row r="2646">
+      <c r="A2646" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2646" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2646" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2646" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2646" s="16" t="n">
+        <v>89.3</v>
+      </c>
+    </row>
+    <row r="2647">
+      <c r="A2647" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2647" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2647" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2647" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2647" s="19" t="n">
+        <v>123.35</v>
+      </c>
+    </row>
+    <row r="2648">
+      <c r="A2648" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2648" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2648" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2648" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2648" s="16" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2649">
+      <c r="A2649" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2649" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2649" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2649" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2649" s="19" t="n">
+        <v>133.9</v>
+      </c>
+    </row>
+    <row r="2650">
+      <c r="A2650" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2650" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2650" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2650" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2650" s="16" t="n">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="2651">
+      <c r="A2651" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2651" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2651" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2651" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2651" s="19" t="n">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="2652">
+      <c r="A2652" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2652" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2652" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2652" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2652" s="16" t="n">
+        <v>72.09999999999999</v>
+      </c>
+    </row>
+    <row r="2653">
+      <c r="A2653" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2653" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2653" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2653" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2653" s="19" t="n">
+        <v>115.2</v>
+      </c>
+    </row>
+    <row r="2654">
+      <c r="A2654" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2654" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2654" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2654" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2654" s="16" t="n">
+        <v>174.55</v>
+      </c>
+    </row>
+    <row r="2655">
+      <c r="A2655" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2655" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2655" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2655" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2655" s="19" t="n">
+        <v>177.25</v>
+      </c>
+    </row>
+    <row r="2656">
+      <c r="A2656" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2656" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2656" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2656" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2656" s="16" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2657">
+      <c r="A2657" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2657" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2657" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2657" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2657" s="19" t="n">
+        <v>109.9</v>
+      </c>
+    </row>
+    <row r="2658">
+      <c r="A2658" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2658" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2658" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2658" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2658" s="16" t="n">
+        <v>168.4</v>
+      </c>
+    </row>
+    <row r="2659">
+      <c r="A2659" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2659" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2659" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2659" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2659" s="19" t="n">
+        <v>171.6</v>
+      </c>
+    </row>
+    <row r="2660">
+      <c r="A2660" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2660" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2660" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2660" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2660" s="16" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2661">
+      <c r="A2661" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2661" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2661" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2661" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2661" s="19" t="n">
+        <v>75.05</v>
+      </c>
+    </row>
+    <row r="2662">
+      <c r="A2662" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2662" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2662" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2662" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2662" s="16" t="n">
+        <v>77.09999999999999</v>
+      </c>
+    </row>
+    <row r="2663">
+      <c r="A2663" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2663" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2663" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2663" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2663" s="19" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2664">
+      <c r="A2664" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2664" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2664" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2664" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2664" s="16" t="n">
+        <v>126.65</v>
+      </c>
+    </row>
+    <row r="2665">
+      <c r="A2665" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2665" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2665" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2665" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2665" s="19" t="n">
+        <v>96.65000000000001</v>
+      </c>
+    </row>
+    <row r="2666">
+      <c r="A2666" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2666" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2666" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2666" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2666" s="16" t="n">
+        <v>80.7</v>
+      </c>
+    </row>
+    <row r="2667">
+      <c r="A2667" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2667" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2667" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2667" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2667" s="19" t="n">
+        <v>66.25</v>
+      </c>
+    </row>
+    <row r="2668">
+      <c r="A2668" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2668" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2668" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2668" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2668" s="16" t="n">
+        <v>61.6</v>
+      </c>
+    </row>
+    <row r="2669">
+      <c r="A2669" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2669" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2669" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2669" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2669" s="19" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="2670">
+      <c r="A2670" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2670" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2670" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2670" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2670" s="16" t="n">
+        <v>114.3</v>
+      </c>
+    </row>
+    <row r="2671">
+      <c r="A2671" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2671" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2671" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2671" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2671" s="19" t="n">
+        <v>69.55</v>
+      </c>
+    </row>
+    <row r="2672">
+      <c r="A2672" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2672" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2672" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2672" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2672" s="16" t="n">
+        <v>112.25</v>
+      </c>
+    </row>
+    <row r="2673">
+      <c r="A2673" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2673" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2673" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2673" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2673" s="19" t="n">
+        <v>167.5</v>
+      </c>
+    </row>
+    <row r="2674">
+      <c r="A2674" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2674" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2674" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2674" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2674" s="16" t="n">
+        <v>165.85</v>
+      </c>
+    </row>
+    <row r="2675">
+      <c r="A2675" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2675" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2675" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2675" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2675" s="19" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2676">
+      <c r="A2676" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2676" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2676" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2676" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2676" s="16" t="n">
+        <v>96.84999999999999</v>
+      </c>
+    </row>
+    <row r="2677">
+      <c r="A2677" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2677" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2677" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2677" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2677" s="19" t="n">
+        <v>161.95</v>
+      </c>
+    </row>
+    <row r="2678">
+      <c r="A2678" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2678" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2678" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2678" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2678" s="16" t="n">
+        <v>160.65</v>
+      </c>
+    </row>
+    <row r="2679">
+      <c r="A2679" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2679" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2679" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2679" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2679" s="19" t="n">
+        <v>61.25</v>
+      </c>
+    </row>
+    <row r="2680">
+      <c r="A2680" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2680" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2680" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2680" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2680" s="16" t="n">
+        <v>91.25</v>
+      </c>
+    </row>
+    <row r="2681">
+      <c r="A2681" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2681" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2681" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2681" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2681" s="19" t="n">
+        <v>154.25</v>
+      </c>
+    </row>
+    <row r="2682">
+      <c r="A2682" s="20" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2682" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2682" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2682" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2682" s="16" t="n">
+        <v>153.8</v>
+      </c>
+    </row>
+    <row r="2683">
+      <c r="A2683" s="21" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2683" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2683" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2683" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2683" s="19" t="n">
+        <v>59.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-29
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2683"/>
+  <dimension ref="A1:E2729"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -62305,6 +62305,1064 @@
         <v>59.75</v>
       </c>
     </row>
+    <row r="2684">
+      <c r="A2684" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2684" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2684" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2684" s="15" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2684" s="16" t="n">
+        <v>81.25</v>
+      </c>
+    </row>
+    <row r="2685">
+      <c r="A2685" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2685" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2685" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2685" s="18" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2685" s="19" t="n">
+        <v>84.3</v>
+      </c>
+    </row>
+    <row r="2686">
+      <c r="A2686" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2686" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2686" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2686" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2686" s="16" t="n">
+        <v>122.95</v>
+      </c>
+    </row>
+    <row r="2687">
+      <c r="A2687" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2687" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2687" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2687" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2687" s="19" t="n">
+        <v>131.25</v>
+      </c>
+    </row>
+    <row r="2688">
+      <c r="A2688" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2688" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2688" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2688" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2688" s="16" t="n">
+        <v>101.35</v>
+      </c>
+    </row>
+    <row r="2689">
+      <c r="A2689" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2689" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2689" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2689" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2689" s="19" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2690">
+      <c r="A2690" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2690" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2690" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2690" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2690" s="16" t="n">
+        <v>76.8</v>
+      </c>
+    </row>
+    <row r="2691">
+      <c r="A2691" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2691" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2691" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2691" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2691" s="19" t="n">
+        <v>70.75</v>
+      </c>
+    </row>
+    <row r="2692">
+      <c r="A2692" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2692" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2692" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2692" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2692" s="16" t="n">
+        <v>89.2</v>
+      </c>
+    </row>
+    <row r="2693">
+      <c r="A2693" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2693" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2693" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2693" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2693" s="19" t="n">
+        <v>118.7</v>
+      </c>
+    </row>
+    <row r="2694">
+      <c r="A2694" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2694" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2694" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2694" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2694" s="16" t="n">
+        <v>77.5</v>
+      </c>
+    </row>
+    <row r="2695">
+      <c r="A2695" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2695" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2695" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2695" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2695" s="19" t="n">
+        <v>132.15</v>
+      </c>
+    </row>
+    <row r="2696">
+      <c r="A2696" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2696" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2696" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2696" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2696" s="16" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="2697">
+      <c r="A2697" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2697" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2697" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2697" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2697" s="19" t="n">
+        <v>181.75</v>
+      </c>
+    </row>
+    <row r="2698">
+      <c r="A2698" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2698" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2698" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2698" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2698" s="16" t="n">
+        <v>73.09999999999999</v>
+      </c>
+    </row>
+    <row r="2699">
+      <c r="A2699" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2699" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2699" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2699" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2699" s="19" t="n">
+        <v>116.5</v>
+      </c>
+    </row>
+    <row r="2700">
+      <c r="A2700" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2700" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2700" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2700" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2700" s="16" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2701">
+      <c r="A2701" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2701" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2701" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2701" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2701" s="19" t="n">
+        <v>174.85</v>
+      </c>
+    </row>
+    <row r="2702">
+      <c r="A2702" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2702" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2702" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2702" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2702" s="16" t="n">
+        <v>71.84999999999999</v>
+      </c>
+    </row>
+    <row r="2703">
+      <c r="A2703" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2703" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2703" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2703" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2703" s="19" t="n">
+        <v>111.5</v>
+      </c>
+    </row>
+    <row r="2704">
+      <c r="A2704" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2704" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2704" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2704" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2704" s="16" t="n">
+        <v>172.5</v>
+      </c>
+    </row>
+    <row r="2705">
+      <c r="A2705" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2705" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2705" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2705" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2705" s="19" t="n">
+        <v>174.5</v>
+      </c>
+    </row>
+    <row r="2706">
+      <c r="A2706" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2706" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2706" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2706" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2706" s="16" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2707">
+      <c r="A2707" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2707" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2707" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2707" s="18" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="E2707" s="19" t="n">
+        <v>75.5</v>
+      </c>
+    </row>
+    <row r="2708">
+      <c r="A2708" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2708" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2708" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2708" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2708" s="16" t="n">
+        <v>76.55</v>
+      </c>
+    </row>
+    <row r="2709">
+      <c r="A2709" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2709" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2709" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2709" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2709" s="19" t="n">
+        <v>112.7</v>
+      </c>
+    </row>
+    <row r="2710">
+      <c r="A2710" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2710" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2710" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2710" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2710" s="16" t="n">
+        <v>119.75</v>
+      </c>
+    </row>
+    <row r="2711">
+      <c r="A2711" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2711" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2711" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2711" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2711" s="19" t="n">
+        <v>92.8</v>
+      </c>
+    </row>
+    <row r="2712">
+      <c r="A2712" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2712" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2712" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2712" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2712" s="16" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2713">
+      <c r="A2713" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2713" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2713" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2713" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2713" s="19" t="n">
+        <v>64.2</v>
+      </c>
+    </row>
+    <row r="2714">
+      <c r="A2714" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2714" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2714" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2714" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2714" s="16" t="n">
+        <v>59.7</v>
+      </c>
+    </row>
+    <row r="2715">
+      <c r="A2715" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2715" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2715" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2715" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2715" s="19" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="2716">
+      <c r="A2716" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2716" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2716" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2716" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2716" s="16" t="n">
+        <v>108.6</v>
+      </c>
+    </row>
+    <row r="2717">
+      <c r="A2717" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2717" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2717" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2717" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2717" s="19" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2718">
+      <c r="A2718" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2718" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2718" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2718" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2718" s="16" t="n">
+        <v>112.35</v>
+      </c>
+    </row>
+    <row r="2719">
+      <c r="A2719" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2719" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2719" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2719" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2719" s="19" t="n">
+        <v>167.1</v>
+      </c>
+    </row>
+    <row r="2720">
+      <c r="A2720" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2720" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2720" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2720" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2720" s="16" t="n">
+        <v>167.5</v>
+      </c>
+    </row>
+    <row r="2721">
+      <c r="A2721" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2721" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2721" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2721" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2721" s="19" t="n">
+        <v>63.5</v>
+      </c>
+    </row>
+    <row r="2722">
+      <c r="A2722" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2722" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2722" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2722" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2722" s="16" t="n">
+        <v>97.25</v>
+      </c>
+    </row>
+    <row r="2723">
+      <c r="A2723" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2723" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2723" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2723" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2723" s="19" t="n">
+        <v>162.05</v>
+      </c>
+    </row>
+    <row r="2724">
+      <c r="A2724" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2724" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2724" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2724" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2724" s="16" t="n">
+        <v>163.65</v>
+      </c>
+    </row>
+    <row r="2725">
+      <c r="A2725" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2725" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2725" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2725" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2725" s="19" t="n">
+        <v>62.25</v>
+      </c>
+    </row>
+    <row r="2726">
+      <c r="A2726" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2726" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2726" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2726" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2726" s="16" t="n">
+        <v>91.25</v>
+      </c>
+    </row>
+    <row r="2727">
+      <c r="A2727" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2727" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2727" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2727" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2727" s="19" t="n">
+        <v>155.55</v>
+      </c>
+    </row>
+    <row r="2728">
+      <c r="A2728" s="20" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2728" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2728" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2728" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2728" s="16" t="n">
+        <v>154.95</v>
+      </c>
+    </row>
+    <row r="2729">
+      <c r="A2729" s="21" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B2729" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2729" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2729" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2729" s="19" t="n">
+        <v>60.85</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-30
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2729"/>
+  <dimension ref="A1:E2773"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63363,6 +63363,1018 @@
         <v>60.85</v>
       </c>
     </row>
+    <row r="2730">
+      <c r="A2730" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2730" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2730" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2730" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2730" s="16" t="n">
+        <v>84.3</v>
+      </c>
+    </row>
+    <row r="2731">
+      <c r="A2731" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2731" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2731" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2731" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2731" s="19" t="n">
+        <v>122.95</v>
+      </c>
+    </row>
+    <row r="2732">
+      <c r="A2732" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2732" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2732" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2732" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2732" s="16" t="n">
+        <v>131.25</v>
+      </c>
+    </row>
+    <row r="2733">
+      <c r="A2733" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2733" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2733" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2733" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2733" s="19" t="n">
+        <v>101.35</v>
+      </c>
+    </row>
+    <row r="2734">
+      <c r="A2734" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2734" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2734" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2734" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2734" s="16" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2735">
+      <c r="A2735" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2735" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2735" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2735" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2735" s="19" t="n">
+        <v>76.8</v>
+      </c>
+    </row>
+    <row r="2736">
+      <c r="A2736" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2736" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2736" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2736" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2736" s="16" t="n">
+        <v>70.75</v>
+      </c>
+    </row>
+    <row r="2737">
+      <c r="A2737" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2737" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2737" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2737" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2737" s="19" t="n">
+        <v>89.2</v>
+      </c>
+    </row>
+    <row r="2738">
+      <c r="A2738" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2738" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2738" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2738" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2738" s="16" t="n">
+        <v>118.7</v>
+      </c>
+    </row>
+    <row r="2739">
+      <c r="A2739" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2739" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2739" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2739" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2739" s="19" t="n">
+        <v>77.5</v>
+      </c>
+    </row>
+    <row r="2740">
+      <c r="A2740" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2740" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2740" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2740" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2740" s="16" t="n">
+        <v>132.15</v>
+      </c>
+    </row>
+    <row r="2741">
+      <c r="A2741" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2741" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2741" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2741" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2741" s="19" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="2742">
+      <c r="A2742" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2742" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2742" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2742" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2742" s="16" t="n">
+        <v>181.75</v>
+      </c>
+    </row>
+    <row r="2743">
+      <c r="A2743" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2743" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2743" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2743" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2743" s="19" t="n">
+        <v>73.09999999999999</v>
+      </c>
+    </row>
+    <row r="2744">
+      <c r="A2744" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2744" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2744" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2744" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2744" s="16" t="n">
+        <v>116.5</v>
+      </c>
+    </row>
+    <row r="2745">
+      <c r="A2745" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2745" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2745" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2745" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2745" s="19" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2746">
+      <c r="A2746" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2746" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2746" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2746" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2746" s="16" t="n">
+        <v>174.85</v>
+      </c>
+    </row>
+    <row r="2747">
+      <c r="A2747" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2747" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2747" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2747" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2747" s="19" t="n">
+        <v>71.84999999999999</v>
+      </c>
+    </row>
+    <row r="2748">
+      <c r="A2748" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2748" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2748" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2748" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2748" s="16" t="n">
+        <v>111.5</v>
+      </c>
+    </row>
+    <row r="2749">
+      <c r="A2749" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2749" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2749" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2749" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2749" s="19" t="n">
+        <v>172.5</v>
+      </c>
+    </row>
+    <row r="2750">
+      <c r="A2750" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2750" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2750" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2750" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2750" s="16" t="n">
+        <v>174.5</v>
+      </c>
+    </row>
+    <row r="2751">
+      <c r="A2751" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2751" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2751" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2751" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2751" s="19" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2752">
+      <c r="A2752" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2752" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2752" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2752" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2752" s="16" t="n">
+        <v>76.55</v>
+      </c>
+    </row>
+    <row r="2753">
+      <c r="A2753" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2753" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2753" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2753" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2753" s="19" t="n">
+        <v>112.7</v>
+      </c>
+    </row>
+    <row r="2754">
+      <c r="A2754" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2754" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2754" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2754" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2754" s="16" t="n">
+        <v>119.75</v>
+      </c>
+    </row>
+    <row r="2755">
+      <c r="A2755" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2755" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2755" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2755" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2755" s="19" t="n">
+        <v>92.8</v>
+      </c>
+    </row>
+    <row r="2756">
+      <c r="A2756" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2756" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2756" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2756" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2756" s="16" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2757">
+      <c r="A2757" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2757" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2757" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2757" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2757" s="19" t="n">
+        <v>64.2</v>
+      </c>
+    </row>
+    <row r="2758">
+      <c r="A2758" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2758" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2758" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2758" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2758" s="16" t="n">
+        <v>59.7</v>
+      </c>
+    </row>
+    <row r="2759">
+      <c r="A2759" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2759" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2759" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2759" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2759" s="19" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="2760">
+      <c r="A2760" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2760" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2760" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2760" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2760" s="16" t="n">
+        <v>108.6</v>
+      </c>
+    </row>
+    <row r="2761">
+      <c r="A2761" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2761" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2761" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2761" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2761" s="19" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2762">
+      <c r="A2762" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2762" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2762" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2762" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2762" s="16" t="n">
+        <v>112.35</v>
+      </c>
+    </row>
+    <row r="2763">
+      <c r="A2763" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2763" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2763" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2763" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2763" s="19" t="n">
+        <v>167.1</v>
+      </c>
+    </row>
+    <row r="2764">
+      <c r="A2764" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2764" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2764" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2764" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2764" s="16" t="n">
+        <v>167.5</v>
+      </c>
+    </row>
+    <row r="2765">
+      <c r="A2765" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2765" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2765" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2765" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2765" s="19" t="n">
+        <v>63.5</v>
+      </c>
+    </row>
+    <row r="2766">
+      <c r="A2766" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2766" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2766" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2766" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2766" s="16" t="n">
+        <v>97.25</v>
+      </c>
+    </row>
+    <row r="2767">
+      <c r="A2767" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2767" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2767" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2767" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2767" s="19" t="n">
+        <v>162.05</v>
+      </c>
+    </row>
+    <row r="2768">
+      <c r="A2768" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2768" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2768" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2768" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2768" s="16" t="n">
+        <v>163.65</v>
+      </c>
+    </row>
+    <row r="2769">
+      <c r="A2769" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2769" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2769" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2769" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2769" s="19" t="n">
+        <v>62.25</v>
+      </c>
+    </row>
+    <row r="2770">
+      <c r="A2770" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2770" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2770" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2770" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2770" s="16" t="n">
+        <v>91.25</v>
+      </c>
+    </row>
+    <row r="2771">
+      <c r="A2771" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2771" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2771" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2771" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2771" s="19" t="n">
+        <v>155.55</v>
+      </c>
+    </row>
+    <row r="2772">
+      <c r="A2772" s="20" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2772" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2772" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2772" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2772" s="16" t="n">
+        <v>154.95</v>
+      </c>
+    </row>
+    <row r="2773">
+      <c r="A2773" s="21" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2773" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2773" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2773" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2773" s="19" t="n">
+        <v>60.85</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-05-31
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2773"/>
+  <dimension ref="A1:E2817"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64375,6 +64375,1018 @@
         <v>60.85</v>
       </c>
     </row>
+    <row r="2774">
+      <c r="A2774" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2774" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2774" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2774" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2774" s="16" t="n">
+        <v>84.3</v>
+      </c>
+    </row>
+    <row r="2775">
+      <c r="A2775" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2775" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2775" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2775" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2775" s="19" t="n">
+        <v>122.95</v>
+      </c>
+    </row>
+    <row r="2776">
+      <c r="A2776" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2776" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2776" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2776" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2776" s="16" t="n">
+        <v>131.25</v>
+      </c>
+    </row>
+    <row r="2777">
+      <c r="A2777" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2777" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2777" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2777" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2777" s="19" t="n">
+        <v>101.35</v>
+      </c>
+    </row>
+    <row r="2778">
+      <c r="A2778" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2778" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2778" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2778" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2778" s="16" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2779">
+      <c r="A2779" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2779" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2779" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2779" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2779" s="19" t="n">
+        <v>76.8</v>
+      </c>
+    </row>
+    <row r="2780">
+      <c r="A2780" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2780" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2780" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2780" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2780" s="16" t="n">
+        <v>70.75</v>
+      </c>
+    </row>
+    <row r="2781">
+      <c r="A2781" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2781" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2781" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2781" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2781" s="19" t="n">
+        <v>89.2</v>
+      </c>
+    </row>
+    <row r="2782">
+      <c r="A2782" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2782" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2782" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2782" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2782" s="16" t="n">
+        <v>118.7</v>
+      </c>
+    </row>
+    <row r="2783">
+      <c r="A2783" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2783" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2783" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2783" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2783" s="19" t="n">
+        <v>77.5</v>
+      </c>
+    </row>
+    <row r="2784">
+      <c r="A2784" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2784" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2784" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2784" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2784" s="16" t="n">
+        <v>132.15</v>
+      </c>
+    </row>
+    <row r="2785">
+      <c r="A2785" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2785" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2785" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2785" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2785" s="19" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="2786">
+      <c r="A2786" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2786" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2786" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2786" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2786" s="16" t="n">
+        <v>181.75</v>
+      </c>
+    </row>
+    <row r="2787">
+      <c r="A2787" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2787" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2787" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2787" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2787" s="19" t="n">
+        <v>73.09999999999999</v>
+      </c>
+    </row>
+    <row r="2788">
+      <c r="A2788" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2788" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2788" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2788" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2788" s="16" t="n">
+        <v>116.5</v>
+      </c>
+    </row>
+    <row r="2789">
+      <c r="A2789" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2789" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2789" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2789" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2789" s="19" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2790">
+      <c r="A2790" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2790" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2790" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2790" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2790" s="16" t="n">
+        <v>174.85</v>
+      </c>
+    </row>
+    <row r="2791">
+      <c r="A2791" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2791" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2791" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2791" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2791" s="19" t="n">
+        <v>71.84999999999999</v>
+      </c>
+    </row>
+    <row r="2792">
+      <c r="A2792" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2792" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2792" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2792" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2792" s="16" t="n">
+        <v>111.5</v>
+      </c>
+    </row>
+    <row r="2793">
+      <c r="A2793" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2793" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2793" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2793" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2793" s="19" t="n">
+        <v>172.5</v>
+      </c>
+    </row>
+    <row r="2794">
+      <c r="A2794" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2794" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2794" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2794" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2794" s="16" t="n">
+        <v>174.5</v>
+      </c>
+    </row>
+    <row r="2795">
+      <c r="A2795" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2795" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2795" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2795" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2795" s="19" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2796">
+      <c r="A2796" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2796" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2796" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2796" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2796" s="16" t="n">
+        <v>76.55</v>
+      </c>
+    </row>
+    <row r="2797">
+      <c r="A2797" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2797" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2797" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2797" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2797" s="19" t="n">
+        <v>112.7</v>
+      </c>
+    </row>
+    <row r="2798">
+      <c r="A2798" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2798" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2798" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2798" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2798" s="16" t="n">
+        <v>119.75</v>
+      </c>
+    </row>
+    <row r="2799">
+      <c r="A2799" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2799" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2799" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2799" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2799" s="19" t="n">
+        <v>92.8</v>
+      </c>
+    </row>
+    <row r="2800">
+      <c r="A2800" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2800" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2800" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2800" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2800" s="16" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2801">
+      <c r="A2801" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2801" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2801" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2801" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2801" s="19" t="n">
+        <v>64.2</v>
+      </c>
+    </row>
+    <row r="2802">
+      <c r="A2802" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2802" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2802" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2802" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2802" s="16" t="n">
+        <v>59.7</v>
+      </c>
+    </row>
+    <row r="2803">
+      <c r="A2803" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2803" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2803" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2803" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2803" s="19" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="2804">
+      <c r="A2804" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2804" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2804" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2804" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2804" s="16" t="n">
+        <v>108.6</v>
+      </c>
+    </row>
+    <row r="2805">
+      <c r="A2805" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2805" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2805" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2805" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2805" s="19" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2806">
+      <c r="A2806" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2806" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2806" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2806" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2806" s="16" t="n">
+        <v>112.35</v>
+      </c>
+    </row>
+    <row r="2807">
+      <c r="A2807" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2807" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2807" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2807" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2807" s="19" t="n">
+        <v>167.1</v>
+      </c>
+    </row>
+    <row r="2808">
+      <c r="A2808" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2808" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2808" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2808" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2808" s="16" t="n">
+        <v>167.5</v>
+      </c>
+    </row>
+    <row r="2809">
+      <c r="A2809" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2809" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2809" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2809" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2809" s="19" t="n">
+        <v>63.5</v>
+      </c>
+    </row>
+    <row r="2810">
+      <c r="A2810" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2810" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2810" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2810" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2810" s="16" t="n">
+        <v>97.25</v>
+      </c>
+    </row>
+    <row r="2811">
+      <c r="A2811" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2811" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2811" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2811" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2811" s="19" t="n">
+        <v>162.05</v>
+      </c>
+    </row>
+    <row r="2812">
+      <c r="A2812" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2812" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2812" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2812" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2812" s="16" t="n">
+        <v>163.65</v>
+      </c>
+    </row>
+    <row r="2813">
+      <c r="A2813" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2813" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2813" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2813" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2813" s="19" t="n">
+        <v>62.25</v>
+      </c>
+    </row>
+    <row r="2814">
+      <c r="A2814" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2814" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2814" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2814" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2814" s="16" t="n">
+        <v>91.25</v>
+      </c>
+    </row>
+    <row r="2815">
+      <c r="A2815" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2815" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2815" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2815" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2815" s="19" t="n">
+        <v>155.55</v>
+      </c>
+    </row>
+    <row r="2816">
+      <c r="A2816" s="20" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2816" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2816" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2816" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2816" s="16" t="n">
+        <v>154.95</v>
+      </c>
+    </row>
+    <row r="2817">
+      <c r="A2817" s="21" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2817" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2817" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2817" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2817" s="19" t="n">
+        <v>60.85</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-02
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2817"/>
+  <dimension ref="A1:E2861"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -65387,6 +65387,1018 @@
         <v>60.85</v>
       </c>
     </row>
+    <row r="2818">
+      <c r="A2818" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2818" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2818" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2818" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2818" s="16" t="n">
+        <v>84.90000000000001</v>
+      </c>
+    </row>
+    <row r="2819">
+      <c r="A2819" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2819" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2819" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2819" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2819" s="19" t="n">
+        <v>122.95</v>
+      </c>
+    </row>
+    <row r="2820">
+      <c r="A2820" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2820" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2820" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2820" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2820" s="16" t="n">
+        <v>131.25</v>
+      </c>
+    </row>
+    <row r="2821">
+      <c r="A2821" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2821" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2821" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2821" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2821" s="19" t="n">
+        <v>101.35</v>
+      </c>
+    </row>
+    <row r="2822">
+      <c r="A2822" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2822" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2822" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2822" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2822" s="16" t="n">
+        <v>84.95</v>
+      </c>
+    </row>
+    <row r="2823">
+      <c r="A2823" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2823" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2823" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2823" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2823" s="19" t="n">
+        <v>76.8</v>
+      </c>
+    </row>
+    <row r="2824">
+      <c r="A2824" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2824" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2824" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2824" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2824" s="16" t="n">
+        <v>70.75</v>
+      </c>
+    </row>
+    <row r="2825">
+      <c r="A2825" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2825" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2825" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2825" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2825" s="19" t="n">
+        <v>89.2</v>
+      </c>
+    </row>
+    <row r="2826">
+      <c r="A2826" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2826" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2826" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2826" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2826" s="16" t="n">
+        <v>118.7</v>
+      </c>
+    </row>
+    <row r="2827">
+      <c r="A2827" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2827" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2827" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2827" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2827" s="19" t="n">
+        <v>77.5</v>
+      </c>
+    </row>
+    <row r="2828">
+      <c r="A2828" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2828" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2828" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2828" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2828" s="16" t="n">
+        <v>132.15</v>
+      </c>
+    </row>
+    <row r="2829">
+      <c r="A2829" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2829" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2829" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2829" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2829" s="19" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="2830">
+      <c r="A2830" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2830" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2830" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2830" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2830" s="16" t="n">
+        <v>181.75</v>
+      </c>
+    </row>
+    <row r="2831">
+      <c r="A2831" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2831" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2831" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2831" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2831" s="19" t="n">
+        <v>73.09999999999999</v>
+      </c>
+    </row>
+    <row r="2832">
+      <c r="A2832" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2832" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2832" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2832" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2832" s="16" t="n">
+        <v>116.5</v>
+      </c>
+    </row>
+    <row r="2833">
+      <c r="A2833" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2833" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2833" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2833" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2833" s="19" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2834">
+      <c r="A2834" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2834" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2834" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2834" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2834" s="16" t="n">
+        <v>174.85</v>
+      </c>
+    </row>
+    <row r="2835">
+      <c r="A2835" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2835" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2835" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2835" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2835" s="19" t="n">
+        <v>71.84999999999999</v>
+      </c>
+    </row>
+    <row r="2836">
+      <c r="A2836" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2836" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2836" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2836" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2836" s="16" t="n">
+        <v>111.5</v>
+      </c>
+    </row>
+    <row r="2837">
+      <c r="A2837" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2837" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2837" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2837" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2837" s="19" t="n">
+        <v>172.5</v>
+      </c>
+    </row>
+    <row r="2838">
+      <c r="A2838" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2838" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2838" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2838" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2838" s="16" t="n">
+        <v>174.5</v>
+      </c>
+    </row>
+    <row r="2839">
+      <c r="A2839" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2839" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2839" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2839" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2839" s="19" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2840">
+      <c r="A2840" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2840" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2840" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2840" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2840" s="16" t="n">
+        <v>77.2</v>
+      </c>
+    </row>
+    <row r="2841">
+      <c r="A2841" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2841" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2841" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2841" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2841" s="19" t="n">
+        <v>112.7</v>
+      </c>
+    </row>
+    <row r="2842">
+      <c r="A2842" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2842" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2842" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2842" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2842" s="16" t="n">
+        <v>119.75</v>
+      </c>
+    </row>
+    <row r="2843">
+      <c r="A2843" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2843" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2843" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2843" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2843" s="19" t="n">
+        <v>92.8</v>
+      </c>
+    </row>
+    <row r="2844">
+      <c r="A2844" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2844" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2844" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2844" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2844" s="16" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2845">
+      <c r="A2845" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2845" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2845" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2845" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2845" s="19" t="n">
+        <v>64.2</v>
+      </c>
+    </row>
+    <row r="2846">
+      <c r="A2846" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2846" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2846" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2846" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2846" s="16" t="n">
+        <v>59.7</v>
+      </c>
+    </row>
+    <row r="2847">
+      <c r="A2847" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2847" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2847" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2847" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2847" s="19" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="2848">
+      <c r="A2848" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2848" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2848" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2848" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2848" s="16" t="n">
+        <v>108.6</v>
+      </c>
+    </row>
+    <row r="2849">
+      <c r="A2849" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2849" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2849" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2849" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2849" s="19" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2850">
+      <c r="A2850" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2850" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2850" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2850" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2850" s="16" t="n">
+        <v>112.35</v>
+      </c>
+    </row>
+    <row r="2851">
+      <c r="A2851" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2851" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2851" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2851" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2851" s="19" t="n">
+        <v>167.1</v>
+      </c>
+    </row>
+    <row r="2852">
+      <c r="A2852" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2852" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2852" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2852" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2852" s="16" t="n">
+        <v>167.5</v>
+      </c>
+    </row>
+    <row r="2853">
+      <c r="A2853" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2853" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2853" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2853" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2853" s="19" t="n">
+        <v>63.5</v>
+      </c>
+    </row>
+    <row r="2854">
+      <c r="A2854" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2854" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2854" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2854" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2854" s="16" t="n">
+        <v>97.25</v>
+      </c>
+    </row>
+    <row r="2855">
+      <c r="A2855" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2855" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2855" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2855" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2855" s="19" t="n">
+        <v>162.05</v>
+      </c>
+    </row>
+    <row r="2856">
+      <c r="A2856" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2856" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2856" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2856" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2856" s="16" t="n">
+        <v>163.65</v>
+      </c>
+    </row>
+    <row r="2857">
+      <c r="A2857" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2857" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2857" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2857" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2857" s="19" t="n">
+        <v>62.25</v>
+      </c>
+    </row>
+    <row r="2858">
+      <c r="A2858" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2858" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2858" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2858" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2858" s="16" t="n">
+        <v>91.25</v>
+      </c>
+    </row>
+    <row r="2859">
+      <c r="A2859" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2859" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2859" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2859" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2859" s="19" t="n">
+        <v>155.55</v>
+      </c>
+    </row>
+    <row r="2860">
+      <c r="A2860" s="20" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2860" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2860" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2860" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2860" s="16" t="n">
+        <v>154.95</v>
+      </c>
+    </row>
+    <row r="2861">
+      <c r="A2861" s="21" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2861" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2861" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2861" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2861" s="19" t="n">
+        <v>60.85</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-04
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2861"/>
+  <dimension ref="A1:E2905"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66399,6 +66399,1018 @@
         <v>60.85</v>
       </c>
     </row>
+    <row r="2862">
+      <c r="A2862" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2862" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2862" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2862" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2862" s="16" t="n">
+        <v>73.95</v>
+      </c>
+    </row>
+    <row r="2863">
+      <c r="A2863" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2863" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2863" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2863" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2863" s="19" t="n">
+        <v>123.1</v>
+      </c>
+    </row>
+    <row r="2864">
+      <c r="A2864" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2864" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2864" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2864" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2864" s="16" t="n">
+        <v>132.35</v>
+      </c>
+    </row>
+    <row r="2865">
+      <c r="A2865" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2865" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2865" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2865" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2865" s="19" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="2866">
+      <c r="A2866" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2866" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2866" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2866" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2866" s="16" t="n">
+        <v>85.2</v>
+      </c>
+    </row>
+    <row r="2867">
+      <c r="A2867" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2867" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2867" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2867" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2867" s="19" t="n">
+        <v>80.09999999999999</v>
+      </c>
+    </row>
+    <row r="2868">
+      <c r="A2868" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2868" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2868" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2868" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2868" s="16" t="n">
+        <v>53.95</v>
+      </c>
+    </row>
+    <row r="2869">
+      <c r="A2869" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2869" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2869" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2869" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2869" s="19" t="n">
+        <v>86.25</v>
+      </c>
+    </row>
+    <row r="2870">
+      <c r="A2870" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2870" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2870" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2870" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2870" s="16" t="n">
+        <v>120.65</v>
+      </c>
+    </row>
+    <row r="2871">
+      <c r="A2871" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2871" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2871" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2871" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2871" s="19" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2872">
+      <c r="A2872" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2872" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2872" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2872" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2872" s="16" t="n">
+        <v>127.95</v>
+      </c>
+    </row>
+    <row r="2873">
+      <c r="A2873" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2873" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2873" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2873" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2873" s="19" t="n">
+        <v>184.75</v>
+      </c>
+    </row>
+    <row r="2874">
+      <c r="A2874" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2874" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2874" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2874" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2874" s="16" t="n">
+        <v>185.1</v>
+      </c>
+    </row>
+    <row r="2875">
+      <c r="A2875" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2875" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2875" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2875" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2875" s="19" t="n">
+        <v>73.09999999999999</v>
+      </c>
+    </row>
+    <row r="2876">
+      <c r="A2876" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2876" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2876" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2876" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2876" s="16" t="n">
+        <v>113.85</v>
+      </c>
+    </row>
+    <row r="2877">
+      <c r="A2877" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2877" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2877" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2877" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2877" s="19" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="2878">
+      <c r="A2878" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2878" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2878" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2878" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2878" s="16" t="n">
+        <v>177.8</v>
+      </c>
+    </row>
+    <row r="2879">
+      <c r="A2879" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2879" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2879" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2879" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2879" s="19" t="n">
+        <v>71.84999999999999</v>
+      </c>
+    </row>
+    <row r="2880">
+      <c r="A2880" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2880" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2880" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2880" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2880" s="16" t="n">
+        <v>111.5</v>
+      </c>
+    </row>
+    <row r="2881">
+      <c r="A2881" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2881" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2881" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2881" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2881" s="19" t="n">
+        <v>172.25</v>
+      </c>
+    </row>
+    <row r="2882">
+      <c r="A2882" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2882" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2882" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2882" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2882" s="16" t="n">
+        <v>173.8</v>
+      </c>
+    </row>
+    <row r="2883">
+      <c r="A2883" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2883" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2883" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2883" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2883" s="19" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2884">
+      <c r="A2884" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2884" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2884" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2884" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2884" s="16" t="n">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="2885">
+      <c r="A2885" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2885" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2885" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2885" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2885" s="19" t="n">
+        <v>109.75</v>
+      </c>
+    </row>
+    <row r="2886">
+      <c r="A2886" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2886" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2886" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2886" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2886" s="16" t="n">
+        <v>121.35</v>
+      </c>
+    </row>
+    <row r="2887">
+      <c r="A2887" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2887" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2887" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2887" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2887" s="19" t="n">
+        <v>95.84999999999999</v>
+      </c>
+    </row>
+    <row r="2888">
+      <c r="A2888" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2888" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2888" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2888" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2888" s="16" t="n">
+        <v>78.65000000000001</v>
+      </c>
+    </row>
+    <row r="2889">
+      <c r="A2889" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2889" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2889" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2889" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2889" s="19" t="n">
+        <v>70.3</v>
+      </c>
+    </row>
+    <row r="2890">
+      <c r="A2890" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2890" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2890" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2890" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2890" s="16" t="n">
+        <v>42.05</v>
+      </c>
+    </row>
+    <row r="2891">
+      <c r="A2891" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2891" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2891" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2891" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2891" s="19" t="n">
+        <v>79.84999999999999</v>
+      </c>
+    </row>
+    <row r="2892">
+      <c r="A2892" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2892" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2892" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2892" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2892" s="16" t="n">
+        <v>109.15</v>
+      </c>
+    </row>
+    <row r="2893">
+      <c r="A2893" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2893" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2893" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2893" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2893" s="19" t="n">
+        <v>63.6</v>
+      </c>
+    </row>
+    <row r="2894">
+      <c r="A2894" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2894" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2894" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2894" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2894" s="16" t="n">
+        <v>105.5</v>
+      </c>
+    </row>
+    <row r="2895">
+      <c r="A2895" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2895" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2895" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2895" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2895" s="19" t="n">
+        <v>167.55</v>
+      </c>
+    </row>
+    <row r="2896">
+      <c r="A2896" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2896" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2896" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2896" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2896" s="16" t="n">
+        <v>167.5</v>
+      </c>
+    </row>
+    <row r="2897">
+      <c r="A2897" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2897" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2897" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2897" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2897" s="19" t="n">
+        <v>63.5</v>
+      </c>
+    </row>
+    <row r="2898">
+      <c r="A2898" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2898" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2898" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2898" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2898" s="16" t="n">
+        <v>96.15000000000001</v>
+      </c>
+    </row>
+    <row r="2899">
+      <c r="A2899" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2899" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2899" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2899" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2899" s="19" t="n">
+        <v>161.55</v>
+      </c>
+    </row>
+    <row r="2900">
+      <c r="A2900" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2900" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2900" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2900" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2900" s="16" t="n">
+        <v>162.2</v>
+      </c>
+    </row>
+    <row r="2901">
+      <c r="A2901" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2901" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2901" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2901" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2901" s="19" t="n">
+        <v>62.75</v>
+      </c>
+    </row>
+    <row r="2902">
+      <c r="A2902" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2902" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2902" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2902" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2902" s="16" t="n">
+        <v>92.15000000000001</v>
+      </c>
+    </row>
+    <row r="2903">
+      <c r="A2903" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2903" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2903" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2903" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2903" s="19" t="n">
+        <v>156.8</v>
+      </c>
+    </row>
+    <row r="2904">
+      <c r="A2904" s="20" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2904" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2904" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2904" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2904" s="16" t="n">
+        <v>157.35</v>
+      </c>
+    </row>
+    <row r="2905">
+      <c r="A2905" s="21" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2905" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2905" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2905" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2905" s="19" t="n">
+        <v>59.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-05
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2905"/>
+  <dimension ref="A1:E2949"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -67411,6 +67411,1018 @@
         <v>59.75</v>
       </c>
     </row>
+    <row r="2906">
+      <c r="A2906" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2906" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2906" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2906" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2906" s="16" t="n">
+        <v>56.55</v>
+      </c>
+    </row>
+    <row r="2907">
+      <c r="A2907" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2907" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2907" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2907" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2907" s="19" t="n">
+        <v>114.1</v>
+      </c>
+    </row>
+    <row r="2908">
+      <c r="A2908" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2908" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2908" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2908" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2908" s="16" t="n">
+        <v>126.05</v>
+      </c>
+    </row>
+    <row r="2909">
+      <c r="A2909" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2909" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2909" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2909" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2909" s="19" t="n">
+        <v>99.75</v>
+      </c>
+    </row>
+    <row r="2910">
+      <c r="A2910" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2910" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2910" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2910" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2910" s="16" t="n">
+        <v>83.5</v>
+      </c>
+    </row>
+    <row r="2911">
+      <c r="A2911" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2911" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2911" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2911" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2911" s="19" t="n">
+        <v>79.05</v>
+      </c>
+    </row>
+    <row r="2912">
+      <c r="A2912" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2912" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2912" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2912" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2912" s="16" t="n">
+        <v>48.5</v>
+      </c>
+    </row>
+    <row r="2913">
+      <c r="A2913" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2913" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2913" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2913" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2913" s="19" t="n">
+        <v>79.65000000000001</v>
+      </c>
+    </row>
+    <row r="2914">
+      <c r="A2914" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2914" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2914" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2914" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2914" s="16" t="n">
+        <v>113.45</v>
+      </c>
+    </row>
+    <row r="2915">
+      <c r="A2915" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2915" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2915" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2915" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2915" s="19" t="n">
+        <v>70.25</v>
+      </c>
+    </row>
+    <row r="2916">
+      <c r="A2916" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2916" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2916" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2916" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2916" s="16" t="n">
+        <v>120.05</v>
+      </c>
+    </row>
+    <row r="2917">
+      <c r="A2917" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2917" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2917" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2917" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2917" s="19" t="n">
+        <v>180.25</v>
+      </c>
+    </row>
+    <row r="2918">
+      <c r="A2918" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2918" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2918" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2918" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2918" s="16" t="n">
+        <v>182.5</v>
+      </c>
+    </row>
+    <row r="2919">
+      <c r="A2919" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2919" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2919" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2919" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2919" s="19" t="n">
+        <v>69.55</v>
+      </c>
+    </row>
+    <row r="2920">
+      <c r="A2920" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2920" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2920" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2920" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2920" s="16" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2921">
+      <c r="A2921" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2921" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2921" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2921" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2921" s="19" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="2922">
+      <c r="A2922" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2922" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2922" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2922" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2922" s="16" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="2923">
+      <c r="A2923" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2923" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2923" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2923" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2923" s="19" t="n">
+        <v>68.55</v>
+      </c>
+    </row>
+    <row r="2924">
+      <c r="A2924" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2924" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2924" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2924" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2924" s="16" t="n">
+        <v>109.5</v>
+      </c>
+    </row>
+    <row r="2925">
+      <c r="A2925" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2925" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2925" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2925" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2925" s="19" t="n">
+        <v>171.85</v>
+      </c>
+    </row>
+    <row r="2926">
+      <c r="A2926" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2926" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2926" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2926" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2926" s="16" t="n">
+        <v>172.85</v>
+      </c>
+    </row>
+    <row r="2927">
+      <c r="A2927" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2927" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C2927" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2927" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2927" s="19" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2928">
+      <c r="A2928" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2928" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2928" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2928" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E2928" s="16" t="n">
+        <v>49.45</v>
+      </c>
+    </row>
+    <row r="2929">
+      <c r="A2929" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2929" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2929" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2929" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E2929" s="19" t="n">
+        <v>101.9</v>
+      </c>
+    </row>
+    <row r="2930">
+      <c r="A2930" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2930" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2930" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2930" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E2930" s="16" t="n">
+        <v>114.8</v>
+      </c>
+    </row>
+    <row r="2931">
+      <c r="A2931" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2931" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2931" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2931" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E2931" s="19" t="n">
+        <v>89.45</v>
+      </c>
+    </row>
+    <row r="2932">
+      <c r="A2932" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2932" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2932" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2932" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2932" s="16" t="n">
+        <v>72.5</v>
+      </c>
+    </row>
+    <row r="2933">
+      <c r="A2933" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2933" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2933" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2933" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E2933" s="19" t="n">
+        <v>66.15000000000001</v>
+      </c>
+    </row>
+    <row r="2934">
+      <c r="A2934" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2934" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2934" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D2934" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E2934" s="16" t="n">
+        <v>38.55</v>
+      </c>
+    </row>
+    <row r="2935">
+      <c r="A2935" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2935" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2935" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2935" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E2935" s="19" t="n">
+        <v>74.25</v>
+      </c>
+    </row>
+    <row r="2936">
+      <c r="A2936" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2936" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2936" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2936" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E2936" s="16" t="n">
+        <v>102.2</v>
+      </c>
+    </row>
+    <row r="2937">
+      <c r="A2937" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2937" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2937" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2937" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2937" s="19" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2938">
+      <c r="A2938" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2938" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2938" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2938" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E2938" s="16" t="n">
+        <v>99.7</v>
+      </c>
+    </row>
+    <row r="2939">
+      <c r="A2939" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2939" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2939" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2939" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E2939" s="19" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="2940">
+      <c r="A2940" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2940" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2940" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2940" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E2940" s="16" t="n">
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="2941">
+      <c r="A2941" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2941" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2941" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2941" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E2941" s="19" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2942">
+      <c r="A2942" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2942" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2942" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2942" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E2942" s="16" t="n">
+        <v>94.40000000000001</v>
+      </c>
+    </row>
+    <row r="2943">
+      <c r="A2943" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2943" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2943" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2943" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E2943" s="19" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2944">
+      <c r="A2944" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2944" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2944" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2944" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E2944" s="16" t="n">
+        <v>161.75</v>
+      </c>
+    </row>
+    <row r="2945">
+      <c r="A2945" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2945" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2945" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2945" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E2945" s="19" t="n">
+        <v>58.9</v>
+      </c>
+    </row>
+    <row r="2946">
+      <c r="A2946" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2946" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2946" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2946" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E2946" s="16" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2947">
+      <c r="A2947" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2947" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2947" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2947" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E2947" s="19" t="n">
+        <v>159.25</v>
+      </c>
+    </row>
+    <row r="2948">
+      <c r="A2948" s="20" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2948" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2948" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2948" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E2948" s="16" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2949">
+      <c r="A2949" s="21" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B2949" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C2949" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D2949" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E2949" s="19" t="n">
+        <v>57</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-09
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Futures Prices" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Futures Prices" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3171"/>
+  <dimension ref="A1:E3215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -73529,6 +73529,1018 @@
         <v>57</v>
       </c>
     </row>
+    <row r="3172">
+      <c r="A3172" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3172" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3172" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3172" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3172" s="16" t="n">
+        <v>45.5</v>
+      </c>
+    </row>
+    <row r="3173">
+      <c r="A3173" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3173" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3173" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3173" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3173" s="19" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3174">
+      <c r="A3174" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3174" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3174" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3174" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3174" s="16" t="n">
+        <v>119.25</v>
+      </c>
+    </row>
+    <row r="3175">
+      <c r="A3175" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3175" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3175" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3175" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3175" s="19" t="n">
+        <v>92.05</v>
+      </c>
+    </row>
+    <row r="3176">
+      <c r="A3176" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3176" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3176" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3176" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3176" s="16" t="n">
+        <v>80.90000000000001</v>
+      </c>
+    </row>
+    <row r="3177">
+      <c r="A3177" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3177" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3177" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3177" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3177" s="19" t="n">
+        <v>75.84999999999999</v>
+      </c>
+    </row>
+    <row r="3178">
+      <c r="A3178" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3178" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3178" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3178" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3178" s="16" t="n">
+        <v>47.8</v>
+      </c>
+    </row>
+    <row r="3179">
+      <c r="A3179" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3179" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3179" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3179" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3179" s="19" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3180">
+      <c r="A3180" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3180" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3180" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3180" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3180" s="16" t="n">
+        <v>105.25</v>
+      </c>
+    </row>
+    <row r="3181">
+      <c r="A3181" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3181" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3181" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3181" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3181" s="19" t="n">
+        <v>68.09999999999999</v>
+      </c>
+    </row>
+    <row r="3182">
+      <c r="A3182" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3182" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3182" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3182" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3182" s="16" t="n">
+        <v>117.5</v>
+      </c>
+    </row>
+    <row r="3183">
+      <c r="A3183" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3183" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3183" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3183" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3183" s="19" t="n">
+        <v>173.05</v>
+      </c>
+    </row>
+    <row r="3184">
+      <c r="A3184" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3184" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3184" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3184" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3184" s="16" t="n">
+        <v>173.5</v>
+      </c>
+    </row>
+    <row r="3185">
+      <c r="A3185" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3185" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3185" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3185" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3185" s="19" t="n">
+        <v>68.90000000000001</v>
+      </c>
+    </row>
+    <row r="3186">
+      <c r="A3186" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3186" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3186" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3186" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3186" s="16" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3187">
+      <c r="A3187" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3187" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3187" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3187" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3187" s="19" t="n">
+        <v>171.95</v>
+      </c>
+    </row>
+    <row r="3188">
+      <c r="A3188" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3188" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3188" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3188" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3188" s="16" t="n">
+        <v>170.4</v>
+      </c>
+    </row>
+    <row r="3189">
+      <c r="A3189" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3189" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3189" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3189" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3189" s="19" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3190">
+      <c r="A3190" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3190" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3190" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3190" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3190" s="16" t="n">
+        <v>108.5</v>
+      </c>
+    </row>
+    <row r="3191">
+      <c r="A3191" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3191" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3191" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3191" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3191" s="19" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3192">
+      <c r="A3192" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3192" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3192" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3192" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3192" s="16" t="n">
+        <v>169.8</v>
+      </c>
+    </row>
+    <row r="3193">
+      <c r="A3193" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3193" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3193" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3193" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3193" s="19" t="n">
+        <v>67.25</v>
+      </c>
+    </row>
+    <row r="3194">
+      <c r="A3194" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3194" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3194" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3194" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3194" s="16" t="n">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="3195">
+      <c r="A3195" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3195" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3195" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3195" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3195" s="19" t="n">
+        <v>96.09999999999999</v>
+      </c>
+    </row>
+    <row r="3196">
+      <c r="A3196" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3196" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3196" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3196" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3196" s="16" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3197">
+      <c r="A3197" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3197" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3197" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3197" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3197" s="19" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="3198">
+      <c r="A3198" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3198" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3198" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3198" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3198" s="16" t="n">
+        <v>69.5</v>
+      </c>
+    </row>
+    <row r="3199">
+      <c r="A3199" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3199" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3199" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3199" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3199" s="19" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3200">
+      <c r="A3200" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3200" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3200" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3200" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3200" s="16" t="n">
+        <v>36.75</v>
+      </c>
+    </row>
+    <row r="3201">
+      <c r="A3201" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3201" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3201" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3201" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3201" s="19" t="n">
+        <v>70.3</v>
+      </c>
+    </row>
+    <row r="3202">
+      <c r="A3202" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3202" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3202" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3202" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3202" s="16" t="n">
+        <v>97.55</v>
+      </c>
+    </row>
+    <row r="3203">
+      <c r="A3203" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3203" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3203" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3203" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3203" s="19" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3204">
+      <c r="A3204" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3204" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3204" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3204" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3204" s="16" t="n">
+        <v>97.5</v>
+      </c>
+    </row>
+    <row r="3205">
+      <c r="A3205" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3205" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3205" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3205" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3205" s="19" t="n">
+        <v>155.05</v>
+      </c>
+    </row>
+    <row r="3206">
+      <c r="A3206" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3206" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3206" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3206" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3206" s="16" t="n">
+        <v>156.45</v>
+      </c>
+    </row>
+    <row r="3207">
+      <c r="A3207" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3207" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3207" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3207" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3207" s="19" t="n">
+        <v>59.25</v>
+      </c>
+    </row>
+    <row r="3208">
+      <c r="A3208" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3208" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3208" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3208" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3208" s="16" t="n">
+        <v>92.45</v>
+      </c>
+    </row>
+    <row r="3209">
+      <c r="A3209" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3209" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3209" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3209" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3209" s="19" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="3210">
+      <c r="A3210" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3210" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3210" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3210" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3210" s="16" t="n">
+        <v>154.05</v>
+      </c>
+    </row>
+    <row r="3211">
+      <c r="A3211" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3211" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3211" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3211" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3211" s="19" t="n">
+        <v>58.6</v>
+      </c>
+    </row>
+    <row r="3212">
+      <c r="A3212" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3212" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3212" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3212" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3212" s="16" t="n">
+        <v>88.65000000000001</v>
+      </c>
+    </row>
+    <row r="3213">
+      <c r="A3213" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3213" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3213" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3213" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3213" s="19" t="n">
+        <v>154.5</v>
+      </c>
+    </row>
+    <row r="3214">
+      <c r="A3214" s="20" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3214" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3214" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3214" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3214" s="16" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3215">
+      <c r="A3215" s="21" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B3215" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3215" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3215" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3215" s="19" t="n">
+        <v>56.7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-10
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3215"/>
+  <dimension ref="A1:E3259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -74541,6 +74541,1018 @@
         <v>59</v>
       </c>
     </row>
+    <row r="3216">
+      <c r="A3216" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3216" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3216" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3216" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3216" s="16" t="n">
+        <v>50.4</v>
+      </c>
+    </row>
+    <row r="3217">
+      <c r="A3217" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3217" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3217" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3217" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3217" s="19" t="n">
+        <v>115.4</v>
+      </c>
+    </row>
+    <row r="3218">
+      <c r="A3218" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3218" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3218" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3218" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3218" s="16" t="n">
+        <v>126.3</v>
+      </c>
+    </row>
+    <row r="3219">
+      <c r="A3219" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3219" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3219" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3219" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3219" s="19" t="n">
+        <v>103.65</v>
+      </c>
+    </row>
+    <row r="3220">
+      <c r="A3220" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3220" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3220" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3220" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3220" s="16" t="n">
+        <v>92.2</v>
+      </c>
+    </row>
+    <row r="3221">
+      <c r="A3221" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3221" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3221" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3221" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3221" s="19" t="n">
+        <v>83.25</v>
+      </c>
+    </row>
+    <row r="3222">
+      <c r="A3222" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3222" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3222" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3222" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3222" s="16" t="n">
+        <v>48.8</v>
+      </c>
+    </row>
+    <row r="3223">
+      <c r="A3223" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3223" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3223" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3223" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3223" s="19" t="n">
+        <v>77.65000000000001</v>
+      </c>
+    </row>
+    <row r="3224">
+      <c r="A3224" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3224" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3224" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3224" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3224" s="16" t="n">
+        <v>115.25</v>
+      </c>
+    </row>
+    <row r="3225">
+      <c r="A3225" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3225" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3225" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3225" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3225" s="19" t="n">
+        <v>74.65000000000001</v>
+      </c>
+    </row>
+    <row r="3226">
+      <c r="A3226" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3226" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3226" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3226" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3226" s="16" t="n">
+        <v>130.45</v>
+      </c>
+    </row>
+    <row r="3227">
+      <c r="A3227" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3227" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3227" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3227" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3227" s="19" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="3228">
+      <c r="A3228" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3228" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3228" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3228" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3228" s="16" t="n">
+        <v>172.9</v>
+      </c>
+    </row>
+    <row r="3229">
+      <c r="A3229" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3229" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3229" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3229" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3229" s="19" t="n">
+        <v>73.09999999999999</v>
+      </c>
+    </row>
+    <row r="3230">
+      <c r="A3230" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3230" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3230" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3230" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3230" s="16" t="n">
+        <v>122.95</v>
+      </c>
+    </row>
+    <row r="3231">
+      <c r="A3231" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3231" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3231" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3231" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3231" s="19" t="n">
+        <v>168.5</v>
+      </c>
+    </row>
+    <row r="3232">
+      <c r="A3232" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3232" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3232" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3232" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3232" s="16" t="n">
+        <v>168.55</v>
+      </c>
+    </row>
+    <row r="3233">
+      <c r="A3233" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3233" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3233" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3233" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3233" s="19" t="n">
+        <v>72.5</v>
+      </c>
+    </row>
+    <row r="3234">
+      <c r="A3234" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3234" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3234" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3234" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3234" s="16" t="n">
+        <v>118.45</v>
+      </c>
+    </row>
+    <row r="3235">
+      <c r="A3235" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3235" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3235" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3235" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3235" s="19" t="n">
+        <v>166.75</v>
+      </c>
+    </row>
+    <row r="3236">
+      <c r="A3236" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3236" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3236" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3236" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3236" s="16" t="n">
+        <v>166.3</v>
+      </c>
+    </row>
+    <row r="3237">
+      <c r="A3237" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3237" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3237" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3237" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3237" s="19" t="n">
+        <v>69.8</v>
+      </c>
+    </row>
+    <row r="3238">
+      <c r="A3238" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3238" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3238" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3238" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3238" s="16" t="n">
+        <v>42.6</v>
+      </c>
+    </row>
+    <row r="3239">
+      <c r="A3239" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3239" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3239" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3239" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3239" s="19" t="n">
+        <v>105.8</v>
+      </c>
+    </row>
+    <row r="3240">
+      <c r="A3240" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3240" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3240" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3240" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3240" s="16" t="n">
+        <v>116.5</v>
+      </c>
+    </row>
+    <row r="3241">
+      <c r="A3241" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3241" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3241" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3241" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3241" s="19" t="n">
+        <v>98.45</v>
+      </c>
+    </row>
+    <row r="3242">
+      <c r="A3242" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3242" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3242" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3242" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3242" s="16" t="n">
+        <v>85.25</v>
+      </c>
+    </row>
+    <row r="3243">
+      <c r="A3243" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3243" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3243" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3243" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3243" s="19" t="n">
+        <v>71.34999999999999</v>
+      </c>
+    </row>
+    <row r="3244">
+      <c r="A3244" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3244" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3244" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3244" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3244" s="16" t="n">
+        <v>41.3</v>
+      </c>
+    </row>
+    <row r="3245">
+      <c r="A3245" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3245" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3245" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3245" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3245" s="19" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3246">
+      <c r="A3246" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3246" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3246" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3246" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3246" s="16" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3247">
+      <c r="A3247" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3247" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3247" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3247" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3247" s="19" t="n">
+        <v>65.90000000000001</v>
+      </c>
+    </row>
+    <row r="3248">
+      <c r="A3248" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3248" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3248" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3248" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3248" s="16" t="n">
+        <v>112.65</v>
+      </c>
+    </row>
+    <row r="3249">
+      <c r="A3249" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3249" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3249" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3249" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3249" s="19" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3250">
+      <c r="A3250" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3250" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3250" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3250" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3250" s="16" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3251">
+      <c r="A3251" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3251" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3251" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3251" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3251" s="19" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3252">
+      <c r="A3252" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3252" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3252" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3252" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3252" s="16" t="n">
+        <v>104.65</v>
+      </c>
+    </row>
+    <row r="3253">
+      <c r="A3253" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3253" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3253" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3253" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3253" s="19" t="n">
+        <v>151.7</v>
+      </c>
+    </row>
+    <row r="3254">
+      <c r="A3254" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3254" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3254" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3254" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3254" s="16" t="n">
+        <v>148.5</v>
+      </c>
+    </row>
+    <row r="3255">
+      <c r="A3255" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3255" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3255" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3255" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3255" s="19" t="n">
+        <v>62.9</v>
+      </c>
+    </row>
+    <row r="3256">
+      <c r="A3256" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3256" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3256" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3256" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3256" s="16" t="n">
+        <v>98.65000000000001</v>
+      </c>
+    </row>
+    <row r="3257">
+      <c r="A3257" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3257" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3257" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3257" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3257" s="19" t="n">
+        <v>150.95</v>
+      </c>
+    </row>
+    <row r="3258">
+      <c r="A3258" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3258" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3258" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3258" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3258" s="16" t="n">
+        <v>149.15</v>
+      </c>
+    </row>
+    <row r="3259">
+      <c r="A3259" s="21" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B3259" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3259" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3259" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3259" s="19" t="n">
+        <v>59.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-11
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3259"/>
+  <dimension ref="A1:E3303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -75553,6 +75553,1018 @@
         <v>59.8</v>
       </c>
     </row>
+    <row r="3260">
+      <c r="A3260" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3260" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3260" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3260" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3260" s="16" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3261">
+      <c r="A3261" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3261" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3261" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3261" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3261" s="19" t="n">
+        <v>111.45</v>
+      </c>
+    </row>
+    <row r="3262">
+      <c r="A3262" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3262" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3262" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3262" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3262" s="16" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3263">
+      <c r="A3263" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3263" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3263" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3263" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3263" s="19" t="n">
+        <v>101.75</v>
+      </c>
+    </row>
+    <row r="3264">
+      <c r="A3264" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3264" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3264" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3264" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3264" s="16" t="n">
+        <v>91.59999999999999</v>
+      </c>
+    </row>
+    <row r="3265">
+      <c r="A3265" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3265" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3265" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3265" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3265" s="19" t="n">
+        <v>82.5</v>
+      </c>
+    </row>
+    <row r="3266">
+      <c r="A3266" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3266" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3266" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3266" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3266" s="16" t="n">
+        <v>60.65</v>
+      </c>
+    </row>
+    <row r="3267">
+      <c r="A3267" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3267" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3267" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3267" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3267" s="19" t="n">
+        <v>76.84999999999999</v>
+      </c>
+    </row>
+    <row r="3268">
+      <c r="A3268" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3268" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3268" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3268" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3268" s="16" t="n">
+        <v>111.85</v>
+      </c>
+    </row>
+    <row r="3269">
+      <c r="A3269" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3269" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3269" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3269" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3269" s="19" t="n">
+        <v>78.2</v>
+      </c>
+    </row>
+    <row r="3270">
+      <c r="A3270" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3270" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3270" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3270" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3270" s="16" t="n">
+        <v>136.2</v>
+      </c>
+    </row>
+    <row r="3271">
+      <c r="A3271" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3271" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3271" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3271" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3271" s="19" t="n">
+        <v>174.65</v>
+      </c>
+    </row>
+    <row r="3272">
+      <c r="A3272" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3272" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3272" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3272" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3272" s="16" t="n">
+        <v>173.25</v>
+      </c>
+    </row>
+    <row r="3273">
+      <c r="A3273" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3273" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3273" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3273" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3273" s="19" t="n">
+        <v>73.34999999999999</v>
+      </c>
+    </row>
+    <row r="3274">
+      <c r="A3274" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3274" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3274" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3274" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3274" s="16" t="n">
+        <v>126.4</v>
+      </c>
+    </row>
+    <row r="3275">
+      <c r="A3275" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3275" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3275" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3275" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3275" s="19" t="n">
+        <v>168.5</v>
+      </c>
+    </row>
+    <row r="3276">
+      <c r="A3276" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3276" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3276" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3276" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3276" s="16" t="n">
+        <v>169.95</v>
+      </c>
+    </row>
+    <row r="3277">
+      <c r="A3277" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3277" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3277" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3277" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3277" s="19" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3278">
+      <c r="A3278" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3278" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3278" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3278" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3278" s="16" t="n">
+        <v>120.95</v>
+      </c>
+    </row>
+    <row r="3279">
+      <c r="A3279" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3279" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3279" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3279" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3279" s="19" t="n">
+        <v>166.75</v>
+      </c>
+    </row>
+    <row r="3280">
+      <c r="A3280" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3280" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3280" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3280" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3280" s="16" t="n">
+        <v>166.3</v>
+      </c>
+    </row>
+    <row r="3281">
+      <c r="A3281" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3281" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3281" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3281" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3281" s="19" t="n">
+        <v>70.90000000000001</v>
+      </c>
+    </row>
+    <row r="3282">
+      <c r="A3282" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3282" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3282" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3282" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3282" s="16" t="n">
+        <v>39.85</v>
+      </c>
+    </row>
+    <row r="3283">
+      <c r="A3283" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3283" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3283" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3283" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3283" s="19" t="n">
+        <v>99.09999999999999</v>
+      </c>
+    </row>
+    <row r="3284">
+      <c r="A3284" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3284" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3284" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3284" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3284" s="16" t="n">
+        <v>112.7</v>
+      </c>
+    </row>
+    <row r="3285">
+      <c r="A3285" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3285" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3285" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3285" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3285" s="19" t="n">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3286">
+      <c r="A3286" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3286" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3286" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3286" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3286" s="16" t="n">
+        <v>82.40000000000001</v>
+      </c>
+    </row>
+    <row r="3287">
+      <c r="A3287" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3287" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3287" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3287" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3287" s="19" t="n">
+        <v>76.45</v>
+      </c>
+    </row>
+    <row r="3288">
+      <c r="A3288" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3288" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3288" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3288" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3288" s="16" t="n">
+        <v>45.15</v>
+      </c>
+    </row>
+    <row r="3289">
+      <c r="A3289" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3289" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3289" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3289" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3289" s="19" t="n">
+        <v>71.09999999999999</v>
+      </c>
+    </row>
+    <row r="3290">
+      <c r="A3290" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3290" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3290" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3290" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3290" s="16" t="n">
+        <v>101.7</v>
+      </c>
+    </row>
+    <row r="3291">
+      <c r="A3291" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3291" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3291" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3291" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3291" s="19" t="n">
+        <v>67.90000000000001</v>
+      </c>
+    </row>
+    <row r="3292">
+      <c r="A3292" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3292" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3292" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3292" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3292" s="16" t="n">
+        <v>116.6</v>
+      </c>
+    </row>
+    <row r="3293">
+      <c r="A3293" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3293" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3293" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3293" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3293" s="19" t="n">
+        <v>156.3</v>
+      </c>
+    </row>
+    <row r="3294">
+      <c r="A3294" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3294" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3294" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3294" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3294" s="16" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3295">
+      <c r="A3295" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3295" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3295" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3295" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3295" s="19" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3296">
+      <c r="A3296" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3296" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3296" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3296" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3296" s="16" t="n">
+        <v>107.4</v>
+      </c>
+    </row>
+    <row r="3297">
+      <c r="A3297" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3297" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3297" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3297" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3297" s="19" t="n">
+        <v>153.45</v>
+      </c>
+    </row>
+    <row r="3298">
+      <c r="A3298" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3298" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3298" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3298" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3298" s="16" t="n">
+        <v>152.15</v>
+      </c>
+    </row>
+    <row r="3299">
+      <c r="A3299" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3299" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3299" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3299" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3299" s="19" t="n">
+        <v>63.25</v>
+      </c>
+    </row>
+    <row r="3300">
+      <c r="A3300" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3300" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3300" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3300" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3300" s="16" t="n">
+        <v>103.25</v>
+      </c>
+    </row>
+    <row r="3301">
+      <c r="A3301" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3301" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3301" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3301" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3301" s="19" t="n">
+        <v>150.95</v>
+      </c>
+    </row>
+    <row r="3302">
+      <c r="A3302" s="20" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3302" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3302" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3302" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3302" s="16" t="n">
+        <v>149.15</v>
+      </c>
+    </row>
+    <row r="3303">
+      <c r="A3303" s="21" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B3303" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3303" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3303" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3303" s="19" t="n">
+        <v>61.65</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-12
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3303"/>
+  <dimension ref="A1:E3347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -76565,6 +76565,1018 @@
         <v>61.65</v>
       </c>
     </row>
+    <row r="3304">
+      <c r="A3304" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3304" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3304" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3304" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3304" s="16" t="n">
+        <v>47.45</v>
+      </c>
+    </row>
+    <row r="3305">
+      <c r="A3305" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3305" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3305" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3305" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3305" s="19" t="n">
+        <v>106.25</v>
+      </c>
+    </row>
+    <row r="3306">
+      <c r="A3306" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3306" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3306" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3306" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3306" s="16" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="3307">
+      <c r="A3307" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3307" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3307" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3307" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3307" s="19" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3308">
+      <c r="A3308" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3308" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3308" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3308" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3308" s="16" t="n">
+        <v>93.05</v>
+      </c>
+    </row>
+    <row r="3309">
+      <c r="A3309" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3309" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3309" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3309" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3309" s="19" t="n">
+        <v>84.34999999999999</v>
+      </c>
+    </row>
+    <row r="3310">
+      <c r="A3310" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3310" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3310" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3310" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3310" s="16" t="n">
+        <v>62.9</v>
+      </c>
+    </row>
+    <row r="3311">
+      <c r="A3311" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3311" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3311" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3311" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3311" s="19" t="n">
+        <v>76.65000000000001</v>
+      </c>
+    </row>
+    <row r="3312">
+      <c r="A3312" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3312" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3312" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3312" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3312" s="16" t="n">
+        <v>110.85</v>
+      </c>
+    </row>
+    <row r="3313">
+      <c r="A3313" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3313" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3313" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3313" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3313" s="19" t="n">
+        <v>80.05</v>
+      </c>
+    </row>
+    <row r="3314">
+      <c r="A3314" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3314" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3314" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3314" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3314" s="16" t="n">
+        <v>136.7</v>
+      </c>
+    </row>
+    <row r="3315">
+      <c r="A3315" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3315" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3315" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3315" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3315" s="19" t="n">
+        <v>174.65</v>
+      </c>
+    </row>
+    <row r="3316">
+      <c r="A3316" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3316" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3316" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3316" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3316" s="16" t="n">
+        <v>173.25</v>
+      </c>
+    </row>
+    <row r="3317">
+      <c r="A3317" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3317" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3317" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3317" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3317" s="19" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3318">
+      <c r="A3318" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3318" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3318" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3318" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3318" s="16" t="n">
+        <v>126.4</v>
+      </c>
+    </row>
+    <row r="3319">
+      <c r="A3319" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3319" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3319" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3319" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3319" s="19" t="n">
+        <v>168.5</v>
+      </c>
+    </row>
+    <row r="3320">
+      <c r="A3320" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3320" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3320" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3320" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3320" s="16" t="n">
+        <v>169.95</v>
+      </c>
+    </row>
+    <row r="3321">
+      <c r="A3321" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3321" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3321" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3321" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3321" s="19" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3322">
+      <c r="A3322" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3322" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3322" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3322" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3322" s="16" t="n">
+        <v>120.95</v>
+      </c>
+    </row>
+    <row r="3323">
+      <c r="A3323" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3323" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3323" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3323" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3323" s="19" t="n">
+        <v>166.75</v>
+      </c>
+    </row>
+    <row r="3324">
+      <c r="A3324" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3324" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3324" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3324" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3324" s="16" t="n">
+        <v>166.3</v>
+      </c>
+    </row>
+    <row r="3325">
+      <c r="A3325" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3325" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3325" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3325" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3325" s="19" t="n">
+        <v>71.34999999999999</v>
+      </c>
+    </row>
+    <row r="3326">
+      <c r="A3326" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3326" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3326" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3326" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3326" s="16" t="n">
+        <v>39.9</v>
+      </c>
+    </row>
+    <row r="3327">
+      <c r="A3327" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3327" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3327" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3327" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3327" s="19" t="n">
+        <v>94.34999999999999</v>
+      </c>
+    </row>
+    <row r="3328">
+      <c r="A3328" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3328" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3328" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3328" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3328" s="16" t="n">
+        <v>112.05</v>
+      </c>
+    </row>
+    <row r="3329">
+      <c r="A3329" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3329" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3329" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3329" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3329" s="19" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3330">
+      <c r="A3330" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3330" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3330" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3330" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3330" s="16" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3331">
+      <c r="A3331" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3331" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3331" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3331" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3331" s="19" t="n">
+        <v>76.34999999999999</v>
+      </c>
+    </row>
+    <row r="3332">
+      <c r="A3332" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3332" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3332" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3332" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3332" s="16" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3333">
+      <c r="A3333" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3333" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3333" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3333" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3333" s="19" t="n">
+        <v>71.09999999999999</v>
+      </c>
+    </row>
+    <row r="3334">
+      <c r="A3334" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3334" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3334" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3334" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3334" s="16" t="n">
+        <v>100.2</v>
+      </c>
+    </row>
+    <row r="3335">
+      <c r="A3335" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3335" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3335" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3335" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3335" s="19" t="n">
+        <v>69.05</v>
+      </c>
+    </row>
+    <row r="3336">
+      <c r="A3336" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3336" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3336" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3336" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3336" s="16" t="n">
+        <v>118.4</v>
+      </c>
+    </row>
+    <row r="3337">
+      <c r="A3337" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3337" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3337" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3337" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3337" s="19" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="3338">
+      <c r="A3338" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3338" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3338" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3338" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3338" s="16" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3339">
+      <c r="A3339" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3339" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3339" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3339" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3339" s="19" t="n">
+        <v>65.2</v>
+      </c>
+    </row>
+    <row r="3340">
+      <c r="A3340" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3340" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3340" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3340" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3340" s="16" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3341">
+      <c r="A3341" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3341" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3341" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3341" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3341" s="19" t="n">
+        <v>153.45</v>
+      </c>
+    </row>
+    <row r="3342">
+      <c r="A3342" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3342" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3342" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3342" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3342" s="16" t="n">
+        <v>153.9</v>
+      </c>
+    </row>
+    <row r="3343">
+      <c r="A3343" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3343" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3343" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3343" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3343" s="19" t="n">
+        <v>63.25</v>
+      </c>
+    </row>
+    <row r="3344">
+      <c r="A3344" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3344" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3344" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3344" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3344" s="16" t="n">
+        <v>102.75</v>
+      </c>
+    </row>
+    <row r="3345">
+      <c r="A3345" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3345" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3345" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3345" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3345" s="19" t="n">
+        <v>150.95</v>
+      </c>
+    </row>
+    <row r="3346">
+      <c r="A3346" s="20" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3346" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3346" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3346" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3346" s="16" t="n">
+        <v>149.15</v>
+      </c>
+    </row>
+    <row r="3347">
+      <c r="A3347" s="21" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B3347" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3347" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3347" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3347" s="19" t="n">
+        <v>62.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-13
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3347"/>
+  <dimension ref="A1:E3391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -77577,6 +77577,1018 @@
         <v>62.4</v>
       </c>
     </row>
+    <row r="3348">
+      <c r="A3348" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3348" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3348" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3348" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3348" s="16" t="n">
+        <v>47.45</v>
+      </c>
+    </row>
+    <row r="3349">
+      <c r="A3349" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3349" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3349" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3349" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3349" s="19" t="n">
+        <v>106.25</v>
+      </c>
+    </row>
+    <row r="3350">
+      <c r="A3350" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3350" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3350" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3350" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3350" s="16" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="3351">
+      <c r="A3351" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3351" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3351" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3351" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3351" s="19" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3352">
+      <c r="A3352" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3352" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3352" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3352" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3352" s="16" t="n">
+        <v>93.05</v>
+      </c>
+    </row>
+    <row r="3353">
+      <c r="A3353" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3353" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3353" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3353" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3353" s="19" t="n">
+        <v>84.34999999999999</v>
+      </c>
+    </row>
+    <row r="3354">
+      <c r="A3354" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3354" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3354" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3354" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3354" s="16" t="n">
+        <v>62.9</v>
+      </c>
+    </row>
+    <row r="3355">
+      <c r="A3355" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3355" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3355" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3355" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3355" s="19" t="n">
+        <v>76.65000000000001</v>
+      </c>
+    </row>
+    <row r="3356">
+      <c r="A3356" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3356" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3356" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3356" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3356" s="16" t="n">
+        <v>110.85</v>
+      </c>
+    </row>
+    <row r="3357">
+      <c r="A3357" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3357" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3357" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3357" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3357" s="19" t="n">
+        <v>80.05</v>
+      </c>
+    </row>
+    <row r="3358">
+      <c r="A3358" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3358" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3358" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3358" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3358" s="16" t="n">
+        <v>136.7</v>
+      </c>
+    </row>
+    <row r="3359">
+      <c r="A3359" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3359" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3359" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3359" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3359" s="19" t="n">
+        <v>174.65</v>
+      </c>
+    </row>
+    <row r="3360">
+      <c r="A3360" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3360" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3360" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3360" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3360" s="16" t="n">
+        <v>173.25</v>
+      </c>
+    </row>
+    <row r="3361">
+      <c r="A3361" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3361" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3361" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3361" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3361" s="19" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3362">
+      <c r="A3362" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3362" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3362" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3362" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3362" s="16" t="n">
+        <v>126.4</v>
+      </c>
+    </row>
+    <row r="3363">
+      <c r="A3363" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3363" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3363" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3363" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3363" s="19" t="n">
+        <v>168.5</v>
+      </c>
+    </row>
+    <row r="3364">
+      <c r="A3364" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3364" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3364" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3364" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3364" s="16" t="n">
+        <v>169.95</v>
+      </c>
+    </row>
+    <row r="3365">
+      <c r="A3365" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3365" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3365" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3365" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3365" s="19" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3366">
+      <c r="A3366" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3366" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3366" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3366" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3366" s="16" t="n">
+        <v>120.95</v>
+      </c>
+    </row>
+    <row r="3367">
+      <c r="A3367" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3367" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3367" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3367" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3367" s="19" t="n">
+        <v>166.75</v>
+      </c>
+    </row>
+    <row r="3368">
+      <c r="A3368" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3368" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3368" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3368" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3368" s="16" t="n">
+        <v>166.3</v>
+      </c>
+    </row>
+    <row r="3369">
+      <c r="A3369" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3369" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3369" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3369" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3369" s="19" t="n">
+        <v>71.34999999999999</v>
+      </c>
+    </row>
+    <row r="3370">
+      <c r="A3370" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3370" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3370" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3370" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3370" s="16" t="n">
+        <v>39.9</v>
+      </c>
+    </row>
+    <row r="3371">
+      <c r="A3371" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3371" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3371" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3371" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3371" s="19" t="n">
+        <v>94.34999999999999</v>
+      </c>
+    </row>
+    <row r="3372">
+      <c r="A3372" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3372" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3372" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3372" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3372" s="16" t="n">
+        <v>112.05</v>
+      </c>
+    </row>
+    <row r="3373">
+      <c r="A3373" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3373" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3373" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3373" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3373" s="19" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3374">
+      <c r="A3374" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3374" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3374" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3374" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3374" s="16" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3375">
+      <c r="A3375" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3375" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3375" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3375" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3375" s="19" t="n">
+        <v>76.34999999999999</v>
+      </c>
+    </row>
+    <row r="3376">
+      <c r="A3376" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3376" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3376" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3376" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3376" s="16" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3377">
+      <c r="A3377" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3377" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3377" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3377" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3377" s="19" t="n">
+        <v>71.09999999999999</v>
+      </c>
+    </row>
+    <row r="3378">
+      <c r="A3378" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3378" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3378" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3378" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3378" s="16" t="n">
+        <v>100.2</v>
+      </c>
+    </row>
+    <row r="3379">
+      <c r="A3379" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3379" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3379" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3379" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3379" s="19" t="n">
+        <v>69.05</v>
+      </c>
+    </row>
+    <row r="3380">
+      <c r="A3380" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3380" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3380" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3380" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3380" s="16" t="n">
+        <v>118.4</v>
+      </c>
+    </row>
+    <row r="3381">
+      <c r="A3381" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3381" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3381" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3381" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3381" s="19" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="3382">
+      <c r="A3382" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3382" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3382" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3382" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3382" s="16" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3383">
+      <c r="A3383" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3383" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3383" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3383" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3383" s="19" t="n">
+        <v>65.2</v>
+      </c>
+    </row>
+    <row r="3384">
+      <c r="A3384" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3384" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3384" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3384" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3384" s="16" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3385">
+      <c r="A3385" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3385" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3385" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3385" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3385" s="19" t="n">
+        <v>153.45</v>
+      </c>
+    </row>
+    <row r="3386">
+      <c r="A3386" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3386" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3386" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3386" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3386" s="16" t="n">
+        <v>153.9</v>
+      </c>
+    </row>
+    <row r="3387">
+      <c r="A3387" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3387" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3387" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3387" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3387" s="19" t="n">
+        <v>63.25</v>
+      </c>
+    </row>
+    <row r="3388">
+      <c r="A3388" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3388" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3388" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3388" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3388" s="16" t="n">
+        <v>102.75</v>
+      </c>
+    </row>
+    <row r="3389">
+      <c r="A3389" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3389" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3389" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3389" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3389" s="19" t="n">
+        <v>150.95</v>
+      </c>
+    </row>
+    <row r="3390">
+      <c r="A3390" s="20" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3390" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3390" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3390" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3390" s="16" t="n">
+        <v>149.15</v>
+      </c>
+    </row>
+    <row r="3391">
+      <c r="A3391" s="21" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B3391" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3391" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3391" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3391" s="19" t="n">
+        <v>62.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-14
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3391"/>
+  <dimension ref="A1:E3435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -78589,6 +78589,1018 @@
         <v>62.4</v>
       </c>
     </row>
+    <row r="3392">
+      <c r="A3392" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3392" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3392" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3392" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3392" s="16" t="n">
+        <v>47.45</v>
+      </c>
+    </row>
+    <row r="3393">
+      <c r="A3393" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3393" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3393" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3393" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3393" s="19" t="n">
+        <v>106.25</v>
+      </c>
+    </row>
+    <row r="3394">
+      <c r="A3394" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3394" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3394" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3394" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3394" s="16" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="3395">
+      <c r="A3395" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3395" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3395" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3395" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3395" s="19" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3396">
+      <c r="A3396" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3396" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3396" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3396" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3396" s="16" t="n">
+        <v>93.05</v>
+      </c>
+    </row>
+    <row r="3397">
+      <c r="A3397" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3397" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3397" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3397" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3397" s="19" t="n">
+        <v>84.34999999999999</v>
+      </c>
+    </row>
+    <row r="3398">
+      <c r="A3398" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3398" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3398" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3398" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3398" s="16" t="n">
+        <v>62.9</v>
+      </c>
+    </row>
+    <row r="3399">
+      <c r="A3399" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3399" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3399" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3399" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3399" s="19" t="n">
+        <v>76.65000000000001</v>
+      </c>
+    </row>
+    <row r="3400">
+      <c r="A3400" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3400" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3400" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3400" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3400" s="16" t="n">
+        <v>110.85</v>
+      </c>
+    </row>
+    <row r="3401">
+      <c r="A3401" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3401" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3401" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3401" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3401" s="19" t="n">
+        <v>80.05</v>
+      </c>
+    </row>
+    <row r="3402">
+      <c r="A3402" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3402" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3402" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3402" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3402" s="16" t="n">
+        <v>136.7</v>
+      </c>
+    </row>
+    <row r="3403">
+      <c r="A3403" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3403" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3403" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3403" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3403" s="19" t="n">
+        <v>174.65</v>
+      </c>
+    </row>
+    <row r="3404">
+      <c r="A3404" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3404" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3404" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3404" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3404" s="16" t="n">
+        <v>173.25</v>
+      </c>
+    </row>
+    <row r="3405">
+      <c r="A3405" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3405" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3405" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3405" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3405" s="19" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3406">
+      <c r="A3406" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3406" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3406" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3406" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3406" s="16" t="n">
+        <v>126.4</v>
+      </c>
+    </row>
+    <row r="3407">
+      <c r="A3407" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3407" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3407" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3407" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3407" s="19" t="n">
+        <v>168.5</v>
+      </c>
+    </row>
+    <row r="3408">
+      <c r="A3408" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3408" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3408" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3408" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3408" s="16" t="n">
+        <v>169.95</v>
+      </c>
+    </row>
+    <row r="3409">
+      <c r="A3409" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3409" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3409" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3409" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3409" s="19" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3410">
+      <c r="A3410" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3410" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3410" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3410" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3410" s="16" t="n">
+        <v>120.95</v>
+      </c>
+    </row>
+    <row r="3411">
+      <c r="A3411" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3411" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3411" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3411" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3411" s="19" t="n">
+        <v>166.75</v>
+      </c>
+    </row>
+    <row r="3412">
+      <c r="A3412" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3412" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3412" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3412" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3412" s="16" t="n">
+        <v>166.3</v>
+      </c>
+    </row>
+    <row r="3413">
+      <c r="A3413" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3413" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3413" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3413" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3413" s="19" t="n">
+        <v>71.34999999999999</v>
+      </c>
+    </row>
+    <row r="3414">
+      <c r="A3414" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3414" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3414" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3414" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3414" s="16" t="n">
+        <v>39.9</v>
+      </c>
+    </row>
+    <row r="3415">
+      <c r="A3415" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3415" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3415" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3415" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3415" s="19" t="n">
+        <v>94.34999999999999</v>
+      </c>
+    </row>
+    <row r="3416">
+      <c r="A3416" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3416" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3416" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3416" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3416" s="16" t="n">
+        <v>112.05</v>
+      </c>
+    </row>
+    <row r="3417">
+      <c r="A3417" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3417" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3417" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3417" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3417" s="19" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3418">
+      <c r="A3418" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3418" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3418" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3418" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3418" s="16" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3419">
+      <c r="A3419" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3419" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3419" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3419" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3419" s="19" t="n">
+        <v>76.34999999999999</v>
+      </c>
+    </row>
+    <row r="3420">
+      <c r="A3420" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3420" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3420" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3420" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3420" s="16" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3421">
+      <c r="A3421" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3421" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3421" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3421" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3421" s="19" t="n">
+        <v>71.09999999999999</v>
+      </c>
+    </row>
+    <row r="3422">
+      <c r="A3422" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3422" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3422" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3422" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3422" s="16" t="n">
+        <v>100.2</v>
+      </c>
+    </row>
+    <row r="3423">
+      <c r="A3423" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3423" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3423" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3423" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3423" s="19" t="n">
+        <v>69.05</v>
+      </c>
+    </row>
+    <row r="3424">
+      <c r="A3424" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3424" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3424" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3424" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3424" s="16" t="n">
+        <v>118.4</v>
+      </c>
+    </row>
+    <row r="3425">
+      <c r="A3425" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3425" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3425" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3425" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3425" s="19" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="3426">
+      <c r="A3426" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3426" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3426" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3426" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3426" s="16" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3427">
+      <c r="A3427" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3427" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3427" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3427" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3427" s="19" t="n">
+        <v>65.2</v>
+      </c>
+    </row>
+    <row r="3428">
+      <c r="A3428" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3428" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3428" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3428" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3428" s="16" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3429">
+      <c r="A3429" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3429" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3429" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3429" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3429" s="19" t="n">
+        <v>153.45</v>
+      </c>
+    </row>
+    <row r="3430">
+      <c r="A3430" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3430" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3430" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3430" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3430" s="16" t="n">
+        <v>153.9</v>
+      </c>
+    </row>
+    <row r="3431">
+      <c r="A3431" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3431" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3431" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3431" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3431" s="19" t="n">
+        <v>63.25</v>
+      </c>
+    </row>
+    <row r="3432">
+      <c r="A3432" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3432" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3432" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3432" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3432" s="16" t="n">
+        <v>102.75</v>
+      </c>
+    </row>
+    <row r="3433">
+      <c r="A3433" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3433" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3433" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3433" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3433" s="19" t="n">
+        <v>150.95</v>
+      </c>
+    </row>
+    <row r="3434">
+      <c r="A3434" s="20" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3434" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3434" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3434" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3434" s="16" t="n">
+        <v>149.15</v>
+      </c>
+    </row>
+    <row r="3435">
+      <c r="A3435" s="21" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B3435" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3435" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3435" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3435" s="19" t="n">
+        <v>62.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-16
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3435"/>
+  <dimension ref="A1:E3479"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -79601,6 +79601,1018 @@
         <v>62.4</v>
       </c>
     </row>
+    <row r="3436">
+      <c r="A3436" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3436" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3436" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3436" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3436" s="16" t="n">
+        <v>47.45</v>
+      </c>
+    </row>
+    <row r="3437">
+      <c r="A3437" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3437" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3437" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3437" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3437" s="19" t="n">
+        <v>108.25</v>
+      </c>
+    </row>
+    <row r="3438">
+      <c r="A3438" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3438" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3438" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3438" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3438" s="16" t="n">
+        <v>126.75</v>
+      </c>
+    </row>
+    <row r="3439">
+      <c r="A3439" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3439" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3439" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3439" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3439" s="19" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3440">
+      <c r="A3440" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3440" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3440" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3440" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3440" s="16" t="n">
+        <v>93.59999999999999</v>
+      </c>
+    </row>
+    <row r="3441">
+      <c r="A3441" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3441" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3441" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3441" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3441" s="19" t="n">
+        <v>86.05</v>
+      </c>
+    </row>
+    <row r="3442">
+      <c r="A3442" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3442" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3442" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3442" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3442" s="16" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3443">
+      <c r="A3443" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3443" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3443" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3443" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3443" s="19" t="n">
+        <v>76.65000000000001</v>
+      </c>
+    </row>
+    <row r="3444">
+      <c r="A3444" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3444" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3444" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3444" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3444" s="16" t="n">
+        <v>112.8</v>
+      </c>
+    </row>
+    <row r="3445">
+      <c r="A3445" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3445" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3445" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3445" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3445" s="19" t="n">
+        <v>78.8</v>
+      </c>
+    </row>
+    <row r="3446">
+      <c r="A3446" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3446" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3446" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3446" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3446" s="16" t="n">
+        <v>129.5</v>
+      </c>
+    </row>
+    <row r="3447">
+      <c r="A3447" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3447" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3447" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3447" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3447" s="19" t="n">
+        <v>175.4</v>
+      </c>
+    </row>
+    <row r="3448">
+      <c r="A3448" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3448" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3448" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3448" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3448" s="16" t="n">
+        <v>175.05</v>
+      </c>
+    </row>
+    <row r="3449">
+      <c r="A3449" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3449" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3449" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3449" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3449" s="19" t="n">
+        <v>73.3</v>
+      </c>
+    </row>
+    <row r="3450">
+      <c r="A3450" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3450" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3450" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3450" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3450" s="16" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3451">
+      <c r="A3451" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3451" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3451" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3451" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3451" s="19" t="n">
+        <v>168.5</v>
+      </c>
+    </row>
+    <row r="3452">
+      <c r="A3452" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3452" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3452" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3452" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3452" s="16" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="3453">
+      <c r="A3453" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3453" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3453" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3453" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3453" s="19" t="n">
+        <v>70.90000000000001</v>
+      </c>
+    </row>
+    <row r="3454">
+      <c r="A3454" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3454" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3454" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3454" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3454" s="16" t="n">
+        <v>118.2</v>
+      </c>
+    </row>
+    <row r="3455">
+      <c r="A3455" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3455" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3455" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3455" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3455" s="19" t="n">
+        <v>161.5</v>
+      </c>
+    </row>
+    <row r="3456">
+      <c r="A3456" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3456" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3456" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3456" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3456" s="16" t="n">
+        <v>161.1</v>
+      </c>
+    </row>
+    <row r="3457">
+      <c r="A3457" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3457" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3457" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3457" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3457" s="19" t="n">
+        <v>69.75</v>
+      </c>
+    </row>
+    <row r="3458">
+      <c r="A3458" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3458" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3458" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3458" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3458" s="16" t="n">
+        <v>41.1</v>
+      </c>
+    </row>
+    <row r="3459">
+      <c r="A3459" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3459" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3459" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3459" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3459" s="19" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3460">
+      <c r="A3460" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3460" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3460" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3460" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3460" s="16" t="n">
+        <v>114.1</v>
+      </c>
+    </row>
+    <row r="3461">
+      <c r="A3461" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3461" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3461" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3461" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3461" s="19" t="n">
+        <v>95.45</v>
+      </c>
+    </row>
+    <row r="3462">
+      <c r="A3462" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3462" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3462" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3462" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3462" s="16" t="n">
+        <v>82.95</v>
+      </c>
+    </row>
+    <row r="3463">
+      <c r="A3463" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3463" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3463" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3463" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3463" s="19" t="n">
+        <v>75.34999999999999</v>
+      </c>
+    </row>
+    <row r="3464">
+      <c r="A3464" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3464" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3464" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3464" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3464" s="16" t="n">
+        <v>46.85</v>
+      </c>
+    </row>
+    <row r="3465">
+      <c r="A3465" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3465" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3465" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3465" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3465" s="19" t="n">
+        <v>71.5</v>
+      </c>
+    </row>
+    <row r="3466">
+      <c r="A3466" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3466" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3466" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3466" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3466" s="16" t="n">
+        <v>101.9</v>
+      </c>
+    </row>
+    <row r="3467">
+      <c r="A3467" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3467" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3467" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3467" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3467" s="19" t="n">
+        <v>68.3</v>
+      </c>
+    </row>
+    <row r="3468">
+      <c r="A3468" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3468" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3468" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3468" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3468" s="16" t="n">
+        <v>109.7</v>
+      </c>
+    </row>
+    <row r="3469">
+      <c r="A3469" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3469" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3469" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3469" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3469" s="19" t="n">
+        <v>156.4</v>
+      </c>
+    </row>
+    <row r="3470">
+      <c r="A3470" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3470" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3470" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3470" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3470" s="16" t="n">
+        <v>156.05</v>
+      </c>
+    </row>
+    <row r="3471">
+      <c r="A3471" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3471" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3471" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3471" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3471" s="19" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3472">
+      <c r="A3472" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3472" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3472" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3472" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3472" s="16" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3473">
+      <c r="A3473" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3473" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3473" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3473" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3473" s="19" t="n">
+        <v>152.4</v>
+      </c>
+    </row>
+    <row r="3474">
+      <c r="A3474" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3474" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3474" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3474" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3474" s="16" t="n">
+        <v>153.15</v>
+      </c>
+    </row>
+    <row r="3475">
+      <c r="A3475" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3475" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3475" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3475" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3475" s="19" t="n">
+        <v>60.15</v>
+      </c>
+    </row>
+    <row r="3476">
+      <c r="A3476" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3476" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3476" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3476" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3476" s="16" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3477">
+      <c r="A3477" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3477" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3477" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3477" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3477" s="19" t="n">
+        <v>147.45</v>
+      </c>
+    </row>
+    <row r="3478">
+      <c r="A3478" s="20" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3478" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3478" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3478" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3478" s="16" t="n">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3479">
+      <c r="A3479" s="21" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B3479" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3479" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3479" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3479" s="19" t="n">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-17
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3479"/>
+  <dimension ref="A1:E3523"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -80613,6 +80613,1018 @@
         <v>60</v>
       </c>
     </row>
+    <row r="3480">
+      <c r="A3480" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3480" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3480" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3480" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3480" s="16" t="n">
+        <v>48.2</v>
+      </c>
+    </row>
+    <row r="3481">
+      <c r="A3481" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3481" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3481" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3481" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3481" s="19" t="n">
+        <v>104.5</v>
+      </c>
+    </row>
+    <row r="3482">
+      <c r="A3482" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3482" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3482" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3482" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3482" s="16" t="n">
+        <v>123.6</v>
+      </c>
+    </row>
+    <row r="3483">
+      <c r="A3483" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3483" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3483" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3483" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3483" s="19" t="n">
+        <v>97.8</v>
+      </c>
+    </row>
+    <row r="3484">
+      <c r="A3484" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3484" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3484" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3484" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3484" s="16" t="n">
+        <v>91.2</v>
+      </c>
+    </row>
+    <row r="3485">
+      <c r="A3485" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3485" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3485" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3485" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3485" s="19" t="n">
+        <v>84.90000000000001</v>
+      </c>
+    </row>
+    <row r="3486">
+      <c r="A3486" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3486" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3486" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3486" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3486" s="16" t="n">
+        <v>57.45</v>
+      </c>
+    </row>
+    <row r="3487">
+      <c r="A3487" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3487" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3487" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3487" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3487" s="19" t="n">
+        <v>76.90000000000001</v>
+      </c>
+    </row>
+    <row r="3488">
+      <c r="A3488" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3488" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3488" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3488" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3488" s="16" t="n">
+        <v>108.75</v>
+      </c>
+    </row>
+    <row r="3489">
+      <c r="A3489" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3489" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3489" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3489" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3489" s="19" t="n">
+        <v>77.75</v>
+      </c>
+    </row>
+    <row r="3490">
+      <c r="A3490" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3490" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3490" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3490" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3490" s="16" t="n">
+        <v>126.6</v>
+      </c>
+    </row>
+    <row r="3491">
+      <c r="A3491" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3491" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3491" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3491" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3491" s="19" t="n">
+        <v>174.05</v>
+      </c>
+    </row>
+    <row r="3492">
+      <c r="A3492" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3492" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3492" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3492" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3492" s="16" t="n">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3493">
+      <c r="A3493" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3493" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3493" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3493" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3493" s="19" t="n">
+        <v>72.34999999999999</v>
+      </c>
+    </row>
+    <row r="3494">
+      <c r="A3494" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3494" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3494" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3494" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3494" s="16" t="n">
+        <v>118.35</v>
+      </c>
+    </row>
+    <row r="3495">
+      <c r="A3495" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3495" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3495" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3495" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3495" s="19" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="3496">
+      <c r="A3496" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3496" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3496" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3496" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3496" s="16" t="n">
+        <v>167.3</v>
+      </c>
+    </row>
+    <row r="3497">
+      <c r="A3497" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3497" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3497" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3497" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3497" s="19" t="n">
+        <v>71.5</v>
+      </c>
+    </row>
+    <row r="3498">
+      <c r="A3498" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3498" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3498" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3498" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3498" s="16" t="n">
+        <v>116.55</v>
+      </c>
+    </row>
+    <row r="3499">
+      <c r="A3499" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3499" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3499" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3499" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3499" s="19" t="n">
+        <v>164.4</v>
+      </c>
+    </row>
+    <row r="3500">
+      <c r="A3500" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3500" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3500" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3500" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3500" s="16" t="n">
+        <v>164.55</v>
+      </c>
+    </row>
+    <row r="3501">
+      <c r="A3501" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3501" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3501" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3501" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3501" s="19" t="n">
+        <v>70.25</v>
+      </c>
+    </row>
+    <row r="3502">
+      <c r="A3502" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3502" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3502" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3502" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3502" s="16" t="n">
+        <v>42.45</v>
+      </c>
+    </row>
+    <row r="3503">
+      <c r="A3503" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3503" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3503" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3503" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3503" s="19" t="n">
+        <v>91.84999999999999</v>
+      </c>
+    </row>
+    <row r="3504">
+      <c r="A3504" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3504" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3504" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3504" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3504" s="16" t="n">
+        <v>110.3</v>
+      </c>
+    </row>
+    <row r="3505">
+      <c r="A3505" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3505" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3505" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3505" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3505" s="19" t="n">
+        <v>91.5</v>
+      </c>
+    </row>
+    <row r="3506">
+      <c r="A3506" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3506" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3506" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3506" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3506" s="16" t="n">
+        <v>79.65000000000001</v>
+      </c>
+    </row>
+    <row r="3507">
+      <c r="A3507" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3507" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3507" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3507" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3507" s="19" t="n">
+        <v>74.40000000000001</v>
+      </c>
+    </row>
+    <row r="3508">
+      <c r="A3508" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3508" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3508" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3508" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3508" s="16" t="n">
+        <v>47.2</v>
+      </c>
+    </row>
+    <row r="3509">
+      <c r="A3509" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3509" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3509" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3509" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3509" s="19" t="n">
+        <v>71.95</v>
+      </c>
+    </row>
+    <row r="3510">
+      <c r="A3510" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3510" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3510" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3510" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3510" s="16" t="n">
+        <v>97.95</v>
+      </c>
+    </row>
+    <row r="3511">
+      <c r="A3511" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3511" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3511" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3511" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3511" s="19" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3512">
+      <c r="A3512" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3512" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3512" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3512" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3512" s="16" t="n">
+        <v>106.8</v>
+      </c>
+    </row>
+    <row r="3513">
+      <c r="A3513" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3513" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3513" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3513" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3513" s="19" t="n">
+        <v>155.1</v>
+      </c>
+    </row>
+    <row r="3514">
+      <c r="A3514" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3514" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3514" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3514" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3514" s="16" t="n">
+        <v>155.85</v>
+      </c>
+    </row>
+    <row r="3515">
+      <c r="A3515" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3515" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3515" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3515" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3515" s="19" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3516">
+      <c r="A3516" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3516" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3516" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3516" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3516" s="16" t="n">
+        <v>99.75</v>
+      </c>
+    </row>
+    <row r="3517">
+      <c r="A3517" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3517" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3517" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3517" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3517" s="19" t="n">
+        <v>151.5</v>
+      </c>
+    </row>
+    <row r="3518">
+      <c r="A3518" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3518" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3518" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3518" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3518" s="16" t="n">
+        <v>151.55</v>
+      </c>
+    </row>
+    <row r="3519">
+      <c r="A3519" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3519" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3519" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3519" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3519" s="19" t="n">
+        <v>61.95</v>
+      </c>
+    </row>
+    <row r="3520">
+      <c r="A3520" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3520" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3520" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3520" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3520" s="16" t="n">
+        <v>97.09999999999999</v>
+      </c>
+    </row>
+    <row r="3521">
+      <c r="A3521" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3521" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3521" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3521" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3521" s="19" t="n">
+        <v>148.6</v>
+      </c>
+    </row>
+    <row r="3522">
+      <c r="A3522" s="20" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3522" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3522" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3522" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3522" s="16" t="n">
+        <v>148.5</v>
+      </c>
+    </row>
+    <row r="3523">
+      <c r="A3523" s="21" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B3523" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3523" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3523" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3523" s="19" t="n">
+        <v>61.05</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-18
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3523"/>
+  <dimension ref="A1:E3567"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -81625,6 +81625,1018 @@
         <v>59</v>
       </c>
     </row>
+    <row r="3524">
+      <c r="A3524" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3524" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3524" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3524" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3524" s="16" t="n">
+        <v>48.2</v>
+      </c>
+    </row>
+    <row r="3525">
+      <c r="A3525" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3525" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3525" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3525" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3525" s="19" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3526">
+      <c r="A3526" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3526" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3526" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3526" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3526" s="16" t="n">
+        <v>117.9</v>
+      </c>
+    </row>
+    <row r="3527">
+      <c r="A3527" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3527" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3527" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3527" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3527" s="19" t="n">
+        <v>95.75</v>
+      </c>
+    </row>
+    <row r="3528">
+      <c r="A3528" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3528" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3528" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3528" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3528" s="16" t="n">
+        <v>86.3</v>
+      </c>
+    </row>
+    <row r="3529">
+      <c r="A3529" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3529" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3529" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3529" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3529" s="19" t="n">
+        <v>79.75</v>
+      </c>
+    </row>
+    <row r="3530">
+      <c r="A3530" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3530" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3530" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3530" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3530" s="16" t="n">
+        <v>56.6</v>
+      </c>
+    </row>
+    <row r="3531">
+      <c r="A3531" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3531" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3531" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3531" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3531" s="19" t="n">
+        <v>76.90000000000001</v>
+      </c>
+    </row>
+    <row r="3532">
+      <c r="A3532" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3532" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3532" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3532" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3532" s="16" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3533">
+      <c r="A3533" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3533" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3533" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3533" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3533" s="19" t="n">
+        <v>74.15000000000001</v>
+      </c>
+    </row>
+    <row r="3534">
+      <c r="A3534" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3534" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3534" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3534" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3534" s="16" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="3535">
+      <c r="A3535" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3535" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3535" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3535" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3535" s="19" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3536">
+      <c r="A3536" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3536" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3536" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3536" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3536" s="16" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3537">
+      <c r="A3537" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3537" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3537" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3537" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3537" s="19" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="3538">
+      <c r="A3538" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3538" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3538" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3538" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3538" s="16" t="n">
+        <v>117.7</v>
+      </c>
+    </row>
+    <row r="3539">
+      <c r="A3539" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3539" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3539" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3539" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3539" s="19" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="3540">
+      <c r="A3540" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3540" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3540" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3540" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3540" s="16" t="n">
+        <v>165.35</v>
+      </c>
+    </row>
+    <row r="3541">
+      <c r="A3541" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3541" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3541" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3541" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3541" s="19" t="n">
+        <v>70.40000000000001</v>
+      </c>
+    </row>
+    <row r="3542">
+      <c r="A3542" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3542" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3542" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3542" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3542" s="16" t="n">
+        <v>115.1</v>
+      </c>
+    </row>
+    <row r="3543">
+      <c r="A3543" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3543" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3543" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3543" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3543" s="19" t="n">
+        <v>162.85</v>
+      </c>
+    </row>
+    <row r="3544">
+      <c r="A3544" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3544" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3544" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3544" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3544" s="16" t="n">
+        <v>163.5</v>
+      </c>
+    </row>
+    <row r="3545">
+      <c r="A3545" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3545" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3545" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3545" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3545" s="19" t="n">
+        <v>68.5</v>
+      </c>
+    </row>
+    <row r="3546">
+      <c r="A3546" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3546" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3546" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3546" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3546" s="16" t="n">
+        <v>41.95</v>
+      </c>
+    </row>
+    <row r="3547">
+      <c r="A3547" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3547" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3547" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3547" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3547" s="19" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3548">
+      <c r="A3548" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3548" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3548" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3548" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3548" s="16" t="n">
+        <v>107.45</v>
+      </c>
+    </row>
+    <row r="3549">
+      <c r="A3549" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3549" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3549" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3549" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3549" s="19" t="n">
+        <v>87.15000000000001</v>
+      </c>
+    </row>
+    <row r="3550">
+      <c r="A3550" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3550" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3550" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3550" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3550" s="16" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3551">
+      <c r="A3551" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3551" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3551" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3551" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3551" s="19" t="n">
+        <v>69.34999999999999</v>
+      </c>
+    </row>
+    <row r="3552">
+      <c r="A3552" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3552" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3552" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3552" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3552" s="16" t="n">
+        <v>45.25</v>
+      </c>
+    </row>
+    <row r="3553">
+      <c r="A3553" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3553" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3553" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3553" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3553" s="19" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="3554">
+      <c r="A3554" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3554" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3554" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3554" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3554" s="16" t="n">
+        <v>94.3</v>
+      </c>
+    </row>
+    <row r="3555">
+      <c r="A3555" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3555" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3555" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3555" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3555" s="19" t="n">
+        <v>64.15000000000001</v>
+      </c>
+    </row>
+    <row r="3556">
+      <c r="A3556" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3556" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3556" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3556" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3556" s="16" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3557">
+      <c r="A3557" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3557" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3557" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3557" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3557" s="19" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3558">
+      <c r="A3558" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3558" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3558" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3558" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3558" s="16" t="n">
+        <v>153.7</v>
+      </c>
+    </row>
+    <row r="3559">
+      <c r="A3559" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3559" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3559" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3559" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3559" s="19" t="n">
+        <v>60.4</v>
+      </c>
+    </row>
+    <row r="3560">
+      <c r="A3560" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3560" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3560" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3560" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3560" s="16" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3561">
+      <c r="A3561" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3561" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3561" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3561" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3561" s="19" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="3562">
+      <c r="A3562" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3562" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3562" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3562" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3562" s="16" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="3563">
+      <c r="A3563" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3563" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3563" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3563" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3563" s="19" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3564">
+      <c r="A3564" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3564" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3564" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3564" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3564" s="16" t="n">
+        <v>97.8</v>
+      </c>
+    </row>
+    <row r="3565">
+      <c r="A3565" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3565" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3565" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3565" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3565" s="19" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3566">
+      <c r="A3566" s="20" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3566" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3566" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3566" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3566" s="16" t="n">
+        <v>145.1</v>
+      </c>
+    </row>
+    <row r="3567">
+      <c r="A3567" s="21" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B3567" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3567" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3567" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3567" s="19" t="n">
+        <v>59.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-19
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3567"/>
+  <dimension ref="A1:E3611"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -82637,6 +82637,1018 @@
         <v>59.5</v>
       </c>
     </row>
+    <row r="3568">
+      <c r="A3568" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3568" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3568" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3568" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3568" s="16" t="n">
+        <v>45.9</v>
+      </c>
+    </row>
+    <row r="3569">
+      <c r="A3569" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3569" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3569" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3569" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3569" s="19" t="n">
+        <v>98.55</v>
+      </c>
+    </row>
+    <row r="3570">
+      <c r="A3570" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3570" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3570" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3570" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3570" s="16" t="n">
+        <v>115.15</v>
+      </c>
+    </row>
+    <row r="3571">
+      <c r="A3571" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3571" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3571" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3571" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3571" s="19" t="n">
+        <v>92.55</v>
+      </c>
+    </row>
+    <row r="3572">
+      <c r="A3572" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3572" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3572" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3572" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3572" s="16" t="n">
+        <v>86.3</v>
+      </c>
+    </row>
+    <row r="3573">
+      <c r="A3573" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3573" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3573" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3573" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3573" s="19" t="n">
+        <v>79.75</v>
+      </c>
+    </row>
+    <row r="3574">
+      <c r="A3574" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3574" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3574" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3574" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3574" s="16" t="n">
+        <v>56.6</v>
+      </c>
+    </row>
+    <row r="3575">
+      <c r="A3575" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3575" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3575" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3575" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3575" s="19" t="n">
+        <v>76.15000000000001</v>
+      </c>
+    </row>
+    <row r="3576">
+      <c r="A3576" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3576" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3576" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3576" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3576" s="16" t="n">
+        <v>102.2</v>
+      </c>
+    </row>
+    <row r="3577">
+      <c r="A3577" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3577" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3577" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3577" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3577" s="19" t="n">
+        <v>74.15000000000001</v>
+      </c>
+    </row>
+    <row r="3578">
+      <c r="A3578" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3578" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3578" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3578" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3578" s="16" t="n">
+        <v>124.15</v>
+      </c>
+    </row>
+    <row r="3579">
+      <c r="A3579" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3579" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3579" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3579" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3579" s="19" t="n">
+        <v>169.5</v>
+      </c>
+    </row>
+    <row r="3580">
+      <c r="A3580" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3580" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3580" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3580" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3580" s="16" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3581">
+      <c r="A3581" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3581" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3581" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3581" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3581" s="19" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="3582">
+      <c r="A3582" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3582" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3582" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3582" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3582" s="16" t="n">
+        <v>117.7</v>
+      </c>
+    </row>
+    <row r="3583">
+      <c r="A3583" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3583" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3583" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3583" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3583" s="19" t="n">
+        <v>169.25</v>
+      </c>
+    </row>
+    <row r="3584">
+      <c r="A3584" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3584" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3584" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3584" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3584" s="16" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="3585">
+      <c r="A3585" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3585" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3585" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3585" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3585" s="19" t="n">
+        <v>70.40000000000001</v>
+      </c>
+    </row>
+    <row r="3586">
+      <c r="A3586" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3586" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3586" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3586" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3586" s="16" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3587">
+      <c r="A3587" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3587" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3587" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3587" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3587" s="19" t="n">
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="3588">
+      <c r="A3588" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3588" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3588" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3588" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3588" s="16" t="n">
+        <v>165.95</v>
+      </c>
+    </row>
+    <row r="3589">
+      <c r="A3589" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3589" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3589" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3589" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3589" s="19" t="n">
+        <v>68.5</v>
+      </c>
+    </row>
+    <row r="3590">
+      <c r="A3590" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3590" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3590" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3590" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3590" s="16" t="n">
+        <v>39.6</v>
+      </c>
+    </row>
+    <row r="3591">
+      <c r="A3591" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3591" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3591" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3591" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3591" s="19" t="n">
+        <v>85.65000000000001</v>
+      </c>
+    </row>
+    <row r="3592">
+      <c r="A3592" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3592" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3592" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3592" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3592" s="16" t="n">
+        <v>103.2</v>
+      </c>
+    </row>
+    <row r="3593">
+      <c r="A3593" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3593" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3593" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3593" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3593" s="19" t="n">
+        <v>80.84999999999999</v>
+      </c>
+    </row>
+    <row r="3594">
+      <c r="A3594" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3594" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3594" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3594" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3594" s="16" t="n">
+        <v>75.45</v>
+      </c>
+    </row>
+    <row r="3595">
+      <c r="A3595" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3595" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3595" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3595" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3595" s="19" t="n">
+        <v>67.90000000000001</v>
+      </c>
+    </row>
+    <row r="3596">
+      <c r="A3596" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3596" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3596" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3596" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3596" s="16" t="n">
+        <v>44.3</v>
+      </c>
+    </row>
+    <row r="3597">
+      <c r="A3597" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3597" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3597" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3597" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3597" s="19" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3598">
+      <c r="A3598" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3598" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3598" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3598" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3598" s="16" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3599">
+      <c r="A3599" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3599" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3599" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3599" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3599" s="19" t="n">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="3600">
+      <c r="A3600" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3600" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3600" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3600" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3600" s="16" t="n">
+        <v>103.75</v>
+      </c>
+    </row>
+    <row r="3601">
+      <c r="A3601" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3601" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3601" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3601" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3601" s="19" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3602">
+      <c r="A3602" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3602" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3602" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3602" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3602" s="16" t="n">
+        <v>152.45</v>
+      </c>
+    </row>
+    <row r="3603">
+      <c r="A3603" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3603" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3603" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3603" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3603" s="19" t="n">
+        <v>60.5</v>
+      </c>
+    </row>
+    <row r="3604">
+      <c r="A3604" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3604" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3604" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3604" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3604" s="16" t="n">
+        <v>97.34999999999999</v>
+      </c>
+    </row>
+    <row r="3605">
+      <c r="A3605" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3605" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3605" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3605" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3605" s="19" t="n">
+        <v>151.9</v>
+      </c>
+    </row>
+    <row r="3606">
+      <c r="A3606" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3606" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3606" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3606" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3606" s="16" t="n">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3607">
+      <c r="A3607" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3607" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3607" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3607" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3607" s="19" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3608">
+      <c r="A3608" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3608" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3608" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3608" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3608" s="16" t="n">
+        <v>95.15000000000001</v>
+      </c>
+    </row>
+    <row r="3609">
+      <c r="A3609" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3609" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3609" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3609" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3609" s="19" t="n">
+        <v>147.5</v>
+      </c>
+    </row>
+    <row r="3610">
+      <c r="A3610" s="20" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3610" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3610" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3610" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3610" s="16" t="n">
+        <v>146.5</v>
+      </c>
+    </row>
+    <row r="3611">
+      <c r="A3611" s="21" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B3611" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3611" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3611" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3611" s="19" t="n">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-20
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3611"/>
+  <dimension ref="A1:E3655"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -83649,6 +83649,1018 @@
         <v>59</v>
       </c>
     </row>
+    <row r="3612">
+      <c r="A3612" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3612" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3612" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3612" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3612" s="16" t="n">
+        <v>45.9</v>
+      </c>
+    </row>
+    <row r="3613">
+      <c r="A3613" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3613" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3613" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3613" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3613" s="19" t="n">
+        <v>98.55</v>
+      </c>
+    </row>
+    <row r="3614">
+      <c r="A3614" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3614" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3614" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3614" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3614" s="16" t="n">
+        <v>115.15</v>
+      </c>
+    </row>
+    <row r="3615">
+      <c r="A3615" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3615" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3615" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3615" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3615" s="19" t="n">
+        <v>92.55</v>
+      </c>
+    </row>
+    <row r="3616">
+      <c r="A3616" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3616" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3616" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3616" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3616" s="16" t="n">
+        <v>86.3</v>
+      </c>
+    </row>
+    <row r="3617">
+      <c r="A3617" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3617" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3617" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3617" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3617" s="19" t="n">
+        <v>79.75</v>
+      </c>
+    </row>
+    <row r="3618">
+      <c r="A3618" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3618" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3618" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3618" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3618" s="16" t="n">
+        <v>56.6</v>
+      </c>
+    </row>
+    <row r="3619">
+      <c r="A3619" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3619" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3619" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3619" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3619" s="19" t="n">
+        <v>76.15000000000001</v>
+      </c>
+    </row>
+    <row r="3620">
+      <c r="A3620" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3620" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3620" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3620" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3620" s="16" t="n">
+        <v>102.2</v>
+      </c>
+    </row>
+    <row r="3621">
+      <c r="A3621" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3621" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3621" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3621" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3621" s="19" t="n">
+        <v>74.15000000000001</v>
+      </c>
+    </row>
+    <row r="3622">
+      <c r="A3622" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3622" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3622" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3622" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3622" s="16" t="n">
+        <v>124.15</v>
+      </c>
+    </row>
+    <row r="3623">
+      <c r="A3623" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3623" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3623" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3623" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3623" s="19" t="n">
+        <v>169.5</v>
+      </c>
+    </row>
+    <row r="3624">
+      <c r="A3624" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3624" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3624" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3624" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3624" s="16" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3625">
+      <c r="A3625" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3625" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3625" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3625" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3625" s="19" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="3626">
+      <c r="A3626" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3626" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3626" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3626" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3626" s="16" t="n">
+        <v>117.7</v>
+      </c>
+    </row>
+    <row r="3627">
+      <c r="A3627" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3627" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3627" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3627" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3627" s="19" t="n">
+        <v>169.25</v>
+      </c>
+    </row>
+    <row r="3628">
+      <c r="A3628" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3628" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3628" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3628" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3628" s="16" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="3629">
+      <c r="A3629" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3629" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3629" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3629" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3629" s="19" t="n">
+        <v>70.40000000000001</v>
+      </c>
+    </row>
+    <row r="3630">
+      <c r="A3630" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3630" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3630" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3630" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3630" s="16" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3631">
+      <c r="A3631" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3631" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3631" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3631" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3631" s="19" t="n">
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="3632">
+      <c r="A3632" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3632" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3632" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3632" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3632" s="16" t="n">
+        <v>165.95</v>
+      </c>
+    </row>
+    <row r="3633">
+      <c r="A3633" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3633" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3633" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3633" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3633" s="19" t="n">
+        <v>68.5</v>
+      </c>
+    </row>
+    <row r="3634">
+      <c r="A3634" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3634" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3634" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3634" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3634" s="16" t="n">
+        <v>39.6</v>
+      </c>
+    </row>
+    <row r="3635">
+      <c r="A3635" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3635" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3635" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3635" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3635" s="19" t="n">
+        <v>85.65000000000001</v>
+      </c>
+    </row>
+    <row r="3636">
+      <c r="A3636" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3636" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3636" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3636" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3636" s="16" t="n">
+        <v>103.2</v>
+      </c>
+    </row>
+    <row r="3637">
+      <c r="A3637" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3637" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3637" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3637" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3637" s="19" t="n">
+        <v>80.84999999999999</v>
+      </c>
+    </row>
+    <row r="3638">
+      <c r="A3638" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3638" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3638" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3638" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3638" s="16" t="n">
+        <v>75.45</v>
+      </c>
+    </row>
+    <row r="3639">
+      <c r="A3639" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3639" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3639" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3639" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3639" s="19" t="n">
+        <v>67.90000000000001</v>
+      </c>
+    </row>
+    <row r="3640">
+      <c r="A3640" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3640" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3640" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3640" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3640" s="16" t="n">
+        <v>44.3</v>
+      </c>
+    </row>
+    <row r="3641">
+      <c r="A3641" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3641" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3641" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3641" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3641" s="19" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3642">
+      <c r="A3642" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3642" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3642" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3642" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3642" s="16" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3643">
+      <c r="A3643" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3643" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3643" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3643" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3643" s="19" t="n">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="3644">
+      <c r="A3644" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3644" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3644" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3644" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3644" s="16" t="n">
+        <v>103.75</v>
+      </c>
+    </row>
+    <row r="3645">
+      <c r="A3645" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3645" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3645" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3645" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3645" s="19" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3646">
+      <c r="A3646" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3646" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3646" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3646" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3646" s="16" t="n">
+        <v>152.45</v>
+      </c>
+    </row>
+    <row r="3647">
+      <c r="A3647" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3647" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3647" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3647" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3647" s="19" t="n">
+        <v>60.5</v>
+      </c>
+    </row>
+    <row r="3648">
+      <c r="A3648" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3648" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3648" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3648" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3648" s="16" t="n">
+        <v>97.34999999999999</v>
+      </c>
+    </row>
+    <row r="3649">
+      <c r="A3649" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3649" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3649" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3649" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3649" s="19" t="n">
+        <v>151.9</v>
+      </c>
+    </row>
+    <row r="3650">
+      <c r="A3650" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3650" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3650" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3650" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3650" s="16" t="n">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3651">
+      <c r="A3651" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3651" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3651" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3651" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3651" s="19" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3652">
+      <c r="A3652" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3652" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3652" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3652" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3652" s="16" t="n">
+        <v>95.15000000000001</v>
+      </c>
+    </row>
+    <row r="3653">
+      <c r="A3653" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3653" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3653" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3653" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3653" s="19" t="n">
+        <v>147.5</v>
+      </c>
+    </row>
+    <row r="3654">
+      <c r="A3654" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3654" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3654" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3654" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3654" s="16" t="n">
+        <v>146.5</v>
+      </c>
+    </row>
+    <row r="3655">
+      <c r="A3655" s="21" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B3655" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3655" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3655" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3655" s="19" t="n">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-21
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3655"/>
+  <dimension ref="A1:E3699"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -84661,6 +84661,1018 @@
         <v>59</v>
       </c>
     </row>
+    <row r="3656">
+      <c r="A3656" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3656" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3656" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3656" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3656" s="16" t="n">
+        <v>45.9</v>
+      </c>
+    </row>
+    <row r="3657">
+      <c r="A3657" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3657" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3657" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3657" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3657" s="19" t="n">
+        <v>98.55</v>
+      </c>
+    </row>
+    <row r="3658">
+      <c r="A3658" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3658" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3658" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3658" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3658" s="16" t="n">
+        <v>115.15</v>
+      </c>
+    </row>
+    <row r="3659">
+      <c r="A3659" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3659" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3659" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3659" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3659" s="19" t="n">
+        <v>92.55</v>
+      </c>
+    </row>
+    <row r="3660">
+      <c r="A3660" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3660" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3660" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3660" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3660" s="16" t="n">
+        <v>86.3</v>
+      </c>
+    </row>
+    <row r="3661">
+      <c r="A3661" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3661" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3661" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3661" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3661" s="19" t="n">
+        <v>79.75</v>
+      </c>
+    </row>
+    <row r="3662">
+      <c r="A3662" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3662" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3662" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3662" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3662" s="16" t="n">
+        <v>56.6</v>
+      </c>
+    </row>
+    <row r="3663">
+      <c r="A3663" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3663" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3663" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3663" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3663" s="19" t="n">
+        <v>76.15000000000001</v>
+      </c>
+    </row>
+    <row r="3664">
+      <c r="A3664" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3664" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3664" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3664" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3664" s="16" t="n">
+        <v>102.2</v>
+      </c>
+    </row>
+    <row r="3665">
+      <c r="A3665" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3665" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3665" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3665" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3665" s="19" t="n">
+        <v>74.15000000000001</v>
+      </c>
+    </row>
+    <row r="3666">
+      <c r="A3666" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3666" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3666" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3666" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3666" s="16" t="n">
+        <v>124.15</v>
+      </c>
+    </row>
+    <row r="3667">
+      <c r="A3667" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3667" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3667" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3667" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3667" s="19" t="n">
+        <v>169.5</v>
+      </c>
+    </row>
+    <row r="3668">
+      <c r="A3668" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3668" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3668" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3668" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3668" s="16" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3669">
+      <c r="A3669" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3669" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3669" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3669" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3669" s="19" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="3670">
+      <c r="A3670" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3670" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3670" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3670" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3670" s="16" t="n">
+        <v>117.7</v>
+      </c>
+    </row>
+    <row r="3671">
+      <c r="A3671" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3671" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3671" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3671" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3671" s="19" t="n">
+        <v>169.25</v>
+      </c>
+    </row>
+    <row r="3672">
+      <c r="A3672" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3672" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3672" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3672" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3672" s="16" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="3673">
+      <c r="A3673" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3673" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3673" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3673" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3673" s="19" t="n">
+        <v>70.40000000000001</v>
+      </c>
+    </row>
+    <row r="3674">
+      <c r="A3674" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3674" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3674" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3674" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3674" s="16" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3675">
+      <c r="A3675" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3675" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3675" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3675" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3675" s="19" t="n">
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="3676">
+      <c r="A3676" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3676" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3676" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3676" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3676" s="16" t="n">
+        <v>165.95</v>
+      </c>
+    </row>
+    <row r="3677">
+      <c r="A3677" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3677" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3677" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3677" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3677" s="19" t="n">
+        <v>68.5</v>
+      </c>
+    </row>
+    <row r="3678">
+      <c r="A3678" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3678" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3678" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3678" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3678" s="16" t="n">
+        <v>39.6</v>
+      </c>
+    </row>
+    <row r="3679">
+      <c r="A3679" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3679" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3679" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3679" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3679" s="19" t="n">
+        <v>85.65000000000001</v>
+      </c>
+    </row>
+    <row r="3680">
+      <c r="A3680" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3680" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3680" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3680" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3680" s="16" t="n">
+        <v>103.2</v>
+      </c>
+    </row>
+    <row r="3681">
+      <c r="A3681" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3681" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3681" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3681" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3681" s="19" t="n">
+        <v>80.84999999999999</v>
+      </c>
+    </row>
+    <row r="3682">
+      <c r="A3682" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3682" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3682" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3682" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3682" s="16" t="n">
+        <v>75.45</v>
+      </c>
+    </row>
+    <row r="3683">
+      <c r="A3683" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3683" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3683" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3683" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3683" s="19" t="n">
+        <v>67.90000000000001</v>
+      </c>
+    </row>
+    <row r="3684">
+      <c r="A3684" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3684" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3684" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3684" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3684" s="16" t="n">
+        <v>44.3</v>
+      </c>
+    </row>
+    <row r="3685">
+      <c r="A3685" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3685" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3685" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3685" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3685" s="19" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3686">
+      <c r="A3686" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3686" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3686" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3686" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3686" s="16" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3687">
+      <c r="A3687" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3687" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3687" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3687" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3687" s="19" t="n">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="3688">
+      <c r="A3688" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3688" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3688" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3688" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3688" s="16" t="n">
+        <v>103.75</v>
+      </c>
+    </row>
+    <row r="3689">
+      <c r="A3689" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3689" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3689" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3689" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3689" s="19" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3690">
+      <c r="A3690" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3690" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3690" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3690" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3690" s="16" t="n">
+        <v>152.45</v>
+      </c>
+    </row>
+    <row r="3691">
+      <c r="A3691" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3691" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3691" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3691" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3691" s="19" t="n">
+        <v>60.5</v>
+      </c>
+    </row>
+    <row r="3692">
+      <c r="A3692" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3692" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3692" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3692" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3692" s="16" t="n">
+        <v>97.34999999999999</v>
+      </c>
+    </row>
+    <row r="3693">
+      <c r="A3693" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3693" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3693" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3693" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3693" s="19" t="n">
+        <v>151.9</v>
+      </c>
+    </row>
+    <row r="3694">
+      <c r="A3694" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3694" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3694" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3694" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3694" s="16" t="n">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3695">
+      <c r="A3695" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3695" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3695" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3695" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3695" s="19" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3696">
+      <c r="A3696" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3696" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3696" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3696" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3696" s="16" t="n">
+        <v>95.15000000000001</v>
+      </c>
+    </row>
+    <row r="3697">
+      <c r="A3697" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3697" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3697" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3697" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3697" s="19" t="n">
+        <v>147.5</v>
+      </c>
+    </row>
+    <row r="3698">
+      <c r="A3698" s="20" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3698" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3698" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3698" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3698" s="16" t="n">
+        <v>146.5</v>
+      </c>
+    </row>
+    <row r="3699">
+      <c r="A3699" s="21" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B3699" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3699" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3699" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3699" s="19" t="n">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-23
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3699"/>
+  <dimension ref="A1:E3743"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -85673,6 +85673,1018 @@
         <v>59</v>
       </c>
     </row>
+    <row r="3700">
+      <c r="A3700" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3700" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3700" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3700" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3700" s="16" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3701">
+      <c r="A3701" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3701" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3701" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3701" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3701" s="19" t="n">
+        <v>90.90000000000001</v>
+      </c>
+    </row>
+    <row r="3702">
+      <c r="A3702" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3702" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3702" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3702" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3702" s="16" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3703">
+      <c r="A3703" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3703" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3703" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3703" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3703" s="19" t="n">
+        <v>87.09999999999999</v>
+      </c>
+    </row>
+    <row r="3704">
+      <c r="A3704" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3704" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3704" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3704" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3704" s="16" t="n">
+        <v>84.65000000000001</v>
+      </c>
+    </row>
+    <row r="3705">
+      <c r="A3705" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3705" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3705" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3705" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3705" s="19" t="n">
+        <v>76.84999999999999</v>
+      </c>
+    </row>
+    <row r="3706">
+      <c r="A3706" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3706" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3706" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3706" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3706" s="16" t="n">
+        <v>57.2</v>
+      </c>
+    </row>
+    <row r="3707">
+      <c r="A3707" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3707" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3707" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3707" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3707" s="19" t="n">
+        <v>74.2</v>
+      </c>
+    </row>
+    <row r="3708">
+      <c r="A3708" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3708" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3708" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3708" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3708" s="16" t="n">
+        <v>94.75</v>
+      </c>
+    </row>
+    <row r="3709">
+      <c r="A3709" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3709" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3709" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3709" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3709" s="19" t="n">
+        <v>72.84999999999999</v>
+      </c>
+    </row>
+    <row r="3710">
+      <c r="A3710" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3710" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3710" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3710" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3710" s="16" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3711">
+      <c r="A3711" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3711" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3711" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3711" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3711" s="19" t="n">
+        <v>166.1</v>
+      </c>
+    </row>
+    <row r="3712">
+      <c r="A3712" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3712" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3712" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3712" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3712" s="16" t="n">
+        <v>166.2</v>
+      </c>
+    </row>
+    <row r="3713">
+      <c r="A3713" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3713" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3713" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3713" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3713" s="19" t="n">
+        <v>69.45</v>
+      </c>
+    </row>
+    <row r="3714">
+      <c r="A3714" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3714" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3714" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3714" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3714" s="16" t="n">
+        <v>114.6</v>
+      </c>
+    </row>
+    <row r="3715">
+      <c r="A3715" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3715" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3715" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3715" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3715" s="19" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="3716">
+      <c r="A3716" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3716" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3716" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3716" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3716" s="16" t="n">
+        <v>165.65</v>
+      </c>
+    </row>
+    <row r="3717">
+      <c r="A3717" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3717" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3717" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3717" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3717" s="19" t="n">
+        <v>68.95</v>
+      </c>
+    </row>
+    <row r="3718">
+      <c r="A3718" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3718" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3718" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3718" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3718" s="16" t="n">
+        <v>112.4</v>
+      </c>
+    </row>
+    <row r="3719">
+      <c r="A3719" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3719" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3719" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3719" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3719" s="19" t="n">
+        <v>164.4</v>
+      </c>
+    </row>
+    <row r="3720">
+      <c r="A3720" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3720" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3720" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3720" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3720" s="16" t="n">
+        <v>164.4</v>
+      </c>
+    </row>
+    <row r="3721">
+      <c r="A3721" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3721" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3721" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3721" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3721" s="19" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3722">
+      <c r="A3722" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3722" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3722" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3722" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3722" s="16" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3723">
+      <c r="A3723" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3723" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3723" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3723" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3723" s="19" t="n">
+        <v>76.75</v>
+      </c>
+    </row>
+    <row r="3724">
+      <c r="A3724" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3724" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3724" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3724" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3724" s="16" t="n">
+        <v>94.5</v>
+      </c>
+    </row>
+    <row r="3725">
+      <c r="A3725" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3725" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3725" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3725" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3725" s="19" t="n">
+        <v>76.2</v>
+      </c>
+    </row>
+    <row r="3726">
+      <c r="A3726" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3726" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3726" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3726" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3726" s="16" t="n">
+        <v>73.2</v>
+      </c>
+    </row>
+    <row r="3727">
+      <c r="A3727" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3727" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3727" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3727" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3727" s="19" t="n">
+        <v>64.40000000000001</v>
+      </c>
+    </row>
+    <row r="3728">
+      <c r="A3728" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3728" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3728" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3728" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3728" s="16" t="n">
+        <v>43.3</v>
+      </c>
+    </row>
+    <row r="3729">
+      <c r="A3729" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3729" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3729" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3729" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3729" s="19" t="n">
+        <v>69.5</v>
+      </c>
+    </row>
+    <row r="3730">
+      <c r="A3730" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3730" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3730" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3730" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3730" s="16" t="n">
+        <v>82.55</v>
+      </c>
+    </row>
+    <row r="3731">
+      <c r="A3731" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3731" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3731" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3731" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3731" s="19" t="n">
+        <v>60.25</v>
+      </c>
+    </row>
+    <row r="3732">
+      <c r="A3732" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3732" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3732" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3732" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3732" s="16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3733">
+      <c r="A3733" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3733" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3733" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3733" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3733" s="19" t="n">
+        <v>148.55</v>
+      </c>
+    </row>
+    <row r="3734">
+      <c r="A3734" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3734" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3734" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3734" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3734" s="16" t="n">
+        <v>151.4</v>
+      </c>
+    </row>
+    <row r="3735">
+      <c r="A3735" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3735" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3735" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3735" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3735" s="19" t="n">
+        <v>58.65</v>
+      </c>
+    </row>
+    <row r="3736">
+      <c r="A3736" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3736" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3736" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3736" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3736" s="16" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3737">
+      <c r="A3737" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3737" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3737" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3737" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3737" s="19" t="n">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3738">
+      <c r="A3738" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3738" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3738" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3738" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3738" s="16" t="n">
+        <v>148.65</v>
+      </c>
+    </row>
+    <row r="3739">
+      <c r="A3739" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3739" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3739" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3739" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3739" s="19" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3740">
+      <c r="A3740" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3740" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3740" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3740" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3740" s="16" t="n">
+        <v>92.59999999999999</v>
+      </c>
+    </row>
+    <row r="3741">
+      <c r="A3741" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3741" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3741" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3741" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3741" s="19" t="n">
+        <v>145.5</v>
+      </c>
+    </row>
+    <row r="3742">
+      <c r="A3742" s="20" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3742" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3742" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3742" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3742" s="16" t="n">
+        <v>146.5</v>
+      </c>
+    </row>
+    <row r="3743">
+      <c r="A3743" s="21" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B3743" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3743" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3743" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3743" s="19" t="n">
+        <v>58.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-24
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3743"/>
+  <dimension ref="A1:E3787"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -86685,6 +86685,1018 @@
         <v>59.25</v>
       </c>
     </row>
+    <row r="3744">
+      <c r="A3744" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3744" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3744" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3744" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3744" s="16" t="n">
+        <v>40.45</v>
+      </c>
+    </row>
+    <row r="3745">
+      <c r="A3745" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3745" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3745" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3745" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3745" s="19" t="n">
+        <v>90.15000000000001</v>
+      </c>
+    </row>
+    <row r="3746">
+      <c r="A3746" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3746" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3746" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3746" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3746" s="16" t="n">
+        <v>103.75</v>
+      </c>
+    </row>
+    <row r="3747">
+      <c r="A3747" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3747" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3747" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3747" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3747" s="19" t="n">
+        <v>85.59999999999999</v>
+      </c>
+    </row>
+    <row r="3748">
+      <c r="A3748" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3748" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3748" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3748" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3748" s="16" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3749">
+      <c r="A3749" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3749" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3749" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3749" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3749" s="19" t="n">
+        <v>75.8</v>
+      </c>
+    </row>
+    <row r="3750">
+      <c r="A3750" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3750" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3750" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3750" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3750" s="16" t="n">
+        <v>55.55</v>
+      </c>
+    </row>
+    <row r="3751">
+      <c r="A3751" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3751" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3751" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3751" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3751" s="19" t="n">
+        <v>74.34999999999999</v>
+      </c>
+    </row>
+    <row r="3752">
+      <c r="A3752" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3752" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3752" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3752" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3752" s="16" t="n">
+        <v>93.25</v>
+      </c>
+    </row>
+    <row r="3753">
+      <c r="A3753" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3753" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3753" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3753" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3753" s="19" t="n">
+        <v>71.40000000000001</v>
+      </c>
+    </row>
+    <row r="3754">
+      <c r="A3754" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3754" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3754" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3754" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3754" s="16" t="n">
+        <v>120.5</v>
+      </c>
+    </row>
+    <row r="3755">
+      <c r="A3755" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3755" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3755" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3755" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3755" s="19" t="n">
+        <v>167.7</v>
+      </c>
+    </row>
+    <row r="3756">
+      <c r="A3756" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3756" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3756" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3756" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3756" s="16" t="n">
+        <v>165.1</v>
+      </c>
+    </row>
+    <row r="3757">
+      <c r="A3757" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3757" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3757" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3757" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3757" s="19" t="n">
+        <v>70.2</v>
+      </c>
+    </row>
+    <row r="3758">
+      <c r="A3758" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3758" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3758" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3758" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3758" s="16" t="n">
+        <v>116.9</v>
+      </c>
+    </row>
+    <row r="3759">
+      <c r="A3759" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3759" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3759" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3759" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3759" s="19" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="3760">
+      <c r="A3760" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3760" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3760" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3760" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3760" s="16" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="3761">
+      <c r="A3761" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3761" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3761" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3761" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3761" s="19" t="n">
+        <v>69.55</v>
+      </c>
+    </row>
+    <row r="3762">
+      <c r="A3762" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3762" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3762" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3762" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3762" s="16" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3763">
+      <c r="A3763" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3763" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3763" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3763" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3763" s="19" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3764">
+      <c r="A3764" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3764" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3764" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3764" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3764" s="16" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3765">
+      <c r="A3765" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3765" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3765" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3765" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3765" s="19" t="n">
+        <v>69.5</v>
+      </c>
+    </row>
+    <row r="3766">
+      <c r="A3766" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3766" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3766" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3766" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3766" s="16" t="n">
+        <v>35.5</v>
+      </c>
+    </row>
+    <row r="3767">
+      <c r="A3767" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3767" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3767" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3767" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3767" s="19" t="n">
+        <v>73.40000000000001</v>
+      </c>
+    </row>
+    <row r="3768">
+      <c r="A3768" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3768" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3768" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3768" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3768" s="16" t="n">
+        <v>89.8</v>
+      </c>
+    </row>
+    <row r="3769">
+      <c r="A3769" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3769" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3769" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3769" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3769" s="19" t="n">
+        <v>75.45</v>
+      </c>
+    </row>
+    <row r="3770">
+      <c r="A3770" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3770" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3770" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3770" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3770" s="16" t="n">
+        <v>71.84999999999999</v>
+      </c>
+    </row>
+    <row r="3771">
+      <c r="A3771" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3771" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3771" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3771" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3771" s="19" t="n">
+        <v>63.3</v>
+      </c>
+    </row>
+    <row r="3772">
+      <c r="A3772" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3772" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3772" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3772" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3772" s="16" t="n">
+        <v>44.2</v>
+      </c>
+    </row>
+    <row r="3773">
+      <c r="A3773" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3773" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3773" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3773" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3773" s="19" t="n">
+        <v>69.65000000000001</v>
+      </c>
+    </row>
+    <row r="3774">
+      <c r="A3774" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3774" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3774" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3774" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3774" s="16" t="n">
+        <v>79.59999999999999</v>
+      </c>
+    </row>
+    <row r="3775">
+      <c r="A3775" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3775" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3775" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3775" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3775" s="19" t="n">
+        <v>59.75</v>
+      </c>
+    </row>
+    <row r="3776">
+      <c r="A3776" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3776" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3776" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3776" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3776" s="16" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3777">
+      <c r="A3777" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3777" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3777" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3777" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3777" s="19" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3778">
+      <c r="A3778" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3778" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3778" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3778" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3778" s="16" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3779">
+      <c r="A3779" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3779" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3779" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3779" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3779" s="19" t="n">
+        <v>60.25</v>
+      </c>
+    </row>
+    <row r="3780">
+      <c r="A3780" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3780" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3780" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3780" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3780" s="16" t="n">
+        <v>96.8</v>
+      </c>
+    </row>
+    <row r="3781">
+      <c r="A3781" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3781" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3781" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3781" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3781" s="19" t="n">
+        <v>149.75</v>
+      </c>
+    </row>
+    <row r="3782">
+      <c r="A3782" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3782" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3782" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3782" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3782" s="16" t="n">
+        <v>150.4</v>
+      </c>
+    </row>
+    <row r="3783">
+      <c r="A3783" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3783" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3783" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3783" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3783" s="19" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3784">
+      <c r="A3784" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3784" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3784" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3784" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3784" s="16" t="n">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3785">
+      <c r="A3785" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3785" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3785" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3785" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3785" s="19" t="n">
+        <v>145.9</v>
+      </c>
+    </row>
+    <row r="3786">
+      <c r="A3786" s="20" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3786" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3786" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3786" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3786" s="16" t="n">
+        <v>146.65</v>
+      </c>
+    </row>
+    <row r="3787">
+      <c r="A3787" s="21" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B3787" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3787" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3787" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3787" s="19" t="n">
+        <v>59.25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-25
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3787"/>
+  <dimension ref="A1:E3831"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -87697,6 +87697,1018 @@
         <v>59.25</v>
       </c>
     </row>
+    <row r="3788">
+      <c r="A3788" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3788" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3788" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3788" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3788" s="16" t="n">
+        <v>41.5</v>
+      </c>
+    </row>
+    <row r="3789">
+      <c r="A3789" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3789" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3789" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3789" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3789" s="19" t="n">
+        <v>90.3</v>
+      </c>
+    </row>
+    <row r="3790">
+      <c r="A3790" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3790" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3790" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3790" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3790" s="16" t="n">
+        <v>103.75</v>
+      </c>
+    </row>
+    <row r="3791">
+      <c r="A3791" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3791" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3791" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3791" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3791" s="19" t="n">
+        <v>85.95</v>
+      </c>
+    </row>
+    <row r="3792">
+      <c r="A3792" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3792" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3792" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3792" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3792" s="16" t="n">
+        <v>82.5</v>
+      </c>
+    </row>
+    <row r="3793">
+      <c r="A3793" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3793" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3793" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3793" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3793" s="19" t="n">
+        <v>74.5</v>
+      </c>
+    </row>
+    <row r="3794">
+      <c r="A3794" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3794" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3794" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3794" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3794" s="16" t="n">
+        <v>57.3</v>
+      </c>
+    </row>
+    <row r="3795">
+      <c r="A3795" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3795" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3795" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3795" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3795" s="19" t="n">
+        <v>74.7</v>
+      </c>
+    </row>
+    <row r="3796">
+      <c r="A3796" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3796" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3796" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3796" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3796" s="16" t="n">
+        <v>93.40000000000001</v>
+      </c>
+    </row>
+    <row r="3797">
+      <c r="A3797" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3797" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3797" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3797" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3797" s="19" t="n">
+        <v>71.40000000000001</v>
+      </c>
+    </row>
+    <row r="3798">
+      <c r="A3798" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3798" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3798" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3798" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3798" s="16" t="n">
+        <v>120.5</v>
+      </c>
+    </row>
+    <row r="3799">
+      <c r="A3799" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3799" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3799" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3799" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3799" s="19" t="n">
+        <v>167.7</v>
+      </c>
+    </row>
+    <row r="3800">
+      <c r="A3800" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3800" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3800" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3800" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3800" s="16" t="n">
+        <v>165.05</v>
+      </c>
+    </row>
+    <row r="3801">
+      <c r="A3801" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3801" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3801" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3801" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3801" s="19" t="n">
+        <v>71.84999999999999</v>
+      </c>
+    </row>
+    <row r="3802">
+      <c r="A3802" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3802" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3802" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3802" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3802" s="16" t="n">
+        <v>116.9</v>
+      </c>
+    </row>
+    <row r="3803">
+      <c r="A3803" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3803" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3803" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3803" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3803" s="19" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="3804">
+      <c r="A3804" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3804" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3804" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3804" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3804" s="16" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3805">
+      <c r="A3805" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3805" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3805" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3805" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3805" s="19" t="n">
+        <v>71.34999999999999</v>
+      </c>
+    </row>
+    <row r="3806">
+      <c r="A3806" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3806" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3806" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3806" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3806" s="16" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3807">
+      <c r="A3807" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3807" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3807" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3807" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3807" s="19" t="n">
+        <v>161.05</v>
+      </c>
+    </row>
+    <row r="3808">
+      <c r="A3808" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3808" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3808" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3808" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3808" s="16" t="n">
+        <v>161.5</v>
+      </c>
+    </row>
+    <row r="3809">
+      <c r="A3809" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3809" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3809" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3809" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3809" s="19" t="n">
+        <v>69.5</v>
+      </c>
+    </row>
+    <row r="3810">
+      <c r="A3810" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3810" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3810" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3810" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3810" s="16" t="n">
+        <v>35.95</v>
+      </c>
+    </row>
+    <row r="3811">
+      <c r="A3811" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3811" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3811" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3811" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3811" s="19" t="n">
+        <v>74.84999999999999</v>
+      </c>
+    </row>
+    <row r="3812">
+      <c r="A3812" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3812" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3812" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3812" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3812" s="16" t="n">
+        <v>90.25</v>
+      </c>
+    </row>
+    <row r="3813">
+      <c r="A3813" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3813" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3813" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3813" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3813" s="19" t="n">
+        <v>76.84999999999999</v>
+      </c>
+    </row>
+    <row r="3814">
+      <c r="A3814" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3814" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3814" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3814" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3814" s="16" t="n">
+        <v>71.34999999999999</v>
+      </c>
+    </row>
+    <row r="3815">
+      <c r="A3815" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3815" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3815" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3815" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3815" s="19" t="n">
+        <v>62.6</v>
+      </c>
+    </row>
+    <row r="3816">
+      <c r="A3816" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3816" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3816" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3816" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3816" s="16" t="n">
+        <v>43.9</v>
+      </c>
+    </row>
+    <row r="3817">
+      <c r="A3817" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3817" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3817" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3817" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3817" s="19" t="n">
+        <v>69.8</v>
+      </c>
+    </row>
+    <row r="3818">
+      <c r="A3818" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3818" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3818" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3818" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3818" s="16" t="n">
+        <v>80.7</v>
+      </c>
+    </row>
+    <row r="3819">
+      <c r="A3819" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3819" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3819" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3819" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3819" s="19" t="n">
+        <v>59.25</v>
+      </c>
+    </row>
+    <row r="3820">
+      <c r="A3820" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3820" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3820" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3820" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3820" s="16" t="n">
+        <v>100.9</v>
+      </c>
+    </row>
+    <row r="3821">
+      <c r="A3821" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3821" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3821" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3821" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3821" s="19" t="n">
+        <v>151.45</v>
+      </c>
+    </row>
+    <row r="3822">
+      <c r="A3822" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3822" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3822" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3822" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3822" s="16" t="n">
+        <v>152.4</v>
+      </c>
+    </row>
+    <row r="3823">
+      <c r="A3823" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3823" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3823" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3823" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3823" s="19" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3824">
+      <c r="A3824" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3824" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3824" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3824" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3824" s="16" t="n">
+        <v>96.8</v>
+      </c>
+    </row>
+    <row r="3825">
+      <c r="A3825" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3825" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3825" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3825" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3825" s="19" t="n">
+        <v>148.35</v>
+      </c>
+    </row>
+    <row r="3826">
+      <c r="A3826" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3826" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3826" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3826" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3826" s="16" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3827">
+      <c r="A3827" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3827" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3827" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3827" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3827" s="19" t="n">
+        <v>60.45</v>
+      </c>
+    </row>
+    <row r="3828">
+      <c r="A3828" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3828" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3828" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3828" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3828" s="16" t="n">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3829">
+      <c r="A3829" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3829" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3829" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3829" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3829" s="19" t="n">
+        <v>145.9</v>
+      </c>
+    </row>
+    <row r="3830">
+      <c r="A3830" s="20" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3830" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3830" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3830" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3830" s="16" t="n">
+        <v>145.65</v>
+      </c>
+    </row>
+    <row r="3831">
+      <c r="A3831" s="21" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B3831" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3831" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3831" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3831" s="19" t="n">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-26
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3831"/>
+  <dimension ref="A1:E3875"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -88709,6 +88709,1018 @@
         <v>60</v>
       </c>
     </row>
+    <row r="3832">
+      <c r="A3832" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3832" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3832" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3832" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3832" s="16" t="n">
+        <v>41.5</v>
+      </c>
+    </row>
+    <row r="3833">
+      <c r="A3833" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3833" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3833" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3833" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3833" s="19" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3834">
+      <c r="A3834" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3834" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3834" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3834" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3834" s="16" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3835">
+      <c r="A3835" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3835" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3835" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3835" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3835" s="19" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3836">
+      <c r="A3836" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3836" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3836" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3836" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3836" s="16" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3837">
+      <c r="A3837" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3837" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3837" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3837" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3837" s="19" t="n">
+        <v>67.90000000000001</v>
+      </c>
+    </row>
+    <row r="3838">
+      <c r="A3838" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3838" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3838" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3838" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3838" s="16" t="n">
+        <v>54.05</v>
+      </c>
+    </row>
+    <row r="3839">
+      <c r="A3839" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3839" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3839" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3839" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3839" s="19" t="n">
+        <v>74.7</v>
+      </c>
+    </row>
+    <row r="3840">
+      <c r="A3840" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3840" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3840" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3840" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3840" s="16" t="n">
+        <v>88.05</v>
+      </c>
+    </row>
+    <row r="3841">
+      <c r="A3841" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3841" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3841" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3841" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3841" s="19" t="n">
+        <v>66.3</v>
+      </c>
+    </row>
+    <row r="3842">
+      <c r="A3842" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3842" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3842" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3842" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3842" s="16" t="n">
+        <v>118.5</v>
+      </c>
+    </row>
+    <row r="3843">
+      <c r="A3843" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3843" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3843" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3843" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3843" s="19" t="n">
+        <v>164.25</v>
+      </c>
+    </row>
+    <row r="3844">
+      <c r="A3844" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3844" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3844" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3844" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3844" s="16" t="n">
+        <v>163.6</v>
+      </c>
+    </row>
+    <row r="3845">
+      <c r="A3845" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3845" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3845" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3845" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3845" s="19" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="3846">
+      <c r="A3846" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3846" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3846" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3846" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3846" s="16" t="n">
+        <v>116.9</v>
+      </c>
+    </row>
+    <row r="3847">
+      <c r="A3847" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3847" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3847" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3847" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3847" s="19" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3848">
+      <c r="A3848" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3848" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3848" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3848" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3848" s="16" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3849">
+      <c r="A3849" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3849" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3849" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3849" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3849" s="19" t="n">
+        <v>71.34999999999999</v>
+      </c>
+    </row>
+    <row r="3850">
+      <c r="A3850" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3850" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3850" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3850" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3850" s="16" t="n">
+        <v>112.85</v>
+      </c>
+    </row>
+    <row r="3851">
+      <c r="A3851" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3851" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3851" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3851" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3851" s="19" t="n">
+        <v>161.05</v>
+      </c>
+    </row>
+    <row r="3852">
+      <c r="A3852" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3852" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3852" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3852" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3852" s="16" t="n">
+        <v>161.5</v>
+      </c>
+    </row>
+    <row r="3853">
+      <c r="A3853" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3853" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3853" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3853" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3853" s="19" t="n">
+        <v>68.8</v>
+      </c>
+    </row>
+    <row r="3854">
+      <c r="A3854" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3854" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3854" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3854" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3854" s="16" t="n">
+        <v>35.95</v>
+      </c>
+    </row>
+    <row r="3855">
+      <c r="A3855" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3855" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3855" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3855" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3855" s="19" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3856">
+      <c r="A3856" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3856" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3856" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3856" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3856" s="16" t="n">
+        <v>86.55</v>
+      </c>
+    </row>
+    <row r="3857">
+      <c r="A3857" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3857" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3857" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3857" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3857" s="19" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3858">
+      <c r="A3858" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3858" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3858" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3858" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3858" s="16" t="n">
+        <v>66.55</v>
+      </c>
+    </row>
+    <row r="3859">
+      <c r="A3859" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3859" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3859" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3859" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3859" s="19" t="n">
+        <v>59.7</v>
+      </c>
+    </row>
+    <row r="3860">
+      <c r="A3860" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3860" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3860" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3860" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3860" s="16" t="n">
+        <v>43.8</v>
+      </c>
+    </row>
+    <row r="3861">
+      <c r="A3861" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3861" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3861" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3861" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3861" s="19" t="n">
+        <v>69.8</v>
+      </c>
+    </row>
+    <row r="3862">
+      <c r="A3862" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3862" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3862" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3862" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3862" s="16" t="n">
+        <v>77.55</v>
+      </c>
+    </row>
+    <row r="3863">
+      <c r="A3863" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3863" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3863" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3863" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3863" s="19" t="n">
+        <v>56.65</v>
+      </c>
+    </row>
+    <row r="3864">
+      <c r="A3864" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3864" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3864" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3864" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3864" s="16" t="n">
+        <v>97.59999999999999</v>
+      </c>
+    </row>
+    <row r="3865">
+      <c r="A3865" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3865" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3865" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3865" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3865" s="19" t="n">
+        <v>148.9</v>
+      </c>
+    </row>
+    <row r="3866">
+      <c r="A3866" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3866" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3866" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3866" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3866" s="16" t="n">
+        <v>147.6</v>
+      </c>
+    </row>
+    <row r="3867">
+      <c r="A3867" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3867" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3867" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3867" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3867" s="19" t="n">
+        <v>61.35</v>
+      </c>
+    </row>
+    <row r="3868">
+      <c r="A3868" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3868" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3868" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3868" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3868" s="16" t="n">
+        <v>96.8</v>
+      </c>
+    </row>
+    <row r="3869">
+      <c r="A3869" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3869" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3869" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3869" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3869" s="19" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3870">
+      <c r="A3870" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3870" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3870" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3870" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3870" s="16" t="n">
+        <v>147.5</v>
+      </c>
+    </row>
+    <row r="3871">
+      <c r="A3871" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3871" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3871" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3871" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3871" s="19" t="n">
+        <v>60.85</v>
+      </c>
+    </row>
+    <row r="3872">
+      <c r="A3872" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3872" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3872" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3872" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3872" s="16" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3873">
+      <c r="A3873" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3873" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3873" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3873" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3873" s="19" t="n">
+        <v>145.9</v>
+      </c>
+    </row>
+    <row r="3874">
+      <c r="A3874" s="20" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3874" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3874" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3874" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3874" s="16" t="n">
+        <v>145.65</v>
+      </c>
+    </row>
+    <row r="3875">
+      <c r="A3875" s="21" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B3875" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3875" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3875" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3875" s="19" t="n">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-27
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3875"/>
+  <dimension ref="A1:E3919"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -89721,6 +89721,1018 @@
         <v>60</v>
       </c>
     </row>
+    <row r="3876">
+      <c r="A3876" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3876" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3876" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3876" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3876" s="16" t="n">
+        <v>41.5</v>
+      </c>
+    </row>
+    <row r="3877">
+      <c r="A3877" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3877" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3877" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3877" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3877" s="19" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3878">
+      <c r="A3878" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3878" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3878" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3878" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3878" s="16" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3879">
+      <c r="A3879" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3879" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3879" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3879" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3879" s="19" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3880">
+      <c r="A3880" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3880" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3880" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3880" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3880" s="16" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3881">
+      <c r="A3881" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3881" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3881" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3881" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3881" s="19" t="n">
+        <v>67.90000000000001</v>
+      </c>
+    </row>
+    <row r="3882">
+      <c r="A3882" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3882" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3882" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3882" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3882" s="16" t="n">
+        <v>54.05</v>
+      </c>
+    </row>
+    <row r="3883">
+      <c r="A3883" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3883" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3883" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3883" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3883" s="19" t="n">
+        <v>74.7</v>
+      </c>
+    </row>
+    <row r="3884">
+      <c r="A3884" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3884" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3884" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3884" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3884" s="16" t="n">
+        <v>88.05</v>
+      </c>
+    </row>
+    <row r="3885">
+      <c r="A3885" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3885" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3885" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3885" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3885" s="19" t="n">
+        <v>66.3</v>
+      </c>
+    </row>
+    <row r="3886">
+      <c r="A3886" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3886" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3886" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3886" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3886" s="16" t="n">
+        <v>118.5</v>
+      </c>
+    </row>
+    <row r="3887">
+      <c r="A3887" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3887" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3887" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3887" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3887" s="19" t="n">
+        <v>164.25</v>
+      </c>
+    </row>
+    <row r="3888">
+      <c r="A3888" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3888" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3888" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3888" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3888" s="16" t="n">
+        <v>163.6</v>
+      </c>
+    </row>
+    <row r="3889">
+      <c r="A3889" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3889" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3889" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3889" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3889" s="19" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="3890">
+      <c r="A3890" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3890" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3890" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3890" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3890" s="16" t="n">
+        <v>116.9</v>
+      </c>
+    </row>
+    <row r="3891">
+      <c r="A3891" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3891" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3891" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3891" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3891" s="19" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3892">
+      <c r="A3892" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3892" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3892" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3892" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3892" s="16" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3893">
+      <c r="A3893" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3893" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3893" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3893" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3893" s="19" t="n">
+        <v>71.34999999999999</v>
+      </c>
+    </row>
+    <row r="3894">
+      <c r="A3894" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3894" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3894" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3894" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3894" s="16" t="n">
+        <v>112.85</v>
+      </c>
+    </row>
+    <row r="3895">
+      <c r="A3895" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3895" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3895" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3895" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3895" s="19" t="n">
+        <v>161.05</v>
+      </c>
+    </row>
+    <row r="3896">
+      <c r="A3896" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3896" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3896" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3896" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3896" s="16" t="n">
+        <v>161.5</v>
+      </c>
+    </row>
+    <row r="3897">
+      <c r="A3897" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3897" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3897" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3897" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3897" s="19" t="n">
+        <v>68.8</v>
+      </c>
+    </row>
+    <row r="3898">
+      <c r="A3898" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3898" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3898" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3898" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3898" s="16" t="n">
+        <v>35.95</v>
+      </c>
+    </row>
+    <row r="3899">
+      <c r="A3899" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3899" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3899" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3899" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3899" s="19" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3900">
+      <c r="A3900" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3900" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3900" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3900" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3900" s="16" t="n">
+        <v>86.55</v>
+      </c>
+    </row>
+    <row r="3901">
+      <c r="A3901" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3901" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3901" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3901" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3901" s="19" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3902">
+      <c r="A3902" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3902" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3902" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3902" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3902" s="16" t="n">
+        <v>66.55</v>
+      </c>
+    </row>
+    <row r="3903">
+      <c r="A3903" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3903" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3903" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3903" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3903" s="19" t="n">
+        <v>59.7</v>
+      </c>
+    </row>
+    <row r="3904">
+      <c r="A3904" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3904" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3904" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3904" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3904" s="16" t="n">
+        <v>43.8</v>
+      </c>
+    </row>
+    <row r="3905">
+      <c r="A3905" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3905" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3905" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3905" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3905" s="19" t="n">
+        <v>69.8</v>
+      </c>
+    </row>
+    <row r="3906">
+      <c r="A3906" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3906" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3906" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3906" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3906" s="16" t="n">
+        <v>77.55</v>
+      </c>
+    </row>
+    <row r="3907">
+      <c r="A3907" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3907" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3907" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3907" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3907" s="19" t="n">
+        <v>56.65</v>
+      </c>
+    </row>
+    <row r="3908">
+      <c r="A3908" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3908" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3908" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3908" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3908" s="16" t="n">
+        <v>97.59999999999999</v>
+      </c>
+    </row>
+    <row r="3909">
+      <c r="A3909" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3909" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3909" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3909" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3909" s="19" t="n">
+        <v>148.9</v>
+      </c>
+    </row>
+    <row r="3910">
+      <c r="A3910" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3910" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3910" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3910" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3910" s="16" t="n">
+        <v>147.6</v>
+      </c>
+    </row>
+    <row r="3911">
+      <c r="A3911" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3911" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3911" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3911" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3911" s="19" t="n">
+        <v>61.35</v>
+      </c>
+    </row>
+    <row r="3912">
+      <c r="A3912" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3912" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3912" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3912" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3912" s="16" t="n">
+        <v>96.8</v>
+      </c>
+    </row>
+    <row r="3913">
+      <c r="A3913" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3913" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3913" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3913" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3913" s="19" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3914">
+      <c r="A3914" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3914" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3914" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3914" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3914" s="16" t="n">
+        <v>147.5</v>
+      </c>
+    </row>
+    <row r="3915">
+      <c r="A3915" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3915" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3915" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3915" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3915" s="19" t="n">
+        <v>60.85</v>
+      </c>
+    </row>
+    <row r="3916">
+      <c r="A3916" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3916" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3916" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3916" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3916" s="16" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3917">
+      <c r="A3917" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3917" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3917" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3917" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3917" s="19" t="n">
+        <v>145.9</v>
+      </c>
+    </row>
+    <row r="3918">
+      <c r="A3918" s="20" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3918" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3918" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3918" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3918" s="16" t="n">
+        <v>145.65</v>
+      </c>
+    </row>
+    <row r="3919">
+      <c r="A3919" s="21" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B3919" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3919" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3919" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3919" s="19" t="n">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-28
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3919"/>
+  <dimension ref="A1:E3963"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -90733,6 +90733,1018 @@
         <v>60</v>
       </c>
     </row>
+    <row r="3920">
+      <c r="A3920" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3920" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3920" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3920" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3920" s="16" t="n">
+        <v>41.5</v>
+      </c>
+    </row>
+    <row r="3921">
+      <c r="A3921" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3921" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3921" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3921" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3921" s="19" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3922">
+      <c r="A3922" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3922" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3922" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3922" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3922" s="16" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3923">
+      <c r="A3923" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3923" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3923" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3923" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3923" s="19" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3924">
+      <c r="A3924" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3924" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3924" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3924" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3924" s="16" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3925">
+      <c r="A3925" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3925" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3925" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3925" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3925" s="19" t="n">
+        <v>67.90000000000001</v>
+      </c>
+    </row>
+    <row r="3926">
+      <c r="A3926" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3926" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3926" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3926" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3926" s="16" t="n">
+        <v>54.05</v>
+      </c>
+    </row>
+    <row r="3927">
+      <c r="A3927" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3927" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3927" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3927" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3927" s="19" t="n">
+        <v>74.7</v>
+      </c>
+    </row>
+    <row r="3928">
+      <c r="A3928" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3928" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3928" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3928" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3928" s="16" t="n">
+        <v>88.05</v>
+      </c>
+    </row>
+    <row r="3929">
+      <c r="A3929" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3929" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3929" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3929" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3929" s="19" t="n">
+        <v>66.3</v>
+      </c>
+    </row>
+    <row r="3930">
+      <c r="A3930" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3930" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3930" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3930" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3930" s="16" t="n">
+        <v>118.5</v>
+      </c>
+    </row>
+    <row r="3931">
+      <c r="A3931" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3931" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3931" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3931" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3931" s="19" t="n">
+        <v>164.25</v>
+      </c>
+    </row>
+    <row r="3932">
+      <c r="A3932" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3932" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3932" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3932" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3932" s="16" t="n">
+        <v>163.6</v>
+      </c>
+    </row>
+    <row r="3933">
+      <c r="A3933" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3933" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3933" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3933" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3933" s="19" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="3934">
+      <c r="A3934" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3934" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3934" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3934" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3934" s="16" t="n">
+        <v>116.9</v>
+      </c>
+    </row>
+    <row r="3935">
+      <c r="A3935" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3935" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3935" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3935" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3935" s="19" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3936">
+      <c r="A3936" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3936" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3936" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3936" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3936" s="16" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3937">
+      <c r="A3937" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3937" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3937" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3937" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3937" s="19" t="n">
+        <v>71.34999999999999</v>
+      </c>
+    </row>
+    <row r="3938">
+      <c r="A3938" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3938" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3938" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3938" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3938" s="16" t="n">
+        <v>112.85</v>
+      </c>
+    </row>
+    <row r="3939">
+      <c r="A3939" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3939" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3939" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3939" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3939" s="19" t="n">
+        <v>161.05</v>
+      </c>
+    </row>
+    <row r="3940">
+      <c r="A3940" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3940" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3940" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3940" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3940" s="16" t="n">
+        <v>161.5</v>
+      </c>
+    </row>
+    <row r="3941">
+      <c r="A3941" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3941" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3941" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3941" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3941" s="19" t="n">
+        <v>68.8</v>
+      </c>
+    </row>
+    <row r="3942">
+      <c r="A3942" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3942" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3942" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3942" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3942" s="16" t="n">
+        <v>35.95</v>
+      </c>
+    </row>
+    <row r="3943">
+      <c r="A3943" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3943" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3943" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3943" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3943" s="19" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3944">
+      <c r="A3944" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3944" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3944" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3944" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3944" s="16" t="n">
+        <v>86.55</v>
+      </c>
+    </row>
+    <row r="3945">
+      <c r="A3945" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3945" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3945" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3945" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3945" s="19" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3946">
+      <c r="A3946" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3946" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3946" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3946" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3946" s="16" t="n">
+        <v>66.55</v>
+      </c>
+    </row>
+    <row r="3947">
+      <c r="A3947" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3947" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3947" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3947" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3947" s="19" t="n">
+        <v>59.7</v>
+      </c>
+    </row>
+    <row r="3948">
+      <c r="A3948" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3948" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3948" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3948" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3948" s="16" t="n">
+        <v>43.8</v>
+      </c>
+    </row>
+    <row r="3949">
+      <c r="A3949" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3949" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3949" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3949" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3949" s="19" t="n">
+        <v>69.8</v>
+      </c>
+    </row>
+    <row r="3950">
+      <c r="A3950" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3950" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3950" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3950" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3950" s="16" t="n">
+        <v>77.55</v>
+      </c>
+    </row>
+    <row r="3951">
+      <c r="A3951" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3951" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3951" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3951" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3951" s="19" t="n">
+        <v>56.65</v>
+      </c>
+    </row>
+    <row r="3952">
+      <c r="A3952" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3952" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3952" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3952" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3952" s="16" t="n">
+        <v>97.59999999999999</v>
+      </c>
+    </row>
+    <row r="3953">
+      <c r="A3953" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3953" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3953" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3953" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3953" s="19" t="n">
+        <v>148.9</v>
+      </c>
+    </row>
+    <row r="3954">
+      <c r="A3954" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3954" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3954" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3954" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3954" s="16" t="n">
+        <v>147.6</v>
+      </c>
+    </row>
+    <row r="3955">
+      <c r="A3955" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3955" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3955" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3955" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3955" s="19" t="n">
+        <v>61.35</v>
+      </c>
+    </row>
+    <row r="3956">
+      <c r="A3956" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3956" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3956" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3956" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3956" s="16" t="n">
+        <v>96.8</v>
+      </c>
+    </row>
+    <row r="3957">
+      <c r="A3957" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3957" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3957" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3957" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3957" s="19" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3958">
+      <c r="A3958" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3958" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3958" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3958" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3958" s="16" t="n">
+        <v>147.5</v>
+      </c>
+    </row>
+    <row r="3959">
+      <c r="A3959" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3959" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3959" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3959" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3959" s="19" t="n">
+        <v>60.85</v>
+      </c>
+    </row>
+    <row r="3960">
+      <c r="A3960" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3960" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3960" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3960" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3960" s="16" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3961">
+      <c r="A3961" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3961" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3961" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3961" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3961" s="19" t="n">
+        <v>145.9</v>
+      </c>
+    </row>
+    <row r="3962">
+      <c r="A3962" s="20" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3962" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3962" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3962" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3962" s="16" t="n">
+        <v>145.65</v>
+      </c>
+    </row>
+    <row r="3963">
+      <c r="A3963" s="21" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B3963" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3963" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3963" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3963" s="19" t="n">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-06-30
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3963"/>
+  <dimension ref="A1:E4007"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -91745,6 +91745,1018 @@
         <v>60</v>
       </c>
     </row>
+    <row r="3964">
+      <c r="A3964" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3964" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3964" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3964" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3964" s="16" t="n">
+        <v>41.4</v>
+      </c>
+    </row>
+    <row r="3965">
+      <c r="A3965" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3965" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3965" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3965" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3965" s="19" t="n">
+        <v>79.3</v>
+      </c>
+    </row>
+    <row r="3966">
+      <c r="A3966" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3966" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3966" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3966" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3966" s="16" t="n">
+        <v>92.3</v>
+      </c>
+    </row>
+    <row r="3967">
+      <c r="A3967" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3967" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3967" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3967" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3967" s="19" t="n">
+        <v>77.5</v>
+      </c>
+    </row>
+    <row r="3968">
+      <c r="A3968" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3968" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3968" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3968" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3968" s="16" t="n">
+        <v>72.09999999999999</v>
+      </c>
+    </row>
+    <row r="3969">
+      <c r="A3969" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3969" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3969" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3969" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3969" s="19" t="n">
+        <v>63.85</v>
+      </c>
+    </row>
+    <row r="3970">
+      <c r="A3970" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3970" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3970" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3970" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3970" s="16" t="n">
+        <v>50.85</v>
+      </c>
+    </row>
+    <row r="3971">
+      <c r="A3971" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3971" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3971" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3971" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3971" s="19" t="n">
+        <v>74.65000000000001</v>
+      </c>
+    </row>
+    <row r="3972">
+      <c r="A3972" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3972" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3972" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3972" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3972" s="16" t="n">
+        <v>83.09999999999999</v>
+      </c>
+    </row>
+    <row r="3973">
+      <c r="A3973" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3973" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3973" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3973" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3973" s="19" t="n">
+        <v>62.25</v>
+      </c>
+    </row>
+    <row r="3974">
+      <c r="A3974" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3974" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3974" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3974" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3974" s="16" t="n">
+        <v>116.4</v>
+      </c>
+    </row>
+    <row r="3975">
+      <c r="A3975" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3975" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3975" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3975" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3975" s="19" t="n">
+        <v>162.5</v>
+      </c>
+    </row>
+    <row r="3976">
+      <c r="A3976" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3976" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3976" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3976" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3976" s="16" t="n">
+        <v>164.15</v>
+      </c>
+    </row>
+    <row r="3977">
+      <c r="A3977" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3977" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3977" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3977" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3977" s="19" t="n">
+        <v>73.15000000000001</v>
+      </c>
+    </row>
+    <row r="3978">
+      <c r="A3978" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3978" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3978" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3978" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E3978" s="16" t="n">
+        <v>116.15</v>
+      </c>
+    </row>
+    <row r="3979">
+      <c r="A3979" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3979" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3979" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3979" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E3979" s="19" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3980">
+      <c r="A3980" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3980" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3980" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3980" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E3980" s="16" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3981">
+      <c r="A3981" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3981" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3981" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3981" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E3981" s="19" t="n">
+        <v>71.05</v>
+      </c>
+    </row>
+    <row r="3982">
+      <c r="A3982" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3982" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3982" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3982" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E3982" s="16" t="n">
+        <v>112.85</v>
+      </c>
+    </row>
+    <row r="3983">
+      <c r="A3983" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3983" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3983" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3983" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E3983" s="19" t="n">
+        <v>161.05</v>
+      </c>
+    </row>
+    <row r="3984">
+      <c r="A3984" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3984" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3984" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3984" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E3984" s="16" t="n">
+        <v>161.05</v>
+      </c>
+    </row>
+    <row r="3985">
+      <c r="A3985" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3985" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C3985" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3985" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E3985" s="19" t="n">
+        <v>68.8</v>
+      </c>
+    </row>
+    <row r="3986">
+      <c r="A3986" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3986" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3986" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3986" s="15" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="E3986" s="16" t="n">
+        <v>35.65</v>
+      </c>
+    </row>
+    <row r="3987">
+      <c r="A3987" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3987" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3987" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3987" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E3987" s="19" t="n">
+        <v>66.5</v>
+      </c>
+    </row>
+    <row r="3988">
+      <c r="A3988" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3988" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3988" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3988" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E3988" s="16" t="n">
+        <v>80.40000000000001</v>
+      </c>
+    </row>
+    <row r="3989">
+      <c r="A3989" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3989" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3989" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3989" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E3989" s="19" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3990">
+      <c r="A3990" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3990" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3990" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3990" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3990" s="16" t="n">
+        <v>61.5</v>
+      </c>
+    </row>
+    <row r="3991">
+      <c r="A3991" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3991" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3991" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3991" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E3991" s="19" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3992">
+      <c r="A3992" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3992" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3992" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D3992" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E3992" s="16" t="n">
+        <v>40.55</v>
+      </c>
+    </row>
+    <row r="3993">
+      <c r="A3993" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3993" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3993" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3993" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="E3993" s="19" t="n">
+        <v>69.7</v>
+      </c>
+    </row>
+    <row r="3994">
+      <c r="A3994" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3994" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3994" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3994" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E3994" s="16" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3995">
+      <c r="A3995" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3995" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3995" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3995" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E3995" s="19" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3996">
+      <c r="A3996" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3996" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3996" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3996" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E3996" s="16" t="n">
+        <v>95.84999999999999</v>
+      </c>
+    </row>
+    <row r="3997">
+      <c r="A3997" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3997" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3997" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3997" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E3997" s="19" t="n">
+        <v>148.5</v>
+      </c>
+    </row>
+    <row r="3998">
+      <c r="A3998" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3998" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3998" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3998" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E3998" s="16" t="n">
+        <v>148.5</v>
+      </c>
+    </row>
+    <row r="3999">
+      <c r="A3999" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B3999" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C3999" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D3999" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E3999" s="19" t="n">
+        <v>60.55</v>
+      </c>
+    </row>
+    <row r="4000">
+      <c r="A4000" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B4000" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4000" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4000" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E4000" s="16" t="n">
+        <v>94.8</v>
+      </c>
+    </row>
+    <row r="4001">
+      <c r="A4001" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B4001" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4001" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4001" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E4001" s="19" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4002">
+      <c r="A4002" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B4002" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4002" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4002" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E4002" s="16" t="n">
+        <v>147.5</v>
+      </c>
+    </row>
+    <row r="4003">
+      <c r="A4003" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B4003" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4003" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4003" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E4003" s="19" t="n">
+        <v>59.95</v>
+      </c>
+    </row>
+    <row r="4004">
+      <c r="A4004" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B4004" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4004" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4004" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E4004" s="16" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4005">
+      <c r="A4005" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B4005" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4005" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4005" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E4005" s="19" t="n">
+        <v>145.9</v>
+      </c>
+    </row>
+    <row r="4006">
+      <c r="A4006" s="20" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B4006" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4006" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4006" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E4006" s="16" t="n">
+        <v>145.65</v>
+      </c>
+    </row>
+    <row r="4007">
+      <c r="A4007" s="21" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B4007" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4007" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4007" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E4007" s="19" t="n">
+        <v>59.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-07-01
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4007"/>
+  <dimension ref="A1:E4053"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -92757,6 +92757,1064 @@
         <v>59.95</v>
       </c>
     </row>
+    <row r="4008">
+      <c r="A4008" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4008" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4008" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4008" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E4008" s="16" t="n">
+        <v>76.25</v>
+      </c>
+    </row>
+    <row r="4009">
+      <c r="A4009" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4009" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4009" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4009" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E4009" s="19" t="n">
+        <v>86.05</v>
+      </c>
+    </row>
+    <row r="4010">
+      <c r="A4010" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4010" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4010" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4010" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E4010" s="16" t="n">
+        <v>76.09999999999999</v>
+      </c>
+    </row>
+    <row r="4011">
+      <c r="A4011" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4011" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4011" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4011" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E4011" s="19" t="n">
+        <v>70.90000000000001</v>
+      </c>
+    </row>
+    <row r="4012">
+      <c r="A4012" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4012" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4012" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4012" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E4012" s="16" t="n">
+        <v>59.95</v>
+      </c>
+    </row>
+    <row r="4013">
+      <c r="A4013" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4013" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4013" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4013" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E4013" s="19" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4014">
+      <c r="A4014" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4014" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4014" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4014" s="15" t="inlineStr">
+        <is>
+          <t>Jan 2027</t>
+        </is>
+      </c>
+      <c r="E4014" s="16" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4015">
+      <c r="A4015" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4015" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4015" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4015" s="18" t="inlineStr">
+        <is>
+          <t>Feb 2027</t>
+        </is>
+      </c>
+      <c r="E4015" s="19" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4016">
+      <c r="A4016" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4016" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4016" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4016" s="15" t="inlineStr">
+        <is>
+          <t>Mar 2027</t>
+        </is>
+      </c>
+      <c r="E4016" s="16" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4017">
+      <c r="A4017" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4017" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4017" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4017" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E4017" s="19" t="n">
+        <v>79.5</v>
+      </c>
+    </row>
+    <row r="4018">
+      <c r="A4018" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4018" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4018" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4018" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E4018" s="16" t="n">
+        <v>58.6</v>
+      </c>
+    </row>
+    <row r="4019">
+      <c r="A4019" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4019" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4019" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4019" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E4019" s="19" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4020">
+      <c r="A4020" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4020" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4020" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4020" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E4020" s="16" t="n">
+        <v>167.35</v>
+      </c>
+    </row>
+    <row r="4021">
+      <c r="A4021" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4021" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4021" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4021" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E4021" s="19" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="4022">
+      <c r="A4022" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4022" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4022" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4022" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E4022" s="16" t="n">
+        <v>73.15000000000001</v>
+      </c>
+    </row>
+    <row r="4023">
+      <c r="A4023" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4023" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4023" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4023" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E4023" s="19" t="n">
+        <v>113.25</v>
+      </c>
+    </row>
+    <row r="4024">
+      <c r="A4024" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4024" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4024" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4024" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E4024" s="16" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4025">
+      <c r="A4025" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4025" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4025" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4025" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E4025" s="19" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4026">
+      <c r="A4026" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4026" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4026" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4026" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E4026" s="16" t="n">
+        <v>73.09999999999999</v>
+      </c>
+    </row>
+    <row r="4027">
+      <c r="A4027" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4027" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4027" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4027" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E4027" s="19" t="n">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4028">
+      <c r="A4028" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4028" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4028" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4028" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E4028" s="16" t="n">
+        <v>161.05</v>
+      </c>
+    </row>
+    <row r="4029">
+      <c r="A4029" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4029" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4029" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4029" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E4029" s="19" t="n">
+        <v>161.05</v>
+      </c>
+    </row>
+    <row r="4030">
+      <c r="A4030" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4030" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4030" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4030" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E4030" s="16" t="n">
+        <v>70.84999999999999</v>
+      </c>
+    </row>
+    <row r="4031">
+      <c r="A4031" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4031" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4031" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4031" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E4031" s="19" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4032">
+      <c r="A4032" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4032" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4032" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4032" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E4032" s="16" t="n">
+        <v>72.75</v>
+      </c>
+    </row>
+    <row r="4033">
+      <c r="A4033" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4033" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4033" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4033" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E4033" s="19" t="n">
+        <v>66.75</v>
+      </c>
+    </row>
+    <row r="4034">
+      <c r="A4034" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4034" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4034" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4034" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E4034" s="16" t="n">
+        <v>60.75</v>
+      </c>
+    </row>
+    <row r="4035">
+      <c r="A4035" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4035" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4035" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4035" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E4035" s="19" t="n">
+        <v>50.1</v>
+      </c>
+    </row>
+    <row r="4036">
+      <c r="A4036" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4036" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4036" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4036" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E4036" s="16" t="n">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="4037">
+      <c r="A4037" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4037" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4037" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4037" s="18" t="inlineStr">
+        <is>
+          <t>Jan 2027</t>
+        </is>
+      </c>
+      <c r="E4037" s="19" t="n">
+        <v>93.25</v>
+      </c>
+    </row>
+    <row r="4038">
+      <c r="A4038" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4038" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4038" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4038" s="15" t="inlineStr">
+        <is>
+          <t>Feb 2027</t>
+        </is>
+      </c>
+      <c r="E4038" s="16" t="n">
+        <v>93.25</v>
+      </c>
+    </row>
+    <row r="4039">
+      <c r="A4039" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4039" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4039" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4039" s="18" t="inlineStr">
+        <is>
+          <t>Mar 2027</t>
+        </is>
+      </c>
+      <c r="E4039" s="19" t="n">
+        <v>93.25</v>
+      </c>
+    </row>
+    <row r="4040">
+      <c r="A4040" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4040" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4040" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4040" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E4040" s="16" t="n">
+        <v>67.5</v>
+      </c>
+    </row>
+    <row r="4041">
+      <c r="A4041" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4041" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4041" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4041" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E4041" s="19" t="n">
+        <v>48.7</v>
+      </c>
+    </row>
+    <row r="4042">
+      <c r="A4042" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4042" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4042" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4042" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E4042" s="16" t="n">
+        <v>93.25</v>
+      </c>
+    </row>
+    <row r="4043">
+      <c r="A4043" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4043" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4043" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4043" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E4043" s="19" t="n">
+        <v>150.3</v>
+      </c>
+    </row>
+    <row r="4044">
+      <c r="A4044" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4044" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4044" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4044" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E4044" s="16" t="n">
+        <v>150.35</v>
+      </c>
+    </row>
+    <row r="4045">
+      <c r="A4045" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4045" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4045" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4045" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E4045" s="19" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4046">
+      <c r="A4046" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4046" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4046" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4046" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E4046" s="16" t="n">
+        <v>93.75</v>
+      </c>
+    </row>
+    <row r="4047">
+      <c r="A4047" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4047" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4047" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4047" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E4047" s="19" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4048">
+      <c r="A4048" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4048" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4048" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4048" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E4048" s="16" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4049">
+      <c r="A4049" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4049" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4049" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4049" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E4049" s="19" t="n">
+        <v>61.85</v>
+      </c>
+    </row>
+    <row r="4050">
+      <c r="A4050" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4050" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4050" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4050" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E4050" s="16" t="n">
+        <v>90.65000000000001</v>
+      </c>
+    </row>
+    <row r="4051">
+      <c r="A4051" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4051" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4051" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4051" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E4051" s="19" t="n">
+        <v>145.9</v>
+      </c>
+    </row>
+    <row r="4052">
+      <c r="A4052" s="20" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4052" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4052" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4052" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E4052" s="16" t="n">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4053">
+      <c r="A4053" s="21" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4053" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4053" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4053" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E4053" s="19" t="n">
+        <v>61.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-07-02
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4053"/>
+  <dimension ref="A1:E4099"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -93815,6 +93815,1064 @@
         <v>61.4</v>
       </c>
     </row>
+    <row r="4054">
+      <c r="A4054" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4054" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4054" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4054" s="15" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E4054" s="16" t="n">
+        <v>72.90000000000001</v>
+      </c>
+    </row>
+    <row r="4055">
+      <c r="A4055" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4055" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4055" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4055" s="18" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E4055" s="19" t="n">
+        <v>83.05</v>
+      </c>
+    </row>
+    <row r="4056">
+      <c r="A4056" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4056" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4056" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4056" s="15" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E4056" s="16" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4057">
+      <c r="A4057" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4057" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4057" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4057" s="18" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E4057" s="19" t="n">
+        <v>68.25</v>
+      </c>
+    </row>
+    <row r="4058">
+      <c r="A4058" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4058" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4058" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4058" s="15" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E4058" s="16" t="n">
+        <v>58.95</v>
+      </c>
+    </row>
+    <row r="4059">
+      <c r="A4059" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4059" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4059" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4059" s="18" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E4059" s="19" t="n">
+        <v>43.15</v>
+      </c>
+    </row>
+    <row r="4060">
+      <c r="A4060" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4060" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4060" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4060" s="15" t="inlineStr">
+        <is>
+          <t>Jan 2027</t>
+        </is>
+      </c>
+      <c r="E4060" s="16" t="n">
+        <v>78.75</v>
+      </c>
+    </row>
+    <row r="4061">
+      <c r="A4061" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4061" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4061" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4061" s="18" t="inlineStr">
+        <is>
+          <t>Feb 2027</t>
+        </is>
+      </c>
+      <c r="E4061" s="19" t="n">
+        <v>122.95</v>
+      </c>
+    </row>
+    <row r="4062">
+      <c r="A4062" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4062" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4062" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4062" s="15" t="inlineStr">
+        <is>
+          <t>Mar 2027</t>
+        </is>
+      </c>
+      <c r="E4062" s="16" t="n">
+        <v>133.75</v>
+      </c>
+    </row>
+    <row r="4063">
+      <c r="A4063" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4063" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4063" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4063" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E4063" s="19" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4064">
+      <c r="A4064" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4064" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4064" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4064" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E4064" s="16" t="n">
+        <v>56.75</v>
+      </c>
+    </row>
+    <row r="4065">
+      <c r="A4065" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4065" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4065" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4065" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E4065" s="19" t="n">
+        <v>111.45</v>
+      </c>
+    </row>
+    <row r="4066">
+      <c r="A4066" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4066" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4066" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4066" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E4066" s="16" t="n">
+        <v>166.5</v>
+      </c>
+    </row>
+    <row r="4067">
+      <c r="A4067" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4067" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4067" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4067" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E4067" s="19" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="4068">
+      <c r="A4068" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4068" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4068" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4068" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E4068" s="16" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4069">
+      <c r="A4069" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4069" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4069" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4069" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E4069" s="19" t="n">
+        <v>112.65</v>
+      </c>
+    </row>
+    <row r="4070">
+      <c r="A4070" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4070" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4070" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4070" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E4070" s="16" t="n">
+        <v>163.75</v>
+      </c>
+    </row>
+    <row r="4071">
+      <c r="A4071" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4071" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4071" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4071" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E4071" s="19" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4072">
+      <c r="A4072" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4072" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4072" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4072" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E4072" s="16" t="n">
+        <v>73.09999999999999</v>
+      </c>
+    </row>
+    <row r="4073">
+      <c r="A4073" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4073" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4073" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4073" s="18" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E4073" s="19" t="n">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="4074">
+      <c r="A4074" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4074" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4074" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4074" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E4074" s="16" t="n">
+        <v>161.75</v>
+      </c>
+    </row>
+    <row r="4075">
+      <c r="A4075" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4075" s="18" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4075" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4075" s="18" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E4075" s="19" t="n">
+        <v>161.7</v>
+      </c>
+    </row>
+    <row r="4076">
+      <c r="A4076" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4076" s="15" t="inlineStr">
+        <is>
+          <t>OTA2201</t>
+        </is>
+      </c>
+      <c r="C4076" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4076" s="15" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E4076" s="16" t="n">
+        <v>71.15000000000001</v>
+      </c>
+    </row>
+    <row r="4077">
+      <c r="A4077" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4077" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4077" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4077" s="18" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="E4077" s="19" t="n">
+        <v>60.4</v>
+      </c>
+    </row>
+    <row r="4078">
+      <c r="A4078" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4078" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4078" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4078" s="15" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="E4078" s="16" t="n">
+        <v>68.5</v>
+      </c>
+    </row>
+    <row r="4079">
+      <c r="A4079" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4079" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4079" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4079" s="18" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="E4079" s="19" t="n">
+        <v>65.05</v>
+      </c>
+    </row>
+    <row r="4080">
+      <c r="A4080" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4080" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4080" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4080" s="15" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="E4080" s="16" t="n">
+        <v>60.25</v>
+      </c>
+    </row>
+    <row r="4081">
+      <c r="A4081" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4081" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4081" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4081" s="18" t="inlineStr">
+        <is>
+          <t>Nov 2026</t>
+        </is>
+      </c>
+      <c r="E4081" s="19" t="n">
+        <v>49.65</v>
+      </c>
+    </row>
+    <row r="4082">
+      <c r="A4082" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4082" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4082" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4082" s="15" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="E4082" s="16" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4083">
+      <c r="A4083" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4083" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4083" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4083" s="18" t="inlineStr">
+        <is>
+          <t>Jan 2027</t>
+        </is>
+      </c>
+      <c r="E4083" s="19" t="n">
+        <v>66.84999999999999</v>
+      </c>
+    </row>
+    <row r="4084">
+      <c r="A4084" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4084" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4084" s="15" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4084" s="15" t="inlineStr">
+        <is>
+          <t>Feb 2027</t>
+        </is>
+      </c>
+      <c r="E4084" s="16" t="n">
+        <v>94.09999999999999</v>
+      </c>
+    </row>
+    <row r="4085">
+      <c r="A4085" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4085" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4085" s="18" t="inlineStr">
+        <is>
+          <t>Base Month</t>
+        </is>
+      </c>
+      <c r="D4085" s="18" t="inlineStr">
+        <is>
+          <t>Mar 2027</t>
+        </is>
+      </c>
+      <c r="E4085" s="19" t="n">
+        <v>111.05</v>
+      </c>
+    </row>
+    <row r="4086">
+      <c r="A4086" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4086" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4086" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4086" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E4086" s="16" t="n">
+        <v>64.65000000000001</v>
+      </c>
+    </row>
+    <row r="4087">
+      <c r="A4087" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4087" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4087" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4087" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E4087" s="19" t="n">
+        <v>48.3</v>
+      </c>
+    </row>
+    <row r="4088">
+      <c r="A4088" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4088" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4088" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4088" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E4088" s="16" t="n">
+        <v>90.55</v>
+      </c>
+    </row>
+    <row r="4089">
+      <c r="A4089" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4089" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4089" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4089" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="E4089" s="19" t="n">
+        <v>150.3</v>
+      </c>
+    </row>
+    <row r="4090">
+      <c r="A4090" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4090" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4090" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4090" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E4090" s="16" t="n">
+        <v>150.35</v>
+      </c>
+    </row>
+    <row r="4091">
+      <c r="A4091" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4091" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4091" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4091" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2027</t>
+        </is>
+      </c>
+      <c r="E4091" s="19" t="n">
+        <v>63.25</v>
+      </c>
+    </row>
+    <row r="4092">
+      <c r="A4092" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4092" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4092" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4092" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2028</t>
+        </is>
+      </c>
+      <c r="E4092" s="16" t="n">
+        <v>92.25</v>
+      </c>
+    </row>
+    <row r="4093">
+      <c r="A4093" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4093" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4093" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4093" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E4093" s="19" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4094">
+      <c r="A4094" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4094" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4094" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4094" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="E4094" s="16" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4095">
+      <c r="A4095" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4095" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4095" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4095" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="E4095" s="19" t="n">
+        <v>61.95</v>
+      </c>
+    </row>
+    <row r="4096">
+      <c r="A4096" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4096" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4096" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4096" s="15" t="inlineStr">
+        <is>
+          <t>Q1 2029</t>
+        </is>
+      </c>
+      <c r="E4096" s="16" t="n">
+        <v>89.34999999999999</v>
+      </c>
+    </row>
+    <row r="4097">
+      <c r="A4097" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4097" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4097" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4097" s="18" t="inlineStr">
+        <is>
+          <t>Q2 2029</t>
+        </is>
+      </c>
+      <c r="E4097" s="19" t="n">
+        <v>145.9</v>
+      </c>
+    </row>
+    <row r="4098">
+      <c r="A4098" s="20" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4098" s="15" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4098" s="15" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4098" s="15" t="inlineStr">
+        <is>
+          <t>Q3 2029</t>
+        </is>
+      </c>
+      <c r="E4098" s="16" t="n">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4099">
+      <c r="A4099" s="21" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B4099" s="18" t="inlineStr">
+        <is>
+          <t>BEN2201</t>
+        </is>
+      </c>
+      <c r="C4099" s="18" t="inlineStr">
+        <is>
+          <t>Base Quarter</t>
+        </is>
+      </c>
+      <c r="D4099" s="18" t="inlineStr">
+        <is>
+          <t>Q4 2029</t>
+        </is>
+      </c>
+      <c r="E4099" s="19" t="n">
+        <v>60.45</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily scrape 2026-07-03
</commit_message>
<xml_diff>
--- a/asx_nz_futures.xlsx
+++ b/asx_nz_futures.xlsx
@@ -583,